<commit_message>
feat: Add Top 10 analyst report PDFs with 5-metric credibility scoring, monthly subfolder sync, and Sunday weekly briefing
</commit_message>
<xml_diff>
--- a/reports/일자별_누적_데일리_이슈_및_주식_브리핑_마스터.xlsx
+++ b/reports/일자별_누적_데일리_이슈_및_주식_브리핑_마스터.xlsx
@@ -11,6 +11,7 @@
     <sheet name="주식추천_누적" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="시장지표_누적" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="코인추천_누적" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="공식리포트_누적" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -455,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G182"/>
+  <dimension ref="A1:G111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -463,7 +464,7 @@
     <col width="32" customWidth="1" min="3" max="3"/>
     <col width="65" customWidth="1" min="4" max="4"/>
     <col width="65" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
     <col width="53" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -3626,27 +3627,27 @@
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>🔥 [언론사 집중 보도 (4개사)]</t>
+          <t>신규 이슈</t>
         </is>
       </c>
       <c r="D86" s="3" t="inlineStr">
         <is>
-          <t>김지용 중수청장 후보자 오늘 청문회…‘친윤 논란·개혁 적합성’ 시험대</t>
+          <t>태안군, 12월부터 참전명예수당 월 30만원→50만원</t>
         </is>
       </c>
       <c r="E86" s="3" t="inlineStr">
         <is>
-          <t>김지용 중수청장 후보자 오늘 청문회…‘친윤 논란·개혁 적합성’ 시험대  한겨레‘친윤’ 딱지에 임은정 감찰까지…김지용, 중수청장 문턱서 여권 시험대  매일경제김민석, '김지용 비판' 추미애에 "자기 역할에 집중해야"  연합뉴스靑이 해야 할 말, 하지 말아야 할 말[오늘과 내일/장원재]  ...</t>
+          <t>(태안=연합뉴스) 정윤덕 기자 = 충남 태안군은 현재 월 30만원인 참전명예수당을 오는 12월부터 50만원으로 인상할 계획이라고 14일 밝혔다.</t>
         </is>
       </c>
       <c r="F86" s="3" t="inlineStr">
         <is>
-          <t>한겨레</t>
+          <t>주요언론</t>
         </is>
       </c>
       <c r="G86" s="3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMickFVX3lxTE5oYjdZdVl0MTNLWE1zWVI3QWw3aVpjNlpkaklQV2dYVUMwOUFkTXVycmRFNFN1Xy1pSFFDYUZzR3pPamxzUzMwYkQtWW5FRVllOWg0SkQ3TTluWmN4TWdBVFhRdGQxbUVWRzR5YXNTN2YtZw?oc=5</t>
+          <t>https://www.yna.co.kr/view/AKR20261014058000063</t>
         </is>
       </c>
     </row>
@@ -3668,22 +3669,22 @@
       </c>
       <c r="D87" s="3" t="inlineStr">
         <is>
-          <t>첫발 뗀 '북극항로' 개척…사업성 확보가 최대 관건</t>
+          <t>與, 野주진우·이진숙·김태규 직격…"패륜으로 인지도 올리나"</t>
         </is>
       </c>
       <c r="E87" s="3" t="inlineStr">
         <is>
-          <t>첫발 뗀 '북극항로' 개척…사업성 확보가 최대 관건  한국경제[대통령 이재명 말모이] 대한민국의 북극항로 항해일지는 이제 첫 장을 열게 됩니다 - 카드/한컷 | 멀티미디어  정책브리핑이 대통령 “국제사회 신뢰 속 북극항로 열어갈 것…해양강국 대한민국”  KBS 뉴스북극항로 부산 허브화 ...</t>
+          <t>(서울=연합뉴스) 최주성 기자 = 더불어민주당은 14일 국민의힘 주진우·이진숙·김태규 의원의 국정감사 기간 중 발언을 놓고 "막말 정치인 양성소...</t>
         </is>
       </c>
       <c r="F87" s="3" t="inlineStr">
         <is>
-          <t>한국경제</t>
+          <t>주요언론</t>
         </is>
       </c>
       <c r="G87" s="3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTE82ZDF3clBYNzVHVFA3NUd4NTRGUnpPSXVoZ1AwTFhPVUdMSGZGeDdDbzBOaTZSeHhVVkEzTHpMVjUzMWxZR3BwcWMxa09hZXBnUWgxQV9Qbm5aZw?oc=5</t>
+          <t>https://www.yna.co.kr/view/AKR20261014062800001</t>
         </is>
       </c>
     </row>
@@ -3695,32 +3696,32 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>정치</t>
+          <t>사회/사건사고</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>신규 이슈</t>
+          <t>🔥 [언론사 집중 보도 (4개사)]</t>
         </is>
       </c>
       <c r="D88" s="3" t="inlineStr">
         <is>
-          <t>국감서 배제된 이진숙… '尹정부 방통위원장 출신' 이해충돌 공방</t>
+          <t>주미대사관 “강경화 ‘불의의 사고 아니다’ 발언, 이 대통령 반박 아냐”</t>
         </is>
       </c>
       <c r="E88" s="3" t="inlineStr">
         <is>
-          <t>국감서 배제된 이진숙… '尹정부 방통위원장 출신' 이해충돌 공방  한국일보“투쟁 선봉” “선 넘는다” 이진숙·주진우에 국힘서도 이견  경향신문‘사상 초유’ 발언권 2명 정지·위원 제척까지…국감서 위원장 칼 휘두르는 與  서울경제국힘 "與, 억지 프레임 씌워 이진숙 제척…내로남불·의회폭거...</t>
+          <t>주미대사관 “강경화 ‘불의의 사고 아니다’ 발언, 이 대통령 반박 아냐”  한겨레"불의의 사고 아니다" 강경화 발언 수습에… 한동훈 "국민이 우습나"  조선일보‘북 DMZ 지뢰’ 대처 공방…“안보리 차원 대응 검토 중”  KBS 뉴스[연합뉴스 이 시각 헤드라인] - 07:30  연합뉴스...</t>
         </is>
       </c>
       <c r="F88" s="3" t="inlineStr">
         <is>
-          <t>한국일보</t>
+          <t>한겨레</t>
         </is>
       </c>
       <c r="G88" s="3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMibkFVX3lxTE9kYVNBRVlPNnliZTREaWdUT3doR0lrWVRTUlVHbmNJT1R5ZEpjS3VIazFrYWpPRkwyZlNiVkFCRlE0MUNYd1pSdVQ3MGdpLUQ4dGxsSkxINzV5bUZnaE9RMndMTE1nNU9IcmFIbUJR0gFzQVVfeXFMTV9ybWJfNmZzNDRBNmlyVkZIVnRUd1JzNGVqcV9TMDJoVjhCTHdOT2lEZjRjTlN1VzZRaWdrU2FyMWRwNjgwUVVBbUM0R2Y3RlV3NFNoMmZpdXdQNnI2MElnb2dBcjdTcUdQQ2FWWFY1RkJiQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMia0FVX3lxTFBvaWlRcEhkSXFzQU56OW1VOEFZdjFYZGh1akJIVUkwOFE4Y2NweUVpaVVxQjhSaGd2bG9FZzZKSExzTU8zY0FocWZTS3diZHZlSGxBaW9TazZ2b1RtWXBhS09tYzRsTHFMNVBR?oc=5</t>
         </is>
       </c>
     </row>
@@ -3732,7 +3733,7 @@
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>정치</t>
+          <t>사회/사건사고</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
@@ -3742,12 +3743,12 @@
       </c>
       <c r="D89" s="3" t="inlineStr">
         <is>
-          <t>지난해 아파트 관리비 최고는 나인원 한남…"월 평균 170만원"</t>
+          <t>경남도, 육상풍력 7개단지 48기 전수 점검…위험요인 사전 확인</t>
         </is>
       </c>
       <c r="E89" s="3" t="inlineStr">
         <is>
-          <t>(서울=연합뉴스) 노선웅 기자 = 지난해 전국 아파트 가운데 서울 용산구 '나인원 한남'의 세대당 월평균 관리비가 월평균 170만1천847원으로...</t>
+          <t>(창원=연합뉴스) 김선경 기자 = 경남도는 오는 30일까지 도내 육상풍력 발전단지 7곳을 전수 점검한다고 14일 밝혔다.</t>
         </is>
       </c>
       <c r="F89" s="3" t="inlineStr">
@@ -3757,7 +3758,7 @@
       </c>
       <c r="G89" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261014047900001</t>
+          <t>https://www.yna.co.kr/view/AKR20261014066600052</t>
         </is>
       </c>
     </row>
@@ -3769,22 +3770,22 @@
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>정치</t>
+          <t>사회/사건사고</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>🔥 [언론사 집중 보도 (3개사)]</t>
+          <t>신규 이슈</t>
         </is>
       </c>
       <c r="D90" s="3" t="inlineStr">
         <is>
-          <t>한병도 "중수청, 리더십 절실…김지용, 소신·비전 제시해달라"</t>
+          <t>세종시-홍익대, 청년 창업·실험실 '금남대평시장 리빙랩' 운영</t>
         </is>
       </c>
       <c r="E90" s="3" t="inlineStr">
         <is>
-          <t>(서울=연합뉴스) 박경준 안정훈 기자 = 더불어민주당 한병도 원내대표는 주진우 의원이 SNS에 '이재 명을 끊을 때'라는 댓글을 적는 등 국민의...</t>
+          <t>(세종=연합뉴스) 양영석 기자 = 세종시와 홍익대학교 세종캠퍼스는 청년 창업·실험 공간인 '금남대평시장 가치회복 리빙랩'을 운영한다고 14일 밝...</t>
         </is>
       </c>
       <c r="F90" s="3" t="inlineStr">
@@ -3794,7 +3795,7 @@
       </c>
       <c r="G90" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261014044800001</t>
+          <t>https://www.yna.co.kr/view/AKR20261014068900063</t>
         </is>
       </c>
     </row>
@@ -3806,7 +3807,7 @@
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>정치</t>
+          <t>사회/사건사고</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
@@ -3816,12 +3817,12 @@
       </c>
       <c r="D91" s="3" t="inlineStr">
         <is>
-          <t>주진우, 2026 여수 세계섬박람회 국민감사 청구</t>
+          <t>AI 전환부터 수출까지…산업부·식약처, 바이오산업 전주기 협력</t>
         </is>
       </c>
       <c r="E91" s="3" t="inlineStr">
         <is>
-          <t>(여수=연합뉴스) 손상원 기자 = 국민의힘 주진우 의원이 부실 지적을 받아온 2026 여수 세계섬박람회에 대한 국민감사를 청구한다.</t>
+          <t>(서울=연합뉴스) 장보인 기자 = 바이오산업 육성을 담당하는 산업통상부와 의약품·의료기기 규제를 책임지는 식품의약품안전처가 바이오산업 전 주기에...</t>
         </is>
       </c>
       <c r="F91" s="3" t="inlineStr">
@@ -3831,7 +3832,7 @@
       </c>
       <c r="G91" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261014048400054</t>
+          <t>https://www.yna.co.kr/view/AKR20261014025800003</t>
         </is>
       </c>
     </row>
@@ -3843,7 +3844,7 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>정치</t>
+          <t>사회/사건사고</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
@@ -3853,12 +3854,12 @@
       </c>
       <c r="D92" s="3" t="inlineStr">
         <is>
-          <t>어기구 "가습기살균제 피해 재심사 결과 받는 데 최장 4년 반"</t>
+          <t>강원 고성군, 재난 안전상황실 전담 인력 배치…내달 본격 운영</t>
         </is>
       </c>
       <c r="E92" s="3" t="inlineStr">
         <is>
-          <t>(당진=연합뉴스) 정윤덕 기자 = 가습기살균제 피해 재심사를 신청한 뒤 결과를 받기까지 길게는 4년 반이 걸린 것으로 나타났다.</t>
+          <t>(강원 고성=연합뉴스) 류호준 기자 = 강원 고성군은 기후 변화와 각종 재난 사고에 신속하게 대응하기 위해 다음 달부터 재난 안전상황실 전담 운...</t>
         </is>
       </c>
       <c r="F92" s="3" t="inlineStr">
@@ -3868,7 +3869,7 @@
       </c>
       <c r="G92" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261014044600063</t>
+          <t>https://www.yna.co.kr/view/AKR20261014066400062</t>
         </is>
       </c>
     </row>
@@ -3880,22 +3881,22 @@
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>정치</t>
+          <t>사회/사건사고</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>🔥 [언론사 집중 보도 (3개사)]</t>
+          <t>신규 이슈</t>
         </is>
       </c>
       <c r="D93" s="3" t="inlineStr">
         <is>
-          <t>전작권 조건충족 이견 속…한미 국방장관 이달말 첫 대면 가능성</t>
+          <t>설악권 현안 두고 머리 맞댄 속초시·고성군 의회…"상생 협력"</t>
         </is>
       </c>
       <c r="E93" s="3" t="inlineStr">
         <is>
-          <t>(서울=연합뉴스) 김효정 기자 = 전시작전통제권(전작권) 전환 조건 충족 여부를 두고 한미가 이견을 보이는 가운데 이달 말 국제회의를 계기로 강...</t>
+          <t>(속초=연합뉴스) 류호준 기자 = 강원 속초시의회와 고성군의회 의장이 만나 울산바위 인근 공동주택 개발 문제 등 설악권 주요 현안과 관련해 지역...</t>
         </is>
       </c>
       <c r="F93" s="3" t="inlineStr">
@@ -3905,7 +3906,7 @@
       </c>
       <c r="G93" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261014039900504</t>
+          <t>https://www.yna.co.kr/view/AKR20261014065100062</t>
         </is>
       </c>
     </row>
@@ -3917,7 +3918,7 @@
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>정치</t>
+          <t>사회/사건사고</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
@@ -3927,12 +3928,12 @@
       </c>
       <c r="D94" s="3" t="inlineStr">
         <is>
-          <t>조의장, 그리스서 경제협력 간담회…방산·첨단산업 세일즈외교</t>
+          <t>AI로 '옥외영업 인허가' 판단…고양시, 직원 아이디어 특허</t>
         </is>
       </c>
       <c r="E94" s="3" t="inlineStr">
         <is>
-          <t>(아테네=연합뉴스) 오규진 기자 = 그리스를 공식 방문 중인 조정식 국회의장은 13일(현지시간) 그리스 의원들과 경제협력 오찬 간담회를 열어 방...</t>
+          <t>(고양=연합뉴스) 노승혁 기자 = 경기 고양시는 현장 공무원이 직접 고안한 '인공지능(AI) 기반 옥외영업 가능 대상 자동 판단 및 인허가 검증...</t>
         </is>
       </c>
       <c r="F94" s="3" t="inlineStr">
@@ -3942,7 +3943,7 @@
       </c>
       <c r="G94" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261013189300001</t>
+          <t>https://www.yna.co.kr/view/AKR20261014064100060</t>
         </is>
       </c>
     </row>
@@ -3954,7 +3955,7 @@
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>정치</t>
+          <t>사회/사건사고</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
@@ -3964,12 +3965,12 @@
       </c>
       <c r="D95" s="3" t="inlineStr">
         <is>
-          <t>김민석 "曺 헌법훼손 차고 넘쳐…잘못 바로잡는 모든 방안 검토"</t>
+          <t>AI 코딩부터 데이터 활용까지…'AI 체험 축제' 열린다</t>
         </is>
       </c>
       <c r="E95" s="3" t="inlineStr">
         <is>
-          <t>(서울=연합뉴스) 김남권 안정훈 기자 = 더불어민주당 김민석 대표는 14일 조희대 대법원장의 대법관 후보자 재제청 거부와 대법관 격려금 지급 논...</t>
+          <t>(서울=연합뉴스) 권하영 기자 = 전 국민이 참여할 수 있는 인공지능(AI) 체험의 장이 열린다.</t>
         </is>
       </c>
       <c r="F95" s="3" t="inlineStr">
@@ -3979,7 +3980,7 @@
       </c>
       <c r="G95" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261014044000001</t>
+          <t>https://www.yna.co.kr/view/AKR20261014065400017</t>
         </is>
       </c>
     </row>
@@ -3991,22 +3992,22 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>정치</t>
+          <t>사회/사건사고</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>연결 이슈 (후속)</t>
+          <t>신규 이슈</t>
         </is>
       </c>
       <c r="D96" s="3" t="inlineStr">
         <is>
-          <t>"농진청, '57만명 개인정보 유출' 제재받은 업체와 재계약"</t>
+          <t>김해진영단감축제 30일 개막…사흘간 공연·체험 행사 풍성</t>
         </is>
       </c>
       <c r="E96" s="3" t="inlineStr">
         <is>
-          <t>(서울=연합뉴스) 노선웅 기자 = 농촌진흥청이 농민 57만여명의 개인정보 유출 사고에 책임이 있는 업체와 별도의 보안 강화 조치 없이 계약을 유...</t>
+          <t>(김해=연합뉴스) 이준영 기자 = 경남 김해시는 오는 30일부터 내달 1일까지 진영운동장 일원에서 '제42회 김해진영단감축제'를 개최한다고 14...</t>
         </is>
       </c>
       <c r="F96" s="3" t="inlineStr">
@@ -4016,7 +4017,7 @@
       </c>
       <c r="G96" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261014035700001</t>
+          <t>https://www.yna.co.kr/view/AKR20261014065600052</t>
         </is>
       </c>
     </row>
@@ -4033,27 +4034,27 @@
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>연결 이슈 (후속)</t>
+          <t>신규 이슈</t>
         </is>
       </c>
       <c r="D97" s="3" t="inlineStr">
         <is>
-          <t>유엔 국감장서도 北 지뢰 논쟁… 野 “유엔대표부 할 일 하고 있나” 공세</t>
+          <t>목포해경, 안전사고 위험 '주의보' 발령</t>
         </is>
       </c>
       <c r="E97" s="3" t="inlineStr">
         <is>
-          <t>유엔 국감장서도 北 지뢰 논쟁… 野 “유엔대표부 할 일 하고 있나” 공세  동아일보‘불의의 사고’ 아니란 강경화 대사 발언 해명 나선 주미 대사관···“기존 표현 맞는지와 무관”  경향신문‘북 DMZ 지뢰’ 대처 공방…“안보리 차원 대응 검토 중”  KBS 뉴스[연합뉴스 이 시각 헤드라...</t>
+          <t>(목포=연합뉴스) 조근영 기자 = 목포해양경찰서는 14일 목포·신안·무안·진도 등 전남광주 8개 시·군 지역에 안전사고 위험예보제 '주의보' 단...</t>
         </is>
       </c>
       <c r="F97" s="3" t="inlineStr">
         <is>
-          <t>동아일보</t>
+          <t>주요언론</t>
         </is>
       </c>
       <c r="G97" s="3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMic0FVX3lxTE00bXFtc1dxeWdEWG9yY0o1WWVYeUNqUVZhc0Q2djhFT1pfdEtaaUdIemQyQWJnMkdfVTZwNDFULV9jYWszR2FuT0EwVjU3dWZJWUdoMFZMVFVuOE5sQ2NsREpqMDE3ek9aT29UaDUxNWxJOXfSAWZBVV95cUxOdktGVFlUOGNCOXhINTh2YWVEQ3k0RDFERDlJbVFVNmdGTTVTaHNPaGxQY0h4a3F2RE85eGN4VzltZDI2a2lYenNsbFh0YldmS2VNUENXNnJHVWdnZlA3cVpIWDhtN1E?oc=5</t>
+          <t>https://www.yna.co.kr/view/AKR20261014065700054</t>
         </is>
       </c>
     </row>
@@ -4075,22 +4076,22 @@
       </c>
       <c r="D98" s="3" t="inlineStr">
         <is>
-          <t>마라톤 결승선 앞두고 숨진 카이스트 대학원생…SNS 추모 물결</t>
+          <t>거래소·배출권시장協, 배출권거래제 정책·산업계 대응 논의</t>
         </is>
       </c>
       <c r="E98" s="3" t="inlineStr">
         <is>
-          <t>마라톤 결승선 앞두고 숨진 카이스트 대학원생…SNS 추모 물결  한국경제'서울 달리기' 마라톤대회 참가했던 20대 여성 사망  연합뉴스황영조 “사망에 이르는 러닝” 경고···SNS 과시형 기록 문화도 지적  경향신문“SNS 인증샷 찍다 죽습니다”…마라톤 기록 경쟁 과열에 황영조 당부 -...</t>
+          <t>(서울=연합뉴스) 임은진 기자 = 한국거래소는 14일 오후 서울 사옥에서 배출권시장협의회와 함께 '2026년 하반기 자문위원회 세미나'를 연다.</t>
         </is>
       </c>
       <c r="F98" s="3" t="inlineStr">
         <is>
-          <t>한국경제</t>
+          <t>주요언론</t>
         </is>
       </c>
       <c r="G98" s="3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTE1nRG1XbzVKbGFySjZMU1FFZ1FHOHNKYjVQNk1nbGdVeE1WYnhXWTdZNGVORlFMMnp1YVppbTZXVDVOY2JJTG96MjhrVkhVN0ZGMmVqUWZOZ05jUQ?oc=5</t>
+          <t>https://www.yna.co.kr/view/AKR20261014066900008</t>
         </is>
       </c>
     </row>
@@ -4112,22 +4113,22 @@
       </c>
       <c r="D99" s="3" t="inlineStr">
         <is>
-          <t>[단독] 美 DNI가 ‘정보공유 제한’ 결정… 李, 정동영·이종석 경질론 선 그어</t>
+          <t>법원, '푸틴 반대' 러시아인 체류연장 불허에 "취소해야"</t>
         </is>
       </c>
       <c r="E99" s="3" t="inlineStr">
         <is>
-          <t>[단독] 美 DNI가 ‘정보공유 제한’ 결정… 李, 정동영·이종석 경질론 선 그어  조선일보국민의힘 “동맹 지키자는게 굴종?…이재명 정부 백해무익 외교”  KBS 뉴스조갑제 “李대통령, 김정은엔 굴종적·美엔 당당하게? 말이 되나”  문화일보한·미 정보 갈등에도 “국익 최우선”… 이 대통...</t>
+          <t>(인천=연합뉴스) 김상연 기자 = 국내에서 러시아·우크라이나 전쟁 반대 시위에 수백회 참여한 러시아인에게 난민인정 신청 결과가 나올 때까지 임시...</t>
         </is>
       </c>
       <c r="F99" s="3" t="inlineStr">
         <is>
-          <t>조선일보</t>
+          <t>주요언론</t>
         </is>
       </c>
       <c r="G99" s="3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxORUxjVnJDQjk3WU9KdllpN3hRcnRSUWNGUDlKc1NQSlZtaHBVWVlGTW1zQ1ROQUJzal9kS1ZJUFF0eGhzS0xEQVZETXpGN1pNTTVxUEtyRlFrYkxLV1MtQ3QtY1Vld0pJbGQ0SWtvMkdCWWYxX0hJNkNmdEhYTURDRDhyaktRSjJGZTJOMUpobkg?oc=5</t>
+          <t>https://www.yna.co.kr/view/AKR20261014065900065</t>
         </is>
       </c>
     </row>
@@ -4139,32 +4140,32 @@
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>사회/사건사고</t>
+          <t>거시경제/비즈니스</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>🔥 [언론사 집중 보도 (3개사)]</t>
+          <t>신규 이슈</t>
         </is>
       </c>
       <c r="D100" s="3" t="inlineStr">
         <is>
-          <t>민간건물 임차 27곳 내년 이전…‘행정수도 세종’ 2031년 완성</t>
+          <t>산업부, 2030년까지 국가·지역 대표 전시회 5개 이상 육성</t>
         </is>
       </c>
       <c r="E100" s="3" t="inlineStr">
         <is>
-          <t>민간건물 임차 27곳 내년 이전…‘행정수도 세종’ 2031년 완성  한겨레안철수, 외교·통일·국방부 ‘세종 이전’ 발표에 “북한에 수도 헌납할건가”  경향신문[전국 주요 신문 톱뉴스](14일 조간)  연합뉴스금융위·법무부 등 44개 기관 9929명, 내년부터 세종 본격 이전  정책브리핑...</t>
+          <t>산업부, 2030년까지 국가·지역 대표 전시회 5개 이상 육성  KBS 뉴스Google 뉴스에서 헤드라인 및 의견 더보기</t>
         </is>
       </c>
       <c r="F100" s="3" t="inlineStr">
         <is>
-          <t>한겨레</t>
+          <t>KBS 뉴스</t>
         </is>
       </c>
       <c r="G100" s="3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiakFVX3lxTE5nRVl0ZVdQRld3OGtSZFp3WmdOZWFmRk1HWkNFZTMtVDJvYWRfQURGNUFLRUFYRVFtVC1wU1VJSGZrR01sMXBsZ2g1eTQ5aldSY0xydHhiUHl3dmpqOTJPLTN2Wl9CdzdLTlE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE0wbFFDM0djVl8tRTVjVUhwS0dfdjFGWkZYVURJNTZnaUZIeEVNdzUtMWZYRTY0VTFSYXMwdk9RVVVOR2FLMTFpSlQ2ZE1xRzFxa2pMdnBfT0pHa3M?oc=5</t>
         </is>
       </c>
     </row>
@@ -4176,32 +4177,32 @@
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>사회/사건사고</t>
+          <t>거시경제/비즈니스</t>
         </is>
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>신규 이슈</t>
+          <t>🔥 [언론사 집중 보도 (3개사)]</t>
         </is>
       </c>
       <c r="D101" s="3" t="inlineStr">
         <is>
-          <t>혼인무효 소송 중 장모 살해·아내 납치한 20대 남성 구속영장심사</t>
+          <t>필라델피아 반도체 지수 5일 연속 하락...7월 말 이후 처음</t>
         </is>
       </c>
       <c r="E101" s="3" t="inlineStr">
         <is>
-          <t>혼인무효 소송 중 장모 살해·아내 납치한 20대 남성 구속영장심사  MBC 뉴스[단독] 장모 살해범, 이미 ‘수차례 전과’…상습범의 계획범죄 정황  JTBC[단독] “경찰 신고 전에 뭐라 했어”…송파 ‘장모 살해범’ 보복 범죄 정황  KBS 뉴스장모 살해 20대, 가족 신변 볼모로 아내...</t>
+          <t>필라델피아 반도체 지수 5일 연속 하락...7월 말 이후 처음  YTN메모리, 제2 소프트웨어?…"내년 정말 힘들 것" PTJ의 경고 [김현석의 월스트리트나우]  한국경제반도체 손실로 월가 하락 후 미국 증시 선물 보합세…CPI 발표 대기  Investing.com 한국어中 반도체 추격...</t>
         </is>
       </c>
       <c r="F101" s="3" t="inlineStr">
         <is>
-          <t>MBC 뉴스</t>
+          <t>YTN</t>
         </is>
       </c>
       <c r="G101" s="3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE5JM3lPYzJGVjJJclh2cUx3cFdzby1sOHF1Q1ktQnIyWkVRVmRPcWdhOEhMTHNUYTNpSDNMWUwyR2NZRnRRc19OMDVHMG1rS2NEYUkzTndob3JxZHk4Wk5FUFp6LTA5Sy1SZzE4UFpvX0ZLWG9sWlRJ0gF3QVVfeXFMTVMwZVl2TXltUlZXd2dwUzVaRXlpOVJuUnlYMHlQLXk5NTBQb2oyNG9PR0xQb1djRGJnd1dtbzQ3ZlJvWmdwVnoxSEhrbmdhVUFxYV9ZcmdoUENGOUtINTBUVXlVcmVEXzY5aXkzVzVZYkNZTDd4c00?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiXkFVX3lxTFByT3A4M2N1UEF1c211Rll3UHdCX2F6ZkttQ3YwY0U3OTlJSE00ZDlwR1Y2X1dRT09zakFLRnd6TEs0RlBCcVhUSURyNF9BLVBHeld6bERydDZUQmxLY1E?oc=5</t>
         </is>
       </c>
     </row>
@@ -4213,32 +4214,32 @@
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>사회/사건사고</t>
+          <t>거시경제/비즈니스</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>🔥 [언론사 집중 보도 (4개사)]</t>
+          <t>신규 이슈</t>
         </is>
       </c>
       <c r="D102" s="3" t="inlineStr">
         <is>
-          <t>추미애 “관사 계약, 사치라 보기 어려워”···이재명 대통령 SNS글엔 “저라고 생각 안 해”</t>
+          <t>삼성전자 '100조 잭팟' 뒤 서늘한 경고…"한국이 흔들린다" [테크로그]</t>
         </is>
       </c>
       <c r="E102" s="3" t="inlineStr">
         <is>
-          <t>추미애 “관사 계약, 사치라 보기 어려워”···이재명 대통령 SNS글엔 “저라고 생각 안 해”  경향신문경기도 아닌 ‘추미애 국정감사’?…여야, ‘예산 삭감’·‘SNS 정치’ 질타  KBS 뉴스"일방독주" "여의도지사" 與도 野도 秋 난타  조선일보秋국감서 與공세성 질의에 '내분 분수령...</t>
+          <t>삼성전자 '100조 잭팟' 뒤 서늘한 경고…"한국이 흔들린다" [테크로그]  한국경제100조원 벌었지만 증가율은 반토막…외국인 올들어 232조원 ‘엑소더스’  한국경제삼성전자·SK하이닉스, 두번째 바닥 찍었나…“W자 반등 기대”  마켓인거침없는 외인 매도...반도체 역대급 실적에도 급락...</t>
         </is>
       </c>
       <c r="F102" s="3" t="inlineStr">
         <is>
-          <t>경향신문</t>
+          <t>한국경제</t>
         </is>
       </c>
       <c r="G102" s="3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTE1ZMXNSbkp5MlNtcXZuQ3R4TjBqek1vQ0NYa1IyRDFKaTBrdXZpZE9SSWVycGVsNHlkRVZCcnpVV2RfZEgxaWdYQV92d05Ja0pUbk04eDlhOGhDd9IBX0FVX3lxTE9lTmFkSV9mNWpFX210TXBZelIzOXU3NF9zQ0w3T25rcjFUbzRBTFhtelpGQlR0QUpCcm9WYW9EaVpxbG9CaUNhZkxEOGdhbzBOS24zMXZ3WGJwdGZnZURZ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTE0ybTlfNDRfSnlTM3l0VzBjYm5QNmpPeW9wLWJ6UGE1dTF2ZEd3Nll1LTA4dW0wVFlneHNqaWlMTzFDY21VbEF3eDluN2FVSXAyR0FQcVRuVm1kUQ?oc=5</t>
         </is>
       </c>
     </row>
@@ -4250,32 +4251,32 @@
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>사회/사건사고</t>
+          <t>거시경제/비즈니스</t>
         </is>
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>신규 이슈</t>
+          <t>연결 이슈 (후속)</t>
         </is>
       </c>
       <c r="D103" s="3" t="inlineStr">
         <is>
-          <t>뇌동맥류 수술 후 사망…법원 "대안 치료 설명 의무 위반"</t>
+          <t>새마을금고·OK저축은행도 고객 정보 유출…금융당국에 신고</t>
         </is>
       </c>
       <c r="E103" s="3" t="inlineStr">
         <is>
-          <t>(부산=연합뉴스) 차근호 기자 = 별다른 증상이 없던 환자가 비파열성 뇌동맥류 수술을 받은 뒤 뇌출혈로 숨진 사건에서 의료진의 수술상 과실은 인...</t>
+          <t>새마을금고·OK저축은행도 고객 정보 유출…금융당국에 신고  조선일보새마을금고 400명대 개인정보 유출... 계좌정보도 포함  보안뉴스금융당국, 해킹 2금융권 확산에 긴급 점검  전자신문OK저축은행, 대출신청 페이지에서 정보 유출… 고객 183명 정보 유출 - 조선비즈  Chosunbiz...</t>
         </is>
       </c>
       <c r="F103" s="3" t="inlineStr">
         <is>
-          <t>주요언론</t>
+          <t>조선일보</t>
         </is>
       </c>
       <c r="G103" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261014049500051</t>
+          <t>https://news.google.com/rss/articles/CBMiiwFBVV95cUxNdUg3TWo4c01LMHZnOXFZOFdfZDRXRWpuMld3TlRzTXBNdjdvQTJyUFZmcGRfOGJCc3dnRFZQbW9pLVYtWDNPSXFDQkR0dTR3ZnVud0NlbjhhYWVhTnpvYm85SUNncUJvYzVqY0FRRlVrU2pvQnhSaDJ6aGFWM0s1bUJwaFdrd3dvQzQw?oc=5</t>
         </is>
       </c>
     </row>
@@ -4287,7 +4288,7 @@
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>사회/사건사고</t>
+          <t>거시경제/비즈니스</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
@@ -4297,12 +4298,12 @@
       </c>
       <c r="D104" s="3" t="inlineStr">
         <is>
-          <t>강북구, 고령자 운전면허 반납지원 확대…차 없애면 20만원 추가</t>
+          <t>횡성군, 임도 사면 녹화 기술 도입…식생 정착·시공 품질 향상</t>
         </is>
       </c>
       <c r="E104" s="3" t="inlineStr">
         <is>
-          <t>(서울=연합뉴스) 정준영 기자 = 서울 강북구(구청장 정창수)는 고령운전자의 교통사고를 예방하고자 오는 15일부터 '고령운전자 운전면허 자진반납...</t>
+          <t>(횡성=연합뉴스) 류호준 기자 = 강원 횡성군은 횡성군산림조합, 구루이엔티와 임도 사면 녹화 기술의 현장 적용과 기술 협력을 위한 업무협약(MO...</t>
         </is>
       </c>
       <c r="F104" s="3" t="inlineStr">
@@ -4312,7 +4313,7 @@
       </c>
       <c r="G104" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261014054900004</t>
+          <t>https://www.yna.co.kr/view/AKR20261014068000062</t>
         </is>
       </c>
     </row>
@@ -4324,7 +4325,7 @@
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>사회/사건사고</t>
+          <t>거시경제/비즈니스</t>
         </is>
       </c>
       <c r="C105" s="2" t="inlineStr">
@@ -4334,12 +4335,12 @@
       </c>
       <c r="D105" s="3" t="inlineStr">
         <is>
-          <t>광주 온 도시철도 2호선 전동차…내년부터 시운전</t>
+          <t>충남도, 올해 마지막 '동네창업학교' 교육생 100명 모집</t>
         </is>
       </c>
       <c r="E105" s="3" t="inlineStr">
         <is>
-          <t>(전남광주=연합뉴스) 장덕종 기자 = 광주도시철도 2호선 1단계(시청∼월드컵경기장∼백운광장∼조선대∼광주역)를 달릴 전동차가 14일 첫 입고돼 본...</t>
+          <t>(홍성=연합뉴스) 김준범 기자 = 충남도는 청년 예비·초기 창업자를 대상으로 올해 마지막 '동네창업학교' 교육생 100명을 모집한다고 14일 밝...</t>
         </is>
       </c>
       <c r="F105" s="3" t="inlineStr">
@@ -4349,7 +4350,7 @@
       </c>
       <c r="G105" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261014044500054</t>
+          <t>https://www.yna.co.kr/view/AKR20261014068300063</t>
         </is>
       </c>
     </row>
@@ -4361,7 +4362,7 @@
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>사회/사건사고</t>
+          <t>거시경제/비즈니스</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
@@ -4371,12 +4372,12 @@
       </c>
       <c r="D106" s="3" t="inlineStr">
         <is>
-          <t>저소득층 '실명 예방' 공로…강동구, 보건복지부장관 표창</t>
+          <t>공공수주 반등에도 민간 부진…8월 건설수주 8% 감소</t>
         </is>
       </c>
       <c r="E106" s="3" t="inlineStr">
         <is>
-          <t>(서울=연합뉴스) 김준태 기자 = 강동구는 지난 8일 송파여성문화회관에서 열린 '제56회 눈의 날 기념식'에서 보건복지부장관 표창을 받았다고 1...</t>
+          <t>(세종=연합뉴스) 오진송 기자 = 올해 8월 국내 건설수주가 공공 부문의 반등에도 민간 부진이 이어지면서 3개월 연속 감소한 것으로 나타났다.</t>
         </is>
       </c>
       <c r="F106" s="3" t="inlineStr">
@@ -4386,7 +4387,7 @@
       </c>
       <c r="G106" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261014048800004</t>
+          <t>https://www.yna.co.kr/view/AKR20261014059000003</t>
         </is>
       </c>
     </row>
@@ -4398,32 +4399,32 @@
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>사회/사건사고</t>
+          <t>세계/국제</t>
         </is>
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>신규 이슈</t>
+          <t>연결 이슈 (후속)</t>
         </is>
       </c>
       <c r="D107" s="3" t="inlineStr">
         <is>
-          <t>음성 사정리 동학군·항일의병 추정 묘소 보존·활용 방향은</t>
+          <t>레오 14세 교황, 폐암 진단…오른쪽 폐 일부 절제 수술</t>
         </is>
       </c>
       <c r="E107" s="3" t="inlineStr">
         <is>
-          <t>(음성=연합뉴스) 박재천 기자 = 충북 음성군은 충북역사문화연구원과 함께 오는 16일 오전 10시 30분 음성생활문화센터에서 사정리 동학군(항일...</t>
+          <t>레오 14세 교황, 폐암 진단…오른쪽 폐 일부 절제 수술  한국경제71살 교황 레오 14세 폐암 진단…“오른쪽 폐 일부 절제”  한겨레레오 14세 교황, 폐 결절 아닌 폐암…오른쪽 폐 일부 절제 수술  동아일보교황청 "레오 14세, 폐 결절 수술 성공적 완료"…남미순방 갈듯  마켓인교황...</t>
         </is>
       </c>
       <c r="F107" s="3" t="inlineStr">
         <is>
-          <t>주요언론</t>
+          <t>한국경제</t>
         </is>
       </c>
       <c r="G107" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261014053100064</t>
+          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTE52ak40R0pZMTk1NVRHM3lZNGNsYnFsYW1Ud2RGbXYzRzJZbUZFRjlxb2V2ZGVVRm5MaVFLOW5HZmM2eE5iSTcyLVowc2cydUc5WS1XRG9uVU53dw?oc=5</t>
         </is>
       </c>
     </row>
@@ -4435,7 +4436,7 @@
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>사회/사건사고</t>
+          <t>세계/국제</t>
         </is>
       </c>
       <c r="C108" s="2" t="inlineStr">
@@ -4445,12 +4446,12 @@
       </c>
       <c r="D108" s="3" t="inlineStr">
         <is>
-          <t>[바이오스냅] 셀트리온, 미국 처방집 추가 등재 추진</t>
+          <t>美검찰, '韓 정부 대리' 혐의 수미 테리 '기소유예 합의'</t>
         </is>
       </c>
       <c r="E108" s="3" t="inlineStr">
         <is>
-          <t>(서울=연합뉴스) 박상현 기자 = 셀트리온[068270]이 미국에서 대형 처방약급여관리업체(PBM) 처방집 추가 등재를 추진하며 매출 확대를 모...</t>
+          <t>(서울=연합뉴스) 임화섭 기자 = 한국 정부를 위해 비밀리에 활동하고 고가 선물을 수수했다는 혐의를 받아온 전직 미국 중앙정보국(CIA) 분석가...</t>
         </is>
       </c>
       <c r="F108" s="3" t="inlineStr">
@@ -4460,7 +4461,7 @@
       </c>
       <c r="G108" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261014055200017</t>
+          <t>https://www.yna.co.kr/view/AKR20261014067100009</t>
         </is>
       </c>
     </row>
@@ -4472,7 +4473,7 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>사회/사건사고</t>
+          <t>IT/과학/신상품</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
@@ -4482,12 +4483,12 @@
       </c>
       <c r="D109" s="3" t="inlineStr">
         <is>
-          <t>서울대 80주년 유홍림총장 "왜 대학이어야 하는가 다시 물어야"</t>
+          <t>해양진흥공사, 지속가능경영보고서 최고 등급</t>
         </is>
       </c>
       <c r="E109" s="3" t="inlineStr">
         <is>
-          <t>(서울=연합뉴스) 윤민혁 기자 = 유홍림 서울대 총장은 14일 제80주년 개교기념사에서 대학의 위상과 의미가 근본적으로 도전받고 있다며 "왜 대...</t>
+          <t>(부산=연합뉴스) 박창수 기자 = 한국해양진흥공사는 지난 5월 발간한 '2025 지속가능경영보고서'가 미국 커뮤니케이션연맹(LACP)이 주관하는...</t>
         </is>
       </c>
       <c r="F109" s="3" t="inlineStr">
@@ -4497,7 +4498,7 @@
       </c>
       <c r="G109" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261014048000004</t>
+          <t>https://www.yna.co.kr/view/AKR20261014067400051</t>
         </is>
       </c>
     </row>
@@ -4509,7 +4510,7 @@
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>사회/사건사고</t>
+          <t>IT/과학/신상품</t>
         </is>
       </c>
       <c r="C110" s="2" t="inlineStr">
@@ -4519,12 +4520,12 @@
       </c>
       <c r="D110" s="3" t="inlineStr">
         <is>
-          <t>[게시판] 소진공, 대전 종합사회복지관 등에 '로컬푸드 꾸러미' 전달</t>
+          <t>1∼8월 배터리 분리막 적재량 25%↑…중국 제외 41% 성장</t>
         </is>
       </c>
       <c r="E110" s="3" t="inlineStr">
         <is>
-          <t>▲ 소상공인시장진흥공단은 지역 농가의 소득 증대와 지역경제 활성화를 돕고자 대전 유성구 종합사회복지관과 그냥드림센터에 '로컬푸드 꾸러미'를 전달...</t>
+          <t>(서울=연합뉴스) 김민지 기자 = 올해 1∼8월 글로벌 전기차용 배터리 분리막 적재량이 배터리 탑재량 증가와 중국 제외 시장의 빠른 성장에 힘입...</t>
         </is>
       </c>
       <c r="F110" s="3" t="inlineStr">
@@ -4534,7 +4535,7 @@
       </c>
       <c r="G110" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261014022600030</t>
+          <t>https://www.yna.co.kr/view/AKR20261014062600003</t>
         </is>
       </c>
     </row>
@@ -4546,7 +4547,7 @@
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>사회/사건사고</t>
+          <t>IT/과학/신상품</t>
         </is>
       </c>
       <c r="C111" s="2" t="inlineStr">
@@ -4556,12 +4557,12 @@
       </c>
       <c r="D111" s="3" t="inlineStr">
         <is>
-          <t>[부고] 홍성권(강원대학교병원 외과 과장)씨 부친상</t>
+          <t>음성군, '전통시장·상점가 활성화 유공' 중기부 장관상 수상</t>
         </is>
       </c>
       <c r="E111" s="3" t="inlineStr">
         <is>
-          <t>▲ 홍홍표(향년 86세)씨 별세, 홍성권(강원대학교병원 외과 과장)씨 부친상 = 14일 오전, 강원대학교병원장례식장 2호실, 발인 16일 오전 ...</t>
+          <t>(음성=연합뉴스) 박재천 기자 = 충북 음성군은 중소벤처기업부의 '2026년 전통시장 및 상점가 활성화 유공' 평가에서 우수 지방자치단체로 선정...</t>
         </is>
       </c>
       <c r="F111" s="3" t="inlineStr">
@@ -4571,2634 +4572,7 @@
       </c>
       <c r="G111" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261014051800062</t>
-        </is>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B112" s="2" t="inlineStr">
-        <is>
-          <t>사회/사건사고</t>
-        </is>
-      </c>
-      <c r="C112" s="2" t="inlineStr">
-        <is>
-          <t>신규 이슈</t>
-        </is>
-      </c>
-      <c r="D112" s="3" t="inlineStr">
-        <is>
-          <t>속초시, 상반기 사업체·청년 창업기업 증가세… 지역경제 활기</t>
-        </is>
-      </c>
-      <c r="E112" s="3" t="inlineStr">
-        <is>
-          <t>(속초=연합뉴스) 류호준 기자 = 강원 속초지역 전체 사업체 수와 청년 창업기업 수가 올해 상반기 매월 증가한 것으로 나타났다.</t>
-        </is>
-      </c>
-      <c r="F112" s="3" t="inlineStr">
-        <is>
-          <t>주요언론</t>
-        </is>
-      </c>
-      <c r="G112" s="3" t="inlineStr">
-        <is>
-          <t>https://www.yna.co.kr/view/AKR20261014051100062</t>
-        </is>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B113" s="2" t="inlineStr">
-        <is>
-          <t>사회/사건사고</t>
-        </is>
-      </c>
-      <c r="C113" s="2" t="inlineStr">
-        <is>
-          <t>신규 이슈</t>
-        </is>
-      </c>
-      <c r="D113" s="3" t="inlineStr">
-        <is>
-          <t>순천향대-국군대전병원, 미래 군 의료 및 과학기술 융합 협약</t>
-        </is>
-      </c>
-      <c r="E113" s="3" t="inlineStr">
-        <is>
-          <t>(아산=연합뉴스) 유의주 기자 = 순천향대는 최근 국군대전병원과 '미래 군 의료 및 과학기술 융합을 위한 업무협약'을 맺었다고 14일 밝혔다.</t>
-        </is>
-      </c>
-      <c r="F113" s="3" t="inlineStr">
-        <is>
-          <t>주요언론</t>
-        </is>
-      </c>
-      <c r="G113" s="3" t="inlineStr">
-        <is>
-          <t>https://www.yna.co.kr/view/AKR20261014051400063</t>
-        </is>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B114" s="2" t="inlineStr">
-        <is>
-          <t>사회/사건사고</t>
-        </is>
-      </c>
-      <c r="C114" s="2" t="inlineStr">
-        <is>
-          <t>신규 이슈</t>
-        </is>
-      </c>
-      <c r="D114" s="3" t="inlineStr">
-        <is>
-          <t>다천 김종원, 추사 김정희 '충효가전' 편액 국립창원대에 기증</t>
-        </is>
-      </c>
-      <c r="E114" s="3" t="inlineStr">
-        <is>
-          <t>(창원=연합뉴스) 박영민 기자 = 국립창원대학교는 경남도립미술관장을 지낸 서예가 다천 김종원이 추사 김정희(1786∼1856)의 '충효가전'(忠...</t>
-        </is>
-      </c>
-      <c r="F114" s="3" t="inlineStr">
-        <is>
-          <t>주요언론</t>
-        </is>
-      </c>
-      <c r="G114" s="3" t="inlineStr">
-        <is>
-          <t>https://www.yna.co.kr/view/AKR20261014052700052</t>
-        </is>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B115" s="2" t="inlineStr">
-        <is>
-          <t>사회/사건사고</t>
-        </is>
-      </c>
-      <c r="C115" s="2" t="inlineStr">
-        <is>
-          <t>신규 이슈</t>
-        </is>
-      </c>
-      <c r="D115" s="3" t="inlineStr">
-        <is>
-          <t>전자발찌 차고 또 흉기난동…이상동기범죄자 80% '전과 있음'</t>
-        </is>
-      </c>
-      <c r="E115" s="3" t="inlineStr">
-        <is>
-          <t>(서울=연합뉴스) 한지은 기자 = 인천에서 전자발찌를 착용한 출소자가 불특정 다수를 상대로 흉기를 휘두르면서 고위험 범죄자의 재범을 막기 위한 ...</t>
-        </is>
-      </c>
-      <c r="F115" s="3" t="inlineStr">
-        <is>
-          <t>주요언론</t>
-        </is>
-      </c>
-      <c r="G115" s="3" t="inlineStr">
-        <is>
-          <t>https://www.yna.co.kr/view/AKR20261014042000004</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B116" s="2" t="inlineStr">
-        <is>
-          <t>사회/사건사고</t>
-        </is>
-      </c>
-      <c r="C116" s="2" t="inlineStr">
-        <is>
-          <t>연결 이슈 (후속)</t>
-        </is>
-      </c>
-      <c r="D116" s="3" t="inlineStr">
-        <is>
-          <t>'8명 부상' 인천 흉기난동 사건에 프로파일러 3명 투입</t>
-        </is>
-      </c>
-      <c r="E116" s="3" t="inlineStr">
-        <is>
-          <t>(인천=연합뉴스) 홍현기 기자 = 인천 대형 상업시설에서 흉기를 휘둘러 8명을 다치게 한 50대 남성을 상대로 경찰이 범행 동기를 밝히기 위해 ...</t>
-        </is>
-      </c>
-      <c r="F116" s="3" t="inlineStr">
-        <is>
-          <t>주요언론</t>
-        </is>
-      </c>
-      <c r="G116" s="3" t="inlineStr">
-        <is>
-          <t>https://www.yna.co.kr/view/AKR20261014050800065</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B117" s="2" t="inlineStr">
-        <is>
-          <t>사회/사건사고</t>
-        </is>
-      </c>
-      <c r="C117" s="2" t="inlineStr">
-        <is>
-          <t>신규 이슈</t>
-        </is>
-      </c>
-      <c r="D117" s="3" t="inlineStr">
-        <is>
-          <t>농민 매년 300명 사망에도…농진청, 안전장비 보급사업 중단</t>
-        </is>
-      </c>
-      <c r="E117" s="3" t="inlineStr">
-        <is>
-          <t>(전주=연합뉴스) 김진방 기자 = 농업인의 재해율이 전체 산업 대비 8배를 웃도는 상황에서 농촌진흥청이 'IoT 농기계 교통안전 및 사고 감지 ...</t>
-        </is>
-      </c>
-      <c r="F117" s="3" t="inlineStr">
-        <is>
-          <t>주요언론</t>
-        </is>
-      </c>
-      <c r="G117" s="3" t="inlineStr">
-        <is>
-          <t>https://www.yna.co.kr/view/AKR20261014048200055</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B118" s="2" t="inlineStr">
-        <is>
-          <t>거시경제/비즈니스</t>
-        </is>
-      </c>
-      <c r="C118" s="2" t="inlineStr">
-        <is>
-          <t>연결 이슈 (후속)</t>
-        </is>
-      </c>
-      <c r="D118" s="3" t="inlineStr">
-        <is>
-          <t>[속보]홍라희 관장, 아들 이재용 회장에 삼성전자 주식 2.6조 증여</t>
-        </is>
-      </c>
-      <c r="E118" s="3" t="inlineStr">
-        <is>
-          <t>[속보]홍라희 관장, 아들 이재용 회장에 삼성전자 주식 2.6조 증여  문화일보이재용, 장외매수로 삼성전자 766만주 매수…1.9조 규모  연합인포맥스홍라희 관장, 이재용 회장에 삼성전자 지분 2.6조 증여  조선일보홍라희, 이재용에 삼성전자 주식 1천115만주 증여…이재용 지분율 1....</t>
-        </is>
-      </c>
-      <c r="F118" s="3" t="inlineStr">
-        <is>
-          <t>문화일보</t>
-        </is>
-      </c>
-      <c r="G118" s="3" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiUEFVX3lxTFBGRllSNUNuOTVwTGl2OXM5a1RKazk3NnRwR2I2Z1ZqOTdveWpNZHYtLUZpVlZTOFlWS2FMNnNYLWpZbkFjTkM3RGNhY0I1UHgy?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B119" s="2" t="inlineStr">
-        <is>
-          <t>거시경제/비즈니스</t>
-        </is>
-      </c>
-      <c r="C119" s="2" t="inlineStr">
-        <is>
-          <t>신규 이슈</t>
-        </is>
-      </c>
-      <c r="D119" s="3" t="inlineStr">
-        <is>
-          <t>[은행이 뚫린다-진단③] 보안업계 제안은? “IP 차단은 임시... 자산식별·행위분석·접점 숨기기 필요”</t>
-        </is>
-      </c>
-      <c r="E119" s="3" t="inlineStr">
-        <is>
-          <t>[은행이 뚫린다-진단③] 보안업계 제안은? “IP 차단은 임시... 자산식별·행위분석·접점 숨기기 필요”  보안뉴스[금융현미경]AI·해킹 위협에 금융권 내부통제 경고등…커지는 '임원 책임' 강화론  아시아경제[단독]망분리 완화 금융사 10곳, 보안계획만 세우고 이행 안해···내부망 해킹...</t>
-        </is>
-      </c>
-      <c r="F119" s="3" t="inlineStr">
-        <is>
-          <t>보안뉴스</t>
-        </is>
-      </c>
-      <c r="G119" s="3" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMia0FVX3lxTE9ESmY2WkEzNVVwVGNGWm9GZjhVUVpRMXp4UWlWMDhwY0ZxTHJ6VllQUXpiOXFEUUtqbFdERk9ERDNzYUt4UklRelNWWEk3TGNFZ2szZDFxb2F0ODlzYm0tT05aVzBLbVdHZGVz?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B120" s="2" t="inlineStr">
-        <is>
-          <t>거시경제/비즈니스</t>
-        </is>
-      </c>
-      <c r="C120" s="2" t="inlineStr">
-        <is>
-          <t>🔥 [언론사 집중 보도 (4개사)]</t>
-        </is>
-      </c>
-      <c r="D120" s="3" t="inlineStr">
-        <is>
-          <t>반도체, 이익 전망 대비 과도한 하락…"분할매수 대응“</t>
-        </is>
-      </c>
-      <c r="E120" s="3" t="inlineStr">
-        <is>
-          <t>반도체, 이익 전망 대비 과도한 하락…"분할매수 대응“  비즈워치“이젠 반도체 미련 버려야?”...내년 증시 주도주 바뀌나  매일경제반도체주 반등 언제쯤…“소부장이 투자 대안”  마켓인메모리 호황인데 '삼전닉스' 왜 떨어지나…"공급 과잉 우려·환율이 발목"  뉴시스반도체 미련 버릴까요?...</t>
-        </is>
-      </c>
-      <c r="F120" s="3" t="inlineStr">
-        <is>
-          <t>비즈워치</t>
-        </is>
-      </c>
-      <c r="G120" s="3" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiakFVX3lxTE8zZUN5TmF3dXFaQktYdkxDdlV6SUFTRndrcnVFZG1PcW92SUhkMzZpa3BLRDVZTFdHNzFRbDNfSWFjbEdUNnhZb2V0Zld6QmI0c3JjNzNPVWZCMXNpc2lpZTg3Y3BPSVRjTFE?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B121" s="2" t="inlineStr">
-        <is>
-          <t>거시경제/비즈니스</t>
-        </is>
-      </c>
-      <c r="C121" s="2" t="inlineStr">
-        <is>
-          <t>연결 이슈 (후속)</t>
-        </is>
-      </c>
-      <c r="D121" s="3" t="inlineStr">
-        <is>
-          <t>삼성·LG, 일상·산업 속 AI 기술 한눈에…’KES 2026’ 개최</t>
-        </is>
-      </c>
-      <c r="E121" s="3" t="inlineStr">
-        <is>
-          <t>삼성·LG, 일상·산업 속 AI 기술 한눈에…’KES 2026’ 개최  연합뉴스TVKTC, 한국전자전서 AI·소프트웨어·스마트가전 역량 선보여  전기신문산업부, 2030년까지 국가·지역 대표 전시회 5개 이상 육성  연합뉴스허공 위 버튼에 로봇손 학습까지...한국판 CES 개막  YTN...</t>
-        </is>
-      </c>
-      <c r="F121" s="3" t="inlineStr">
-        <is>
-          <t>연합뉴스TV</t>
-        </is>
-      </c>
-      <c r="G121" s="3" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiZ0FVX3lxTFBfbWtIOGxCdFNuNW9Eb1lhaG9uMVlRNmVxRHJSSE1zTUlwdFY1bV9ORmI2NFkxcVhFSWlRZGwwSm11RVNzZGJKYkRWNm5kTFVnMGJCY0J1MEtwcmhaekp6NUQ4eWZrdU0?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B122" s="2" t="inlineStr">
-        <is>
-          <t>거시경제/비즈니스</t>
-        </is>
-      </c>
-      <c r="C122" s="2" t="inlineStr">
-        <is>
-          <t>신규 이슈</t>
-        </is>
-      </c>
-      <c r="D122" s="3" t="inlineStr">
-        <is>
-          <t>NDF, 1,341.90/ 1,342.30원…2.05원↓</t>
-        </is>
-      </c>
-      <c r="E122" s="3" t="inlineStr">
-        <is>
-          <t>NDF, 1,341.90/ 1,342.30원…2.05원↓  연합인포맥스중동발 유가상승·증시 급락에…환율 10원 오른 1,345.1원  연합뉴스반도체 호황에 ‘센’ 원화…1200이냐, 다시 1400이냐  경향신문원·달러 환율, 1340원대 초반 등락  뉴시스외인 증시 순매수 전환에…달러·...</t>
-        </is>
-      </c>
-      <c r="F122" s="3" t="inlineStr">
-        <is>
-          <t>연합인포맥스</t>
-        </is>
-      </c>
-      <c r="G122" s="3" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE5HaGJxTHJkaTFEM1JDS09WTkNEX1ZMLUNuZEpYQ0Vjb0VhN1ZDb1FZeGo2S1hXM08yZDh6RTFqQUVxek9sVXNXUElXQnMwbGg0eGkyMDhOSmVFYUdjSDdjOGQxS0dycEJjYm8xXzZLaHXSAXRBVV95cUxQNjVRWjlpWDJNa1RiZVljNW5mOTQ4QjhmT1JkdXlfRU4tUEJEOE9XUTlTX1JGbmhBTFRRb1FtVUdnVVdHeTBpQ1ljNkRfRTBqQ19falEyN0thbmZiNHNtaTlab0JtREJnZHU0Wk5UdnBUVldzeQ?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B123" s="2" t="inlineStr">
-        <is>
-          <t>거시경제/비즈니스</t>
-        </is>
-      </c>
-      <c r="C123" s="2" t="inlineStr">
-        <is>
-          <t>신규 이슈</t>
-        </is>
-      </c>
-      <c r="D123" s="3" t="inlineStr">
-        <is>
-          <t>中 차세대 D램, 삼전닉스 주도판 흔든다?…"기술격차 3년" 업계 선긋기 - 머니투데이</t>
-        </is>
-      </c>
-      <c r="E123" s="3" t="inlineStr">
-        <is>
-          <t>中 차세대 D램, 삼전닉스 주도판 흔든다?…"기술격차 3년" 업계 선긋기 - 머니투데이  머니투데이삼성證 "中 CXMT 리스크, 더 반영할 이유 없어…반도체 소부장 주목"  뉴시스창신메모리, 사실이면 "삼전닉스보다 빠르다"…긴장  JTBC애널리스트, 중국 CXMT의 주장이 마이크론 테크...</t>
-        </is>
-      </c>
-      <c r="F123" s="3" t="inlineStr">
-        <is>
-          <t>머니투데이</t>
-        </is>
-      </c>
-      <c r="G123" s="3" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiaEFVX3lxTFBGZE5NWFB1MmgwZjZ2YWdqYl9XamNORTBzS2Zxb3ZwdHhqWWJRc0U2a2t5ZlE2VUFDT1l5YUxLTEQ0Z05kMXk0ODZ6OUxUTTlyMWxOWVpoQWpmVWwwUUI4akYzMDdzZDVY0gFuQVVfeXFMTkc5Rnc2ek9rNy00amdwbFBaZDU1blI1ODBoclpMUzVOQy0xTWlscENENUhJUjVJbU93UzV0UzNoMk11dm1WaTZuRzBkN1FVRHlELThlWkVJVUU0enFxQldEUnI3WkEtNmZTdTR6dGc?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B124" s="2" t="inlineStr">
-        <is>
-          <t>거시경제/비즈니스</t>
-        </is>
-      </c>
-      <c r="C124" s="2" t="inlineStr">
-        <is>
-          <t>🔥 [언론사 집중 보도 (3개사)]</t>
-        </is>
-      </c>
-      <c r="D124" s="3" t="inlineStr">
-        <is>
-          <t>한화생명, '필요할 때 쓰는 종신보험' 출시</t>
-        </is>
-      </c>
-      <c r="E124" s="3" t="inlineStr">
-        <is>
-          <t>(서울=연합뉴스) 강수련 기자 = 한화생명[088350]은 14일 보장이 필요할 때는 사망보험금을, 생애 자금이 필요할 때는 납입보험료 전액을 ...</t>
-        </is>
-      </c>
-      <c r="F124" s="3" t="inlineStr">
-        <is>
-          <t>주요언론</t>
-        </is>
-      </c>
-      <c r="G124" s="3" t="inlineStr">
-        <is>
-          <t>https://www.yna.co.kr/view/AKR20261014053900002</t>
-        </is>
-      </c>
-    </row>
-    <row r="125">
-      <c r="A125" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B125" s="2" t="inlineStr">
-        <is>
-          <t>거시경제/비즈니스</t>
-        </is>
-      </c>
-      <c r="C125" s="2" t="inlineStr">
-        <is>
-          <t>신규 이슈</t>
-        </is>
-      </c>
-      <c r="D125" s="3" t="inlineStr">
-        <is>
-          <t>[게시판] CJ프레시웨이, 상생협력 아카데미 개최</t>
-        </is>
-      </c>
-      <c r="E125" s="3" t="inlineStr">
-        <is>
-          <t>▲ CJ프레시웨이[051500]는 지난 13일 서울 마포구 본사에서 중소식품 협력사의 식품안전 역량 강화를 위한 프로그램 '상생협력 아카데미'를...</t>
-        </is>
-      </c>
-      <c r="F125" s="3" t="inlineStr">
-        <is>
-          <t>주요언론</t>
-        </is>
-      </c>
-      <c r="G125" s="3" t="inlineStr">
-        <is>
-          <t>https://www.yna.co.kr/view/AKR20261014026300030</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B126" s="2" t="inlineStr">
-        <is>
-          <t>거시경제/비즈니스</t>
-        </is>
-      </c>
-      <c r="C126" s="2" t="inlineStr">
-        <is>
-          <t>🔥 [언론사 집중 보도 (5개사)]</t>
-        </is>
-      </c>
-      <c r="D126" s="3" t="inlineStr">
-        <is>
-          <t>카카오, 인적분할 앞두고 CEO 총출동…새 성장전략 공개</t>
-        </is>
-      </c>
-      <c r="E126" s="3" t="inlineStr">
-        <is>
-          <t>(서울=연합뉴스) 한상용 기자 = 카카오[035720]는 인적분할을 앞두고 증권사 애널리스트 등을 대상으로 주요 계열사 최고경영자(CEO)들이 ...</t>
-        </is>
-      </c>
-      <c r="F126" s="3" t="inlineStr">
-        <is>
-          <t>주요언론</t>
-        </is>
-      </c>
-      <c r="G126" s="3" t="inlineStr">
-        <is>
-          <t>https://www.yna.co.kr/view/AKR20261014055100017</t>
-        </is>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B127" s="2" t="inlineStr">
-        <is>
-          <t>거시경제/비즈니스</t>
-        </is>
-      </c>
-      <c r="C127" s="2" t="inlineStr">
-        <is>
-          <t>신규 이슈</t>
-        </is>
-      </c>
-      <c r="D127" s="3" t="inlineStr">
-        <is>
-          <t>[보령소식] 종합체육관서 20일 취·창업 박람회</t>
-        </is>
-      </c>
-      <c r="E127" s="3" t="inlineStr">
-        <is>
-          <t>(보령=연합뉴스) ▲ 종합체육관서 20일 취·창업 박람회 = 충남 보령시는 아주자동차대학교와 함께 오는 20일 오후 1시 30분부터 보령종합체육...</t>
-        </is>
-      </c>
-      <c r="F127" s="3" t="inlineStr">
-        <is>
-          <t>주요언론</t>
-        </is>
-      </c>
-      <c r="G127" s="3" t="inlineStr">
-        <is>
-          <t>https://www.yna.co.kr/view/AKR20261014050500063</t>
-        </is>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B128" s="2" t="inlineStr">
-        <is>
-          <t>거시경제/비즈니스</t>
-        </is>
-      </c>
-      <c r="C128" s="2" t="inlineStr">
-        <is>
-          <t>🔥 [언론사 집중 보도 (3개사)]</t>
-        </is>
-      </c>
-      <c r="D128" s="3" t="inlineStr">
-        <is>
-          <t>카카오페이, 마이데이터 기반 '멤버십 사후 적립' 출시</t>
-        </is>
-      </c>
-      <c r="E128" s="3" t="inlineStr">
-        <is>
-          <t>(서울=연합뉴스) 오지은 기자 = 카카오페이[377300]가 마이데이터를 활용해 결제 당시 놓친 멤버십 포인트를 나중에 적립할 수 있는 서비스를...</t>
-        </is>
-      </c>
-      <c r="F128" s="3" t="inlineStr">
-        <is>
-          <t>주요언론</t>
-        </is>
-      </c>
-      <c r="G128" s="3" t="inlineStr">
-        <is>
-          <t>https://www.yna.co.kr/view/AKR20261014043700017</t>
-        </is>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B129" s="2" t="inlineStr">
-        <is>
-          <t>거시경제/비즈니스</t>
-        </is>
-      </c>
-      <c r="C129" s="2" t="inlineStr">
-        <is>
-          <t>신규 이슈</t>
-        </is>
-      </c>
-      <c r="D129" s="3" t="inlineStr">
-        <is>
-          <t>hy "자체 개발 유산균, 알코올성 간손상 완화"…국제학술지 게재</t>
-        </is>
-      </c>
-      <c r="E129" s="3" t="inlineStr">
-        <is>
-          <t>(서울=연합뉴스) 한주홍 기자 = hy는 자체 개발한 프로바이오틱스 균주 'HY7804'의 알코올성 간손상 완화 가능성을 확인한 연구 논문이 국...</t>
-        </is>
-      </c>
-      <c r="F129" s="3" t="inlineStr">
-        <is>
-          <t>주요언론</t>
-        </is>
-      </c>
-      <c r="G129" s="3" t="inlineStr">
-        <is>
-          <t>https://www.yna.co.kr/view/AKR20261014044100030</t>
-        </is>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B130" s="2" t="inlineStr">
-        <is>
-          <t>거시경제/비즈니스</t>
-        </is>
-      </c>
-      <c r="C130" s="2" t="inlineStr">
-        <is>
-          <t>신규 이슈</t>
-        </is>
-      </c>
-      <c r="D130" s="3" t="inlineStr">
-        <is>
-          <t>카이아, 490만개 KAIA 소각…JPYC도 기여보상 대상</t>
-        </is>
-      </c>
-      <c r="E130" s="3" t="inlineStr">
-        <is>
-          <t>(서울=연합뉴스) 유동현 기자 = 카이아 DLT 재단이 자체 블록체인 네트워크의 토큰인 카이아(KAIA) 490만개를 소각한다고 14일 밝혔다.</t>
-        </is>
-      </c>
-      <c r="F130" s="3" t="inlineStr">
-        <is>
-          <t>주요언론</t>
-        </is>
-      </c>
-      <c r="G130" s="3" t="inlineStr">
-        <is>
-          <t>https://www.yna.co.kr/view/AKR20261014051200002</t>
-        </is>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B131" s="2" t="inlineStr">
-        <is>
-          <t>거시경제/비즈니스</t>
-        </is>
-      </c>
-      <c r="C131" s="2" t="inlineStr">
-        <is>
-          <t>신규 이슈</t>
-        </is>
-      </c>
-      <c r="D131" s="3" t="inlineStr">
-        <is>
-          <t>[게시판] 토스증권, 앱에 '시장' 탭 신설…AI시황 요약 제공</t>
-        </is>
-      </c>
-      <c r="E131" s="3" t="inlineStr">
-        <is>
-          <t>▲ 토스증권은 앱 내 '시장' 탭을 새롭게 도입했다고 14일 밝혔다. 이 탭에서는 주요 국내외 지수와 수급 등을 확인할 수 있다. 특히 'AI(...</t>
-        </is>
-      </c>
-      <c r="F131" s="3" t="inlineStr">
-        <is>
-          <t>주요언론</t>
-        </is>
-      </c>
-      <c r="G131" s="3" t="inlineStr">
-        <is>
-          <t>https://www.yna.co.kr/view/AKR20261014049900008</t>
-        </is>
-      </c>
-    </row>
-    <row r="132">
-      <c r="A132" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B132" s="2" t="inlineStr">
-        <is>
-          <t>거시경제/비즈니스</t>
-        </is>
-      </c>
-      <c r="C132" s="2" t="inlineStr">
-        <is>
-          <t>🔥 [언론사 집중 보도 (3개사)]</t>
-        </is>
-      </c>
-      <c r="D132" s="3" t="inlineStr">
-        <is>
-          <t>KB국민은행, 기업고객용 'KB B2B우대통장' 출시</t>
-        </is>
-      </c>
-      <c r="E132" s="3" t="inlineStr">
-        <is>
-          <t>(서울=연합뉴스) 한지훈 기자 = KB국민은행은 14일 기업 전용 파킹통장 'KB B2B우대통장'을 출시했다.</t>
-        </is>
-      </c>
-      <c r="F132" s="3" t="inlineStr">
-        <is>
-          <t>주요언론</t>
-        </is>
-      </c>
-      <c r="G132" s="3" t="inlineStr">
-        <is>
-          <t>https://www.yna.co.kr/view/AKR20261014051700002</t>
-        </is>
-      </c>
-    </row>
-    <row r="133">
-      <c r="A133" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B133" s="2" t="inlineStr">
-        <is>
-          <t>거시경제/비즈니스</t>
-        </is>
-      </c>
-      <c r="C133" s="2" t="inlineStr">
-        <is>
-          <t>신규 이슈</t>
-        </is>
-      </c>
-      <c r="D133" s="3" t="inlineStr">
-        <is>
-          <t>[게시판] LS증권, 국내 선물·옵션 수수료 할인 이벤트</t>
-        </is>
-      </c>
-      <c r="E133" s="3" t="inlineStr">
-        <is>
-          <t>▲ LS증권[078020]은 국내 선물·옵션 신규 및 휴면 고객을 대상으로 거래 수수료를 할인해주는 이벤트를 12월 31일까지 진행한다고 14일...</t>
-        </is>
-      </c>
-      <c r="F133" s="3" t="inlineStr">
-        <is>
-          <t>주요언론</t>
-        </is>
-      </c>
-      <c r="G133" s="3" t="inlineStr">
-        <is>
-          <t>https://www.yna.co.kr/view/AKR20261014050100008</t>
-        </is>
-      </c>
-    </row>
-    <row r="134">
-      <c r="A134" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B134" s="2" t="inlineStr">
-        <is>
-          <t>거시경제/비즈니스</t>
-        </is>
-      </c>
-      <c r="C134" s="2" t="inlineStr">
-        <is>
-          <t>신규 이슈</t>
-        </is>
-      </c>
-      <c r="D134" s="3" t="inlineStr">
-        <is>
-          <t>메리츠증권, 캔톤 재단과 금융자산 토큰화 협약체결</t>
-        </is>
-      </c>
-      <c r="E134" s="3" t="inlineStr">
-        <is>
-          <t>(서울=연합뉴스) 김유아 기자 = 메리츠증권은 캔톤 네트워크(Canton Network) 운영 재단인 캔톤 재단(CantonFoundation)...</t>
-        </is>
-      </c>
-      <c r="F134" s="3" t="inlineStr">
-        <is>
-          <t>주요언론</t>
-        </is>
-      </c>
-      <c r="G134" s="3" t="inlineStr">
-        <is>
-          <t>https://www.yna.co.kr/view/AKR20261014050900008</t>
-        </is>
-      </c>
-    </row>
-    <row r="135">
-      <c r="A135" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B135" s="2" t="inlineStr">
-        <is>
-          <t>거시경제/비즈니스</t>
-        </is>
-      </c>
-      <c r="C135" s="2" t="inlineStr">
-        <is>
-          <t>신규 이슈</t>
-        </is>
-      </c>
-      <c r="D135" s="3" t="inlineStr">
-        <is>
-          <t>코람코라이프인프라리츠, 전국 주유소 19곳 매각 추진</t>
-        </is>
-      </c>
-      <c r="E135" s="3" t="inlineStr">
-        <is>
-          <t>(서울=연합뉴스) 정회인 기자 = 코람코자산신탁이 운용하는 코람코라이프인프라리츠가 포트폴리오 재편과 신규 성장자산 투자를 위해 전국 주유소 19...</t>
-        </is>
-      </c>
-      <c r="F135" s="3" t="inlineStr">
-        <is>
-          <t>주요언론</t>
-        </is>
-      </c>
-      <c r="G135" s="3" t="inlineStr">
-        <is>
-          <t>https://www.yna.co.kr/view/AKR20261014049700008</t>
-        </is>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B136" s="2" t="inlineStr">
-        <is>
-          <t>거시경제/비즈니스</t>
-        </is>
-      </c>
-      <c r="C136" s="2" t="inlineStr">
-        <is>
-          <t>신규 이슈</t>
-        </is>
-      </c>
-      <c r="D136" s="3" t="inlineStr">
-        <is>
-          <t>관세청 "최근 5년 국회 반복지적 전면 점검…8건 개선 완료"</t>
-        </is>
-      </c>
-      <c r="E136" s="3" t="inlineStr">
-        <is>
-          <t>(세종=연합뉴스) 안채원 기자 = 관세청은 최근 5년간 국정감사에서 반복적으로 지적돼온 사항을 전면 점검해 총 8건의 개선 조치를 완료했다고 1...</t>
-        </is>
-      </c>
-      <c r="F136" s="3" t="inlineStr">
-        <is>
-          <t>주요언론</t>
-        </is>
-      </c>
-      <c r="G136" s="3" t="inlineStr">
-        <is>
-          <t>https://www.yna.co.kr/view/AKR20261014047700002</t>
-        </is>
-      </c>
-    </row>
-    <row r="137">
-      <c r="A137" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B137" s="2" t="inlineStr">
-        <is>
-          <t>거시경제/비즈니스</t>
-        </is>
-      </c>
-      <c r="C137" s="2" t="inlineStr">
-        <is>
-          <t>신규 이슈</t>
-        </is>
-      </c>
-      <c r="D137" s="3" t="inlineStr">
-        <is>
-          <t>LH, 공동주택 중대하자 4년새 90% 감소…"품질관리 강화"</t>
-        </is>
-      </c>
-      <c r="E137" s="3" t="inlineStr">
-        <is>
-          <t>(서울=연합뉴스) 오예진 기자 = 한국토지주택공사(LH)는 공동주택 품질 개선에 노력한 결과 올해 균열, 누수 등 중대하자 발생 건수가 크게 감...</t>
-        </is>
-      </c>
-      <c r="F137" s="3" t="inlineStr">
-        <is>
-          <t>주요언론</t>
-        </is>
-      </c>
-      <c r="G137" s="3" t="inlineStr">
-        <is>
-          <t>https://www.yna.co.kr/view/AKR20261014047500003</t>
-        </is>
-      </c>
-    </row>
-    <row r="138">
-      <c r="A138" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B138" s="2" t="inlineStr">
-        <is>
-          <t>거시경제/비즈니스</t>
-        </is>
-      </c>
-      <c r="C138" s="2" t="inlineStr">
-        <is>
-          <t>🔥 [언론사 집중 보도 (4개사)]</t>
-        </is>
-      </c>
-      <c r="D138" s="3" t="inlineStr">
-        <is>
-          <t>섬박람회 논란 큰데 이번엔 K컬처 전시회?…117억 투입 지역행사 키운다</t>
-        </is>
-      </c>
-      <c r="E138" s="3" t="inlineStr">
-        <is>
-          <t>2030년까지 전시회 5개 이상 육성 첨단 제조산업·K-컬처 등 연계 계획 기존 전시장들 낮은 가동률은 문제정부가 2030년까지 국가·지역 대표 전시회를 5개 이상 육성하고 관련 ..</t>
-        </is>
-      </c>
-      <c r="F138" s="3" t="inlineStr">
-        <is>
-          <t>주요언론</t>
-        </is>
-      </c>
-      <c r="G138" s="3" t="inlineStr">
-        <is>
-          <t>https://www.mk.co.kr/news/economy/12175201</t>
-        </is>
-      </c>
-    </row>
-    <row r="139">
-      <c r="A139" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B139" s="2" t="inlineStr">
-        <is>
-          <t>세계/국제</t>
-        </is>
-      </c>
-      <c r="C139" s="2" t="inlineStr">
-        <is>
-          <t>연결 이슈 (후속)</t>
-        </is>
-      </c>
-      <c r="D139" s="3" t="inlineStr">
-        <is>
-          <t>교황 레오 14세 폐암 진단…“오른쪽 폐 일부 절제”</t>
-        </is>
-      </c>
-      <c r="E139" s="3" t="inlineStr">
-        <is>
-          <t>교황 레오 14세 폐암 진단…“오른쪽 폐 일부 절제”  한겨레교황청 "레오 14세, 폐 결절 수술 성공적 완료"…남미순방 갈듯  마켓인교황, 폐 결절 제거술 위해 로마 병원에 입원  연합뉴스바티칸 "교황 레오 14세 폐암 진단…수술 성공적" - 머니투데이  머니투데이[속보]교황 레오16...</t>
-        </is>
-      </c>
-      <c r="F139" s="3" t="inlineStr">
-        <is>
-          <t>한겨레</t>
-        </is>
-      </c>
-      <c r="G139" s="3" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxNSFNnUnVzUU4taDNoM1NEcmU5YlpXaVozdzFjT3N5UENKS2hTU3o4LW1hN0FtUzNYNDJ6WDBxVS0ydGFxSHJZUTd2LWpzbFFaZDNRMGM2X3hzRm5STUxLcmlHR2Y2M1FTQlBIa1AxbFRZazJpS0dmdHBEQWlyT0doM1h3?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="140">
-      <c r="A140" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B140" s="2" t="inlineStr">
-        <is>
-          <t>세계/국제</t>
-        </is>
-      </c>
-      <c r="C140" s="2" t="inlineStr">
-        <is>
-          <t>신규 이슈</t>
-        </is>
-      </c>
-      <c r="D140" s="3" t="inlineStr">
-        <is>
-          <t>여객기 납치경보에 교신까지 끊겨 독일 발칵…알고보니 시스템 오류</t>
-        </is>
-      </c>
-      <c r="E140" s="3" t="inlineStr">
-        <is>
-          <t>여객기 납치경보에 교신까지 끊겨 독일 발칵…알고보니 시스템 오류  연합뉴스TV“드론 추정 물체 목격, 항공 비상 상황”···독일 뉘른베르크 공항, 항공기 운항 중단  경향신문독일행 여객기 납치경보 잘못 보내 전투기 출격 소동  MBC 뉴스'7500' 여객기 하이재킹 오경보에 獨전투기 2...</t>
-        </is>
-      </c>
-      <c r="F140" s="3" t="inlineStr">
-        <is>
-          <t>연합뉴스TV</t>
-        </is>
-      </c>
-      <c r="G140" s="3" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiZ0FVX3lxTE81QWVvWkFRaTBZYmdkb25GbnZyOWFoR2tCUzNhMWxoVHpsUkR6dzFnRm9ZSmZBemxLQW5ZNExNVnRqaWxjbWx4bldiamd6WmlXM0NrS3ZKd29mXy1zdW5tOG5JNVJnU1k?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="141">
-      <c r="A141" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B141" s="2" t="inlineStr">
-        <is>
-          <t>세계/국제</t>
-        </is>
-      </c>
-      <c r="C141" s="2" t="inlineStr">
-        <is>
-          <t>🔥 [언론사 집중 보도 (4개사)]</t>
-        </is>
-      </c>
-      <c r="D141" s="3" t="inlineStr">
-        <is>
-          <t>트럼프 "우크라이나와 정보 공유 중단 안 해…푸틴, 종전 더 원해"(종합)</t>
-        </is>
-      </c>
-      <c r="E141" s="3" t="inlineStr">
-        <is>
-          <t>트럼프 "우크라이나와 정보 공유 중단 안 해…푸틴, 종전 더 원해"(종합)  뉴스1‘경유 딜’ 우크라 반발에… “美, 종전 협상단 방러 보류”  동아일보트럼프 ‘에너지 휴전’ 후폭풍 속 침묵하는 푸틴…왜?  경향신문공화·민주 상원의원 12명 "러시아 경유 합의는 적국에 주는 선물"  뉴...</t>
-        </is>
-      </c>
-      <c r="F141" s="3" t="inlineStr">
-        <is>
-          <t>뉴스1</t>
-        </is>
-      </c>
-      <c r="G141" s="3" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiWEFVX3lxTFBCYmM0WHNQd01tM3A3MThrZ3FEbVBySlQ0OFVKZVVsSjg2SmVCYndZRXBLWGVOX201Ukhjd3ZwSzNJQnBGVVJITWRVdVRmYWFFdEdOMllZRHk?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="142">
-      <c r="A142" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B142" s="2" t="inlineStr">
-        <is>
-          <t>세계/국제</t>
-        </is>
-      </c>
-      <c r="C142" s="2" t="inlineStr">
-        <is>
-          <t>🔥 [언론사 집중 보도 (3개사)]</t>
-        </is>
-      </c>
-      <c r="D142" s="3" t="inlineStr">
-        <is>
-          <t>美 정보공유 안했나?…러 미사일, 공습경보 발령 전 키이우 타격</t>
-        </is>
-      </c>
-      <c r="E142" s="3" t="inlineStr">
-        <is>
-          <t>美 정보공유 안했나?…러 미사일, 공습경보 발령 전 키이우 타격  뉴스1우크라 드론이 러시아 데이터센터 때리자 중앙아시아 앱 '멈춤'  연합뉴스러 미사일 공격으로 부상한 여성 옮기는 구조대  뉴시스러 데이터센터 피격에 카자흐 주요 플랫폼 마비…디지털 인프라 의존 한계  아시아투데이[포착...</t>
-        </is>
-      </c>
-      <c r="F142" s="3" t="inlineStr">
-        <is>
-          <t>뉴스1</t>
-        </is>
-      </c>
-      <c r="G142" s="3" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiU0FVX3lxTFA5cFVCdDlfQ1VyOFp0ZEpsRVh1MUxrVnM4SFlvYVl1WE5SRVJWWC14VXNQWXo2VnplQVk1ZFhqanNlcnd0NjQ1bklEV3RsV0FieEsw?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="143">
-      <c r="A143" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B143" s="2" t="inlineStr">
-        <is>
-          <t>세계/국제</t>
-        </is>
-      </c>
-      <c r="C143" s="2" t="inlineStr">
-        <is>
-          <t>🔥 [언론사 집중 보도 (4개사)]</t>
-        </is>
-      </c>
-      <c r="D143" s="3" t="inlineStr">
-        <is>
-          <t>‘트럼프 장남 전 연인’ 주그리스 미국 대사 비위 의혹에 사임</t>
-        </is>
-      </c>
-      <c r="E143" s="3" t="inlineStr">
-        <is>
-          <t>‘트럼프 장남 전 연인’ 주그리스 미국 대사 비위 의혹에 사임  경향신문"가족은 아니었다"…트럼프, '아들 전 약혼녀' 그리스 대사 해임  마켓인백악관, '각종 비위 의혹' 그리스 대사에 "사퇴 요구했다"  연합뉴스트럼프와 측근 인사 부패 의혹, 미 중간선거 쟁점 부상  뉴시스"억대 빚...</t>
-        </is>
-      </c>
-      <c r="F143" s="3" t="inlineStr">
-        <is>
-          <t>경향신문</t>
-        </is>
-      </c>
-      <c r="G143" s="3" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTFBsanNzT0RJMzI1SGI4b3ByWUJPUXRzdEgzTGtkZl90Wmo5dUhrSE53MmFpbDBuQmdEcXNUVy1vV1dFSGlQMG5EdVFfQmhTZHVOcG1taUVubS0yd9IBX0FVX3lxTE5nUV8yQUZXOUZ2SV9JeUpLa2lzc0t5QXlOREoyYmh6STFLX0VKd2hJTTg2WnllWTBRQ1JTdlZDbFVpT2VXa2k1MGE2N05qQjI5R1J0WTZZZmMweEJySnRz?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="144">
-      <c r="A144" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B144" s="2" t="inlineStr">
-        <is>
-          <t>세계/국제</t>
-        </is>
-      </c>
-      <c r="C144" s="2" t="inlineStr">
-        <is>
-          <t>연결 이슈 (후속)</t>
-        </is>
-      </c>
-      <c r="D144" s="3" t="inlineStr">
-        <is>
-          <t>신압록강대교 북한 쪽 관문에 인공기·오성홍기 내걸려‥개통 임박 정황</t>
-        </is>
-      </c>
-      <c r="E144" s="3" t="inlineStr">
-        <is>
-          <t>신압록강대교 북한 쪽 관문에 인공기·오성홍기 내걸려‥개통 임박 정황  MBC 뉴스北中신압록강대교 개통 임박했나…북측 관문 북중 대형국기 포착  연합뉴스[특파원리포트] 두 개의 다리와 북한의 몸값  세계일보북한 남포항 컨테이너 단지를 촬영한 위성사진. 올해 10월 7일 촬영된 위성사진에서...</t>
-        </is>
-      </c>
-      <c r="F144" s="3" t="inlineStr">
-        <is>
-          <t>MBC 뉴스</t>
-        </is>
-      </c>
-      <c r="G144" s="3" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMidEFVX3lxTE1tYXFLZnE3VmpmekdBZnpWM2FfalNNejBfT2oxMTVYRUR5cEY4WFMtamE0X1pscGNvZ0x3VjRiN2JtbFEtTEFRbXdlR25xczVZemMwUHZqbVNZTzJMdzhBRWtKX1NSU1BjWUJVUzZqSHlSS2dx0gF0QVVfeXFMTjdRbDZnbU5wdFBtMVJQY1RMZjRwRS1JQjdmQVRNR2lDUFNPQzlZVEhEWURZb25wWGptQXNMR1lrT0czSmMxc1lEakhHNVVqYjJkdkM3OVFPUUQwU01lNUEzNk1EZUpZVkZhV3dJYkIzbDFRWmU?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="145">
-      <c r="A145" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B145" s="2" t="inlineStr">
-        <is>
-          <t>세계/국제</t>
-        </is>
-      </c>
-      <c r="C145" s="2" t="inlineStr">
-        <is>
-          <t>연결 이슈 (후속)</t>
-        </is>
-      </c>
-      <c r="D145" s="3" t="inlineStr">
-        <is>
-          <t>"호르무즈 선박 피격 2주간 24건…이란전 이후 최다"</t>
-        </is>
-      </c>
-      <c r="E145" s="3" t="inlineStr">
-        <is>
-          <t>"호르무즈 선박 피격 2주간 24건…이란전 이후 최다"  연합뉴스TV"호르무즈 선박 피격 2주간 24건…개전 이후 최다"  연합뉴스이란군 “호르무즈 동부 선박 주시…금지 구역서 유조선 화재”  KBS 뉴스호르무즈 유조선 연쇄 공격… '중동 원유' 수출 회복세 또 꺾이나  마켓인호르무즈 ...</t>
-        </is>
-      </c>
-      <c r="F145" s="3" t="inlineStr">
-        <is>
-          <t>연합뉴스TV</t>
-        </is>
-      </c>
-      <c r="G145" s="3" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiZ0FVX3lxTE80R1Ezc0hlaWJRSUNQUk1XWmNDU1JDYVNSOWxwWm1JY0lTblpSZ055YXNwWmhKcDJSN3VMUk9HcTk2dnluSkpkX1lLSXRYWTJhSmRXV2RCVGxlY1dva3NwRlBOa2hkMms?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="146">
-      <c r="A146" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B146" s="2" t="inlineStr">
-        <is>
-          <t>세계/국제</t>
-        </is>
-      </c>
-      <c r="C146" s="2" t="inlineStr">
-        <is>
-          <t>신규 이슈</t>
-        </is>
-      </c>
-      <c r="D146" s="3" t="inlineStr">
-        <is>
-          <t>PAK DA 지연에 Kh-BD 부상…러시아 공중 핵억지력의 불확실성</t>
-        </is>
-      </c>
-      <c r="E146" s="3" t="inlineStr">
-        <is>
-          <t>PAK DA 지연에 Kh-BD 부상…러시아 공중 핵억지력의 불확실성  Meta-Defense</t>
-        </is>
-      </c>
-      <c r="F146" s="3" t="inlineStr">
-        <is>
-          <t>Meta-Defense</t>
-        </is>
-      </c>
-      <c r="G146" s="3" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxQbEEyUy02aDN4OG5KVVdhSUl2TkZzck83eVhHRFB2eHZqMEY0U21BemgtS3VKNDBZOHlmWHN2MTg1M2xsMWF1RENwNl9kbkJGUEx2V1dRcUMxLTRNSXBBUVY2UU1oYk01RWE0Vk94emxHQ3VWVzg4U1N3ZGVVeFFQRlJqY0ptR2Ez?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="147">
-      <c r="A147" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B147" s="2" t="inlineStr">
-        <is>
-          <t>세계/국제</t>
-        </is>
-      </c>
-      <c r="C147" s="2" t="inlineStr">
-        <is>
-          <t>신규 이슈</t>
-        </is>
-      </c>
-      <c r="D147" s="3" t="inlineStr">
-        <is>
-          <t>다급한 룰라, '소상공인 부채탕감' 대선 결선용 선심법안</t>
-        </is>
-      </c>
-      <c r="E147" s="3" t="inlineStr">
-        <is>
-          <t>다급한 룰라, '소상공인 부채탕감' 대선 결선용 선심법안  연합뉴스[브라질증시] 이보베스파 1.04% 하락…룰라·플라비우 지지율 격차 주시  뉴스핌트럼프 ‘블루 타이드’ 마지막 퍼즐 완성하나…‘보우소나루 정치 왕조’ 계승자 [더 비저너리-플라비우 보우소나루]  헤럴드경제브라질 대법원, ...</t>
-        </is>
-      </c>
-      <c r="F147" s="3" t="inlineStr">
-        <is>
-          <t>연합뉴스</t>
-        </is>
-      </c>
-      <c r="G147" s="3" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE1QYjRyYU1pSUdDc2x4SVotMktwUTRfSk5XTEFIanI1UzVGWHdKeVZlWnpfQThvV3BNbTJ0X2t2SjBUa21UUnVaR0NDVWJGV2QyNlM4ZVM4TlBoY0nSAWBBVV95cUxOaTNpZ0FuR0plZ0k4ZE5GLTBlS2NaTjR2Vkp5M2Y3NExOZ0hoUmJ6cmQ1ZGZTc2l6bHNtbVh2dkZ2QjRZUENiVUlUM1NuQWp1bU9HTUQ3OV95UTJpRnRkcEE?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="148">
-      <c r="A148" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B148" s="2" t="inlineStr">
-        <is>
-          <t>세계/국제</t>
-        </is>
-      </c>
-      <c r="C148" s="2" t="inlineStr">
-        <is>
-          <t>신규 이슈</t>
-        </is>
-      </c>
-      <c r="D148" s="3" t="inlineStr">
-        <is>
-          <t>"오픈AI, 사이버보안업체 '트레일오브비츠' 인수 추진"</t>
-        </is>
-      </c>
-      <c r="E148" s="3" t="inlineStr">
-        <is>
-          <t>(서울=연합뉴스) 이성한 기자 = 오픈AI가 사이버보안 업체인 '트레일 오브 비츠'를 인수하기 위한 협상을 진행하고 있다고 미국 IT전문매체 디...</t>
-        </is>
-      </c>
-      <c r="F148" s="3" t="inlineStr">
-        <is>
-          <t>주요언론</t>
-        </is>
-      </c>
-      <c r="G148" s="3" t="inlineStr">
-        <is>
-          <t>https://www.yna.co.kr/view/AKR20261014042500009</t>
-        </is>
-      </c>
-    </row>
-    <row r="149">
-      <c r="A149" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B149" s="2" t="inlineStr">
-        <is>
-          <t>세계/국제</t>
-        </is>
-      </c>
-      <c r="C149" s="2" t="inlineStr">
-        <is>
-          <t>🔥 [언론사 집중 보도 (5개사)]</t>
-        </is>
-      </c>
-      <c r="D149" s="3" t="inlineStr">
-        <is>
-          <t>앤트로픽, 14일 공식 재무상황 공개</t>
-        </is>
-      </c>
-      <c r="E149" s="3" t="inlineStr">
-        <is>
-          <t>(서울=연합뉴스) 주종국 기자 = 기업공개(IPO)를 준비 중인 인공지능(AI) 모델 개발 기업 앤트로픽이 14일(이하 현지시간) 기관투자가들과...</t>
-        </is>
-      </c>
-      <c r="F149" s="3" t="inlineStr">
-        <is>
-          <t>주요언론</t>
-        </is>
-      </c>
-      <c r="G149" s="3" t="inlineStr">
-        <is>
-          <t>https://www.yna.co.kr/view/AKR20261014050400009</t>
-        </is>
-      </c>
-    </row>
-    <row r="150">
-      <c r="A150" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B150" s="2" t="inlineStr">
-        <is>
-          <t>세계/국제</t>
-        </is>
-      </c>
-      <c r="C150" s="2" t="inlineStr">
-        <is>
-          <t>신규 이슈</t>
-        </is>
-      </c>
-      <c r="D150" s="3" t="inlineStr">
-        <is>
-          <t>국방비 연 112조원 쓰고도 난타당하는 사우디…"지킬 게 많다"</t>
-        </is>
-      </c>
-      <c r="E150" s="3" t="inlineStr">
-        <is>
-          <t>(서울=연합뉴스) 임화섭 기자 = 사우디아라비아는 막대한 국방비 지출이 무색하게도 최근 예멘 후티 반군이 쏘는 미사일과 드론에 공항, 정유소, ...</t>
-        </is>
-      </c>
-      <c r="F150" s="3" t="inlineStr">
-        <is>
-          <t>주요언론</t>
-        </is>
-      </c>
-      <c r="G150" s="3" t="inlineStr">
-        <is>
-          <t>https://www.yna.co.kr/view/AKR20261014046300009</t>
-        </is>
-      </c>
-    </row>
-    <row r="151">
-      <c r="A151" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B151" s="2" t="inlineStr">
-        <is>
-          <t>세계/국제</t>
-        </is>
-      </c>
-      <c r="C151" s="2" t="inlineStr">
-        <is>
-          <t>🔥 [언론사 집중 보도 (3개사)]</t>
-        </is>
-      </c>
-      <c r="D151" s="3" t="inlineStr">
-        <is>
-          <t>다저스 감독 "오타니 3차전도 출전"…선발 제외 가능성 일축(종합)</t>
-        </is>
-      </c>
-      <c r="E151" s="3" t="inlineStr">
-        <is>
-          <t>(서울=연합뉴스) 천병혁 기자 = 미국프로야구 메이저리그(MLB) 로스앤젤레스 다저스가 간판스타 오타니 쇼헤이(32)에 대한 신뢰를 재확인했다.</t>
-        </is>
-      </c>
-      <c r="F151" s="3" t="inlineStr">
-        <is>
-          <t>주요언론</t>
-        </is>
-      </c>
-      <c r="G151" s="3" t="inlineStr">
-        <is>
-          <t>https://www.yna.co.kr/view/AKR20261014019651007</t>
-        </is>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B152" s="2" t="inlineStr">
-        <is>
-          <t>세계/국제</t>
-        </is>
-      </c>
-      <c r="C152" s="2" t="inlineStr">
-        <is>
-          <t>신규 이슈</t>
-        </is>
-      </c>
-      <c r="D152" s="3" t="inlineStr">
-        <is>
-          <t>베트남에 'K-문화유산 보존법' 전한다…22일까지 현지 교육</t>
-        </is>
-      </c>
-      <c r="E152" s="3" t="inlineStr">
-        <is>
-          <t>(서울=연합뉴스) 김예나 기자 = 한국의 문화유산 보존과학 전문가들이 베트남 현지에서 문화유산 보존·관리 노하우를 전한다.</t>
-        </is>
-      </c>
-      <c r="F152" s="3" t="inlineStr">
-        <is>
-          <t>주요언론</t>
-        </is>
-      </c>
-      <c r="G152" s="3" t="inlineStr">
-        <is>
-          <t>https://www.yna.co.kr/view/AKR20261014042800005</t>
-        </is>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B153" s="2" t="inlineStr">
-        <is>
-          <t>세계/국제</t>
-        </is>
-      </c>
-      <c r="C153" s="2" t="inlineStr">
-        <is>
-          <t>신규 이슈</t>
-        </is>
-      </c>
-      <c r="D153" s="3" t="inlineStr">
-        <is>
-          <t>세레브라스 CEO "데이터센터 반발은 공포 마케팅 탓"</t>
-        </is>
-      </c>
-      <c r="E153" s="3" t="inlineStr">
-        <is>
-          <t>(샌프란시스코=연합뉴스) 권영전 특파원 = 엔비디아 대항마로 꼽히는 인공지능(AI) 칩 개발사 세레브라스의 앤드루 펠드먼 최고경영자(CEO)는 ...</t>
-        </is>
-      </c>
-      <c r="F153" s="3" t="inlineStr">
-        <is>
-          <t>주요언론</t>
-        </is>
-      </c>
-      <c r="G153" s="3" t="inlineStr">
-        <is>
-          <t>https://www.yna.co.kr/view/AKR20261014022500091</t>
-        </is>
-      </c>
-    </row>
-    <row r="154">
-      <c r="A154" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B154" s="2" t="inlineStr">
-        <is>
-          <t>IT/과학/신상품</t>
-        </is>
-      </c>
-      <c r="C154" s="2" t="inlineStr">
-        <is>
-          <t>연결 이슈 (후속)</t>
-        </is>
-      </c>
-      <c r="D154" s="3" t="inlineStr">
-        <is>
-          <t>NASA 화성 로버, 45.22㎞ 주행 신기록…마라톤 풀코스보다 더 달려 [여기는 화성]</t>
-        </is>
-      </c>
-      <c r="E154" s="3" t="inlineStr">
-        <is>
-          <t>NASA 화성 로버, 45.22㎞ 주행 신기록…마라톤 풀코스보다 더 달려 [여기는 화성]  지디넷코리아화성에서 45.2km…퍼시비런스, 지구 밖 천체 주행 신기록  한겨레NASA 화성탐사 로버 퍼서비어런스, 지구밖 최장 주행  연합뉴스화성서 45.2㎞ 달린 퍼서비어런스… 지구 밖 로버 ...</t>
-        </is>
-      </c>
-      <c r="F154" s="3" t="inlineStr">
-        <is>
-          <t>지디넷코리아</t>
-        </is>
-      </c>
-      <c r="G154" s="3" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiVkFVX3lxTE1sV0ZxS09JU05rdnJhclRvVlFwbFR6X1p1ZWQ1WnFxSFdic1VzZXdubHhGVmhyVHpEaEhQNk1oQWsxbWQ3cXQ0akp1cldsR3A3RWR4TEdR?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="155">
-      <c r="A155" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B155" s="2" t="inlineStr">
-        <is>
-          <t>IT/과학/신상품</t>
-        </is>
-      </c>
-      <c r="C155" s="2" t="inlineStr">
-        <is>
-          <t>신규 이슈</t>
-        </is>
-      </c>
-      <c r="D155" s="3" t="inlineStr">
-        <is>
-          <t>XBOX, AI 에이전트와 게임 디컴파일을 탐구하는 XBOX LABS 출범</t>
-        </is>
-      </c>
-      <c r="E155" s="3" t="inlineStr">
-        <is>
-          <t>XBOX, AI 에이전트와 게임 디컴파일을 탐구하는 XBOX LABS 출범  Unite.AI엑스박스, 신기술 실험조직 ‘엑스박스 랩스’ 출범  지디넷코리아게임 넘어 디즈니처럼… MS, 엑스박스 엔터 사업부 ‘XP’ 신설  IT조선Xbox, 영화, TV, 라이브 이벤트 및 소비재를 전담하...</t>
-        </is>
-      </c>
-      <c r="F155" s="3" t="inlineStr">
-        <is>
-          <t>Unite.AI</t>
-        </is>
-      </c>
-      <c r="G155" s="3" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxPV1A1WUZhSVlvQnZxSlNLeG1xZFFROHVKVzc5YkJxTFVnVnR4Q0x4TS1GdXJ0QUEtOW54Ym1JaWVfVmlUZTNoWlZWVlp5SEhfaXo1cGpwbW1ESHhoUXhLLWJubXZRbW1KX1FnZnlWa190Y1padmc3bG04NGxYenp4dHFKUEFGbi1JVHRlaTdhTEJZWFlhMmc?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="156">
-      <c r="A156" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B156" s="2" t="inlineStr">
-        <is>
-          <t>IT/과학/신상품</t>
-        </is>
-      </c>
-      <c r="C156" s="2" t="inlineStr">
-        <is>
-          <t>🔥 [언론사 집중 보도 (3개사)]</t>
-        </is>
-      </c>
-      <c r="D156" s="3" t="inlineStr">
-        <is>
-          <t>[이슈] 컬렉터스 에디션인데 게임이 없다?</t>
-        </is>
-      </c>
-      <c r="E156" s="3" t="inlineStr">
-        <is>
-          <t>[이슈] 컬렉터스 에디션인데 게임이 없다?  인벤</t>
-        </is>
-      </c>
-      <c r="F156" s="3" t="inlineStr">
-        <is>
-          <t>인벤</t>
-        </is>
-      </c>
-      <c r="G156" s="3" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiXkFVX3lxTE1WV3lvcVpSZTVFQ0lzNTZob1RNYVFmNUwwMGFVSHFnSWRQZndnNlhCdDF0T1cwSm5xbG9MUnl1dUVPelVNa1NrVThZcFRhWWxMQmVWd043NlhnU2JZRmc?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="157">
-      <c r="A157" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B157" s="2" t="inlineStr">
-        <is>
-          <t>IT/과학/신상품</t>
-        </is>
-      </c>
-      <c r="C157" s="2" t="inlineStr">
-        <is>
-          <t>🔥 [언론사 집중 보도 (3개사)]</t>
-        </is>
-      </c>
-      <c r="D157" s="3" t="inlineStr">
-        <is>
-          <t>메트로 2039 예약 판매가 시작되었으며, 동시에 컬렉터스 에디션 출시 소식도 발표되었습니다.</t>
-        </is>
-      </c>
-      <c r="E157" s="3" t="inlineStr">
-        <is>
-          <t>메트로 2039 예약 판매가 시작되었으며, 동시에 컬렉터스 에디션 출시 소식도 발표되었습니다.  GameGPU</t>
-        </is>
-      </c>
-      <c r="F157" s="3" t="inlineStr">
-        <is>
-          <t>GameGPU</t>
-        </is>
-      </c>
-      <c r="G157" s="3" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiqwFBVV95cUxPTXZTOVBsSVAyaXBaOW1DdmktV285RVpQbDlveGs3NUVnNkFDMlBVWFBSQXg0UWhBNjJuTG1HWjZkRmgteDk4aGtwYVdIUHNObFRyUGRabnUxY0F5RXgxOTMzN1FrNTU4Y3IzS0NjVXJPSFROY1MwUk1HSEtTekFRZk9GTHJOY2dNTUY1bFRaWnlEMm03NUE0SjNCbG1YdS0tajI1QUJFXzkyR2s?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="158">
-      <c r="A158" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B158" s="2" t="inlineStr">
-        <is>
-          <t>IT/과학/신상품</t>
-        </is>
-      </c>
-      <c r="C158" s="2" t="inlineStr">
-        <is>
-          <t>🔥 [언론사 집중 보도 (3개사)]</t>
-        </is>
-      </c>
-      <c r="D158" s="3" t="inlineStr">
-        <is>
-          <t>독성 약품 투입량 5분의 1로 낮춰···'청정 원전 해체' 가능성</t>
-        </is>
-      </c>
-      <c r="E158" s="3" t="inlineStr">
-        <is>
-          <t>독성 약품 투입량 5분의 1로 낮춰···'청정 원전 해체' 가능성  이데일리</t>
-        </is>
-      </c>
-      <c r="F158" s="3" t="inlineStr">
-        <is>
-          <t>이데일리</t>
-        </is>
-      </c>
-      <c r="G158" s="3" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxNNGxxUG1PSF8taVVIQXp0bGJteS1Ga3NkdkdmOGRqbEpBbGxaSDYzMTJDZUxPRjcyNTRvUzdiSWRBSlJaOFZPYTVkS3pZMEVrQTN5ZVlRYjF1NDdxTElsU1c0SG0xRnlJTU01SEhtRS1NYWZva0dWYVZWVlhWZ2c0bw?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="159">
-      <c r="A159" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B159" s="2" t="inlineStr">
-        <is>
-          <t>IT/과학/신상품</t>
-        </is>
-      </c>
-      <c r="C159" s="2" t="inlineStr">
-        <is>
-          <t>🔥 [언론사 집중 보도 (3개사)]</t>
-        </is>
-      </c>
-      <c r="D159" s="3" t="inlineStr">
-        <is>
-          <t>“죽으면 전 재산 증발”…요즘 세상보다 더 살벌한 생존 게임 ‘빌로우 더 스톤’ 11/17 정식 출시</t>
-        </is>
-      </c>
-      <c r="E159" s="3" t="inlineStr">
-        <is>
-          <t>“죽으면 전 재산 증발”…요즘 세상보다 더 살벌한 생존 게임 ‘빌로우 더 스톤’ 11/17 정식 출시  헝그리앱</t>
-        </is>
-      </c>
-      <c r="F159" s="3" t="inlineStr">
-        <is>
-          <t>헝그리앱</t>
-        </is>
-      </c>
-      <c r="G159" s="3" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMidEFVX3lxTE9xUFY5bFV3Q1hidUJJVy1TajdHbnc5VjVqQzYwaEVUMVBIVUFvN1dvcjhFWkdUZkFvMnY0cFF2djRPcTNCS3BoOEdPWGF0Q0F1LXpnYzZWUXF6cW85RHo5UWxFU2stZklYNkc2WFRPSTJyWGJV?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="160">
-      <c r="A160" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B160" s="2" t="inlineStr">
-        <is>
-          <t>IT/과학/신상품</t>
-        </is>
-      </c>
-      <c r="C160" s="2" t="inlineStr">
-        <is>
-          <t>🔥 [언론사 집중 보도 (3개사)]</t>
-        </is>
-      </c>
-      <c r="D160" s="3" t="inlineStr">
-        <is>
-          <t>파페 산의 한국 식료점, 파리에서 비밀리에 열리는 콜 오브 듀티 팝업을 선보인다</t>
-        </is>
-      </c>
-      <c r="E160" s="3" t="inlineStr">
-        <is>
-          <t>파페 산의 한국 식료점, 파리에서 비밀리에 열리는 콜 오브 듀티 팝업을 선보인다  Sortir à Paris콜오브듀티: 모던 워페어4, 캠페인에 이어 'DMZ'도 미리 한다  인벤콜 오브 듀티: 모던 워페어 4의 DMZ 모드에 대해 알아야 할 모든 것  PlayStationDMZ 모드에...</t>
-        </is>
-      </c>
-      <c r="F160" s="3" t="inlineStr">
-        <is>
-          <t>Sortir à Paris</t>
-        </is>
-      </c>
-      <c r="G160" s="3" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMi9gFBVV95cUxOS3dMSHNXSGFZaV9uV3d0ZTFLaldzWG9zcW1XRnBwczRpaUladnZWcjNqZU5DeWJwV2lDamtGY1FVek1SQkdnNW03ZVV5ckpOMzZMWFFNRjhtekVKMHRzY3RKNVVZQ1dEZE80cU1SZnUxWFhCUDJQY0FBcEVvY0MxSEM3c01uX25MT1RWR0FiaXNoc0ZPVkVtSHFxWF9Mc2FHU2VrV2RDeWpZeFVOc1NOTmdEeTdMZEItWjFSNXJCNWZuOFdsT3IwQVBIcXFZTkVyWXNCcTE4ZzRPejkzQU02cldhalZnREprSkR4QzlFZE5vRHNKN1E?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="161">
-      <c r="A161" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B161" s="2" t="inlineStr">
-        <is>
-          <t>IT/과학/신상품</t>
-        </is>
-      </c>
-      <c r="C161" s="2" t="inlineStr">
-        <is>
-          <t>연결 이슈 (후속)</t>
-        </is>
-      </c>
-      <c r="D161" s="3" t="inlineStr">
-        <is>
-          <t>남극 얼음에 탐지기 심어 우주 중성미자 잡았다…할젠 교수 노벨 물리학상 수상</t>
-        </is>
-      </c>
-      <c r="E161" s="3" t="inlineStr">
-        <is>
-          <t>남극 얼음에 탐지기 심어 우주 중성미자 잡았다…할젠 교수 노벨 물리학상 수상  교수신문남극 빙하를 거대 망원경으로...'유령 입자'로 노벨상  YTN 사이언스[금주의인물] 프란시스 할전, ‘노벨 물리학상’ 단독 수상  한국아이닷컴벨기에 13년 만에 또 노벨 물리학상…과학 강소국 저력 과...</t>
-        </is>
-      </c>
-      <c r="F161" s="3" t="inlineStr">
-        <is>
-          <t>교수신문</t>
-        </is>
-      </c>
-      <c r="G161" s="3" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiZ0FVX3lxTE92WF9yMDViT0RjQjNiWHA0c19DVnBPSHRnRGdWbXhJRElzMEZpM05Fdmd2dlJreURYS2V4VGtwMVBhSGozdDZFNkRPMVViMkd5dmxGbXRUNmp5cEg0ZkhkVDlPN3ptclk?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="162">
-      <c r="A162" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B162" s="2" t="inlineStr">
-        <is>
-          <t>IT/과학/신상품</t>
-        </is>
-      </c>
-      <c r="C162" s="2" t="inlineStr">
-        <is>
-          <t>연결 이슈 (후속)</t>
-        </is>
-      </c>
-      <c r="D162" s="3" t="inlineStr">
-        <is>
-          <t>[리뷰] 채찍으로 날아다니는 화려한 악마성, '캐슬바니아: 벨몬트의 저주'</t>
-        </is>
-      </c>
-      <c r="E162" s="3" t="inlineStr">
-        <is>
-          <t>[리뷰] 채찍으로 날아다니는 화려한 악마성, '캐슬바니아: 벨몬트의 저주'  디스이즈게임캐슬바니아신작 '벨몬트의 저주' 10월 15일 출시, 무료 데모 이미 공개  디지털포커스캐슬바니아: 벨몬트의 저주 - 리뷰  IGN Korea18년 만에 정사로 복귀, 캐슬바니아: 벨몬트의 저주  게...</t>
-        </is>
-      </c>
-      <c r="F162" s="3" t="inlineStr">
-        <is>
-          <t>디스이즈게임</t>
-        </is>
-      </c>
-      <c r="G162" s="3" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiVEFVX3lxTE45bEhmaWlTVDMxUW1hMjV6RzltOFRHeV9VZTdoc0p6am5JcUJiY1NBaGVmeFYyZEk3WHUydWJRcGlUS0ZpWWk0YlBwclJrcVEzZWJXMg?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="163">
-      <c r="A163" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B163" s="2" t="inlineStr">
-        <is>
-          <t>IT/과학/신상품</t>
-        </is>
-      </c>
-      <c r="C163" s="2" t="inlineStr">
-        <is>
-          <t>신규 이슈</t>
-        </is>
-      </c>
-      <c r="D163" s="3" t="inlineStr">
-        <is>
-          <t>Mafia Definitive Edition이 10월 22일까지 PlayStation Store에서 85% 할인된 가격으로 판매됩니다.</t>
-        </is>
-      </c>
-      <c r="E163" s="3" t="inlineStr">
-        <is>
-          <t>Mafia Definitive Edition이 10월 22일까지 PlayStation Store에서 85% 할인된 가격으로 판매됩니다.  GameGPUMafia III는 현재 고화질 HDR을 지원하며, 향후 DLSS 및 FSR도 지원할 예정입니다.  GameGPU마피아 3가 버그 수정 ...</t>
-        </is>
-      </c>
-      <c r="F163" s="3" t="inlineStr">
-        <is>
-          <t>GameGPU</t>
-        </is>
-      </c>
-      <c r="G163" s="3" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxNZUVrXzhrQmRqZE1Ia0RzM2lJaG5MYmdSdVZpQXNkMkNnbE15Vmt5eGw3REFBYlExOGt2em5nMGVUN2Y4dXBwUllnUk9Oa280SGlEYzBSUjRSMjhKMkNHUUFHZERDZDN5My1rbGtNTGotMm90M0tLanhzazYwLW1CaXBQM3JBR0FkQW9DWENNYXdkaWExYzgybTVGdk9HVFZRVTV6Z0NzdkdIM21GdWhVRzN3WQ?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="164">
-      <c r="A164" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B164" s="2" t="inlineStr">
-        <is>
-          <t>IT/과학/신상품</t>
-        </is>
-      </c>
-      <c r="C164" s="2" t="inlineStr">
-        <is>
-          <t>신규 이슈</t>
-        </is>
-      </c>
-      <c r="D164" s="3" t="inlineStr">
-        <is>
-          <t>새로운 보도에 따르면 소니는 플레이스테이션 6를 세 가지 구성으로 출시할 계획입니다.</t>
-        </is>
-      </c>
-      <c r="E164" s="3" t="inlineStr">
-        <is>
-          <t>새로운 보도에 따르면 소니는 플레이스테이션 6를 세 가지 구성으로 출시할 계획입니다.  GameGPU플스5 소니의 잇단 '반 게이머' 정책에 소비자 불만 급증  글로벌EPS5 탈옥 스토어까지...소니 향한 게이머들의 '반란' 왜?  게임플“어차피 사라질 운명” 사이버커넥트2 대표 디스크...</t>
-        </is>
-      </c>
-      <c r="F164" s="3" t="inlineStr">
-        <is>
-          <t>GameGPU</t>
-        </is>
-      </c>
-      <c r="G164" s="3" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMitAFBVV95cUxOdWJQZGg0bDQ2RTNsbjlDM0pIZnlFYmZnYnJza21KckdWWHVkZXYzRmhaaFFteHYzWEQwOG9GZ0wyV3QtbHE1ZktCQ29jczF6c1ZPWkJydTBjRE4zLWxRdGRlWi1OUjViajBsb1gzLWhPUVV6ZmR0d2Y2dXlNRnhvQzVjSjdDNmwtTG1UU0NDcmp6LVBPMzV4djBEVFRsSmdCaTRtWGwxbV9lVDRaYVpmMnU3MVU?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="165">
-      <c r="A165" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B165" s="2" t="inlineStr">
-        <is>
-          <t>IT/과학/신상품</t>
-        </is>
-      </c>
-      <c r="C165" s="2" t="inlineStr">
-        <is>
-          <t>신규 이슈</t>
-        </is>
-      </c>
-      <c r="D165" s="3" t="inlineStr">
-        <is>
-          <t>[속초소식] 착한가격업소 2곳 신규 선정…16일까지 신청</t>
-        </is>
-      </c>
-      <c r="E165" s="3" t="inlineStr">
-        <is>
-          <t>(속초=연합뉴스) ▲ 착한가격업소 2곳 신규 선정…16일까지 신청 = 강원 속초시는 오는 16일까지 '2026년 2차 착한가격업소' 신규 지정 ...</t>
-        </is>
-      </c>
-      <c r="F165" s="3" t="inlineStr">
-        <is>
-          <t>주요언론</t>
-        </is>
-      </c>
-      <c r="G165" s="3" t="inlineStr">
-        <is>
-          <t>https://www.yna.co.kr/view/AKR20261014054400062</t>
-        </is>
-      </c>
-    </row>
-    <row r="166">
-      <c r="A166" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B166" s="2" t="inlineStr">
-        <is>
-          <t>IT/과학/신상품</t>
-        </is>
-      </c>
-      <c r="C166" s="2" t="inlineStr">
-        <is>
-          <t>신규 이슈</t>
-        </is>
-      </c>
-      <c r="D166" s="3" t="inlineStr">
-        <is>
-          <t>소노인터내셔널, 비발디파크 스키장 '26·27 시즌패스' 판매</t>
-        </is>
-      </c>
-      <c r="E166" s="3" t="inlineStr">
-        <is>
-          <t>(서울=연합뉴스) 구정모 기자 = 소노인터내셔널은 2026∼2027년 겨울 시즌을 맞아 비발디파크 스키장 시즌패스를 판매한다고 14일 밝혔다.</t>
-        </is>
-      </c>
-      <c r="F166" s="3" t="inlineStr">
-        <is>
-          <t>주요언론</t>
-        </is>
-      </c>
-      <c r="G166" s="3" t="inlineStr">
-        <is>
-          <t>https://www.yna.co.kr/view/AKR20261014049100030</t>
-        </is>
-      </c>
-    </row>
-    <row r="167">
-      <c r="A167" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B167" s="2" t="inlineStr">
-        <is>
-          <t>IT/과학/신상품</t>
-        </is>
-      </c>
-      <c r="C167" s="2" t="inlineStr">
-        <is>
-          <t>신규 이슈</t>
-        </is>
-      </c>
-      <c r="D167" s="3" t="inlineStr">
-        <is>
-          <t>파라다이스, 인천서 '넥스트 가스트로노미' 포럼…ESG 실천 모색</t>
-        </is>
-      </c>
-      <c r="E167" s="3" t="inlineStr">
-        <is>
-          <t>(서울=연합뉴스) 이상서 기자 = 파라다이스[034230]그룹은 지난 12일 인천 파라다이스시티에서 글로벌 미식 가이드인 '라 리스트 2027 ...</t>
-        </is>
-      </c>
-      <c r="F167" s="3" t="inlineStr">
-        <is>
-          <t>주요언론</t>
-        </is>
-      </c>
-      <c r="G167" s="3" t="inlineStr">
-        <is>
-          <t>https://www.yna.co.kr/view/AKR20261014048500030</t>
-        </is>
-      </c>
-    </row>
-    <row r="168">
-      <c r="A168" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B168" s="2" t="inlineStr">
-        <is>
-          <t>IT/과학/신상품</t>
-        </is>
-      </c>
-      <c r="C168" s="2" t="inlineStr">
-        <is>
-          <t>신규 이슈</t>
-        </is>
-      </c>
-      <c r="D168" s="3" t="inlineStr">
-        <is>
-          <t>신한은행, 모바일 신분증 발급 서비스 개시</t>
-        </is>
-      </c>
-      <c r="E168" s="3" t="inlineStr">
-        <is>
-          <t>(서울=연합뉴스) 한지훈 기자 = 신한은행은 14일 신한 슈퍼SOL에서 모바일 신분증을 발급하는 서비스를 시작했다.</t>
-        </is>
-      </c>
-      <c r="F168" s="3" t="inlineStr">
-        <is>
-          <t>주요언론</t>
-        </is>
-      </c>
-      <c r="G168" s="3" t="inlineStr">
-        <is>
-          <t>https://www.yna.co.kr/view/AKR20261014052900002</t>
-        </is>
-      </c>
-    </row>
-    <row r="169">
-      <c r="A169" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B169" s="2" t="inlineStr">
-        <is>
-          <t>IT/과학/신상품</t>
-        </is>
-      </c>
-      <c r="C169" s="2" t="inlineStr">
-        <is>
-          <t>신규 이슈</t>
-        </is>
-      </c>
-      <c r="D169" s="3" t="inlineStr">
-        <is>
-          <t>[인사] 한국방송광고진흥공사</t>
-        </is>
-      </c>
-      <c r="E169" s="3" t="inlineStr">
-        <is>
-          <t>▲ 상임감사 이수호 (서울=연합뉴스)</t>
-        </is>
-      </c>
-      <c r="F169" s="3" t="inlineStr">
-        <is>
-          <t>주요언론</t>
-        </is>
-      </c>
-      <c r="G169" s="3" t="inlineStr">
-        <is>
-          <t>https://www.yna.co.kr/view/AKR20261014051300017</t>
-        </is>
-      </c>
-    </row>
-    <row r="170">
-      <c r="A170" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B170" s="2" t="inlineStr">
-        <is>
-          <t>IT/과학/신상품</t>
-        </is>
-      </c>
-      <c r="C170" s="2" t="inlineStr">
-        <is>
-          <t>신규 이슈</t>
-        </is>
-      </c>
-      <c r="D170" s="3" t="inlineStr">
-        <is>
-          <t>위메이드, 서틱과 위믹스 3.0 보안 강화…최대 1만 달러 포상</t>
-        </is>
-      </c>
-      <c r="E170" s="3" t="inlineStr">
-        <is>
-          <t>(서울=연합뉴스) 김주환 기자 = 위메이드[112040]의 위믹스 재단은 미국 소재 블록체인 보안 기업 서틱(CertiK)과 함께 블록체인 메인...</t>
-        </is>
-      </c>
-      <c r="F170" s="3" t="inlineStr">
-        <is>
-          <t>주요언론</t>
-        </is>
-      </c>
-      <c r="G170" s="3" t="inlineStr">
-        <is>
-          <t>https://www.yna.co.kr/view/AKR20261014040300017</t>
-        </is>
-      </c>
-    </row>
-    <row r="171">
-      <c r="A171" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B171" s="2" t="inlineStr">
-        <is>
-          <t>연예/대중문화</t>
-        </is>
-      </c>
-      <c r="C171" s="2" t="inlineStr">
-        <is>
-          <t>🔥 [언론사 집중 보도 (5개사)]</t>
-        </is>
-      </c>
-      <c r="D171" s="3" t="inlineStr">
-        <is>
-          <t>이수만 “새 문 열겠다” 3년 만에 K팝 복귀…보이·걸그룹 동시 공개</t>
-        </is>
-      </c>
-      <c r="E171" s="3" t="inlineStr">
-        <is>
-          <t>이수만 “새 문 열겠다” 3년 만에 K팝 복귀…보이·걸그룹 동시 공개  국민일보이수만, 유영진과 돌아왔다…24명 아이돌로 K팝 흔들까  한겨레A20 LITE의 데뷔 쇼  뉴시스[ET포토] A2O 라이트 라다, '호수에서 백조가 발레하듯'  전자신문'이수만 표' 새 바람…A2O 소울·A2...</t>
-        </is>
-      </c>
-      <c r="F171" s="3" t="inlineStr">
-        <is>
-          <t>국민일보</t>
-        </is>
-      </c>
-      <c r="G171" s="3" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxOamxndXRINVdISDF1N2VpMUdjM0R4dmVYR09fazVNYzExZTh1QXh6bk1DWEtUV21VcFhNTktOei0xYlp6aTlSYkZ5VjJ1WjE3ZUdzRGdmZTRjVEQxbmpuT0dhVkp0X3BzNDBhaHlfNHRfUDhVSHZLT0VFXy01REtPeEh0RHg4T3VPX3pyRWRna2Vzdw?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="172">
-      <c r="A172" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B172" s="2" t="inlineStr">
-        <is>
-          <t>연예/대중문화</t>
-        </is>
-      </c>
-      <c r="C172" s="2" t="inlineStr">
-        <is>
-          <t>🔥 [언론사 집중 보도 (5개사)]</t>
-        </is>
-      </c>
-      <c r="D172" s="3" t="inlineStr">
-        <is>
-          <t>'나를 충전해줘', 공개 3일 만에 글로벌 톱10 비영어 쇼 3위</t>
-        </is>
-      </c>
-      <c r="E172" s="3" t="inlineStr">
-        <is>
-          <t>'나를 충전해줘', 공개 3일 만에 글로벌 톱10 비영어 쇼 3위  뉴스핌차우민, '최애의 사원' 이어 '나를 충전해줘'까지…로맨스 연타 흥행 예고  YTN김영광·채수빈 ‘나를 충전해줘’, 공개 3일 만에 넷플릭스 글로벌 비영어권 3위  스포츠동아‘국민엄마’ 김미경, 백발됐다…이번엔 재...</t>
-        </is>
-      </c>
-      <c r="F172" s="3" t="inlineStr">
-        <is>
-          <t>뉴스핌</t>
-        </is>
-      </c>
-      <c r="G172" s="3" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiXEFVX3lxTE1PUG5VSTdieXRQZ0lrVmJGVWZieHdqRjhqYkZieWZ1cV9SN3Y2ZlBFdlBodzNORkNtbjh2Q1ZReklxQy1YR2l0aS1oYkROSDA1WVNkNjV3VXZTbFdm?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="173">
-      <c r="A173" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B173" s="2" t="inlineStr">
-        <is>
-          <t>연예/대중문화</t>
-        </is>
-      </c>
-      <c r="C173" s="2" t="inlineStr">
-        <is>
-          <t>🔥 [언론사 집중 보도 (3개사)]</t>
-        </is>
-      </c>
-      <c r="D173" s="3" t="inlineStr">
-        <is>
-          <t>[스브스夜] '틈만나면' 남지현, "전파견문록 출신, 출연 이후 드라마 캐스팅"…유재석 '사과 방송' 예고</t>
-        </is>
-      </c>
-      <c r="E173" s="3" t="inlineStr">
-        <is>
-          <t>[스브스夜] '틈만나면' 남지현, "전파견문록 출신, 출연 이후 드라마 캐스팅"…유재석 '사과 방송' 예고  news.sbs.co.krGoogle 뉴스에서 헤드라인 및 의견 더보기</t>
-        </is>
-      </c>
-      <c r="F173" s="3" t="inlineStr">
-        <is>
-          <t>news.sbs.co.kr</t>
-        </is>
-      </c>
-      <c r="G173" s="3" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMihgFBVV95cUxPZ202a3RsUTFDVEJxU1A3eGpIT3lDZlhJbmdhank3dk8tRlVzVnVIcHZlUG9hWjRiSGxIdEpJVVZ5bjFHVUxvV1FkSlp0S2xCVWNQYUlhS2JYclZFampIcHRlVnlONGY0Wl9PSjBVR0RmNUozOFhQRGRHOUFIOE9XN1NDeTF6Zw?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="174">
-      <c r="A174" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B174" s="2" t="inlineStr">
-        <is>
-          <t>연예/대중문화</t>
-        </is>
-      </c>
-      <c r="C174" s="2" t="inlineStr">
-        <is>
-          <t>🔥 [언론사 집중 보도 (4개사)]</t>
-        </is>
-      </c>
-      <c r="D174" s="3" t="inlineStr">
-        <is>
-          <t>시크릿, 17주년 자축…송지은, 박위 논란 불똥 속 '침묵' - 머니투데이</t>
-        </is>
-      </c>
-      <c r="E174" s="3" t="inlineStr">
-        <is>
-          <t>시크릿, 17주년 자축…송지은, 박위 논란 불똥 속 '침묵' - 머니투데이  머니투데이'♥박위' 발목잡힌 송지은-잘나가는 한선화-3크릿, 엇갈린 시크릿 17주년[SC이슈]  조선일보전효성, 데뷔 17주년 생일 카페에서 전한 팬 사랑 다짐  톱스타뉴스시크릿, 송지은 없이 17주년 맞았다…...</t>
-        </is>
-      </c>
-      <c r="F174" s="3" t="inlineStr">
-        <is>
-          <t>머니투데이</t>
-        </is>
-      </c>
-      <c r="G174" s="3" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMic0FVX3lxTFBuTXhMcGtwMGVIR3ZvQkVMMkh5Wjc1TDFNNUloenNzY1kxZVVNYnJrNXMxVjVvSjZrLUtMT2IzVVNIVndpRF9IdnItcEhhQjQ1RFVZN0xTWEZJa1owNWgwcUZ1ZGxjQlpGNG1hRTB6NHpkNVHSAXhBVV95cUxPNkptTVNtRWZxWDVYLU1NNXdzVTYybVVRWC1zYzhuYlpzQVh6dEluMEFRWVNSNUQ1b2VRZWlFbkt2ZDk1U0ZOa2RISUxMaVJxanRZT2pvRlZJbEVCLW83NE9DQ0NVenhWWUtWNVczeXJ3Mk9ZS01sUXY?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="175">
-      <c r="A175" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B175" s="2" t="inlineStr">
-        <is>
-          <t>연예/대중문화</t>
-        </is>
-      </c>
-      <c r="C175" s="2" t="inlineStr">
-        <is>
-          <t>신규 이슈</t>
-        </is>
-      </c>
-      <c r="D175" s="3" t="inlineStr">
-        <is>
-          <t>국힘 달성 군의회와 당원, \'암살자(들)\'영화 상영중지 촉구</t>
-        </is>
-      </c>
-      <c r="E175" s="3" t="inlineStr">
-        <is>
-          <t>국힘 달성 군의회와 당원, \'암살자(들)\'영화 상영중지 촉구  세명일보‘암살자(들)’ 실제 기자 “우리 패던 중정…영화가 잘 그려”  한겨레‘암살자(들)’ 논란, 하다하다 ‘100분 토론’ 간다  스포츠경향‘기립박수받은 배우가 위협받고 있다’ 외신도 주목  JTBC[시론] 권력자의 ...</t>
-        </is>
-      </c>
-      <c r="F175" s="3" t="inlineStr">
-        <is>
-          <t>세명일보</t>
-        </is>
-      </c>
-      <c r="G175" s="3" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTFBnSG5LUDhaVXZFcDR6ZE9fbUdhMDN6MnpmN0p3eUF0YUZLQUR4YkZIWldSMTloUm9ncWdWd2NEWVNfNkxBU1JwSFNuNG1Lbk1WMWk4YWgzbmszOEVON2hBNnZMaU1SQ3VsSlprTldUcWo?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="176">
-      <c r="A176" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B176" s="2" t="inlineStr">
-        <is>
-          <t>연예/대중문화</t>
-        </is>
-      </c>
-      <c r="C176" s="2" t="inlineStr">
-        <is>
-          <t>신규 이슈</t>
-        </is>
-      </c>
-      <c r="D176" s="3" t="inlineStr">
-        <is>
-          <t>김새론에 “언제 안고 잘 수 있어” 다른 연예인이었다…김수현 미성년 성착취 의혹 해소</t>
-        </is>
-      </c>
-      <c r="E176" s="3" t="inlineStr">
-        <is>
-          <t>김새론에 “언제 안고 잘 수 있어” 다른 연예인이었다…김수현 미성년 성착취 의혹 해소  헤럴드경제김수현 아니었다…"너 안고 잠들 수 있어" 발신자는 연예인 A씨  뉴시스‘누명 벗은’ 김수현 측, 허위사실 유포에 강경 대응…“합의 없이 형사 고소·민사소송”  스포츠동아“언제 안고 잘 수 ...</t>
-        </is>
-      </c>
-      <c r="F176" s="3" t="inlineStr">
-        <is>
-          <t>헤럴드경제</t>
-        </is>
-      </c>
-      <c r="G176" s="3" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiV0FVX3lxTE4wVEI2bnllQmlsZ2JUcmxBQ05mdmpGQnZLVW9ueXpPVTV2Q0VDaE5IX2lKV2tBY3R3NWQ0ZEU1TWMzVTU2RXA2aEt2NHVnSUtvRnhQcktWaw?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="177">
-      <c r="A177" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B177" s="2" t="inlineStr">
-        <is>
-          <t>연예/대중문화</t>
-        </is>
-      </c>
-      <c r="C177" s="2" t="inlineStr">
-        <is>
-          <t>연결 이슈 (후속)</t>
-        </is>
-      </c>
-      <c r="D177" s="3" t="inlineStr">
-        <is>
-          <t>베이비몬스터, 23일 신곡 ‘디저브’로 컴백…“강렬한 에너지”</t>
-        </is>
-      </c>
-      <c r="E177" s="3" t="inlineStr">
-        <is>
-          <t>베이비몬스터, 23일 신곡 ‘디저브’로 컴백…“강렬한 에너지”  KBS 뉴스베이비몬스터, 23일 신곡 '디저브'로 컴백…"강렬한 에너지"  연합뉴스YG 5인조 보이그룹·4인조 걸그룹 데뷔 구체화..양현석 직접 밝혔다 - 조선비즈  Chosunbiz‘가창력 과시’ 베이비몬스터, ‘힙합 노...</t>
-        </is>
-      </c>
-      <c r="F177" s="3" t="inlineStr">
-        <is>
-          <t>KBS 뉴스</t>
-        </is>
-      </c>
-      <c r="G177" s="3" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiZkFVX3lxTE00bjZ2YkUwcmZ3MW1GZjF5dnViZVpNbzdaYmpzSllMYnFpakNidzhMN3hyV0FMVERfcUR4em5pTHcwdkp2YXRYN09PaVBqRm1MbkxIN3ZtSmxzMjZiUEVFWWVqT0t3UQ?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="178">
-      <c r="A178" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B178" s="2" t="inlineStr">
-        <is>
-          <t>연예/대중문화</t>
-        </is>
-      </c>
-      <c r="C178" s="2" t="inlineStr">
-        <is>
-          <t>신규 이슈</t>
-        </is>
-      </c>
-      <c r="D178" s="3" t="inlineStr">
-        <is>
-          <t>맨발로 비스듬히 느릿느릿… 차이밍량·이강생 “기존 영화 지겨워져 걸었다”</t>
-        </is>
-      </c>
-      <c r="E178" s="3" t="inlineStr">
-        <is>
-          <t>맨발로 비스듬히 느릿느릿… 차이밍량·이강생 “기존 영화 지겨워져 걸었다”  문화일보</t>
-        </is>
-      </c>
-      <c r="F178" s="3" t="inlineStr">
-        <is>
-          <t>문화일보</t>
-        </is>
-      </c>
-      <c r="G178" s="3" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiUEFVX3lxTE53dlVHR0diVUc0YTRVMHhBWXFDUXhlUnpIOXVBUVIxZGdtZHNNbG1FR3BST0FwdVAzUVBQY0FqUXUtQ2ZUT28yMGJZbmRHMlJJ?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="179">
-      <c r="A179" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B179" s="2" t="inlineStr">
-        <is>
-          <t>연예/대중문화</t>
-        </is>
-      </c>
-      <c r="C179" s="2" t="inlineStr">
-        <is>
-          <t>신규 이슈</t>
-        </is>
-      </c>
-      <c r="D179" s="3" t="inlineStr">
-        <is>
-          <t>[가요소식] '정엽 밴드' 코스믹 칩스, 2집 '테이스트'</t>
-        </is>
-      </c>
-      <c r="E179" s="3" t="inlineStr">
-        <is>
-          <t>(서울=연합뉴스) 이태수 기자 = ▲ 코스믹 칩스 정규 2집 = 가수 정엽이 결성한 밴드 코스믹 칩스가 14일 오후 6시 두 번째 정규앨범 '테...</t>
-        </is>
-      </c>
-      <c r="F179" s="3" t="inlineStr">
-        <is>
-          <t>주요언론</t>
-        </is>
-      </c>
-      <c r="G179" s="3" t="inlineStr">
-        <is>
-          <t>https://www.yna.co.kr/view/AKR20261014054000005</t>
-        </is>
-      </c>
-    </row>
-    <row r="180">
-      <c r="A180" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B180" s="2" t="inlineStr">
-        <is>
-          <t>연예/대중문화</t>
-        </is>
-      </c>
-      <c r="C180" s="2" t="inlineStr">
-        <is>
-          <t>🔥 [언론사 집중 보도 (3개사)]</t>
-        </is>
-      </c>
-      <c r="D180" s="3" t="inlineStr">
-        <is>
-          <t>KBS '드라마스페셜 2026'…연말까지 단막극 8편 방송</t>
-        </is>
-      </c>
-      <c r="E180" s="3" t="inlineStr">
-        <is>
-          <t>(서울=연합뉴스) 장진리 기자 = KBS는 2TV '드라마스페셜 2026'을 편성해 연말까지 단막극 8편을 방송한다고 14일 밝혔다.</t>
-        </is>
-      </c>
-      <c r="F180" s="3" t="inlineStr">
-        <is>
-          <t>주요언론</t>
-        </is>
-      </c>
-      <c r="G180" s="3" t="inlineStr">
-        <is>
-          <t>https://www.yna.co.kr/view/AKR20261014048100005</t>
-        </is>
-      </c>
-    </row>
-    <row r="181">
-      <c r="A181" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B181" s="2" t="inlineStr">
-        <is>
-          <t>연예/대중문화</t>
-        </is>
-      </c>
-      <c r="C181" s="2" t="inlineStr">
-        <is>
-          <t>연결 이슈 (후속)</t>
-        </is>
-      </c>
-      <c r="D181" s="3" t="inlineStr">
-        <is>
-          <t>베이비몬스터, 23일 신곡 '디저브'로 컴백…"강렬한 에너지"</t>
-        </is>
-      </c>
-      <c r="E181" s="3" t="inlineStr">
-        <is>
-          <t>(서울=연합뉴스) 이태수 기자 = 걸그룹 베이비몬스터가 오는 23일 오후 1시 새 디지털 싱글 '디저브'(DESERVE)를 발매하고 가을 K팝 ...</t>
-        </is>
-      </c>
-      <c r="F181" s="3" t="inlineStr">
-        <is>
-          <t>주요언론</t>
-        </is>
-      </c>
-      <c r="G181" s="3" t="inlineStr">
-        <is>
-          <t>https://www.yna.co.kr/view/AKR20261014047000005</t>
-        </is>
-      </c>
-    </row>
-    <row r="182">
-      <c r="A182" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B182" s="2" t="inlineStr">
-        <is>
-          <t>연예/대중문화</t>
-        </is>
-      </c>
-      <c r="C182" s="2" t="inlineStr">
-        <is>
-          <t>신규 이슈</t>
-        </is>
-      </c>
-      <c r="D182" s="3" t="inlineStr">
-        <is>
-          <t>BTS '아리랑', 스포티파이 50억 스트리밍…올해 발매 최고 기록</t>
-        </is>
-      </c>
-      <c r="E182" s="3" t="inlineStr">
-        <is>
-          <t>(서울=연합뉴스) 이태수 기자 = 그룹 방탄소년단(BTS)의 정규 5집 '아리랑'(ARIRANG)이 세계 최대 음원 플랫폼 스포티파이에서 누적 ...</t>
-        </is>
-      </c>
-      <c r="F182" s="3" t="inlineStr">
-        <is>
-          <t>주요언론</t>
-        </is>
-      </c>
-      <c r="G182" s="3" t="inlineStr">
-        <is>
-          <t>https://www.yna.co.kr/view/AKR20261014039500005</t>
+          <t>https://www.yna.co.kr/view/AKR20261014066300064</t>
         </is>
       </c>
     </row>
@@ -8521,42 +5895,42 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>240,000원</t>
+          <t>236,000원</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>+33,500.0원 (+16.22%)</t>
+          <t>+29,500.0원 (+14.29%)</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>237,500원</t>
+          <t>220,500원</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>257,000원</t>
+          <t>233,500원</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>231,500원</t>
+          <t>229,000원</t>
         </is>
       </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
-          <t>+8.2%</t>
+          <t>+6.0%</t>
         </is>
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>🟢 오늘 단기 매수 (저점 반등)</t>
+          <t>🔴 단기 비중 축소 (악재 주의)</t>
         </is>
       </c>
       <c r="L15" s="3" t="inlineStr">
         <is>
-          <t>RSI 39.3로 단기 과매도 구간 진입, 기술적 반등 노림</t>
+          <t>악재 보도 및 5일 연속 약세로 단기 추가 하락 위험</t>
         </is>
       </c>
       <c r="M15" s="3" t="inlineStr">
@@ -8570,21 +5944,21 @@
         </is>
       </c>
       <c r="O15" s="3" t="n">
-        <v>39.3</v>
+        <v>37</v>
       </c>
       <c r="P15" s="3" t="inlineStr">
         <is>
-          <t>-8.5%</t>
+          <t>-10.0%</t>
         </is>
       </c>
       <c r="Q15" s="3" t="inlineStr">
         <is>
-          <t>52.7%</t>
+          <t>51.3%</t>
         </is>
       </c>
       <c r="R15" s="3" t="inlineStr">
         <is>
-          <t>[속보]홍라희 관장, 아들 이재용 회장에 삼성전자 주식 2.6조 증여 (문화일보)</t>
+          <t>필라델피아 반도체 지수 5일 연속 하락...7월 말 이후 처음 (YTN)</t>
         </is>
       </c>
     </row>
@@ -8611,42 +5985,42 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>1,487,000원</t>
+          <t>1,458,000원</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>+384,000.0원 (+34.81%)</t>
+          <t>+355,000.0원 (+32.18%)</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>1,472,000원</t>
+          <t>1,371,000원</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>1,706,500원</t>
+          <t>1,443,500원</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>1,435,000원</t>
+          <t>1,414,500원</t>
         </is>
       </c>
       <c r="J16" s="3" t="inlineStr">
         <is>
-          <t>+15.9%</t>
+          <t>+5.3%</t>
         </is>
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>🟢 오늘 단기 매수 (저점 반등)</t>
+          <t>🔴 단기 비중 축소 (악재 주의)</t>
         </is>
       </c>
       <c r="L16" s="3" t="inlineStr">
         <is>
-          <t>RSI 35.1로 단기 과매도 구간 진입, 기술적 반등 노림</t>
+          <t>악재 보도 및 5일 연속 약세로 단기 추가 하락 위험</t>
         </is>
       </c>
       <c r="M16" s="3" t="inlineStr">
@@ -8660,21 +6034,21 @@
         </is>
       </c>
       <c r="O16" s="3" t="n">
-        <v>35.1</v>
+        <v>32.7</v>
       </c>
       <c r="P16" s="3" t="inlineStr">
         <is>
-          <t>-14.6%</t>
+          <t>-16.2%</t>
         </is>
       </c>
       <c r="Q16" s="3" t="inlineStr">
         <is>
-          <t>41.9%</t>
+          <t>40.7%</t>
         </is>
       </c>
       <c r="R16" s="3" t="inlineStr">
         <is>
-          <t>[개장시황] 코스피 1.29% 상승 출발…삼성전자·SK하이닉스 반등 (남도일보)</t>
+          <t>삼성전자 '100조 잭팟' 뒤 서늘한 경고…"한국이 흔들린다" [테크로그] (한국경제)</t>
         </is>
       </c>
     </row>
@@ -8701,17 +6075,17 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>321,000원</t>
+          <t>318,500원</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>-170,500.0원 (-34.69%)</t>
+          <t>-173,000.0원 (-35.20%)</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>318,000원</t>
+          <t>315,500원</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
@@ -8721,12 +6095,12 @@
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>310,000원</t>
+          <t>307,500원</t>
         </is>
       </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
-          <t>+7.8%</t>
+          <t>+8.6%</t>
         </is>
       </c>
       <c r="K17" s="3" t="inlineStr">
@@ -8736,7 +6110,7 @@
       </c>
       <c r="L17" s="3" t="inlineStr">
         <is>
-          <t>RSI 27.4로 단기 과매도 구간 진입, 기술적 반등 노림</t>
+          <t>RSI 25.2로 단기 과매도 구간 진입, 기술적 반등 노림</t>
         </is>
       </c>
       <c r="M17" s="3" t="inlineStr">
@@ -8750,21 +6124,21 @@
         </is>
       </c>
       <c r="O17" s="3" t="n">
-        <v>27.4</v>
+        <v>25.2</v>
       </c>
       <c r="P17" s="3" t="inlineStr">
         <is>
-          <t>-8.2%</t>
+          <t>-8.9%</t>
         </is>
       </c>
       <c r="Q17" s="3" t="inlineStr">
         <is>
-          <t>18.2%</t>
+          <t>17.8%</t>
         </is>
       </c>
       <c r="R17" s="3" t="inlineStr">
         <is>
-          <t>최근 특이 뉴스 없음</t>
+          <t>1∼8월 배터리 분리막 적재량 25%↑…중국 제외 41% 성장 (주요언론)</t>
         </is>
       </c>
     </row>
@@ -8796,7 +6170,7 @@
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>-39,100.0원 (-26.21%)</t>
+          <t>-39,300.0원 (-26.34%)</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
@@ -8826,7 +6200,7 @@
       </c>
       <c r="L18" s="3" t="inlineStr">
         <is>
-          <t>RSI 34.0로 단기 과매도 구간 진입, 기술적 반등 노림</t>
+          <t>RSI 33.5로 단기 과매도 구간 진입, 기술적 반등 노림</t>
         </is>
       </c>
       <c r="M18" s="3" t="inlineStr">
@@ -8840,16 +6214,16 @@
         </is>
       </c>
       <c r="O18" s="3" t="n">
-        <v>34</v>
+        <v>33.5</v>
       </c>
       <c r="P18" s="3" t="inlineStr">
         <is>
-          <t>-5.0%</t>
+          <t>-5.2%</t>
         </is>
       </c>
       <c r="Q18" s="3" t="inlineStr">
         <is>
-          <t>8.6%</t>
+          <t>8.4%</t>
         </is>
       </c>
       <c r="R18" s="3" t="inlineStr">
@@ -8886,7 +6260,7 @@
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>-19,250.0원 (-9.55%)</t>
+          <t>-19,400.0원 (-9.63%)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -8901,7 +6275,7 @@
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>176,000원</t>
+          <t>175,500원</t>
         </is>
       </c>
       <c r="J19" s="3" t="inlineStr">
@@ -8916,7 +6290,7 @@
       </c>
       <c r="L19" s="3" t="inlineStr">
         <is>
-          <t>RSI 33.6로 단기 과매도 구간 진입, 기술적 반등 노림</t>
+          <t>RSI 33.3로 단기 과매도 구간 진입, 기술적 반등 노림</t>
         </is>
       </c>
       <c r="M19" s="3" t="inlineStr">
@@ -8930,16 +6304,16 @@
         </is>
       </c>
       <c r="O19" s="3" t="n">
-        <v>33.6</v>
+        <v>33.3</v>
       </c>
       <c r="P19" s="3" t="inlineStr">
         <is>
-          <t>-6.1%</t>
+          <t>-6.2%</t>
         </is>
       </c>
       <c r="Q19" s="3" t="inlineStr">
         <is>
-          <t>3.4%</t>
+          <t>3.3%</t>
         </is>
       </c>
       <c r="R19" s="3" t="inlineStr">
@@ -8976,12 +6350,12 @@
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>-16,100.0원 (-33.47%)</t>
+          <t>-16,150.0원 (-33.58%)</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>31,700원</t>
+          <t>31,600원</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
@@ -8991,7 +6365,7 @@
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>30,900원</t>
+          <t>30,800원</t>
         </is>
       </c>
       <c r="J20" s="3" t="inlineStr">
@@ -9006,7 +6380,7 @@
       </c>
       <c r="L20" s="3" t="inlineStr">
         <is>
-          <t>RSI 35.4로 단기 과매도 구간 진입, 기술적 반등 노림</t>
+          <t>RSI 34.9로 단기 과매도 구간 진입, 기술적 반등 노림</t>
         </is>
       </c>
       <c r="M20" s="3" t="inlineStr">
@@ -9020,21 +6394,21 @@
         </is>
       </c>
       <c r="O20" s="3" t="n">
-        <v>35.4</v>
+        <v>34.9</v>
       </c>
       <c r="P20" s="3" t="inlineStr">
         <is>
-          <t>-4.1%</t>
+          <t>-4.3%</t>
         </is>
       </c>
       <c r="Q20" s="3" t="inlineStr">
         <is>
-          <t>2.2%</t>
+          <t>2.1%</t>
         </is>
       </c>
       <c r="R20" s="3" t="inlineStr">
         <is>
-          <t>카카오, 인적분할 앞두고 CEO 총출동…새 성장전략 공개 (주요언론)</t>
+          <t>최근 특이 뉴스 없음</t>
         </is>
       </c>
     </row>
@@ -9066,7 +6440,7 @@
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>-5,919.049999999988원 (-3.12%)</t>
+          <t>-6,019.049999999988원 (-3.17%)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -9086,7 +6460,7 @@
       </c>
       <c r="J21" s="3" t="inlineStr">
         <is>
-          <t>+7.2%</t>
+          <t>+7.1%</t>
         </is>
       </c>
       <c r="K21" s="3" t="inlineStr">
@@ -9110,21 +6484,21 @@
         </is>
       </c>
       <c r="O21" s="3" t="n">
-        <v>53</v>
+        <v>52.9</v>
       </c>
       <c r="P21" s="3" t="inlineStr">
         <is>
-          <t>+2.1%</t>
+          <t>+2.0%</t>
         </is>
       </c>
       <c r="Q21" s="3" t="inlineStr">
         <is>
-          <t>31.3%</t>
+          <t>31.2%</t>
         </is>
       </c>
       <c r="R21" s="3" t="inlineStr">
         <is>
-          <t>[바이오스냅] 셀트리온, 미국 처방집 추가 등재 추진 (주요언론)</t>
+          <t>최근 특이 뉴스 없음</t>
         </is>
       </c>
     </row>
@@ -9151,17 +6525,17 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>832,000원</t>
+          <t>828,000원</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>-691,000.0원 (-45.37%)</t>
+          <t>-695,000.0원 (-45.63%)</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>823,500원</t>
+          <t>819,500원</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
@@ -9171,12 +6545,12 @@
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>803,000원</t>
+          <t>799,000원</t>
         </is>
       </c>
       <c r="J22" s="3" t="inlineStr">
         <is>
-          <t>+20.4%</t>
+          <t>+20.9%</t>
         </is>
       </c>
       <c r="K22" s="3" t="inlineStr">
@@ -9186,7 +6560,7 @@
       </c>
       <c r="L22" s="3" t="inlineStr">
         <is>
-          <t>RSI 29.1로 단기 과매도 구간 진입, 기술적 반등 노림</t>
+          <t>RSI 28.8로 단기 과매도 구간 진입, 기술적 반등 노림</t>
         </is>
       </c>
       <c r="M22" s="3" t="inlineStr">
@@ -9200,16 +6574,16 @@
         </is>
       </c>
       <c r="O22" s="3" t="n">
-        <v>29.1</v>
+        <v>28.8</v>
       </c>
       <c r="P22" s="3" t="inlineStr">
         <is>
-          <t>-17.8%</t>
+          <t>-18.1%</t>
         </is>
       </c>
       <c r="Q22" s="3" t="inlineStr">
         <is>
-          <t>5.6%</t>
+          <t>5.2%</t>
         </is>
       </c>
       <c r="R22" s="3" t="inlineStr">
@@ -9241,12 +6615,12 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>421,500원</t>
+          <t>419,500원</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>+21,500.0원 (+5.38%)</t>
+          <t>+19,500.0원 (+4.88%)</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -9256,17 +6630,17 @@
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>421,500원</t>
+          <t>419,500원</t>
         </is>
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>413,000원</t>
+          <t>411,000원</t>
         </is>
       </c>
       <c r="J23" s="3" t="inlineStr">
         <is>
-          <t>+13.3%</t>
+          <t>+12.7%</t>
         </is>
       </c>
       <c r="K23" s="3" t="inlineStr">
@@ -9276,7 +6650,7 @@
       </c>
       <c r="L23" s="3" t="inlineStr">
         <is>
-          <t>RSI 70.9, 20일선 이격도 +13.2%로 단기 과열권, 분할 차익 실현 권고</t>
+          <t>RSI 70.4, 20일선 이격도 +12.8%로 단기 과열권, 분할 차익 실현 권고</t>
         </is>
       </c>
       <c r="M23" s="3" t="inlineStr">
@@ -9290,21 +6664,21 @@
         </is>
       </c>
       <c r="O23" s="3" t="n">
-        <v>70.90000000000001</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="P23" s="3" t="inlineStr">
         <is>
-          <t>+13.2%</t>
+          <t>+12.8%</t>
         </is>
       </c>
       <c r="Q23" s="3" t="inlineStr">
         <is>
-          <t>55.4%</t>
+          <t>54.5%</t>
         </is>
       </c>
       <c r="R23" s="3" t="inlineStr">
         <is>
-          <t>최근 특이 뉴스 없음</t>
+          <t>1∼8월 배터리 분리막 적재량 25%↑…중국 제외 41% 성장 (주요언론)</t>
         </is>
       </c>
     </row>
@@ -9331,17 +6705,17 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>308,500원</t>
+          <t>309,500원</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>-53,000.0원 (-14.66%)</t>
+          <t>-52,000.0원 (-14.38%)</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>302,500원</t>
+          <t>303,500원</t>
         </is>
       </c>
       <c r="H24" s="3" t="inlineStr">
@@ -9351,12 +6725,12 @@
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>293,000원</t>
+          <t>294,000원</t>
         </is>
       </c>
       <c r="J24" s="3" t="inlineStr">
         <is>
-          <t>+10.5%</t>
+          <t>+10.1%</t>
         </is>
       </c>
       <c r="K24" s="3" t="inlineStr">
@@ -9380,16 +6754,16 @@
         </is>
       </c>
       <c r="O24" s="3" t="n">
-        <v>45</v>
+        <v>45.7</v>
       </c>
       <c r="P24" s="3" t="inlineStr">
         <is>
-          <t>-2.0%</t>
+          <t>-1.7%</t>
         </is>
       </c>
       <c r="Q24" s="3" t="inlineStr">
         <is>
-          <t>14.9%</t>
+          <t>15.3%</t>
         </is>
       </c>
       <c r="R24" s="3" t="inlineStr">
@@ -9484,7 +6858,7 @@
       </c>
       <c r="R25" s="3" t="inlineStr">
         <is>
-          <t>세레브라스 CEO "데이터센터 반발은 공포 마케팅 탓" (주요언론)</t>
+          <t>최근 특이 뉴스 없음</t>
         </is>
       </c>
     </row>
@@ -9896,12 +7270,12 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>6,168.13</t>
+          <t>6,094.87</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>+132.78 (+2.20%)</t>
+          <t>+59.52 (+0.99%)</t>
         </is>
       </c>
     </row>
@@ -9923,12 +7297,12 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>845.03</t>
+          <t>830.88</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>+8.00 (+0.96%)</t>
+          <t>-6.15 (-0.73%)</t>
         </is>
       </c>
     </row>
@@ -9950,7 +7324,7 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>1,340.88원</t>
+          <t>1,340.88</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
@@ -9977,7 +7351,7 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>847.01원</t>
+          <t>847.01</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -10004,7 +7378,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>1,500.84원</t>
+          <t>1,500.84</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -10031,7 +7405,7 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>199.98원</t>
+          <t>199.98</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
@@ -10142,27 +7516,27 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>112,822,000원</t>
+          <t>112,595,000원</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>+0.20%</t>
+          <t>+0.00%</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>112,258,000원</t>
+          <t>112,032,000원</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>121,848,000원</t>
+          <t>121,603,000원</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>110,586,000원</t>
+          <t>110,576,000원</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
@@ -10199,27 +7573,27 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>3,391,000원</t>
+          <t>3,385,000원</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>+0.30%</t>
+          <t>+0.12%</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>3,364,000원</t>
+          <t>3,358,000원</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>3,594,500원</t>
+          <t>3,588,000원</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>3,272,500원</t>
+          <t>3,266,500원</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
@@ -10234,7 +7608,7 @@
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>RSI 47.2로 단기 과매도 구간 진입, 기술적 반등 기대</t>
+          <t>RSI 46.8로 단기 과매도 구간 진입, 기술적 반등 기대</t>
         </is>
       </c>
     </row>
@@ -10256,17 +7630,17 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>145,300원</t>
+          <t>144,900원</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>+0.48%</t>
+          <t>+0.21%</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>144,100원</t>
+          <t>143,700원</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -10276,12 +7650,12 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>140,200원</t>
+          <t>139,800원</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>+8.1%</t>
+          <t>+8.4%</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
@@ -10291,7 +7665,529 @@
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>RSI 47.6로 단기 과매도 구간 진입, 기술적 반등 기대</t>
+          <t>RSI 47.1로 단기 과매도 구간 진입, 기술적 반등 기대</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="65" customWidth="1" min="8" max="8"/>
+    <col width="65" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>수집일자</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>신뢰도점수</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>증권사</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>종목명</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>리포트제목</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>목표주가</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>투자의견</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>핵심요약</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>PDF파일명</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>79</v>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>신한투자증권</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>팬오션</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>빛을 보기 시작한 포트폴리오 변화</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>매수</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>한 단계 진화한 실적, 한 단계 진화할 주가 레벨 수급 영향으로 단기 주가의 변동폭은 과거 대비 커졌으나 우호적인 벌크·탱커 시황 감안 시 중기 우상향 흐름 지속될 것으로 판단. 환율 방향성이원화 환산 실적에 부담이나 펀더멘털에 미치는 영향은 제한적</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-14_신한투자증권_팬오션_빛을 보기 시작한 포트폴리오 변화.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>76</v>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>신한투자증권</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>일진전기</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>가장 저평가된 전력기기</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>매수</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>변압기 29년 수주 논의 및 전선 상반기 수주 급증 5월 시가총액 약 6.9조원 도달 이후 7월말 2.2조원까지 약 68% 하락. 전선업체들의 수주잔고총계 연간 증가율은 24년 25.4%, 25년 21.2%에서 26년 상반기에만 23.2% 증가. 변압기에 이은 전선 부문의 호황이 확대되는 것을 감안할 때 펀더멘털 문제가 아닌 수급 측면의 주가 하락으로 판단</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-14_신한투자증권_일진전기_가장 저평가된 전력기기.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>신한투자증권</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>HMM</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>우려도 있지만 너무 잠잠한 주가</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>매수</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>거버넌스 우려로 덮어놓기엔 아까운 실적 글로벌 컨테이너선사들은 가이던스 상향과 함께 주가도 상승했으나 동사 반응은 제한적. 거버넌스 불확실성에도 예상보다 큰 이익 회복에 주목</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-14_신한투자증권_HMM_우려도 있지만 너무 잠잠한 주가.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>73</v>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>하나증권</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>한미약품</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>더 안정적인 성장을 위한 정비 작업(3Q26 Pre)</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>선급금 4Q26 반영, 북경한미 정비 작업과 앱토즈 인수로 전체적인 실적은 부진 3Q26 실적은 연결기준 매출액 3,794억원(YoY+4.7%), 영업이익 381억원(YoY-30.8%, OPM 10.0%)으로 예상된다. 컨센서스와 크게 어긋나 보이지만, Genentech향 HM17321 L/O 선급금이 미국 HSR 행정절차가 10월 초 완료됨에 따라 4Q26에 인식되는데 컨센서스가 미리 3Q에 이를 반영했기 때문이다. 2Q에 Lilly향 L/O에 따른 선급금이 반영되었기 때문에 QoQ로 비교하는 것도 큰 의미가 없다. 선급금이 없던</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-14_하나증권_한미약품_더 안정적인 성장을 위한 정비 작업(3Q26 Pre).pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>73</v>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>신한투자증권</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>현대글로비스</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>환율은 야속하지만 너무 좋은 해운 업황</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>매수</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>자동차 밸류체인이지만 해운사이기도 함 단기 실적 가시성은 다소 낮아졌으나 이익 방향성은 여전히 긍정적. 비계열 고객 호조로 이익 개선이 뚜렷한 사업부를 가진 점은 차별화 포인트</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-14_신한투자증권_현대글로비스_환율은 야속하지만 너무 좋은 해운 업황.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>미래에셋증권</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>휴젤</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>3Q26 Preview: 단기 실적 눈높이 조정</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>매수</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3분기 실적은 미국 판매체계 전환 영향으로 부진 휴젤의 3Q26 매출액은 1,009억원(-4.7% YoY), 영업이익 211억원(-55.5% YoY)으로 추정했다. 3Q26 영업이익은 미국 판매체계 전환 영향으로 전년 동기 대비 55.5% 감소할 것으로 보인다. 3분기는 미국 유통사 모델에서 CSO 모델로 전환하는 과정에서 일회성 매출 차감과 비용 증가가 동반되는 구간이었기 때문이다. 기존 유통사 재고 바이백으로 미국 매출은 마이너스가 예상된다. ASP가 높은 미국향 톡신 매출 공백으로 매출총이익률도 전년 동기 대비 6%p 하락이 </t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-14_미래에셋증권_휴젤_3Q26 Preview 단기 실적 눈높이 조정.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>69</v>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>하나증권</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>삼성화재</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>3Q26 Pre - 단기 실적보다 중요한 것은</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026년 3분기 실적은 컨센서스 하회 전망 3분기 연결 지배순이익은 4,863억원으로 컨센서스(5,825억원)를 하회할 것으로 전망한다. 장기보험손익이 사업비 부담 확대로 예상대비 부한 가운데, 증시 부진과 금리 상승에 따른 투자손익 악화도 실적에 부담으로 작용할 것으로 예상한다. [보험손익] 보험손익은 4,006억원(YoY +8.6%, QoQ -27.5%)으로 추정한다. 장기보험손익은 3,560억원으로 YoY/QoQ 모두 감소할 것으로 예상하며, 사업비 부담 확대가 주요 원인이다. 자동차보험손익은 전분기대비 감소하겠으나 YoY </t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-14_하나증권_삼성화재_3Q26 Pre - 단기 실적보다 중요한 것은.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>하나증권</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>세아베스틸지주</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>3분기는 다소 부진하겠지만 4분기부터 회복 기대</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3Q26 주력 자회사들 판매 감소와 스프레드 축소 2026년 3분기 세아베스틸지주의 매출액과 영업이익은 각각 1.0조원(YoY +10.3%, QoQ -10.6%)과 236억원(YoY -12.4%, QoQ -60.6%)으로 영업이익은 시장컨센서스인 398억원을 크게 하회할 것으로 예상된다. 계절적 비수기와 9월 추석 연휴 영향으로 세아베스틸의 특수강 판매는 41.2만톤(YoY +5.0%, QoQ -9.8%)에 그치며 고정비 부담이 확대될 전망이다. 원가 상승분 가격 전가를 위한 노력으로 8월초까지 적극적인 가격 인상을 시도한 결과, </t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-14_하나증권_세아베스틸지주_3분기는 다소 부진하겠지만 4분기부터 회복 기대.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>하나증권</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>한화손해보험</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>3Q26 Pre - 보험손익 개선세에 주목</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>2026년 3분기 실적은 컨센서스 소폭 하회 전망 3분기 별도 당기순이익은 903억원으로 컨센서스(939억원)를 소폭 하회할 것으로 전망한다. 증시 부진 및 금리 상승에 따른 투자손익 악화가 예상되나, 보험손익은 전반적으로 개선될 전망이다. [보험손익] 보험손익은 1,377억원(YoY +44.5%, QoQ +35.2%)으로 추정한다. 장기·자동차·일반보험손익 모두 예상대비 양호한 수준을 기록할 전망이다. 장기보험손익은 1,411억원으로 YoY/QoQ 모두 큰 폭 증가할 것으로 예상한다. 관리급여 효과에 따른 보험금 예실차 개선이 주</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-14_하나증권_한화손해보험_3Q26 Pre - 보험손익 개선세에 주목.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>67</v>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>하나증권</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>세아제강</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>어려운 영업환경!</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>3Q26 내수와 수출 모두 수익성 악화 2026년 3분기 세아제강의 매출액과 영업이익은 각각 4,318억원(YoY +30.2%, QoQ -12.8%)과 195억원(YoY 흑.전, QoQ -44.2%)으로 영업이익은 시장컨센서스인 254억원을 하회할 것으로 예상된다. 3분기 내수 강관 시장은 계절적 비수기와 추석 연휴 영향으로 다소 부진할 것으로 예상되는 가운데 수출의 경우 캐나다 LNG와 같은 프로젝트 덕분에 소폭 증가한 것으로 추정되어 결과적으로 세아제강의 3분기 전체 강관 판매는 22.8만톤(YoY +21.4%, QoQ -6.8</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-14_하나증권_세아제강_어려운 영업환경!.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: complete 5 major upgrades - backtesting win rate, cool-down, DART disclosures, US Big Tech 4, and analyst PDF table extraction
</commit_message>
<xml_diff>
--- a/reports/일자별_누적_데일리_이슈_및_주식_브리핑_마스터.xlsx
+++ b/reports/일자별_누적_데일리_이슈_및_주식_브리핑_마스터.xlsx
@@ -12,6 +12,8 @@
     <sheet name="시장지표_누적" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="코인추천_누적" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="공식리포트_누적" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="추천성과_검증누적" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="특수공시_누적" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -456,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G111"/>
+  <dimension ref="A1:G107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3632,12 +3634,12 @@
       </c>
       <c r="D86" s="3" t="inlineStr">
         <is>
-          <t>태안군, 12월부터 참전명예수당 월 30만원→50만원</t>
+          <t>김용태 "은퇴봉사동물 지원예산 편성 2곳뿐…관리체계 개선해야"</t>
         </is>
       </c>
       <c r="E86" s="3" t="inlineStr">
         <is>
-          <t>(태안=연합뉴스) 정윤덕 기자 = 충남 태안군은 현재 월 30만원인 참전명예수당을 오는 12월부터 50만원으로 인상할 계획이라고 14일 밝혔다.</t>
+          <t>(서울=연합뉴스) 김세린 기자 = 국가봉사동물 운용 기관 대부분이 은퇴 동물에 대한 별도 지원 예산을 편성하지 않아 범부처 차원의 관리체계 개선...</t>
         </is>
       </c>
       <c r="F86" s="3" t="inlineStr">
@@ -3647,7 +3649,7 @@
       </c>
       <c r="G86" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261014058000063</t>
+          <t>https://www.yna.co.kr/view/AKR20261014083900030</t>
         </is>
       </c>
     </row>
@@ -3659,7 +3661,7 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>정치</t>
+          <t>사회/사건사고</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
@@ -3669,22 +3671,22 @@
       </c>
       <c r="D87" s="3" t="inlineStr">
         <is>
-          <t>與, 野주진우·이진숙·김태규 직격…"패륜으로 인지도 올리나"</t>
+          <t>달리기 대회서 20대女 사망에… '마라톤 거목' 황영조가 한 말</t>
         </is>
       </c>
       <c r="E87" s="3" t="inlineStr">
         <is>
-          <t>(서울=연합뉴스) 최주성 기자 = 더불어민주당은 14일 국민의힘 주진우·이진숙·김태규 의원의 국정감사 기간 중 발언을 놓고 "막말 정치인 양성소...</t>
+          <t>달리기 대회서 20대女 사망에… '마라톤 거목' 황영조가 한 말  한국일보황영조 ‘죽음에 이르는 러닝’ 경고···“욕심 부리지 말고, 필요하면 포기할 줄 알아야”  경향신문'서울 달리기' 마라톤대회 참가했던 20대 여성 사망  연합뉴스'서울달리기' 숨진 20대女는 '카이스트 대학원생' ...</t>
         </is>
       </c>
       <c r="F87" s="3" t="inlineStr">
         <is>
-          <t>주요언론</t>
+          <t>한국일보</t>
         </is>
       </c>
       <c r="G87" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261014062800001</t>
+          <t>https://news.google.com/rss/articles/CBMibkFVX3lxTFBNT1l5LUxfQjNUOTIwSDRwdGt0MDBBZXZzVjQwa1RMV21NTTNxOHVMNS1ydjgzZ0wxRlJkY0xPSzVkcDYydUt1SWxRR1FBbVpmMjU0WkJFeW5La1NZSlREczBuVUJuU19vTVdQbGJn0gFzQVVfeXFMTzFCN2tGdVpYMjI0a1Z0emhBR3pPWUZjRXlnRTdpTlRwY0lxTnhPb1dpc2gwekFNYm9LVW1PRnFuRm12eDNzRDkzWkZSUVA2T0VsTUx6UDRHQ0dZM3Z2U2pSbzhWdUxUUXRHaEQ5UldldTFuTQ?oc=5</t>
         </is>
       </c>
     </row>
@@ -3701,27 +3703,27 @@
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>🔥 [언론사 집중 보도 (4개사)]</t>
+          <t>🔥 [언론사 집중 보도 (3개사)]</t>
         </is>
       </c>
       <c r="D88" s="3" t="inlineStr">
         <is>
-          <t>주미대사관 “강경화 ‘불의의 사고 아니다’ 발언, 이 대통령 반박 아냐”</t>
+          <t>울산 온산읍 제조업체서 불‥'대응 1단계'</t>
         </is>
       </c>
       <c r="E88" s="3" t="inlineStr">
         <is>
-          <t>주미대사관 “강경화 ‘불의의 사고 아니다’ 발언, 이 대통령 반박 아냐”  한겨레"불의의 사고 아니다" 강경화 발언 수습에… 한동훈 "국민이 우습나"  조선일보‘북 DMZ 지뢰’ 대처 공방…“안보리 차원 대응 검토 중”  KBS 뉴스[연합뉴스 이 시각 헤드라인] - 07:30  연합뉴스...</t>
+          <t>울산 온산읍 제조업체서 불‥'대응 1단계'  MBC 뉴스[속보] 울산 온산읍 제조업체 큰불...대응 1단계 발령  YTN울산 온산 화학공장서 폭발음 잇따라…공단 근로자 수천명 대피  부산일보울산 울주군 위험물 제조업체서 화재···소방 대응 1단계 발령  경향신문검은 연기 치솟는 울산 화...</t>
         </is>
       </c>
       <c r="F88" s="3" t="inlineStr">
         <is>
-          <t>한겨레</t>
+          <t>MBC 뉴스</t>
         </is>
       </c>
       <c r="G88" s="3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMia0FVX3lxTFBvaWlRcEhkSXFzQU56OW1VOEFZdjFYZGh1akJIVUkwOFE4Y2NweUVpaVVxQjhSaGd2bG9FZzZKSExzTU8zY0FocWZTS3diZHZlSGxBaW9TazZ2b1RtWXBhS09tYzRsTHFMNVBR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE9xZ25EN3hYNlBZZE8yUmZCSHByRkdsbnMyNHA1eGt5VzdrUzV2djlqamdlUUVUWUlFT2k3cjVkSXFTY1hfVThBSGFDaHlTZC1GMlNHa09mQzJGMUxmNjUwYVhkbTdaOGhxS1ZDLTc1QmMyNzlTZkJN0gF3QVVfeXFMT0NFQ2FBa0JYcGdWUjZxSVhFQXZId3haTnNtOFFocExTUUR3R3Q3SWxFV2xaODdSUXNGdkd1bGtIMlRDZlVUYWNkZmxSU01DbXp1ZjVlRE9kaU84MXdIMlFzZElYSjBsMm5ySWZLdFdPLTVhVTk5c3c?oc=5</t>
         </is>
       </c>
     </row>
@@ -3738,17 +3740,17 @@
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>신규 이슈</t>
+          <t>연결 이슈 (후속)</t>
         </is>
       </c>
       <c r="D89" s="3" t="inlineStr">
         <is>
-          <t>경남도, 육상풍력 7개단지 48기 전수 점검…위험요인 사전 확인</t>
+          <t>무면허 중학생 공유 킥보드로 60대 여성 치여 하천 추락</t>
         </is>
       </c>
       <c r="E89" s="3" t="inlineStr">
         <is>
-          <t>(창원=연합뉴스) 김선경 기자 = 경남도는 오는 30일까지 도내 육상풍력 발전단지 7곳을 전수 점검한다고 14일 밝혔다.</t>
+          <t>(양주=연합뉴스) 심민규 기자 = 경기 양주시에서 중학생이 몰던 공유 전동킥보드에 60대 여성이 치여 하천으로 추락하는 사고가 발생했다.</t>
         </is>
       </c>
       <c r="F89" s="3" t="inlineStr">
@@ -3758,7 +3760,7 @@
       </c>
       <c r="G89" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261014066600052</t>
+          <t>https://www.yna.co.kr/view/AKR20261014083700060</t>
         </is>
       </c>
     </row>
@@ -3780,12 +3782,12 @@
       </c>
       <c r="D90" s="3" t="inlineStr">
         <is>
-          <t>세종시-홍익대, 청년 창업·실험실 '금남대평시장 리빙랩' 운영</t>
+          <t>흉기 난동범 재범 위험 '높음'이었는데…예견된 참극</t>
         </is>
       </c>
       <c r="E90" s="3" t="inlineStr">
         <is>
-          <t>(세종=연합뉴스) 양영석 기자 = 세종시와 홍익대학교 세종캠퍼스는 청년 창업·실험 공간인 '금남대평시장 가치회복 리빙랩'을 운영한다고 14일 밝...</t>
+          <t>(인천=연합뉴스) 최은지 기자 = 과거에도 재범 위험성 '높음' 판정을 받은 50대 살인미수 전과자가 도심 한복판에서 시민 8명을 찌르는 참극이...</t>
         </is>
       </c>
       <c r="F90" s="3" t="inlineStr">
@@ -3795,7 +3797,7 @@
       </c>
       <c r="G90" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261014068900063</t>
+          <t>https://www.yna.co.kr/view/AKR20261014081200065</t>
         </is>
       </c>
     </row>
@@ -3807,7 +3809,7 @@
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>사회/사건사고</t>
+          <t>거시경제/비즈니스</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
@@ -3817,22 +3819,22 @@
       </c>
       <c r="D91" s="3" t="inlineStr">
         <is>
-          <t>AI 전환부터 수출까지…산업부·식약처, 바이오산업 전주기 협력</t>
+          <t>9월 ICT 수출 751억달러 '역대 최대'…반도체가 80% 견인</t>
         </is>
       </c>
       <c r="E91" s="3" t="inlineStr">
         <is>
-          <t>(서울=연합뉴스) 장보인 기자 = 바이오산업 육성을 담당하는 산업통상부와 의약품·의료기기 규제를 책임지는 식품의약품안전처가 바이오산업 전 주기에...</t>
+          <t>9월 ICT 수출 751억달러 '역대 최대'…반도체가 80% 견인  연합인포맥스지난달 ICT 수출 “사상 첫 700억 달러 돌파”  KBS 뉴스AI 열풍 탄 K-반도체 폭주…9월 ICT 수출 700억弗 첫 돌파  뉴시스2026년 9월 정보통신산업(ICT) 수출입 동향  서울PnKDI, ...</t>
         </is>
       </c>
       <c r="F91" s="3" t="inlineStr">
         <is>
-          <t>주요언론</t>
+          <t>연합인포맥스</t>
         </is>
       </c>
       <c r="G91" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261014025800003</t>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTFBMdnFvTFQycG1RNDZHcWU3WncxMEpyZHB4Z3lHMlhFc0U1TUs0djFoZ3pLQ2lpZERDTThqXzNjeFNCdnpiOWxOZHFVVjFLeGlrWGNKNWpRLVRRbFRsTnM3TUlBN01iMTRzNXNtdlI5ck8?oc=5</t>
         </is>
       </c>
     </row>
@@ -3844,7 +3846,7 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>사회/사건사고</t>
+          <t>거시경제/비즈니스</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
@@ -3854,12 +3856,12 @@
       </c>
       <c r="D92" s="3" t="inlineStr">
         <is>
-          <t>강원 고성군, 재난 안전상황실 전담 인력 배치…내달 본격 운영</t>
+          <t>완주 테크노밸리 미니복합타운 2천884세대, 내년부터 순차 분양</t>
         </is>
       </c>
       <c r="E92" s="3" t="inlineStr">
         <is>
-          <t>(강원 고성=연합뉴스) 류호준 기자 = 강원 고성군은 기후 변화와 각종 재난 사고에 신속하게 대응하기 위해 다음 달부터 재난 안전상황실 전담 운...</t>
+          <t>(완주=연합뉴스) 최영수 기자 = 전북 완주군은 봉동읍 테크노밸리 제2일반산업단지 옆 미니복합타운을 내년 1월 첫 분양한다고 14일 밝혔다.</t>
         </is>
       </c>
       <c r="F92" s="3" t="inlineStr">
@@ -3869,7 +3871,7 @@
       </c>
       <c r="G92" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261014066400062</t>
+          <t>https://www.yna.co.kr/view/AKR20261014082100055</t>
         </is>
       </c>
     </row>
@@ -3881,22 +3883,22 @@
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>사회/사건사고</t>
+          <t>거시경제/비즈니스</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>신규 이슈</t>
+          <t>🔥 [언론사 집중 보도 (3개사)]</t>
         </is>
       </c>
       <c r="D93" s="3" t="inlineStr">
         <is>
-          <t>설악권 현안 두고 머리 맞댄 속초시·고성군 의회…"상생 협력"</t>
+          <t>한솔제지 등 대전 3개 기업, 공장 증설에 734억 투자</t>
         </is>
       </c>
       <c r="E93" s="3" t="inlineStr">
         <is>
-          <t>(속초=연합뉴스) 류호준 기자 = 강원 속초시의회와 고성군의회 의장이 만나 울산바위 인근 공동주택 개발 문제 등 설악권 주요 현안과 관련해 지역...</t>
+          <t>(대전=연합뉴스) 박주영 기자 = 대전시는 14일 대전 소재 기업 3곳과 734억원 규모의 투자 유치를 위한 업무협약을 했다.</t>
         </is>
       </c>
       <c r="F93" s="3" t="inlineStr">
@@ -3906,7 +3908,7 @@
       </c>
       <c r="G93" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261014065100062</t>
+          <t>https://www.yna.co.kr/view/AKR20261014083600063</t>
         </is>
       </c>
     </row>
@@ -3918,22 +3920,22 @@
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>사회/사건사고</t>
+          <t>거시경제/비즈니스</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>신규 이슈</t>
+          <t>🔥 [언론사 집중 보도 (3개사)]</t>
         </is>
       </c>
       <c r="D94" s="3" t="inlineStr">
         <is>
-          <t>AI로 '옥외영업 인허가' 판단…고양시, 직원 아이디어 특허</t>
+          <t>이란, 레이더 파괴되자 '인간 레이더' 동원…미국과 '유가 전쟁'</t>
         </is>
       </c>
       <c r="E94" s="3" t="inlineStr">
         <is>
-          <t>(고양=연합뉴스) 노승혁 기자 = 경기 고양시는 현장 공무원이 직접 고안한 '인공지능(AI) 기반 옥외영업 가능 대상 자동 판단 및 인허가 검증...</t>
+          <t>(서울=연합뉴스) 임화섭 기자 = 미국 중간선거를 앞두고 이란이 호르무즈 해협을 지나는 선박을 공격하는 데에 '새 전술'을 동원하고 있다고 로이...</t>
         </is>
       </c>
       <c r="F94" s="3" t="inlineStr">
@@ -3943,7 +3945,7 @@
       </c>
       <c r="G94" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261014064100060</t>
+          <t>https://www.yna.co.kr/view/AKR20261014052400009</t>
         </is>
       </c>
     </row>
@@ -3955,7 +3957,7 @@
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>사회/사건사고</t>
+          <t>세계/국제</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
@@ -3965,22 +3967,22 @@
       </c>
       <c r="D95" s="3" t="inlineStr">
         <is>
-          <t>AI 코딩부터 데이터 활용까지…'AI 체험 축제' 열린다</t>
+          <t>불륜녀에게 칼 찔린 남편…살려달라 연락한 사람은 ‘아내’, 日 발칵 [핫이슈]</t>
         </is>
       </c>
       <c r="E95" s="3" t="inlineStr">
         <is>
-          <t>(서울=연합뉴스) 권하영 기자 = 전 국민이 참여할 수 있는 인공지능(AI) 체험의 장이 열린다.</t>
+          <t>불륜녀에게 칼 찔린 남편…살려달라 연락한 사람은 ‘아내’, 日 발칵 [핫이슈]  나우뉴스</t>
         </is>
       </c>
       <c r="F95" s="3" t="inlineStr">
         <is>
-          <t>주요언론</t>
+          <t>나우뉴스</t>
         </is>
       </c>
       <c r="G95" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261014065400017</t>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE5yYlFXd1pIRWNSakJjSmhDT1FGY0doR0NhYlNodFotVmZobWI4Uzh4dENKQnhqbFBoV1ZSNlFORTBxenpLbkh5MUpnN09VTjJPYmxRVWRQX3RRUjNhNnQ0aF9YU3htTUJLc0ZhWFRoMFE?oc=5</t>
         </is>
       </c>
     </row>
@@ -3992,32 +3994,32 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>사회/사건사고</t>
+          <t>세계/국제</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>신규 이슈</t>
+          <t>🔥 [언론사 집중 보도 (5개사)]</t>
         </is>
       </c>
       <c r="D96" s="3" t="inlineStr">
         <is>
-          <t>김해진영단감축제 30일 개막…사흘간 공연·체험 행사 풍성</t>
+          <t>트럼프, '장남 전 약혼녀' 길포일 주그리스 대사 전격 경질</t>
         </is>
       </c>
       <c r="E96" s="3" t="inlineStr">
         <is>
-          <t>(김해=연합뉴스) 이준영 기자 = 경남 김해시는 오는 30일부터 내달 1일까지 진영운동장 일원에서 '제42회 김해진영단감축제'를 개최한다고 14...</t>
+          <t>트럼프, '장남 전 약혼녀' 길포일 주그리스 대사 전격 경질  뉴스핌‘트럼프 장남 전 연인’ 주그리스 미국 대사 비위 의혹에 사임  경향신문"가족은 아니었다"…트럼프, '아들 전 약혼녀' 그리스 대사 해임  마켓인백악관, '각종 비위 의혹' 그리스 대사에 "사퇴 요구했다"  연합뉴스트럼...</t>
         </is>
       </c>
       <c r="F96" s="3" t="inlineStr">
         <is>
-          <t>주요언론</t>
+          <t>뉴스핌</t>
         </is>
       </c>
       <c r="G96" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261014065600052</t>
+          <t>https://news.google.com/rss/articles/CBMiXEFVX3lxTE1FTFlBWGhjbXIyR01pc0Q4bGJGWWFyY01BTzdrS3hZdmlrQ3NzdHJheUV0Nmd2Y21fN3pabXR3YTlnUVZTZE90SWtmdGJYM0hKZGF3c2hlRk1rRlZP?oc=5</t>
         </is>
       </c>
     </row>
@@ -4029,32 +4031,32 @@
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>사회/사건사고</t>
+          <t>세계/국제</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>신규 이슈</t>
+          <t>🔥 [언론사 집중 보도 (5개사)]</t>
         </is>
       </c>
       <c r="D97" s="3" t="inlineStr">
         <is>
-          <t>목포해경, 안전사고 위험 '주의보' 발령</t>
+          <t>트럼프·네타냐후, 선거 전 이란 재공격 저울질…정치적 부담에 딜레마</t>
         </is>
       </c>
       <c r="E97" s="3" t="inlineStr">
         <is>
-          <t>(목포=연합뉴스) 조근영 기자 = 목포해양경찰서는 14일 목포·신안·무안·진도 등 전남광주 8개 시·군 지역에 안전사고 위험예보제 '주의보' 단...</t>
+          <t>트럼프·네타냐후, 선거 전 이란 재공격 저울질…정치적 부담에 딜레마  뉴스핌악시오스 "트럼프, 지난주 네타냐후와 중간선거 전 이란 공격 논의"  MBC 뉴스트럼프 "선거 끝나도 나는 대통령…후티 공격 잊지 않을 것" [이상은의 워싱턴나우]  한국경제트럼프, "러시아·중국이 이란 돕고 있...</t>
         </is>
       </c>
       <c r="F97" s="3" t="inlineStr">
         <is>
-          <t>주요언론</t>
+          <t>뉴스핌</t>
         </is>
       </c>
       <c r="G97" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261014065700054</t>
+          <t>https://news.google.com/rss/articles/CBMiXEFVX3lxTE5IeWdpMkUtOVZFQWRXQ0VERHJKVUNRSWE1M3JZSnB5Y1NfSWFVZHZwUGhiZ0ZqV05QNFdTZzlSNll1YTQyN0tLT0h2R3JEVEdXcVBfYnpJT1phRUFt?oc=5</t>
         </is>
       </c>
     </row>
@@ -4066,22 +4068,22 @@
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>사회/사건사고</t>
+          <t>세계/국제</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>신규 이슈</t>
+          <t>🔥 [언론사 집중 보도 (5개사)]</t>
         </is>
       </c>
       <c r="D98" s="3" t="inlineStr">
         <is>
-          <t>거래소·배출권시장協, 배출권거래제 정책·산업계 대응 논의</t>
+          <t>트럼프 새 대변인 변호사 경력 논란…"중국서 자격 취득" 주장</t>
         </is>
       </c>
       <c r="E98" s="3" t="inlineStr">
         <is>
-          <t>(서울=연합뉴스) 임은진 기자 = 한국거래소는 14일 오후 서울 사옥에서 배출권시장협의회와 함께 '2026년 하반기 자문위원회 세미나'를 연다.</t>
+          <t>(서울=연합뉴스) 이신영 기자 = 도널드 트럼프 미국 대통령이 새로 임명한 백악관 대변인 케이티 재커라이어가 경력 논란에 휩싸였다.</t>
         </is>
       </c>
       <c r="F98" s="3" t="inlineStr">
@@ -4091,7 +4093,7 @@
       </c>
       <c r="G98" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261014066900008</t>
+          <t>https://www.yna.co.kr/view/AKR20261014076000009</t>
         </is>
       </c>
     </row>
@@ -4103,7 +4105,7 @@
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>사회/사건사고</t>
+          <t>세계/국제</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
@@ -4113,12 +4115,12 @@
       </c>
       <c r="D99" s="3" t="inlineStr">
         <is>
-          <t>법원, '푸틴 반대' 러시아인 체류연장 불허에 "취소해야"</t>
+          <t>텐센트, AI 투자용 7.7조원 채권 발행…주문 4배 몰려</t>
         </is>
       </c>
       <c r="E99" s="3" t="inlineStr">
         <is>
-          <t>(인천=연합뉴스) 김상연 기자 = 국내에서 러시아·우크라이나 전쟁 반대 시위에 수백회 참여한 러시아인에게 난민인정 신청 결과가 나올 때까지 임시...</t>
+          <t>(서울=연합뉴스) 정주호 기자 = 중국 텐센트가 인공지능(AI) 투자 자금 마련을 위한 대규모 채권 발행에 4배가 넘는 투자 수요가 몰렸다.</t>
         </is>
       </c>
       <c r="F99" s="3" t="inlineStr">
@@ -4128,7 +4130,7 @@
       </c>
       <c r="G99" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261014065900065</t>
+          <t>https://www.yna.co.kr/view/AKR20261014082900009</t>
         </is>
       </c>
     </row>
@@ -4140,32 +4142,32 @@
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>거시경제/비즈니스</t>
+          <t>IT/과학/신상품</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>신규 이슈</t>
+          <t>🔥 [언론사 집중 보도 (3개사)]</t>
         </is>
       </c>
       <c r="D100" s="3" t="inlineStr">
         <is>
-          <t>산업부, 2030년까지 국가·지역 대표 전시회 5개 이상 육성</t>
+          <t>조이시티, 12월 3일 신작 '프리스타일 풋볼 2' 글로벌 출시</t>
         </is>
       </c>
       <c r="E100" s="3" t="inlineStr">
         <is>
-          <t>산업부, 2030년까지 국가·지역 대표 전시회 5개 이상 육성  KBS 뉴스Google 뉴스에서 헤드라인 및 의견 더보기</t>
+          <t>조이시티, 12월 3일 신작 '프리스타일 풋볼 2' 글로벌 출시  아이뉴스24조이시티, '프리스타일 풋볼 2' 12월 3일 출시…사전 판매 시작  매일경제 마켓26년 9월 월간게임동향  게임트릭스'프리스타일 풋볼 2', 12월 3일 글로벌 출시…사전 판매 시작  인벤조이시티 ‘프리스타일...</t>
         </is>
       </c>
       <c r="F100" s="3" t="inlineStr">
         <is>
-          <t>KBS 뉴스</t>
+          <t>아이뉴스24</t>
         </is>
       </c>
       <c r="G100" s="3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE0wbFFDM0djVl8tRTVjVUhwS0dfdjFGWkZYVURJNTZnaUZIeEVNdzUtMWZYRTY0VTFSYXMwdk9RVVVOR2FLMTFpSlQ2ZE1xRzFxa2pMdnBfT0pHa3M?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiS0FVX3lxTFBLeDN5NXQ2U2xZdjRrYm1TSnJkRjdydDRPc19qbzZzU3E4ZnZMRW5DcWszNWNqRFA3aWp5YklNNG0zeVJyd2lEQ0N3NA?oc=5</t>
         </is>
       </c>
     </row>
@@ -4177,32 +4179,32 @@
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>거시경제/비즈니스</t>
+          <t>IT/과학/신상품</t>
         </is>
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>🔥 [언론사 집중 보도 (3개사)]</t>
+          <t>연결 이슈 (후속)</t>
         </is>
       </c>
       <c r="D101" s="3" t="inlineStr">
         <is>
-          <t>필라델피아 반도체 지수 5일 연속 하락...7월 말 이후 처음</t>
+          <t>RTX 5080 할인에 CPU 쿨러까지…조텍, 탁탁몰 특가 행사</t>
         </is>
       </c>
       <c r="E101" s="3" t="inlineStr">
         <is>
-          <t>필라델피아 반도체 지수 5일 연속 하락...7월 말 이후 처음  YTN메모리, 제2 소프트웨어?…"내년 정말 힘들 것" PTJ의 경고 [김현석의 월스트리트나우]  한국경제반도체 손실로 월가 하락 후 미국 증시 선물 보합세…CPI 발표 대기  Investing.com 한국어中 반도체 추격...</t>
+          <t>RTX 5080 할인에 CPU 쿨러까지…조텍, 탁탁몰 특가 행사  뉴스탭Google 뉴스에서 헤드라인 및 의견 더보기</t>
         </is>
       </c>
       <c r="F101" s="3" t="inlineStr">
         <is>
-          <t>YTN</t>
+          <t>뉴스탭</t>
         </is>
       </c>
       <c r="G101" s="3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiXkFVX3lxTFByT3A4M2N1UEF1c211Rll3UHdCX2F6ZkttQ3YwY0U3OTlJSE00ZDlwR1Y2X1dRT09zakFLRnd6TEs0RlBCcVhUSURyNF9BLVBHeld6bERydDZUQmxLY1E?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMibEFVX3lxTE92UmZLWFY0bG9iOEZPUjVtYTZjcnBNMkRteFZUY2ZkZ2xYaVlKS3lvRG5UMENyNGVMSkxaYUxIREo2ZjdSSjZlY2FFeEZuU1M4NF9EY0w5dU9wZWhBN1VucjB0ZGg5bmUtNmI4SA?oc=5</t>
         </is>
       </c>
     </row>
@@ -4214,7 +4216,7 @@
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>거시경제/비즈니스</t>
+          <t>IT/과학/신상품</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
@@ -4224,22 +4226,22 @@
       </c>
       <c r="D102" s="3" t="inlineStr">
         <is>
-          <t>삼성전자 '100조 잭팟' 뒤 서늘한 경고…"한국이 흔들린다" [테크로그]</t>
+          <t>콘솔게임 보안까지 뚫은 AI, 해적판 등장에 업계 '발칵'</t>
         </is>
       </c>
       <c r="E102" s="3" t="inlineStr">
         <is>
-          <t>삼성전자 '100조 잭팟' 뒤 서늘한 경고…"한국이 흔들린다" [테크로그]  한국경제100조원 벌었지만 증가율은 반토막…외국인 올들어 232조원 ‘엑소더스’  한국경제삼성전자·SK하이닉스, 두번째 바닥 찍었나…“W자 반등 기대”  마켓인거침없는 외인 매도...반도체 역대급 실적에도 급락...</t>
+          <t>(서울=연합뉴스) 김주환 기자 = 인기 콘솔 게임과 플랫폼의 철통 같은 데이터 보안이 에이전틱 인공지능(AI) 고도화에 잇달아 뚫리며 해적판이 ...</t>
         </is>
       </c>
       <c r="F102" s="3" t="inlineStr">
         <is>
-          <t>한국경제</t>
+          <t>주요언론</t>
         </is>
       </c>
       <c r="G102" s="3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTE0ybTlfNDRfSnlTM3l0VzBjYm5QNmpPeW9wLWJ6UGE1dTF2ZEd3Nll1LTA4dW0wVFlneHNqaWlMTzFDY21VbEF3eDluN2FVSXAyR0FQcVRuVm1kUQ?oc=5</t>
+          <t>https://www.yna.co.kr/view/AKR20261014079700017</t>
         </is>
       </c>
     </row>
@@ -4251,32 +4253,32 @@
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>거시경제/비즈니스</t>
+          <t>IT/과학/신상품</t>
         </is>
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>연결 이슈 (후속)</t>
+          <t>신규 이슈</t>
         </is>
       </c>
       <c r="D103" s="3" t="inlineStr">
         <is>
-          <t>새마을금고·OK저축은행도 고객 정보 유출…금융당국에 신고</t>
+          <t>'월가 족집게' 댄 아이브스 "테슬라·스페이스X 내년 합병 가능성 80%"</t>
         </is>
       </c>
       <c r="E103" s="3" t="inlineStr">
         <is>
-          <t>새마을금고·OK저축은행도 고객 정보 유출…금융당국에 신고  조선일보새마을금고 400명대 개인정보 유출... 계좌정보도 포함  보안뉴스금융당국, 해킹 2금융권 확산에 긴급 점검  전자신문OK저축은행, 대출신청 페이지에서 정보 유출… 고객 183명 정보 유출 - 조선비즈  Chosunbiz...</t>
+          <t>(서울=연합뉴스) 정회인 기자 = 월가의 대표적인 기술주 분석가인 댄 아이브스 '요크빌 아이브스' 파트너 겸 선임 전무는 엔비디아와 마이크로소프...</t>
         </is>
       </c>
       <c r="F103" s="3" t="inlineStr">
         <is>
-          <t>조선일보</t>
+          <t>주요언론</t>
         </is>
       </c>
       <c r="G103" s="3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiiwFBVV95cUxNdUg3TWo4c01LMHZnOXFZOFdfZDRXRWpuMld3TlRzTXBNdjdvQTJyUFZmcGRfOGJCc3dnRFZQbW9pLVYtWDNPSXFDQkR0dTR3ZnVud0NlbjhhYWVhTnpvYm85SUNncUJvYzVqY0FRRlVrU2pvQnhSaDJ6aGFWM0s1bUJwaFdrd3dvQzQw?oc=5</t>
+          <t>https://www.yna.co.kr/view/AKR20261014080500008</t>
         </is>
       </c>
     </row>
@@ -4288,7 +4290,7 @@
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>거시경제/비즈니스</t>
+          <t>연예/대중문화</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
@@ -4298,22 +4300,22 @@
       </c>
       <c r="D104" s="3" t="inlineStr">
         <is>
-          <t>횡성군, 임도 사면 녹화 기술 도입…식생 정착·시공 품질 향상</t>
+          <t>‘이병헌♥’ 이민정, 12살 초등학생 아들 사교육 언급..“농구·수학만 시켜”</t>
         </is>
       </c>
       <c r="E104" s="3" t="inlineStr">
         <is>
-          <t>(횡성=연합뉴스) 류호준 기자 = 강원 횡성군은 횡성군산림조합, 구루이엔티와 임도 사면 녹화 기술의 현장 적용과 기술 협력을 위한 업무협약(MO...</t>
+          <t>‘이병헌♥’ 이민정, 12살 초등학생 아들 사교육 언급..“농구·수학만 시켜”  조선일보이민정, 아들 사교육 질문에 "농구·수학 학원만 다녀"  뉴시스‘이병헌♥’ 이민정, 12살 초등학생 아들 사교육 언급..“농구·수학만 시켜” - 조선비즈  Chosunbiz'MJ' 이민정 "어렸을 때...</t>
         </is>
       </c>
       <c r="F104" s="3" t="inlineStr">
         <is>
-          <t>주요언론</t>
+          <t>조선일보</t>
         </is>
       </c>
       <c r="G104" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261014068000062</t>
+          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxQZXdFa0RBNkNZYlBOZ1ZOUzlQWWJWbXlYbjJVUFdLeFBrSFhqcHVvMm5wWVRBMklsTm44MUJJRmMycjRCdzByYTdfTW8xLTFyaDVyN1RIdnZzSVRNOHdIeld1NW15Q2VibGZTUFE2eTlTXzR6MTdtakJ2MDZWRkk1UndvNy0xZUt0a2lRQ0dXbw?oc=5</t>
         </is>
       </c>
     </row>
@@ -4325,32 +4327,32 @@
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>거시경제/비즈니스</t>
+          <t>연예/대중문화</t>
         </is>
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>신규 이슈</t>
+          <t>연결 이슈 (후속)</t>
         </is>
       </c>
       <c r="D105" s="3" t="inlineStr">
         <is>
-          <t>충남도, 올해 마지막 '동네창업학교' 교육생 100명 모집</t>
+          <t>최수종, 모친상 후 끝내 눈물 “왜 쓴소리 했을까” (유퀴즈)</t>
         </is>
       </c>
       <c r="E105" s="3" t="inlineStr">
         <is>
-          <t>(홍성=연합뉴스) 김준범 기자 = 충남도는 청년 예비·초기 창업자를 대상으로 올해 마지막 '동네창업학교' 교육생 100명을 모집한다고 14일 밝...</t>
+          <t>최수종, 모친상 후 끝내 눈물 “왜 쓴소리 했을까” (유퀴즈)  매일경제최수종, 모친상 발인 다음 날 녹화…"엄마에게 쓴소리했던 게 후회"  뉴시스최수종, 모친상 심경.."쓴소리 더 기억나서 마음 아파" 눈물('유퀴즈')[핫피플] - 조선비즈  Chosunbiz“쓴소리했던 기억에 눈물”...</t>
         </is>
       </c>
       <c r="F105" s="3" t="inlineStr">
         <is>
-          <t>주요언론</t>
+          <t>매일경제</t>
         </is>
       </c>
       <c r="G105" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261014068300063</t>
+          <t>https://news.google.com/rss/articles/CBMiZkFVX3lxTE55YkFOMHFYNXc3S1c4MWY4T1ZHRGQxdmwzMjZFWS15d3dtaTZkdW1QbzgxUWlmaWpOcHFJVXN0RFlIcV9rU0dkX3ZpdGI5MG41ME9yeXdKVjF2Yi16cVBYZk1ic21vQQ?oc=5</t>
         </is>
       </c>
     </row>
@@ -4362,32 +4364,32 @@
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>거시경제/비즈니스</t>
+          <t>연예/대중문화</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>신규 이슈</t>
+          <t>🔥 [언론사 집중 보도 (5개사)]</t>
         </is>
       </c>
       <c r="D106" s="3" t="inlineStr">
         <is>
-          <t>공공수주 반등에도 민간 부진…8월 건설수주 8% 감소</t>
+          <t>김영광·채수빈 ‘나를 충전해줘’, 공개 3일 만에 넷플릭스 글로벌 비영어권 3위</t>
         </is>
       </c>
       <c r="E106" s="3" t="inlineStr">
         <is>
-          <t>(세종=연합뉴스) 오진송 기자 = 올해 8월 국내 건설수주가 공공 부문의 반등에도 민간 부진이 이어지면서 3개월 연속 감소한 것으로 나타났다.</t>
+          <t>김영광·채수빈 ‘나를 충전해줘’, 공개 3일 만에 넷플릭스 글로벌 비영어권 3위  스포츠동아차우민, '최애의 사원' 이어 '나를 충전해줘'까지…로맨스 연타 흥행 예고  YTN‘국민엄마’ 김미경, 백발됐다…이번엔 재벌가 회장 변신(‘나를 충전해줘’) - 조선비즈  Chosunbiz‘나를 ...</t>
         </is>
       </c>
       <c r="F106" s="3" t="inlineStr">
         <is>
-          <t>주요언론</t>
+          <t>스포츠동아</t>
         </is>
       </c>
       <c r="G106" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261014059000003</t>
+          <t>https://news.google.com/rss/articles/CBMibkFVX3lxTE9Ra1M4ZWNJS21PN3QtYnBCU3V4bnZoRm44Z2ZITHR1Z1lkUXZqZ2RVWTN1ZU0xWWRkZkJRVlVvOXQzanpDekVYcnBvWDJ0ekRlWElHZVFmVDVOT0IwWnpBbDlPNzk0WmtGdm1TTGZ3?oc=5</t>
         </is>
       </c>
     </row>
@@ -4399,180 +4401,32 @@
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>세계/국제</t>
+          <t>연예/대중문화</t>
         </is>
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>연결 이슈 (후속)</t>
+          <t>🔥 [언론사 집중 보도 (3개사)]</t>
         </is>
       </c>
       <c r="D107" s="3" t="inlineStr">
         <is>
-          <t>레오 14세 교황, 폐암 진단…오른쪽 폐 일부 절제 수술</t>
+          <t>‘계약결혼’ 음주·흡연 갈등 시작</t>
         </is>
       </c>
       <c r="E107" s="3" t="inlineStr">
         <is>
-          <t>레오 14세 교황, 폐암 진단…오른쪽 폐 일부 절제 수술  한국경제71살 교황 레오 14세 폐암 진단…“오른쪽 폐 일부 절제”  한겨레레오 14세 교황, 폐 결절 아닌 폐암…오른쪽 폐 일부 절제 수술  동아일보교황청 "레오 14세, 폐 결절 수술 성공적 완료"…남미순방 갈듯  마켓인교황...</t>
+          <t>‘계약결혼’ 음주·흡연 갈등 시작  BNT뉴스'계약결혼' 남편 담배 냄새에 질색 "안대에서도 냄새나"  뉴시스흥행신화 PD도 0%대 굴욕...새 판 짠 남규홍 ‘계약결혼’ 아쉬운 초반 성적표 [SC이슈]  조선일보16기 상철, 암 수술한 영숙에 술 권유 "한 캔 정도는…"  파이낸셜뉴스...</t>
         </is>
       </c>
       <c r="F107" s="3" t="inlineStr">
         <is>
-          <t>한국경제</t>
+          <t>BNT뉴스</t>
         </is>
       </c>
       <c r="G107" s="3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTE52ak40R0pZMTk1NVRHM3lZNGNsYnFsYW1Ud2RGbXYzRzJZbUZFRjlxb2V2ZGVVRm5MaVFLOW5HZmM2eE5iSTcyLVowc2cydUc5WS1XRG9uVU53dw?oc=5</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B108" s="2" t="inlineStr">
-        <is>
-          <t>세계/국제</t>
-        </is>
-      </c>
-      <c r="C108" s="2" t="inlineStr">
-        <is>
-          <t>신규 이슈</t>
-        </is>
-      </c>
-      <c r="D108" s="3" t="inlineStr">
-        <is>
-          <t>美검찰, '韓 정부 대리' 혐의 수미 테리 '기소유예 합의'</t>
-        </is>
-      </c>
-      <c r="E108" s="3" t="inlineStr">
-        <is>
-          <t>(서울=연합뉴스) 임화섭 기자 = 한국 정부를 위해 비밀리에 활동하고 고가 선물을 수수했다는 혐의를 받아온 전직 미국 중앙정보국(CIA) 분석가...</t>
-        </is>
-      </c>
-      <c r="F108" s="3" t="inlineStr">
-        <is>
-          <t>주요언론</t>
-        </is>
-      </c>
-      <c r="G108" s="3" t="inlineStr">
-        <is>
-          <t>https://www.yna.co.kr/view/AKR20261014067100009</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B109" s="2" t="inlineStr">
-        <is>
-          <t>IT/과학/신상품</t>
-        </is>
-      </c>
-      <c r="C109" s="2" t="inlineStr">
-        <is>
-          <t>신규 이슈</t>
-        </is>
-      </c>
-      <c r="D109" s="3" t="inlineStr">
-        <is>
-          <t>해양진흥공사, 지속가능경영보고서 최고 등급</t>
-        </is>
-      </c>
-      <c r="E109" s="3" t="inlineStr">
-        <is>
-          <t>(부산=연합뉴스) 박창수 기자 = 한국해양진흥공사는 지난 5월 발간한 '2025 지속가능경영보고서'가 미국 커뮤니케이션연맹(LACP)이 주관하는...</t>
-        </is>
-      </c>
-      <c r="F109" s="3" t="inlineStr">
-        <is>
-          <t>주요언론</t>
-        </is>
-      </c>
-      <c r="G109" s="3" t="inlineStr">
-        <is>
-          <t>https://www.yna.co.kr/view/AKR20261014067400051</t>
-        </is>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B110" s="2" t="inlineStr">
-        <is>
-          <t>IT/과학/신상품</t>
-        </is>
-      </c>
-      <c r="C110" s="2" t="inlineStr">
-        <is>
-          <t>신규 이슈</t>
-        </is>
-      </c>
-      <c r="D110" s="3" t="inlineStr">
-        <is>
-          <t>1∼8월 배터리 분리막 적재량 25%↑…중국 제외 41% 성장</t>
-        </is>
-      </c>
-      <c r="E110" s="3" t="inlineStr">
-        <is>
-          <t>(서울=연합뉴스) 김민지 기자 = 올해 1∼8월 글로벌 전기차용 배터리 분리막 적재량이 배터리 탑재량 증가와 중국 제외 시장의 빠른 성장에 힘입...</t>
-        </is>
-      </c>
-      <c r="F110" s="3" t="inlineStr">
-        <is>
-          <t>주요언론</t>
-        </is>
-      </c>
-      <c r="G110" s="3" t="inlineStr">
-        <is>
-          <t>https://www.yna.co.kr/view/AKR20261014062600003</t>
-        </is>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B111" s="2" t="inlineStr">
-        <is>
-          <t>IT/과학/신상품</t>
-        </is>
-      </c>
-      <c r="C111" s="2" t="inlineStr">
-        <is>
-          <t>신규 이슈</t>
-        </is>
-      </c>
-      <c r="D111" s="3" t="inlineStr">
-        <is>
-          <t>음성군, '전통시장·상점가 활성화 유공' 중기부 장관상 수상</t>
-        </is>
-      </c>
-      <c r="E111" s="3" t="inlineStr">
-        <is>
-          <t>(음성=연합뉴스) 박재천 기자 = 충북 음성군은 중소벤처기업부의 '2026년 전통시장 및 상점가 활성화 유공' 평가에서 우수 지방자치단체로 선정...</t>
-        </is>
-      </c>
-      <c r="F111" s="3" t="inlineStr">
-        <is>
-          <t>주요언론</t>
-        </is>
-      </c>
-      <c r="G111" s="3" t="inlineStr">
-        <is>
-          <t>https://www.yna.co.kr/view/AKR20261014066300064</t>
+          <t>https://news.google.com/rss/articles/CBMiZEFVX3lxTE9RbjBZcjlhWHUtcDdJb3V3Q1VlWU9CVTBWSXNzaURtb05heENLNzJ1aHZJM3BqSFBjd2p0WTU0Ym5TODhVSjV5LWxvXzM3LWEyNmlBWVcyRVNhLTRLbEM3VzRpQ1M?oc=5</t>
         </is>
       </c>
     </row>
@@ -4587,17 +4441,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R27"/>
+  <dimension ref="A1:R28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="29" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
     <col width="34" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="25" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="36" customWidth="1" min="11" max="11"/>
@@ -5895,42 +5749,42 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>236,000원</t>
+          <t>238,000원</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>+29,500.0원 (+14.29%)</t>
+          <t>+31,250.0원 (+15.13%)</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>220,500원</t>
+          <t>235,500원</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>233,500원</t>
+          <t>257,000원</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>229,000원</t>
+          <t>229,500원</t>
         </is>
       </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
-          <t>+6.0%</t>
+          <t>+9.2%</t>
         </is>
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>🔴 단기 비중 축소 (악재 주의)</t>
+          <t>🟢 오늘 단기 매수 (저점 반등)</t>
         </is>
       </c>
       <c r="L15" s="3" t="inlineStr">
         <is>
-          <t>악재 보도 및 5일 연속 약세로 단기 추가 하락 위험</t>
+          <t>RSI 38.0로 단기 과매도 구간 진입, 기술적 반등 노림</t>
         </is>
       </c>
       <c r="M15" s="3" t="inlineStr">
@@ -5944,21 +5798,21 @@
         </is>
       </c>
       <c r="O15" s="3" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="P15" s="3" t="inlineStr">
         <is>
-          <t>-10.0%</t>
+          <t>-9.4%</t>
         </is>
       </c>
       <c r="Q15" s="3" t="inlineStr">
         <is>
-          <t>51.3%</t>
+          <t>51.6%</t>
         </is>
       </c>
       <c r="R15" s="3" t="inlineStr">
         <is>
-          <t>필라델피아 반도체 지수 5일 연속 하락...7월 말 이후 처음 (YTN)</t>
+          <t>9월 ICT 수출 751억달러 '역대 최대'…반도체가 80% 견인 (연합인포맥스)</t>
         </is>
       </c>
     </row>
@@ -5985,42 +5839,42 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>1,458,000원</t>
+          <t>1,475,000원</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>+355,000.0원 (+32.18%)</t>
+          <t>+372,000.0원 (+33.73%)</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>1,371,000원</t>
+          <t>1,460,000원</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>1,443,500원</t>
+          <t>1,706,000원</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>1,414,500원</t>
+          <t>1,423,500원</t>
         </is>
       </c>
       <c r="J16" s="3" t="inlineStr">
         <is>
-          <t>+5.3%</t>
+          <t>+16.8%</t>
         </is>
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>🔴 단기 비중 축소 (악재 주의)</t>
+          <t>🟢 오늘 단기 매수 (저점 반등)</t>
         </is>
       </c>
       <c r="L16" s="3" t="inlineStr">
         <is>
-          <t>악재 보도 및 5일 연속 약세로 단기 추가 하락 위험</t>
+          <t>RSI 34.2로 단기 과매도 구간 진입, 기술적 반등 노림</t>
         </is>
       </c>
       <c r="M16" s="3" t="inlineStr">
@@ -6034,21 +5888,21 @@
         </is>
       </c>
       <c r="O16" s="3" t="n">
-        <v>32.7</v>
+        <v>34.2</v>
       </c>
       <c r="P16" s="3" t="inlineStr">
         <is>
-          <t>-16.2%</t>
+          <t>-15.3%</t>
         </is>
       </c>
       <c r="Q16" s="3" t="inlineStr">
         <is>
-          <t>40.7%</t>
+          <t>41.4%</t>
         </is>
       </c>
       <c r="R16" s="3" t="inlineStr">
         <is>
-          <t>삼성전자 '100조 잭팟' 뒤 서늘한 경고…"한국이 흔들린다" [테크로그] (한국경제)</t>
+          <t>최근 특이 뉴스 없음</t>
         </is>
       </c>
     </row>
@@ -6075,42 +5929,42 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>318,500원</t>
+          <t>319,500원</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>-173,000.0원 (-35.20%)</t>
+          <t>-172,000.0원 (-34.99%)</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>315,500원</t>
+          <t>313,000원</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>342,500원</t>
+          <t>382,500원</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>307,500원</t>
+          <t>303,500원</t>
         </is>
       </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
-          <t>+8.6%</t>
+          <t>+22.2%</t>
         </is>
       </c>
       <c r="K17" s="3" t="inlineStr">
         <is>
-          <t>🟢 오늘 단기 매수 (저점 반등)</t>
+          <t>⏸️ 관망/보유 (쿨다운 1일차)</t>
         </is>
       </c>
       <c r="L17" s="3" t="inlineStr">
         <is>
-          <t>RSI 25.2로 단기 과매도 구간 진입, 기술적 반등 노림</t>
+          <t>최근 1일 전(2026-10-13) 단기 매수 추천 이력 존재 ➔ 중복 매수 방지 쿨다운 적용(기존 포지션 분할 보유/관망 권고)</t>
         </is>
       </c>
       <c r="M17" s="3" t="inlineStr">
@@ -6124,21 +5978,21 @@
         </is>
       </c>
       <c r="O17" s="3" t="n">
-        <v>25.2</v>
+        <v>26.1</v>
       </c>
       <c r="P17" s="3" t="inlineStr">
         <is>
-          <t>-8.9%</t>
+          <t>-8.6%</t>
         </is>
       </c>
       <c r="Q17" s="3" t="inlineStr">
         <is>
-          <t>17.8%</t>
+          <t>17.7%</t>
         </is>
       </c>
       <c r="R17" s="3" t="inlineStr">
         <is>
-          <t>1∼8월 배터리 분리막 적재량 25%↑…중국 제외 41% 성장 (주요언론)</t>
+          <t>최근 특이 뉴스 없음</t>
         </is>
       </c>
     </row>
@@ -6165,42 +6019,42 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>110,000원</t>
+          <t>109,500원</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>-39,300.0원 (-26.34%)</t>
+          <t>-39,500.0원 (-26.47%)</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>109,000원</t>
+          <t>107,500원</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>116,500원</t>
+          <t>126,500원</t>
         </is>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>106,000원</t>
+          <t>104,000원</t>
         </is>
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>+7.1%</t>
+          <t>+17.8%</t>
         </is>
       </c>
       <c r="K18" s="3" t="inlineStr">
         <is>
-          <t>🟢 오늘 단기 매수 (저점 반등)</t>
+          <t>⏸️ 관망/보유 (쿨다운 1일차)</t>
         </is>
       </c>
       <c r="L18" s="3" t="inlineStr">
         <is>
-          <t>RSI 33.5로 단기 과매도 구간 진입, 기술적 반등 노림</t>
+          <t>최근 1일 전(2026-10-13) 단기 매수 추천 이력 존재 ➔ 중복 매수 방지 쿨다운 적용(기존 포지션 분할 보유/관망 권고)</t>
         </is>
       </c>
       <c r="M18" s="3" t="inlineStr">
@@ -6214,16 +6068,16 @@
         </is>
       </c>
       <c r="O18" s="3" t="n">
-        <v>33.5</v>
+        <v>33</v>
       </c>
       <c r="P18" s="3" t="inlineStr">
         <is>
-          <t>-5.2%</t>
+          <t>-5.3%</t>
         </is>
       </c>
       <c r="Q18" s="3" t="inlineStr">
         <is>
-          <t>8.4%</t>
+          <t>7.1%</t>
         </is>
       </c>
       <c r="R18" s="3" t="inlineStr">
@@ -6255,42 +6109,42 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>182,000원</t>
+          <t>181,500원</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>-19,400.0원 (-9.63%)</t>
+          <t>-19,900.0원 (-9.88%)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>180,500원</t>
+          <t>178,000원</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>193,000원</t>
+          <t>206,500원</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>175,500원</t>
+          <t>172,500원</t>
         </is>
       </c>
       <c r="J19" s="3" t="inlineStr">
         <is>
-          <t>+7.1%</t>
+          <t>+16.0%</t>
         </is>
       </c>
       <c r="K19" s="3" t="inlineStr">
         <is>
-          <t>🟢 오늘 단기 매수 (저점 반등)</t>
+          <t>⏸️ 관망/보유 (쿨다운 1일차)</t>
         </is>
       </c>
       <c r="L19" s="3" t="inlineStr">
         <is>
-          <t>RSI 33.3로 단기 과매도 구간 진입, 기술적 반등 노림</t>
+          <t>최근 1일 전(2026-10-13) 단기 매수 추천 이력 존재 ➔ 중복 매수 방지 쿨다운 적용(기존 포지션 분할 보유/관망 권고)</t>
         </is>
       </c>
       <c r="M19" s="3" t="inlineStr">
@@ -6304,16 +6158,16 @@
         </is>
       </c>
       <c r="O19" s="3" t="n">
-        <v>33.3</v>
+        <v>32.6</v>
       </c>
       <c r="P19" s="3" t="inlineStr">
         <is>
-          <t>-6.2%</t>
+          <t>-6.4%</t>
         </is>
       </c>
       <c r="Q19" s="3" t="inlineStr">
         <is>
-          <t>3.3%</t>
+          <t>6.4%</t>
         </is>
       </c>
       <c r="R19" s="3" t="inlineStr">
@@ -6345,42 +6199,42 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>32,000원</t>
+          <t>31,900원</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>-16,150.0원 (-33.58%)</t>
+          <t>-16,200.0원 (-33.68%)</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>31,600원</t>
+          <t>31,300원</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>33,900원</t>
+          <t>34,600원</t>
         </is>
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>30,800원</t>
+          <t>30,300원</t>
         </is>
       </c>
       <c r="J20" s="3" t="inlineStr">
         <is>
-          <t>+7.1%</t>
+          <t>+10.8%</t>
         </is>
       </c>
       <c r="K20" s="3" t="inlineStr">
         <is>
-          <t>🟢 오늘 단기 매수 (저점 반등)</t>
+          <t>⏸️ 관망/보유 (쿨다운 1일차)</t>
         </is>
       </c>
       <c r="L20" s="3" t="inlineStr">
         <is>
-          <t>RSI 34.9로 단기 과매도 구간 진입, 기술적 반등 노림</t>
+          <t>최근 1일 전(2026-10-13) 단기 매수 추천 이력 존재 ➔ 중복 매수 방지 쿨다운 적용(기존 포지션 분할 보유/관망 권고)</t>
         </is>
       </c>
       <c r="M20" s="3" t="inlineStr">
@@ -6394,16 +6248,16 @@
         </is>
       </c>
       <c r="O20" s="3" t="n">
-        <v>34.9</v>
+        <v>34.4</v>
       </c>
       <c r="P20" s="3" t="inlineStr">
         <is>
-          <t>-4.3%</t>
+          <t>-4.4%</t>
         </is>
       </c>
       <c r="Q20" s="3" t="inlineStr">
         <is>
-          <t>2.1%</t>
+          <t>4.2%</t>
         </is>
       </c>
       <c r="R20" s="3" t="inlineStr">
@@ -6435,27 +6289,27 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>183,500원</t>
+          <t>182,000원</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>-6,019.049999999988원 (-3.17%)</t>
+          <t>-7,419.049999999988원 (-3.91%)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>180,000원</t>
+          <t>178,500원</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>193,000원</t>
+          <t>191,500원</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>174,500원</t>
+          <t>173,000원</t>
         </is>
       </c>
       <c r="J21" s="3" t="inlineStr">
@@ -6484,16 +6338,16 @@
         </is>
       </c>
       <c r="O21" s="3" t="n">
-        <v>52.9</v>
+        <v>50.3</v>
       </c>
       <c r="P21" s="3" t="inlineStr">
         <is>
-          <t>+2.0%</t>
+          <t>+1.3%</t>
         </is>
       </c>
       <c r="Q21" s="3" t="inlineStr">
         <is>
-          <t>31.2%</t>
+          <t>29.4%</t>
         </is>
       </c>
       <c r="R21" s="3" t="inlineStr">
@@ -6525,42 +6379,42 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>828,000원</t>
+          <t>835,000원</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>-695,000.0원 (-45.63%)</t>
+          <t>-688,000.0원 (-45.17%)</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>819,500원</t>
+          <t>818,500원</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>991,500원</t>
+          <t>1,137,000원</t>
         </is>
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>799,000원</t>
+          <t>793,000원</t>
         </is>
       </c>
       <c r="J22" s="3" t="inlineStr">
         <is>
-          <t>+20.9%</t>
+          <t>+38.9%</t>
         </is>
       </c>
       <c r="K22" s="3" t="inlineStr">
         <is>
-          <t>🟢 오늘 단기 매수 (저점 반등)</t>
+          <t>⏸️ 관망/보유 (쿨다운 1일차)</t>
         </is>
       </c>
       <c r="L22" s="3" t="inlineStr">
         <is>
-          <t>RSI 28.8로 단기 과매도 구간 진입, 기술적 반등 노림</t>
+          <t>최근 1일 전(2026-10-13) 단기 매수 추천 이력 존재 ➔ 중복 매수 방지 쿨다운 적용(기존 포지션 분할 보유/관망 권고)</t>
         </is>
       </c>
       <c r="M22" s="3" t="inlineStr">
@@ -6574,16 +6428,16 @@
         </is>
       </c>
       <c r="O22" s="3" t="n">
-        <v>28.8</v>
+        <v>29.3</v>
       </c>
       <c r="P22" s="3" t="inlineStr">
         <is>
-          <t>-18.1%</t>
+          <t>-17.5%</t>
         </is>
       </c>
       <c r="Q22" s="3" t="inlineStr">
         <is>
-          <t>5.2%</t>
+          <t>6.0%</t>
         </is>
       </c>
       <c r="R22" s="3" t="inlineStr">
@@ -6615,12 +6469,12 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>419,500원</t>
+          <t>422,500원</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>+19,500.0원 (+4.88%)</t>
+          <t>+22,500.0원 (+5.62%)</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -6630,17 +6484,17 @@
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>419,500원</t>
+          <t>422,500원</t>
         </is>
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>411,000원</t>
+          <t>414,000원</t>
         </is>
       </c>
       <c r="J23" s="3" t="inlineStr">
         <is>
-          <t>+12.7%</t>
+          <t>+13.5%</t>
         </is>
       </c>
       <c r="K23" s="3" t="inlineStr">
@@ -6650,7 +6504,7 @@
       </c>
       <c r="L23" s="3" t="inlineStr">
         <is>
-          <t>RSI 70.4, 20일선 이격도 +12.8%로 단기 과열권, 분할 차익 실현 권고</t>
+          <t>RSI 71.1, 20일선 이격도 +13.5%로 단기 과열권, 분할 차익 실현 권고</t>
         </is>
       </c>
       <c r="M23" s="3" t="inlineStr">
@@ -6664,21 +6518,21 @@
         </is>
       </c>
       <c r="O23" s="3" t="n">
-        <v>70.40000000000001</v>
+        <v>71.09999999999999</v>
       </c>
       <c r="P23" s="3" t="inlineStr">
         <is>
-          <t>+12.8%</t>
+          <t>+13.5%</t>
         </is>
       </c>
       <c r="Q23" s="3" t="inlineStr">
         <is>
-          <t>54.5%</t>
+          <t>55.8%</t>
         </is>
       </c>
       <c r="R23" s="3" t="inlineStr">
         <is>
-          <t>1∼8월 배터리 분리막 적재량 25%↑…중국 제외 41% 성장 (주요언론)</t>
+          <t>최근 특이 뉴스 없음</t>
         </is>
       </c>
     </row>
@@ -6705,17 +6559,17 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>309,500원</t>
+          <t>309,000원</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>-52,000.0원 (-14.38%)</t>
+          <t>-52,500.0원 (-14.52%)</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>303,500원</t>
+          <t>303,000원</t>
         </is>
       </c>
       <c r="H24" s="3" t="inlineStr">
@@ -6725,12 +6579,12 @@
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>294,000원</t>
+          <t>293,500원</t>
         </is>
       </c>
       <c r="J24" s="3" t="inlineStr">
         <is>
-          <t>+10.1%</t>
+          <t>+10.3%</t>
         </is>
       </c>
       <c r="K24" s="3" t="inlineStr">
@@ -6754,16 +6608,16 @@
         </is>
       </c>
       <c r="O24" s="3" t="n">
-        <v>45.7</v>
+        <v>45.3</v>
       </c>
       <c r="P24" s="3" t="inlineStr">
         <is>
-          <t>-1.7%</t>
+          <t>-1.9%</t>
         </is>
       </c>
       <c r="Q24" s="3" t="inlineStr">
         <is>
-          <t>15.3%</t>
+          <t>12.7%</t>
         </is>
       </c>
       <c r="R24" s="3" t="inlineStr">
@@ -6795,7 +6649,7 @@
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>$228.52</t>
+          <t>$228.52 (약 306,417원)</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
@@ -6805,12 +6659,12 @@
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>$223.95</t>
+          <t>$223.95 (약 300,289원)</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
-          <t>$239.95</t>
+          <t>$239.95 (약 321,738원)</t>
         </is>
       </c>
       <c r="I25" s="3" t="inlineStr">
@@ -6844,11 +6698,11 @@
         </is>
       </c>
       <c r="O25" s="3" t="n">
-        <v>49.4</v>
+        <v>52</v>
       </c>
       <c r="P25" s="3" t="inlineStr">
         <is>
-          <t>+0.5%</t>
+          <t>+0.1%</t>
         </is>
       </c>
       <c r="Q25" s="3" t="inlineStr">
@@ -6858,7 +6712,7 @@
       </c>
       <c r="R25" s="3" t="inlineStr">
         <is>
-          <t>최근 특이 뉴스 없음</t>
+          <t>'월가 족집게' 댄 아이브스 "테슬라·스페이스X 내년 합병 가능성 80%" (주요언론)</t>
         </is>
       </c>
     </row>
@@ -6885,7 +6739,7 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>$341.27</t>
+          <t>$341.27 (약 457,602원)</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
@@ -6895,12 +6749,12 @@
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>$334.44</t>
+          <t>$334.44 (약 448,450원)</t>
         </is>
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
-          <t>$358.33</t>
+          <t>$358.33 (약 480,482원)</t>
         </is>
       </c>
       <c r="I26" s="3" t="inlineStr">
@@ -6934,11 +6788,11 @@
         </is>
       </c>
       <c r="O26" s="3" t="n">
-        <v>60.2</v>
+        <v>60.5</v>
       </c>
       <c r="P26" s="3" t="inlineStr">
         <is>
-          <t>+1.6%</t>
+          <t>+1.5%</t>
         </is>
       </c>
       <c r="Q26" s="3" t="inlineStr">
@@ -6975,7 +6829,7 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>$375.23</t>
+          <t>$375.23 (약 503,138원)</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
@@ -6985,12 +6839,12 @@
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>$367.73</t>
+          <t>$367.73 (약 493,075원)</t>
         </is>
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>$393.99</t>
+          <t>$393.99 (약 528,295원)</t>
         </is>
       </c>
       <c r="I27" s="3" t="inlineStr">
@@ -7024,11 +6878,11 @@
         </is>
       </c>
       <c r="O27" s="3" t="n">
-        <v>56.4</v>
+        <v>54.5</v>
       </c>
       <c r="P27" s="3" t="inlineStr">
         <is>
-          <t>+1.5%</t>
+          <t>+1.3%</t>
         </is>
       </c>
       <c r="Q27" s="3" t="inlineStr">
@@ -7037,6 +6891,96 @@
         </is>
       </c>
       <c r="R27" s="3" t="inlineStr">
+        <is>
+          <t>'월가 족집게' 댄 아이브스 "테슬라·스페이스X 내년 합병 가능성 80%" (주요언론)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>마이크로소프트 (Microsoft)</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>글로벌 AI/클라우드</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>$543.45 (약 728,701원)</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>+159.08000000000004$ (+41.39%)</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>$514.20 (약 689,480원)</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>$543.45 (약 728,701원)</t>
+        </is>
+      </c>
+      <c r="I28" s="3" t="inlineStr">
+        <is>
+          <t>$532.58</t>
+        </is>
+      </c>
+      <c r="J28" s="3" t="inlineStr">
+        <is>
+          <t>+5.7%</t>
+        </is>
+      </c>
+      <c r="K28" s="3" t="inlineStr">
+        <is>
+          <t>🔴 오늘 단기 매도 (과열 차익실현)</t>
+        </is>
+      </c>
+      <c r="L28" s="3" t="inlineStr">
+        <is>
+          <t>RSI 70.7, 20일선 이격도 +5.7%로 단기 과열권, 분할 차익 실현 권고</t>
+        </is>
+      </c>
+      <c r="M28" s="3" t="inlineStr">
+        <is>
+          <t>보유 / 중립 (HOLD)</t>
+        </is>
+      </c>
+      <c r="N28" s="3" t="inlineStr">
+        <is>
+          <t>장기 추세 유지</t>
+        </is>
+      </c>
+      <c r="O28" s="3" t="n">
+        <v>70.7</v>
+      </c>
+      <c r="P28" s="3" t="inlineStr">
+        <is>
+          <t>+5.7%</t>
+        </is>
+      </c>
+      <c r="Q28" s="3" t="inlineStr">
+        <is>
+          <t>95.0%</t>
+        </is>
+      </c>
+      <c r="R28" s="3" t="inlineStr">
         <is>
           <t>최근 특이 뉴스 없음</t>
         </is>
@@ -7270,12 +7214,12 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>6,094.87</t>
+          <t>6,123.61</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>+59.52 (+0.99%)</t>
+          <t>+88.26 (+1.46%)</t>
         </is>
       </c>
     </row>
@@ -7297,12 +7241,12 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>830.88</t>
+          <t>832.41</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>-6.15 (-0.73%)</t>
+          <t>-4.62 (-0.55%)</t>
         </is>
       </c>
     </row>
@@ -7516,27 +7460,27 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>112,595,000원</t>
+          <t>112,538,000원</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>+0.00%</t>
+          <t>-0.05%</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>112,032,000원</t>
+          <t>111,975,000원</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>121,603,000원</t>
+          <t>121,541,000원</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>110,576,000원</t>
+          <t>110,573,000원</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
@@ -7573,27 +7517,27 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>3,385,000원</t>
+          <t>3,384,000원</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>+0.12%</t>
+          <t>+0.09%</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>3,358,000원</t>
+          <t>3,357,000원</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>3,588,000원</t>
+          <t>3,587,000원</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>3,266,500원</t>
+          <t>3,265,500원</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
@@ -7630,17 +7574,17 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>144,900원</t>
+          <t>145,000원</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>+0.21%</t>
+          <t>+0.28%</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>143,700원</t>
+          <t>143,800원</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -7650,12 +7594,12 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>139,800원</t>
+          <t>139,900원</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>+8.4%</t>
+          <t>+8.3%</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
@@ -7665,7 +7609,7 @@
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>RSI 47.1로 단기 과매도 구간 진입, 기술적 반등 기대</t>
+          <t>RSI 47.3로 단기 과매도 구간 진입, 기술적 반등 기대</t>
         </is>
       </c>
     </row>
@@ -7680,7 +7624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:N11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -7692,6 +7636,11 @@
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="65" customWidth="1" min="8" max="8"/>
     <col width="65" customWidth="1" min="9" max="9"/>
+    <col width="17" customWidth="1" min="10" max="10"/>
+    <col width="19" customWidth="1" min="11" max="11"/>
+    <col width="17" customWidth="1" min="12" max="12"/>
+    <col width="19" customWidth="1" min="13" max="13"/>
+    <col width="65" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7740,6 +7689,31 @@
           <t>PDF파일명</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>2026F_예상매출</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>2026F_예상영업익</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>2027F_예상매출</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>2027F_예상영업익</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>실적전망요약</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -7748,7 +7722,7 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -7783,6 +7757,31 @@
       <c r="I2" s="3" t="inlineStr">
         <is>
           <t>2026-10-14_신한투자증권_팬오션_빛을 보기 시작한 포트폴리오 변화.pdf</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>7,426.1십억원</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="inlineStr">
+        <is>
+          <t>726.2십억원</t>
+        </is>
+      </c>
+      <c r="L2" s="3" t="inlineStr">
+        <is>
+          <t>7,662.9십억원</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>742.3십억원</t>
+        </is>
+      </c>
+      <c r="N2" s="3" t="inlineStr">
+        <is>
+          <t>3Q26 영업이익 2,027억원(+61</t>
         </is>
       </c>
     </row>
@@ -7793,21 +7792,21 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>신한투자증권</t>
+          <t>하나증권</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>일진전기</t>
+          <t>한미약품</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>가장 저평가된 전력기기</t>
+          <t>더 안정적인 성장을 위한 정비 작업(3Q26 Pre)</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
@@ -7817,17 +7816,42 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>매수</t>
+          <t>Buy</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>변압기 29년 수주 논의 및 전선 상반기 수주 급증 5월 시가총액 약 6.9조원 도달 이후 7월말 2.2조원까지 약 68% 하락. 전선업체들의 수주잔고총계 연간 증가율은 24년 25.4%, 25년 21.2%에서 26년 상반기에만 23.2% 증가. 변압기에 이은 전선 부문의 호황이 확대되는 것을 감안할 때 펀더멘털 문제가 아닌 수급 측면의 주가 하락으로 판단</t>
+          <t>선급금 4Q26 반영, 북경한미 정비 작업과 앱토즈 인수로 전체적인 실적은 부진 3Q26 실적은 연결기준 매출액 3,794억원(YoY+4.7%), 영업이익 381억원(YoY-30.8%, OPM 10.0%)으로 예상된다. 컨센서스와 크게 어긋나 보이지만, Genentech향 HM17321 L/O 선급금이 미국 HSR 행정절차가 10월 초 완료됨에 따라 4Q26에 인식되는데 컨센서스가 미리 3Q에 이를 반영했기 때문이다. 2Q에 Lilly향 L/O에 따른 선급금이 반영되었기 때문에 QoQ로 비교하는 것도 큰 의미가 없다. 선급금이 없던</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>2026-10-14_신한투자증권_일진전기_가장 저평가된 전력기기.pdf</t>
+          <t>2026-10-14_하나증권_한미약품_더 안정적인 성장을 위한 정비 작업(3Q26 Pre).pdf</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>1,895.0십억원</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>494.6십억원</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>1,844.1십억원</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>284.7십억원</t>
+        </is>
+      </c>
+      <c r="N3" s="3" t="inlineStr">
+        <is>
+          <t>3Q26 실적은 연결기준 매출액 3,794억원(YoY+4</t>
         </is>
       </c>
     </row>
@@ -7847,12 +7871,12 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>HMM</t>
+          <t>일진전기</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>우려도 있지만 너무 잠잠한 주가</t>
+          <t>가장 저평가된 전력기기</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -7867,12 +7891,37 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>거버넌스 우려로 덮어놓기엔 아까운 실적 글로벌 컨테이너선사들은 가이던스 상향과 함께 주가도 상승했으나 동사 반응은 제한적. 거버넌스 불확실성에도 예상보다 큰 이익 회복에 주목</t>
+          <t>변압기 29년 수주 논의 및 전선 상반기 수주 급증 5월 시가총액 약 6.9조원 도달 이후 7월말 2.2조원까지 약 68% 하락. 전선업체들의 수주잔고총계 연간 증가율은 24년 25.4%, 25년 21.2%에서 26년 상반기에만 23.2% 증가. 변압기에 이은 전선 부문의 호황이 확대되는 것을 감안할 때 펀더멘털 문제가 아닌 수급 측면의 주가 하락으로 판단</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>2026-10-14_신한투자증권_HMM_우려도 있지만 너무 잠잠한 주가.pdf</t>
+          <t>2026-10-14_신한투자증권_일진전기_가장 저평가된 전력기기.pdf</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>2,350.8십억원</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>252.8십억원</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>2,595.2십억원</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>271.7십억원</t>
+        </is>
+      </c>
+      <c r="N4" s="3" t="inlineStr">
+        <is>
+          <t>2026/2027 실적 성장세 및 기업가치 재평가 전망</t>
         </is>
       </c>
     </row>
@@ -7883,21 +7932,21 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>하나증권</t>
+          <t>신한투자증권</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>한미약품</t>
+          <t>HMM</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>더 안정적인 성장을 위한 정비 작업(3Q26 Pre)</t>
+          <t>우려도 있지만 너무 잠잠한 주가</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -7907,17 +7956,42 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Buy</t>
+          <t>매수</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>선급금 4Q26 반영, 북경한미 정비 작업과 앱토즈 인수로 전체적인 실적은 부진 3Q26 실적은 연결기준 매출액 3,794억원(YoY+4.7%), 영업이익 381억원(YoY-30.8%, OPM 10.0%)으로 예상된다. 컨센서스와 크게 어긋나 보이지만, Genentech향 HM17321 L/O 선급금이 미국 HSR 행정절차가 10월 초 완료됨에 따라 4Q26에 인식되는데 컨센서스가 미리 3Q에 이를 반영했기 때문이다. 2Q에 Lilly향 L/O에 따른 선급금이 반영되었기 때문에 QoQ로 비교하는 것도 큰 의미가 없다. 선급금이 없던</t>
+          <t>거버넌스 우려로 덮어놓기엔 아까운 실적 글로벌 컨테이너선사들은 가이던스 상향과 함께 주가도 상승했으나 동사 반응은 제한적. 거버넌스 불확실성에도 예상보다 큰 이익 회복에 주목</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>2026-10-14_하나증권_한미약품_더 안정적인 성장을 위한 정비 작업(3Q26 Pre).pdf</t>
+          <t>2026-10-14_신한투자증권_HMM_우려도 있지만 너무 잠잠한 주가.pdf</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>14,179.9십억원</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>2,497.7십억원</t>
+        </is>
+      </c>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>14,293.1십억원</t>
+        </is>
+      </c>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>1,812.7십억원</t>
+        </is>
+      </c>
+      <c r="N5" s="3" t="inlineStr">
+        <is>
+          <t>3Q26 매출 4조 802억원(+51%, 이하 YoY) 및 영업이익 1조 42억원(+</t>
         </is>
       </c>
     </row>
@@ -7965,6 +8039,31 @@
           <t>2026-10-14_신한투자증권_현대글로비스_환율은 야속하지만 너무 좋은 해운 업황.pdf</t>
         </is>
       </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>33,217.4십억원</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>2,077.2십억원</t>
+        </is>
+      </c>
+      <c r="L6" s="3" t="inlineStr">
+        <is>
+          <t>34,964.5십억원</t>
+        </is>
+      </c>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>2,408.5십억원</t>
+        </is>
+      </c>
+      <c r="N6" s="3" t="inlineStr">
+        <is>
+          <t>2026/2027 실적 성장세 및 기업가치 재평가 전망</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -7977,17 +8076,17 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>미래에셋증권</t>
+          <t>하나증권</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>휴젤</t>
+          <t>삼성화재</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>3Q26 Preview: 단기 실적 눈높이 조정</t>
+          <t>3Q26 Pre - 단기 실적보다 중요한 것은</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
@@ -7997,17 +8096,42 @@
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>매수</t>
+          <t>Buy</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">3분기 실적은 미국 판매체계 전환 영향으로 부진 휴젤의 3Q26 매출액은 1,009억원(-4.7% YoY), 영업이익 211억원(-55.5% YoY)으로 추정했다. 3Q26 영업이익은 미국 판매체계 전환 영향으로 전년 동기 대비 55.5% 감소할 것으로 보인다. 3분기는 미국 유통사 모델에서 CSO 모델로 전환하는 과정에서 일회성 매출 차감과 비용 증가가 동반되는 구간이었기 때문이다. 기존 유통사 재고 바이백으로 미국 매출은 마이너스가 예상된다. ASP가 높은 미국향 톡신 매출 공백으로 매출총이익률도 전년 동기 대비 6%p 하락이 </t>
+          <t xml:space="preserve">2026년 3분기 실적은 컨센서스 하회 전망 3분기 연결 지배순이익은 4,863억원으로 컨센서스(5,825억원)를 하회할 것으로 전망한다. 장기보험손익이 사업비 부담 확대로 예상대비 부한 가운데, 증시 부진과 금리 상승에 따른 투자손익 악화도 실적에 부담으로 작용할 것으로 예상한다. [보험손익] 보험손익은 4,006억원(YoY +8.6%, QoQ -27.5%)으로 추정한다. 장기보험손익은 3,560억원으로 YoY/QoQ 모두 감소할 것으로 예상하며, 사업비 부담 확대가 주요 원인이다. 자동차보험손익은 전분기대비 감소하겠으나 YoY </t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>2026-10-14_미래에셋증권_휴젤_3Q26 Preview 단기 실적 눈높이 조정.pdf</t>
+          <t>2026-10-14_하나증권_삼성화재_3Q26 Pre - 단기 실적보다 중요한 것은.pdf</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>3,496십억원</t>
+        </is>
+      </c>
+      <c r="L7" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M7" s="3" t="inlineStr">
+        <is>
+          <t>4,566십억원</t>
+        </is>
+      </c>
+      <c r="N7" s="3" t="inlineStr">
+        <is>
+          <t>2026/2027 실적 성장세 및 기업가치 재평가 전망</t>
         </is>
       </c>
     </row>
@@ -8018,21 +8142,21 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>하나증권</t>
+          <t>미래에셋증권</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>삼성화재</t>
+          <t>휴젤</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>3Q26 Pre - 단기 실적보다 중요한 것은</t>
+          <t>3Q26 Preview: 단기 실적 눈높이 조정</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -8042,17 +8166,42 @@
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>Buy</t>
+          <t>매수</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026년 3분기 실적은 컨센서스 하회 전망 3분기 연결 지배순이익은 4,863억원으로 컨센서스(5,825억원)를 하회할 것으로 전망한다. 장기보험손익이 사업비 부담 확대로 예상대비 부한 가운데, 증시 부진과 금리 상승에 따른 투자손익 악화도 실적에 부담으로 작용할 것으로 예상한다. [보험손익] 보험손익은 4,006억원(YoY +8.6%, QoQ -27.5%)으로 추정한다. 장기보험손익은 3,560억원으로 YoY/QoQ 모두 감소할 것으로 예상하며, 사업비 부담 확대가 주요 원인이다. 자동차보험손익은 전분기대비 감소하겠으나 YoY </t>
+          <t xml:space="preserve">3분기 실적은 미국 판매체계 전환 영향으로 부진 휴젤의 3Q26 매출액은 1,009억원(-4.7% YoY), 영업이익 211억원(-55.5% YoY)으로 추정했다. 3Q26 영업이익은 미국 판매체계 전환 영향으로 전년 동기 대비 55.5% 감소할 것으로 보인다. 3분기는 미국 유통사 모델에서 CSO 모델로 전환하는 과정에서 일회성 매출 차감과 비용 증가가 동반되는 구간이었기 때문이다. 기존 유통사 재고 바이백으로 미국 매출은 마이너스가 예상된다. ASP가 높은 미국향 톡신 매출 공백으로 매출총이익률도 전년 동기 대비 6%p 하락이 </t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>2026-10-14_하나증권_삼성화재_3Q26 Pre - 단기 실적보다 중요한 것은.pdf</t>
+          <t>2026-10-14_미래에셋증권_휴젤_3Q26 Preview 단기 실적 눈높이 조정.pdf</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>486십억원</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>174십억원</t>
+        </is>
+      </c>
+      <c r="L8" s="3" t="inlineStr">
+        <is>
+          <t>657십억원</t>
+        </is>
+      </c>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>272십억원</t>
+        </is>
+      </c>
+      <c r="N8" s="3" t="inlineStr">
+        <is>
+          <t>3Q26 매출액은 1,009억원(-4</t>
         </is>
       </c>
     </row>
@@ -8063,7 +8212,7 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -8098,6 +8247,31 @@
       <c r="I9" s="3" t="inlineStr">
         <is>
           <t>2026-10-14_하나증권_세아베스틸지주_3분기는 다소 부진하겠지만 4분기부터 회복 기대.pdf</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>4,116.0십억원</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>140.6십억원</t>
+        </is>
+      </c>
+      <c r="L9" s="3" t="inlineStr">
+        <is>
+          <t>4,496.9십억원</t>
+        </is>
+      </c>
+      <c r="M9" s="3" t="inlineStr">
+        <is>
+          <t>223.3십억원</t>
+        </is>
+      </c>
+      <c r="N9" s="3" t="inlineStr">
+        <is>
+          <t>3Q26 영업이익 236억원(YoY -</t>
         </is>
       </c>
     </row>
@@ -8108,7 +8282,7 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -8143,6 +8317,31 @@
       <c r="I10" s="3" t="inlineStr">
         <is>
           <t>2026-10-14_하나증권_한화손해보험_3Q26 Pre - 보험손익 개선세에 주목.pdf</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t>465십억원</t>
+        </is>
+      </c>
+      <c r="L10" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M10" s="3" t="inlineStr">
+        <is>
+          <t>595십억원</t>
+        </is>
+      </c>
+      <c r="N10" s="3" t="inlineStr">
+        <is>
+          <t>2026/2027 실적 성장세 및 기업가치 재평가 전망</t>
         </is>
       </c>
     </row>
@@ -8153,7 +8352,7 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
@@ -8188,6 +8387,991 @@
       <c r="I11" s="3" t="inlineStr">
         <is>
           <t>2026-10-14_하나증권_세아제강_어려운 영업환경!.pdf</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>1,822.7십억원</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>103.1십억원</t>
+        </is>
+      </c>
+      <c r="L11" s="3" t="inlineStr">
+        <is>
+          <t>1,852.8십억원</t>
+        </is>
+      </c>
+      <c r="M11" s="3" t="inlineStr">
+        <is>
+          <t>124.3십억원</t>
+        </is>
+      </c>
+      <c r="N11" s="3" t="inlineStr">
+        <is>
+          <t>2026년 3분기 세아제강의 매출액과 영업이익은 각각 4,318억원(YoY +30</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="32" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>검증기준일</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>추천일자</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>종목명</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>티커</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>추천당시가</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>매수추천가</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>목표매도가</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>손절기준가</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>검증결과</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>실현수익률</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>최고도달가</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>소요일수</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>현대차</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>005380.KS</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>315,000원</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>312,000원</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>349,500원</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>304,000원</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>⏳ 진행 중 (보유 중)</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>+2.2%</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="inlineStr">
+        <is>
+          <t>321,500원</t>
+        </is>
+      </c>
+      <c r="L2" s="3" t="inlineStr">
+        <is>
+          <t>1일 경과</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>기아</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>000270.KS</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>108,500원</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>107,000원</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>115,500원</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>104,500원</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>⏳ 진행 중 (보유 중)</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>+2.5%</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>110,700원</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>1일 경과</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>NAVER</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>035420.KS</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>178,000원</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>176,000원</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>193,000원</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>172,000원</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>⏳ 진행 중 (보유 중)</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>+3.2%</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>183,200원</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>1일 경과</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>카카오</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>035720.KS</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>31,300원</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>31,000원</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>33,200원</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>30,200원</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>⏳ 진행 중 (보유 중)</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>+2.9%</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>32,100원</t>
+        </is>
+      </c>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>1일 경과</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>한화에어로스페이스</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>012450.KS</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>839,000원</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>830,500원</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>1,012,000원</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>809,500원</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>⏳ 진행 중 (보유 중)</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>+0.5%</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>839,000원</t>
+        </is>
+      </c>
+      <c r="L6" s="3" t="inlineStr">
+        <is>
+          <t>1일 경과</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>POSCO홀딩스</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>005490.KS</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>299,000원</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>296,000원</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>317,000원</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>288,500원</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>⏳ 진행 중 (보유 중)</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>+4.4%</t>
+        </is>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>312,000원</t>
+        </is>
+      </c>
+      <c r="L7" s="3" t="inlineStr">
+        <is>
+          <t>1일 경과</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>SK하이닉스</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>000660.KS</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>1,475,000원</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>1,460,000원</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>1,706,000원</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>1,423,500원</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>⏳ 진행 중 (당일 포지션 구축)</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>+1.0%</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>1,475,000원</t>
+        </is>
+      </c>
+      <c r="L8" s="3" t="inlineStr">
+        <is>
+          <t>1일차</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="29" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="65" customWidth="1" min="5" max="5"/>
+    <col width="65" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="53" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>수집일자</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>공시구분</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>공시배지</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>관련기업</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>공시제목</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>영향전망</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>언론사</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>공시일시</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>💎 자사주 취득 (주가 부양)</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>자사주 취득</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>스틱인베스트먼트</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>[공시 Pick] 스틱인베스트먼트, 41억원 자사주 취득에 강세…장중 4%↑</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>기업 자금 투입으로 유통 물량 흡수 및 강력한 주가 바닥 지지 신호</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>뉴스투데이</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>Tue, 13 Oct 2026 05:20:00 GMT</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiXkFVX3lxTE41b0xlNUs4c2FxVTNMaENRVHJFM1prZDE0dWw0dy1CY1VYOVN3LVV4REtOUDJhTTFhU2lCS1RMcDlQeU8tVG8xSXVSbURwRW9oOHNaelhKdktwRjhmSWc?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>💎 자사주 취득 (주가 부양)</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>자사주 취득</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>데스트라 멀티 대체 투자 펀드, 자사주 매입 프로그램 도입·월 배당금 주당 0.115달러로 인상</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>기업 자금 투입으로 유통 물량 흡수 및 강력한 주가 바닥 지지 신호</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>데이터투자</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Tue, 13 Oct 2026 19:52:27 GMT</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMic0FVX3lxTE1lemt2YTFaYUFFeVI4cVJZbjFYOHpWLVJmNTUxN3huQlRtYUVHYXplTUpvQktSZFdKenhkMl9PYXlNci1RbHNtTUdQdXgxelpjaEJVbWNjVmFndWFiaV9KZFAxd2ozbVZXVUd4MHFPNlZYT0U?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>💎 자사주 취득 (주가 부양)</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>자사주 취득</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr"/>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>“역시 주주환원은 뒷전입니까”…코스피 자사주 매입, 삼전닉스 뺐더니 줄었다</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>기업 자금 투입으로 유통 물량 흡수 및 강력한 주가 바닥 지지 신호</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>매일경제 마켓</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Sun, 11 Oct 2026 11:51:10 GMT</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiUkFVX3lxTE0zXzFYa0xGekFCVWtnODd6QVRIRmp1MnFLcXhBWWVadVdXQWZaY3lGcGg3WUl1dzY4M1R1cTBWV1h1a0JBbXdGV3Y0aC1KV25lRmc?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>💎 자사주 취득 (주가 부양)</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>자사주 취득</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>AZZ, 연간 실적 가이던스 상향…2000만 달러 규모 자사주 매입</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>기업 자금 투입으로 유통 물량 흡수 및 강력한 주가 바닥 지지 신호</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>데이터투자</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Tue, 13 Oct 2026 20:20:27 GMT</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMickFVX3lxTE9QR3MyNXVOWndYaXJsdTF5Z2NaQnlGUVRFanBlUjhmN1U0TDNCMXNUZ2RrNTRselZhSGtXTW9YMUJGVWtvSTdDdFhCVVN6ZTVCcTZ0WnlkeUNsRTZlMGZBXzJnSnkxZ1Z3NjI5MlF0N0N3dw?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>💎 자사주 취득 (주가 부양)</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>자사주 취득</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>트러스트</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>선라이즈 리얼티 트러스트, 2000만 달러 자사주 매입 프로그램 승인</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>기업 자금 투입으로 유통 물량 흡수 및 강력한 주가 바닥 지지 신호</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>데이터투자</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>Tue, 13 Oct 2026 12:13:59 GMT</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMic0FVX3lxTE1fQmV2cFR2OFA5M1B6UXE3NF83TmRrd2lGSE1QelFpZWFMUDhZT1lHWHJYUnFBcmtKNUJmRWlwRTU3ME1ydno4cmpDMnpWMTF0Q09HQ0dmOVVubFFIYXNWZ1FhWlRZaEp3dk4xcHd2TmdFQ00?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>💎 자사주 취득 (주가 부양)</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>자사주 취득</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>아웃렛</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>올리스 바겐 아웃렛, 5억 달러 규모 신규 자사주 매입 승인</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>기업 자금 투입으로 유통 물량 흡수 및 강력한 주가 바닥 지지 신호</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>데이터투자</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Tue, 13 Oct 2026 11:09:56 GMT</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMic0FVX3lxTE5nZklvLUJYTTRmYUtlSnZGdWgzaE9aeExETGVnWDF1dXpLTGVMWWpSSEdodW1WMkprQW5oeEMxV0xtM0pIcndVZDVhVk5UWnIwcFNyMlI2X0hjb2M3UHBXME5sRGFCN0pYdDJWTEstSmpqVE0?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>💎 자사주 취득 (주가 부양)</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>자사주 취득</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>엘컴텍</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>엘컴텍, 20억원 규모 자사주 취득 결정</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>기업 자금 투입으로 유통 물량 흡수 및 강력한 주가 바닥 지지 신호</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>데이터투자</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>Tue, 13 Oct 2026 07:22:52 GMT</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMickFVX3lxTE13UXpQT2FyUjBQSkpSdFNtQVpJOHFGMExaeDFtajBra1h5dHl5S2dMbUV5TUdmMzFYZkF6b1RmSTd0TVk1NUZCOGN1Y1pWS3d1Rk50WmRUS19XZkJISzdJX3k1YXpPU2V3X3FhNkloOWs1QQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>💎 자사주 취득 (주가 부양)</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>자사주 취득</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>더핑크퐁컴퍼니</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>더핑크퐁컴퍼니, 50억원 규모 자사주 취득 신탁계약 해지 결정</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>기업 자금 투입으로 유통 물량 흡수 및 강력한 주가 바닥 지지 신호</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>데이터투자</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>Tue, 13 Oct 2026 05:43:38 GMT</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMic0FVX3lxTE1MVmRGS1NqcEJobXNpM01fNTlJbV9MeFZUeXBTVktGWV9XOWFlMHFET09BeW1rQ1RJdzVCR0I1OXM1UkpxM3Nnazk4RnBPbC1EaGFxM0FpVVpqYzZPRnlGb0plTEwyYmZDSXJXNW8yYmh5M0k?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Add YouTube Syuka World style Two-Track Deep Dive Storytelling Engine (Economy/Society & Trend/Lifestyle) with 8-sheet Excel and Email cards
</commit_message>
<xml_diff>
--- a/reports/일자별_누적_데일리_이슈_및_주식_브리핑_마스터.xlsx
+++ b/reports/일자별_누적_데일리_이슈_및_주식_브리핑_마스터.xlsx
@@ -14,6 +14,7 @@
     <sheet name="공식리포트_누적" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="추천성과_검증누적" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="특수공시_누적" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="스토리딥다이브_누적" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -458,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G107"/>
+  <dimension ref="A1:G154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3629,27 +3630,27 @@
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>신규 이슈</t>
+          <t>🔥 [언론사 집중 보도 (3개사)]</t>
         </is>
       </c>
       <c r="D86" s="3" t="inlineStr">
         <is>
-          <t>김용태 "은퇴봉사동물 지원예산 편성 2곳뿐…관리체계 개선해야"</t>
+          <t>김지용 "중수청, 외압 흔들림 없이 법·원칙 따라 공정 수사"</t>
         </is>
       </c>
       <c r="E86" s="3" t="inlineStr">
         <is>
-          <t>(서울=연합뉴스) 김세린 기자 = 국가봉사동물 운용 기관 대부분이 은퇴 동물에 대한 별도 지원 예산을 편성하지 않아 범부처 차원의 관리체계 개선...</t>
+          <t>김지용 "중수청, 외압 흔들림 없이 법·원칙 따라 공정 수사"  MBC 뉴스김지용 중수청장 후보자 "약자 대상 범죄 보완수사 빈틈없이"  조선일보김민석 “각자 역할 집중해야”…‘김지용 비판’ 추미애에 [지금뉴스]  KBS 뉴스김지용 "김학의 불법출금 무리한 기소 인정…책임 없지 않아" ...</t>
         </is>
       </c>
       <c r="F86" s="3" t="inlineStr">
         <is>
-          <t>주요언론</t>
+          <t>MBC 뉴스</t>
         </is>
       </c>
       <c r="G86" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261014083900030</t>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTFB5UDcySVc2Q3hrX1ZxUi1oOXVFTkJCSF9DUHZvVmVYY3BKeC0xdmN4RXVXcGxsRE45enFpYXNLcERDbVRBMWNWUHgydURaRkpTaV9KbHVqTGIwVEFTYkVXUHBzdVFMb1N3Zk80OUVzM1NRRGlNWVh30gF3QVVfeXFMUHgtOG9BQlprR3ZSc0JFeWthUFNsZ29BM0xyR2FmVm9iNkQxWm01REpPUmlPQzdHbUxobnpmVHp1ZE1ldHdRNHpZZ2h4YkFjWGREMzFWemcwUGFBY1JheDhOcHNlTzhsQ2VRUTIyWWRLbVMzZHZkU3M?oc=5</t>
         </is>
       </c>
     </row>
@@ -3661,32 +3662,32 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>사회/사건사고</t>
+          <t>정치</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>신규 이슈</t>
+          <t>연결 이슈 (후속)</t>
         </is>
       </c>
       <c r="D87" s="3" t="inlineStr">
         <is>
-          <t>달리기 대회서 20대女 사망에… '마라톤 거목' 황영조가 한 말</t>
+          <t>[사설]“대출 더 줄여야” “집값 급락 가능성”… LH 사장의 오지랖</t>
         </is>
       </c>
       <c r="E87" s="3" t="inlineStr">
         <is>
-          <t>달리기 대회서 20대女 사망에… '마라톤 거목' 황영조가 한 말  한국일보황영조 ‘죽음에 이르는 러닝’ 경고···“욕심 부리지 말고, 필요하면 포기할 줄 알아야”  경향신문'서울 달리기' 마라톤대회 참가했던 20대 여성 사망  연합뉴스'서울달리기' 숨진 20대女는 '카이스트 대학원생' ...</t>
+          <t>[사설]“대출 더 줄여야” “집값 급락 가능성”… LH 사장의 오지랖  동아일보이성훈 LH 사장, 고양창릉 첫마을 입주 준비 점검…공공임대 품질 강화 주문  전기신문유승민 “LH사장이 집값 예측할 때인가…주택공급이나 열심히 해야”  경기일보[기자수첩]대출 없이 집 산 LH 사장의 대출 ...</t>
         </is>
       </c>
       <c r="F87" s="3" t="inlineStr">
         <is>
-          <t>한국일보</t>
+          <t>동아일보</t>
         </is>
       </c>
       <c r="G87" s="3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMibkFVX3lxTFBNT1l5LUxfQjNUOTIwSDRwdGt0MDBBZXZzVjQwa1RMV21NTTNxOHVMNS1ydjgzZ0wxRlJkY0xPSzVkcDYydUt1SWxRR1FBbVpmMjU0WkJFeW5La1NZSlREczBuVUJuU19vTVdQbGJn0gFzQVVfeXFMTzFCN2tGdVpYMjI0a1Z0emhBR3pPWUZjRXlnRTdpTlRwY0lxTnhPb1dpc2gwekFNYm9LVW1PRnFuRm12eDNzRDkzWkZSUVA2T0VsTUx6UDRHQ0dZM3Z2U2pSbzhWdUxUUXRHaEQ5UldldTFuTQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTE43QTc0VC1rSWlsSzZteVRkOXNDYU5YbmlxVjJoeVV6bFZXNmw2V1NfSklHY2JHVHVLU0pja196Ml91MXhrN3ZxTHQ5SE5ZQUZuTkRHUHVrOGUxbEhuV2phcWF3MllveFEwVzlEaEMyUDFvMHVzMlHSAWZBVV95cUxQZTUtX0dhUVdyNmw0T1JCTzQzc1NtakNnWDJ4MXZ3Vk1SaVBvRmFFakE1MjA5a3NMT0FvTWplYjFBZWF4am5zUnhnQVFHSFNpTVUweHpQMkcxZzFCZnl4Wms1MVpiVkE?oc=5</t>
         </is>
       </c>
     </row>
@@ -3698,32 +3699,32 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>사회/사건사고</t>
+          <t>정치</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>🔥 [언론사 집중 보도 (3개사)]</t>
+          <t>연결 이슈 (후속)</t>
         </is>
       </c>
       <c r="D88" s="3" t="inlineStr">
         <is>
-          <t>울산 온산읍 제조업체서 불‥'대응 1단계'</t>
+          <t>국힘, 與 '신천지 의혹' 확인에 "특검·당원명부 압수수색 해야"</t>
         </is>
       </c>
       <c r="E88" s="3" t="inlineStr">
         <is>
-          <t>울산 온산읍 제조업체서 불‥'대응 1단계'  MBC 뉴스[속보] 울산 온산읍 제조업체 큰불...대응 1단계 발령  YTN울산 온산 화학공장서 폭발음 잇따라…공단 근로자 수천명 대피  부산일보울산 울주군 위험물 제조업체서 화재···소방 대응 1단계 발령  경향신문검은 연기 치솟는 울산 화...</t>
+          <t>(서울=연합뉴스) 박수윤 조다운 기자 = 국민의힘은 14일 더불어민주당이 신천지 교인의 집단 당원 가입 정황을 자체 조사로 공식 확인하자 당원 ...</t>
         </is>
       </c>
       <c r="F88" s="3" t="inlineStr">
         <is>
-          <t>MBC 뉴스</t>
+          <t>주요언론</t>
         </is>
       </c>
       <c r="G88" s="3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE9xZ25EN3hYNlBZZE8yUmZCSHByRkdsbnMyNHA1eGt5VzdrUzV2djlqamdlUUVUWUlFT2k3cjVkSXFTY1hfVThBSGFDaHlTZC1GMlNHa09mQzJGMUxmNjUwYVhkbTdaOGhxS1ZDLTc1QmMyNzlTZkJN0gF3QVVfeXFMT0NFQ2FBa0JYcGdWUjZxSVhFQXZId3haTnNtOFFocExTUUR3R3Q3SWxFV2xaODdSUXNGdkd1bGtIMlRDZlVUYWNkZmxSU01DbXp1ZjVlRE9kaU84MXdIMlFzZElYSjBsMm5ySWZLdFdPLTVhVTk5c3c?oc=5</t>
+          <t>https://www.yna.co.kr/view/AKR20261014089200001</t>
         </is>
       </c>
     </row>
@@ -3735,22 +3736,22 @@
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>사회/사건사고</t>
+          <t>정치</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>연결 이슈 (후속)</t>
+          <t>신규 이슈</t>
         </is>
       </c>
       <c r="D89" s="3" t="inlineStr">
         <is>
-          <t>무면허 중학생 공유 킥보드로 60대 여성 치여 하천 추락</t>
+          <t>교육위서 교부금 개편 도마…여야 '김민석·한동훈 자녀' 겨냥도</t>
         </is>
       </c>
       <c r="E89" s="3" t="inlineStr">
         <is>
-          <t>(양주=연합뉴스) 심민규 기자 = 경기 양주시에서 중학생이 몰던 공유 전동킥보드에 60대 여성이 치여 하천으로 추락하는 사고가 발생했다.</t>
+          <t>(서울=연합뉴스) 류미나 이율립 기자 = 국회 교육위원회가 14일 서울·인천·경기 등 수도권 교육청을 대상으로 실시한 국정감사에서는 정부의 지방...</t>
         </is>
       </c>
       <c r="F89" s="3" t="inlineStr">
@@ -3760,7 +3761,7 @@
       </c>
       <c r="G89" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261014083700060</t>
+          <t>https://www.yna.co.kr/view/AKR20261014088200001</t>
         </is>
       </c>
     </row>
@@ -3772,7 +3773,7 @@
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>사회/사건사고</t>
+          <t>정치</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
@@ -3782,12 +3783,12 @@
       </c>
       <c r="D90" s="3" t="inlineStr">
         <is>
-          <t>흉기 난동범 재범 위험 '높음'이었는데…예견된 참극</t>
+          <t>어린 딸 두고 입대한 6·25전쟁 두 호국영웅 유해 신원확인</t>
         </is>
       </c>
       <c r="E90" s="3" t="inlineStr">
         <is>
-          <t>(인천=연합뉴스) 최은지 기자 = 과거에도 재범 위험성 '높음' 판정을 받은 50대 살인미수 전과자가 도심 한복판에서 시민 8명을 찌르는 참극이...</t>
+          <t>(서울=연합뉴스) 김효정 기자 = 국방부 유해발굴감식단(이하 국유단)은 각기 어린 딸을 두고 입대했다 6·25전쟁에서 전사한 고(故) 진성대 이...</t>
         </is>
       </c>
       <c r="F90" s="3" t="inlineStr">
@@ -3797,7 +3798,7 @@
       </c>
       <c r="G90" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261014081200065</t>
+          <t>https://www.yna.co.kr/view/AKR20261014085600504</t>
         </is>
       </c>
     </row>
@@ -3809,7 +3810,7 @@
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>거시경제/비즈니스</t>
+          <t>정치</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
@@ -3819,22 +3820,22 @@
       </c>
       <c r="D91" s="3" t="inlineStr">
         <is>
-          <t>9월 ICT 수출 751억달러 '역대 최대'…반도체가 80% 견인</t>
+          <t>복지위 '리밸런싱' 충돌…"회의록 공개해야"·"시장영향 우려"</t>
         </is>
       </c>
       <c r="E91" s="3" t="inlineStr">
         <is>
-          <t>9월 ICT 수출 751억달러 '역대 최대'…반도체가 80% 견인  연합인포맥스지난달 ICT 수출 “사상 첫 700억 달러 돌파”  KBS 뉴스AI 열풍 탄 K-반도체 폭주…9월 ICT 수출 700억弗 첫 돌파  뉴시스2026년 9월 정보통신산업(ICT) 수출입 동향  서울PnKDI, ...</t>
+          <t>(서울=연합뉴스) 권희원 기자 = 여야는 14일 국회 보건복지위원회 국민연금공단 국정감사에서 국민연금의 리밸런싱(자산 비중 재조정) 유예 결정 ...</t>
         </is>
       </c>
       <c r="F91" s="3" t="inlineStr">
         <is>
-          <t>연합인포맥스</t>
+          <t>주요언론</t>
         </is>
       </c>
       <c r="G91" s="3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTFBMdnFvTFQycG1RNDZHcWU3WncxMEpyZHB4Z3lHMlhFc0U1TUs0djFoZ3pLQ2lpZERDTThqXzNjeFNCdnpiOWxOZHFVVjFLeGlrWGNKNWpRLVRRbFRsTnM3TUlBN01iMTRzNXNtdlI5ck8?oc=5</t>
+          <t>https://www.yna.co.kr/view/AKR20261014090800001</t>
         </is>
       </c>
     </row>
@@ -3846,7 +3847,7 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>거시경제/비즈니스</t>
+          <t>정치</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
@@ -3856,12 +3857,12 @@
       </c>
       <c r="D92" s="3" t="inlineStr">
         <is>
-          <t>완주 테크노밸리 미니복합타운 2천884세대, 내년부터 순차 분양</t>
+          <t>국정원 '美, 국정원장 방문거부' 보도 정정신청…이례적 법적대응</t>
         </is>
       </c>
       <c r="E92" s="3" t="inlineStr">
         <is>
-          <t>(완주=연합뉴스) 최영수 기자 = 전북 완주군은 봉동읍 테크노밸리 제2일반산업단지 옆 미니복합타운을 내년 1월 첫 분양한다고 14일 밝혔다.</t>
+          <t>(서울=연합뉴스) 하채림 기자 = 국가정보원이 미국 국방부 산하 기관이 이종석 국정원장의 방문을 거부했다는 언론보도에 대해 이례적으로 법적 대응...</t>
         </is>
       </c>
       <c r="F92" s="3" t="inlineStr">
@@ -3871,7 +3872,7 @@
       </c>
       <c r="G92" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261014082100055</t>
+          <t>https://www.yna.co.kr/view/AKR20261014084800504</t>
         </is>
       </c>
     </row>
@@ -3883,22 +3884,22 @@
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>거시경제/비즈니스</t>
+          <t>정치</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>🔥 [언론사 집중 보도 (3개사)]</t>
+          <t>신규 이슈</t>
         </is>
       </c>
       <c r="D93" s="3" t="inlineStr">
         <is>
-          <t>한솔제지 등 대전 3개 기업, 공장 증설에 734억 투자</t>
+          <t>김창국 aT 사장대행 "브라질산 계란 수입, 수입선 다변화 측면"</t>
         </is>
       </c>
       <c r="E93" s="3" t="inlineStr">
         <is>
-          <t>(대전=연합뉴스) 박주영 기자 = 대전시는 14일 대전 소재 기업 3곳과 734억원 규모의 투자 유치를 위한 업무협약을 했다.</t>
+          <t>(서울=연합뉴스) 한주홍 기자 = 김창국 한국농수산식품유통공사(aT) 사장 직무대행은 14일 브라질산 신선란 수입과 관련해 "수입선 다변화 측면...</t>
         </is>
       </c>
       <c r="F93" s="3" t="inlineStr">
@@ -3908,7 +3909,7 @@
       </c>
       <c r="G93" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261014083600063</t>
+          <t>https://www.yna.co.kr/view/AKR20261014091000030</t>
         </is>
       </c>
     </row>
@@ -3920,22 +3921,22 @@
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>거시경제/비즈니스</t>
+          <t>정치</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>🔥 [언론사 집중 보도 (3개사)]</t>
+          <t>신규 이슈</t>
         </is>
       </c>
       <c r="D94" s="3" t="inlineStr">
         <is>
-          <t>이란, 레이더 파괴되자 '인간 레이더' 동원…미국과 '유가 전쟁'</t>
+          <t>특검, '선거용품 입찰비리' 중앙선관위 등 5곳 압수수색</t>
         </is>
       </c>
       <c r="E94" s="3" t="inlineStr">
         <is>
-          <t>(서울=연합뉴스) 임화섭 기자 = 미국 중간선거를 앞두고 이란이 호르무즈 해협을 지나는 선박을 공격하는 데에 '새 전술'을 동원하고 있다고 로이...</t>
+          <t>(서울=연합뉴스) 최원정 기자 = 이태한 선거관리위원회 특별검사팀이 중앙선관위의 선거 용품 입찰 비리 의혹과 관련해 강제수사에 착수했다.</t>
         </is>
       </c>
       <c r="F94" s="3" t="inlineStr">
@@ -3945,7 +3946,7 @@
       </c>
       <c r="G94" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261014052400009</t>
+          <t>https://www.yna.co.kr/view/AKR20261014090600004</t>
         </is>
       </c>
     </row>
@@ -3957,32 +3958,32 @@
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>세계/국제</t>
+          <t>정치</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>신규 이슈</t>
+          <t>🔥 [언론사 집중 보도 (3개사)]</t>
         </is>
       </c>
       <c r="D95" s="3" t="inlineStr">
         <is>
-          <t>불륜녀에게 칼 찔린 남편…살려달라 연락한 사람은 ‘아내’, 日 발칵 [핫이슈]</t>
+          <t>김지용 "정치 편중되지 않게 일했다…부적격이라 생각지 않아"</t>
         </is>
       </c>
       <c r="E95" s="3" t="inlineStr">
         <is>
-          <t>불륜녀에게 칼 찔린 남편…살려달라 연락한 사람은 ‘아내’, 日 발칵 [핫이슈]  나우뉴스</t>
+          <t>(서울=연합뉴스) 황재하 기자 = 김지용 초대 중대범죄수사청장(중수청장) 후보자가 과거 검찰권 남용 사례들에 반대했었다고 재차 밝히면서 정치적 ...</t>
         </is>
       </c>
       <c r="F95" s="3" t="inlineStr">
         <is>
-          <t>나우뉴스</t>
+          <t>주요언론</t>
         </is>
       </c>
       <c r="G95" s="3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE5yYlFXd1pIRWNSakJjSmhDT1FGY0doR0NhYlNodFotVmZobWI4Uzh4dENKQnhqbFBoV1ZSNlFORTBxenpLbkh5MUpnN09VTjJPYmxRVWRQX3RRUjNhNnQ0aF9YU3htTUJLc0ZhWFRoMFE?oc=5</t>
+          <t>https://www.yna.co.kr/view/AKR20261014089000004</t>
         </is>
       </c>
     </row>
@@ -3994,32 +3995,32 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>세계/국제</t>
+          <t>정치</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>🔥 [언론사 집중 보도 (5개사)]</t>
+          <t>신규 이슈</t>
         </is>
       </c>
       <c r="D96" s="3" t="inlineStr">
         <is>
-          <t>트럼프, '장남 전 약혼녀' 길포일 주그리스 대사 전격 경질</t>
+          <t>문체위, 이임생·이동국 국감증인 의결…암살자(들) 채택은 불발</t>
         </is>
       </c>
       <c r="E96" s="3" t="inlineStr">
         <is>
-          <t>트럼프, '장남 전 약혼녀' 길포일 주그리스 대사 전격 경질  뉴스핌‘트럼프 장남 전 연인’ 주그리스 미국 대사 비위 의혹에 사임  경향신문"가족은 아니었다"…트럼프, '아들 전 약혼녀' 그리스 대사 해임  마켓인백악관, '각종 비위 의혹' 그리스 대사에 "사퇴 요구했다"  연합뉴스트럼...</t>
+          <t>(서울=연합뉴스) 박경준 기자 = 국회 문화체육관광위원회는 14일 전체회의를 열어 이용수 대한축구협회 회장 직무대행, 이임생 전 대한축구협회 기...</t>
         </is>
       </c>
       <c r="F96" s="3" t="inlineStr">
         <is>
-          <t>뉴스핌</t>
+          <t>주요언론</t>
         </is>
       </c>
       <c r="G96" s="3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiXEFVX3lxTE1FTFlBWGhjbXIyR01pc0Q4bGJGWWFyY01BTzdrS3hZdmlrQ3NzdHJheUV0Nmd2Y21fN3pabXR3YTlnUVZTZE90SWtmdGJYM0hKZGF3c2hlRk1rRlZP?oc=5</t>
+          <t>https://www.yna.co.kr/view/AKR20261014084500001</t>
         </is>
       </c>
     </row>
@@ -4031,32 +4032,32 @@
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>세계/국제</t>
+          <t>정치</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>🔥 [언론사 집중 보도 (5개사)]</t>
+          <t>🔥 [언론사 집중 보도 (3개사)]</t>
         </is>
       </c>
       <c r="D97" s="3" t="inlineStr">
         <is>
-          <t>트럼프·네타냐후, 선거 전 이란 재공격 저울질…정치적 부담에 딜레마</t>
+          <t>LIG D&amp;A, 미국 방산 스타트업과 유도로켓 추진체계 '맞손'</t>
         </is>
       </c>
       <c r="E97" s="3" t="inlineStr">
         <is>
-          <t>트럼프·네타냐후, 선거 전 이란 재공격 저울질…정치적 부담에 딜레마  뉴스핌악시오스 "트럼프, 지난주 네타냐후와 중간선거 전 이란 공격 논의"  MBC 뉴스트럼프 "선거 끝나도 나는 대통령…후티 공격 잊지 않을 것" [이상은의 워싱턴나우]  한국경제트럼프, "러시아·중국이 이란 돕고 있...</t>
+          <t>(서울=연합뉴스) 홍규빈 기자 = LIG 디펜스&amp;amp;에어로스페이스(LIG D&amp;amp;A)가 미국 방산 스타트업 '파이어호크'와 손잡고 미국 ...</t>
         </is>
       </c>
       <c r="F97" s="3" t="inlineStr">
         <is>
-          <t>뉴스핌</t>
+          <t>주요언론</t>
         </is>
       </c>
       <c r="G97" s="3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiXEFVX3lxTE5IeWdpMkUtOVZFQWRXQ0VERHJKVUNRSWE1M3JZSnB5Y1NfSWFVZHZwUGhiZ0ZqV05QNFdTZzlSNll1YTQyN0tLT0h2R3JEVEdXcVBfYnpJT1phRUFt?oc=5</t>
+          <t>https://www.yna.co.kr/view/AKR20261014087800003</t>
         </is>
       </c>
     </row>
@@ -4068,22 +4069,22 @@
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>세계/국제</t>
+          <t>정치</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>🔥 [언론사 집중 보도 (5개사)]</t>
+          <t>신규 이슈</t>
         </is>
       </c>
       <c r="D98" s="3" t="inlineStr">
         <is>
-          <t>트럼프 새 대변인 변호사 경력 논란…"중국서 자격 취득" 주장</t>
+          <t>육군 1군단, 19∼23일 파주·고양·양주서 호국훈련</t>
         </is>
       </c>
       <c r="E98" s="3" t="inlineStr">
         <is>
-          <t>(서울=연합뉴스) 이신영 기자 = 도널드 트럼프 미국 대통령이 새로 임명한 백악관 대변인 케이티 재커라이어가 경력 논란에 휩싸였다.</t>
+          <t>(고양=연합뉴스) 노승혁 기자 = 육군 1군단은 군사대비태세 유지와 합동 작전 수행 능력 향상을 위해 오는 19∼23일 파주·고양·양주 등 경기...</t>
         </is>
       </c>
       <c r="F98" s="3" t="inlineStr">
@@ -4093,7 +4094,7 @@
       </c>
       <c r="G98" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261014076000009</t>
+          <t>https://www.yna.co.kr/view/AKR20261014087900060</t>
         </is>
       </c>
     </row>
@@ -4105,7 +4106,7 @@
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>세계/국제</t>
+          <t>정치</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
@@ -4115,12 +4116,12 @@
       </c>
       <c r="D99" s="3" t="inlineStr">
         <is>
-          <t>텐센트, AI 투자용 7.7조원 채권 발행…주문 4배 몰려</t>
+          <t>친청계 "허위면 책임져야"…與 '신천지 확인'에 갈등 재점화 조짐</t>
         </is>
       </c>
       <c r="E99" s="3" t="inlineStr">
         <is>
-          <t>(서울=연합뉴스) 정주호 기자 = 중국 텐센트가 인공지능(AI) 투자 자금 마련을 위한 대규모 채권 발행에 4배가 넘는 투자 수요가 몰렸다.</t>
+          <t>(서울=연합뉴스) 김정진 안정훈 기자 = 더불어민주당이 공식적으로 신천지 교인의 집단 당원 가입 사실을 확인하면서 당내 계파 갈등이 재점화하고 ...</t>
         </is>
       </c>
       <c r="F99" s="3" t="inlineStr">
@@ -4130,7 +4131,7 @@
       </c>
       <c r="G99" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261014082900009</t>
+          <t>https://www.yna.co.kr/view/AKR20261014078300001</t>
         </is>
       </c>
     </row>
@@ -4142,32 +4143,32 @@
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>IT/과학/신상품</t>
+          <t>사회/사건사고</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>🔥 [언론사 집중 보도 (3개사)]</t>
+          <t>신규 이슈</t>
         </is>
       </c>
       <c r="D100" s="3" t="inlineStr">
         <is>
-          <t>조이시티, 12월 3일 신작 '프리스타일 풋볼 2' 글로벌 출시</t>
+          <t>'카이스트 러너' 유지원, 마라톤 레이스 중 사망 ...500m 남기고 '심정지' 비보</t>
         </is>
       </c>
       <c r="E100" s="3" t="inlineStr">
         <is>
-          <t>조이시티, 12월 3일 신작 '프리스타일 풋볼 2' 글로벌 출시  아이뉴스24조이시티, '프리스타일 풋볼 2' 12월 3일 출시…사전 판매 시작  매일경제 마켓26년 9월 월간게임동향  게임트릭스'프리스타일 풋볼 2', 12월 3일 글로벌 출시…사전 판매 시작  인벤조이시티 ‘프리스타일...</t>
+          <t>'카이스트 러너' 유지원, 마라톤 레이스 중 사망 ...500m 남기고 '심정지' 비보  스포츠조선황영조 ‘죽음에 이르는 러닝’ 경고···“욕심 부리지 말고, 필요하면 포기할 줄 알아야”  경향신문'서울 달리기' 마라톤대회 참가했던 20대 여성 사망  연합뉴스'서울달리기' 숨진 20대女...</t>
         </is>
       </c>
       <c r="F100" s="3" t="inlineStr">
         <is>
-          <t>아이뉴스24</t>
+          <t>스포츠조선</t>
         </is>
       </c>
       <c r="G100" s="3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiS0FVX3lxTFBLeDN5NXQ2U2xZdjRrYm1TSnJkRjdydDRPc19qbzZzU3E4ZnZMRW5DcWszNWNqRFA3aWp5YklNNG0zeVJyd2lEQ0N3NA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxQSTFXR09uYVhhTEJlb3BRQVg0RndvYkhVNThjcFB6VzNpdDhBa1o5dDFfbnFGXy1WYkFKTG1GOEtKUjBvS01Pc1VzTGtLbFBiYWR4U1dib01JdnZ1cnBfdlFxcGtObjdqSzZTRnE5Mml0WWZlMVJWLVJoVkl0Y3h1eXlJRDU?oc=5</t>
         </is>
       </c>
     </row>
@@ -4179,7 +4180,7 @@
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>IT/과학/신상품</t>
+          <t>사회/사건사고</t>
         </is>
       </c>
       <c r="C101" s="2" t="inlineStr">
@@ -4189,22 +4190,22 @@
       </c>
       <c r="D101" s="3" t="inlineStr">
         <is>
-          <t>RTX 5080 할인에 CPU 쿨러까지…조텍, 탁탁몰 특가 행사</t>
+          <t>생후 2개월 딸 때려 숨지게 한 친부 구속 갈림길‥"죄송하다"</t>
         </is>
       </c>
       <c r="E101" s="3" t="inlineStr">
         <is>
-          <t>RTX 5080 할인에 CPU 쿨러까지…조텍, 탁탁몰 특가 행사  뉴스탭Google 뉴스에서 헤드라인 및 의견 더보기</t>
+          <t>생후 2개월 딸 때려 숨지게 한 친부 구속 갈림길‥"죄송하다"  MBC 뉴스“잠투정한다고” 생후 2개월 딸 숨지게 한 40대 친부 구속 갈림길  경기일보2개월 영아 멍든 채 숨져..."안 자고 울어 때렸다" [뉴스퀘어 2PM]  YTN오산 2개월 여아 살해 사건 수사 중인 경찰, 고의 ...</t>
         </is>
       </c>
       <c r="F101" s="3" t="inlineStr">
         <is>
-          <t>뉴스탭</t>
+          <t>MBC 뉴스</t>
         </is>
       </c>
       <c r="G101" s="3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMibEFVX3lxTE92UmZLWFY0bG9iOEZPUjVtYTZjcnBNMkRteFZUY2ZkZ2xYaVlKS3lvRG5UMENyNGVMSkxaYUxIREo2ZjdSSjZlY2FFeEZuU1M4NF9EY0w5dU9wZWhBN1VucjB0ZGg5bmUtNmI4SA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTFBnRzZabG1wTjhuTjNENmh4OGllVHB3bzJDMmdjWEhualNhYUFJNG9vN2ZyTGx5UjVHTWZBZ0E0bklWZnNBakhmVmVzbVJpaENwSl9sR25IRXpoSXQwLXp2a2RESmxEQ1RJUTRPeWtIaElvY1hadGNF0gF3QVVfeXFMUE5PNHVOWnU4N3NzNEdpR3pLMnlDWTk1NGRQWmdZeFEtU0JvMFdERTZwYnZXQ1Z5dEhQWVdaeTVrcXlXVFo4N2JfaG5sdEdNTGo4NWg5X1pwcUttN3p4OHhFZ1ptNnhHVEk0anJ5WW5JbEhTY0VJcUE?oc=5</t>
         </is>
       </c>
     </row>
@@ -4216,7 +4217,7 @@
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>IT/과학/신상품</t>
+          <t>사회/사건사고</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
@@ -4226,12 +4227,12 @@
       </c>
       <c r="D102" s="3" t="inlineStr">
         <is>
-          <t>콘솔게임 보안까지 뚫은 AI, 해적판 등장에 업계 '발칵'</t>
+          <t>"학대 정황 없어 안전" 판단했지만…비극 못 막은 경찰</t>
         </is>
       </c>
       <c r="E102" s="3" t="inlineStr">
         <is>
-          <t>(서울=연합뉴스) 김주환 기자 = 인기 콘솔 게임과 플랫폼의 철통 같은 데이터 보안이 에이전틱 인공지능(AI) 고도화에 잇달아 뚫리며 해적판이 ...</t>
+          <t>(제주=연합뉴스) 백나용 기자 = 제주에서 부녀가 차 안에서 숨진 채 발견된 사건과 관련해 경찰이 아동학대 의심과 실종 신고에 따른 조사·면담과...</t>
         </is>
       </c>
       <c r="F102" s="3" t="inlineStr">
@@ -4241,7 +4242,7 @@
       </c>
       <c r="G102" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261014079700017</t>
+          <t>https://www.yna.co.kr/view/AKR20261014088500056</t>
         </is>
       </c>
     </row>
@@ -4253,7 +4254,7 @@
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>IT/과학/신상품</t>
+          <t>사회/사건사고</t>
         </is>
       </c>
       <c r="C103" s="2" t="inlineStr">
@@ -4263,12 +4264,12 @@
       </c>
       <c r="D103" s="3" t="inlineStr">
         <is>
-          <t>'월가 족집게' 댄 아이브스 "테슬라·스페이스X 내년 합병 가능성 80%"</t>
+          <t>이진호 원자력환경공단 이사장 취임…"국민 신뢰받는 기관으로"</t>
         </is>
       </c>
       <c r="E103" s="3" t="inlineStr">
         <is>
-          <t>(서울=연합뉴스) 정회인 기자 = 월가의 대표적인 기술주 분석가인 댄 아이브스 '요크빌 아이브스' 파트너 겸 선임 전무는 엔비디아와 마이크로소프...</t>
+          <t>(경주=연합뉴스) 손대성 기자 = 이진호(61) 한국원자력환경공단 신임 이사장이 14일 경북 경주의 본사에서 취임식을 하고 업무에 들어갔다.</t>
         </is>
       </c>
       <c r="F103" s="3" t="inlineStr">
@@ -4278,7 +4279,7 @@
       </c>
       <c r="G103" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261014080500008</t>
+          <t>https://www.yna.co.kr/view/AKR20261014094000053</t>
         </is>
       </c>
     </row>
@@ -4290,32 +4291,32 @@
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>연예/대중문화</t>
+          <t>사회/사건사고</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>신규 이슈</t>
+          <t>🔥 [언론사 집중 보도 (3개사)]</t>
         </is>
       </c>
       <c r="D104" s="3" t="inlineStr">
         <is>
-          <t>‘이병헌♥’ 이민정, 12살 초등학생 아들 사교육 언급..“농구·수학만 시켜”</t>
+          <t>김지용 중수청장 후보 "정치검사 1호는 윤석열…한동훈도 포함"</t>
         </is>
       </c>
       <c r="E104" s="3" t="inlineStr">
         <is>
-          <t>‘이병헌♥’ 이민정, 12살 초등학생 아들 사교육 언급..“농구·수학만 시켜”  조선일보이민정, 아들 사교육 질문에 "농구·수학 학원만 다녀"  뉴시스‘이병헌♥’ 이민정, 12살 초등학생 아들 사교육 언급..“농구·수학만 시켜” - 조선비즈  Chosunbiz'MJ' 이민정 "어렸을 때...</t>
+          <t>(서울=연합뉴스) 이승연 기자 = 김지용 중대범죄수사청장(중수청장) 후보자가 검찰의 개혁 필요성에 동의한다는 입장을 재차 밝히며 그 배경에 윤석...</t>
         </is>
       </c>
       <c r="F104" s="3" t="inlineStr">
         <is>
-          <t>조선일보</t>
+          <t>주요언론</t>
         </is>
       </c>
       <c r="G104" s="3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxQZXdFa0RBNkNZYlBOZ1ZOUzlQWWJWbXlYbjJVUFdLeFBrSFhqcHVvMm5wWVRBMklsTm44MUJJRmMycjRCdzByYTdfTW8xLTFyaDVyN1RIdnZzSVRNOHdIeld1NW15Q2VibGZTUFE2eTlTXzR6MTdtakJ2MDZWRkk1UndvNy0xZUt0a2lRQ0dXbw?oc=5</t>
+          <t>https://www.yna.co.kr/view/AKR20261014093300004</t>
         </is>
       </c>
     </row>
@@ -4327,32 +4328,32 @@
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>연예/대중문화</t>
+          <t>사회/사건사고</t>
         </is>
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>연결 이슈 (후속)</t>
+          <t>신규 이슈</t>
         </is>
       </c>
       <c r="D105" s="3" t="inlineStr">
         <is>
-          <t>최수종, 모친상 후 끝내 눈물 “왜 쓴소리 했을까” (유퀴즈)</t>
+          <t>'채용대가 뇌물수수' 강서구의회 前의장·운영위원장 징역 5년</t>
         </is>
       </c>
       <c r="E105" s="3" t="inlineStr">
         <is>
-          <t>최수종, 모친상 후 끝내 눈물 “왜 쓴소리 했을까” (유퀴즈)  매일경제최수종, 모친상 발인 다음 날 녹화…"엄마에게 쓴소리했던 게 후회"  뉴시스최수종, 모친상 심경.."쓴소리 더 기억나서 마음 아파" 눈물('유퀴즈')[핫피플] - 조선비즈  Chosunbiz“쓴소리했던 기억에 눈물”...</t>
+          <t>(서울=연합뉴스) 김채린 기자 = 공무원 채용 및 계약 연장 대가로 금품을 수수한 혐의로 재판에 넘겨진 구의회 전직 의장과 운영위원장이 1심에서...</t>
         </is>
       </c>
       <c r="F105" s="3" t="inlineStr">
         <is>
-          <t>매일경제</t>
+          <t>주요언론</t>
         </is>
       </c>
       <c r="G105" s="3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiZkFVX3lxTE55YkFOMHFYNXc3S1c4MWY4T1ZHRGQxdmwzMjZFWS15d3dtaTZkdW1QbzgxUWlmaWpOcHFJVXN0RFlIcV9rU0dkX3ZpdGI5MG41ME9yeXdKVjF2Yi16cVBYZk1ic21vQQ?oc=5</t>
+          <t>https://www.yna.co.kr/view/AKR20261014087100004</t>
         </is>
       </c>
     </row>
@@ -4364,32 +4365,32 @@
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>연예/대중문화</t>
+          <t>사회/사건사고</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>🔥 [언론사 집중 보도 (5개사)]</t>
+          <t>신규 이슈</t>
         </is>
       </c>
       <c r="D106" s="3" t="inlineStr">
         <is>
-          <t>김영광·채수빈 ‘나를 충전해줘’, 공개 3일 만에 넷플릭스 글로벌 비영어권 3위</t>
+          <t>평택 아파트 지하실 화재…2살 여아 등 11명 중경상(종합)</t>
         </is>
       </c>
       <c r="E106" s="3" t="inlineStr">
         <is>
-          <t>김영광·채수빈 ‘나를 충전해줘’, 공개 3일 만에 넷플릭스 글로벌 비영어권 3위  스포츠동아차우민, '최애의 사원' 이어 '나를 충전해줘'까지…로맨스 연타 흥행 예고  YTN‘국민엄마’ 김미경, 백발됐다…이번엔 재벌가 회장 변신(‘나를 충전해줘’) - 조선비즈  Chosunbiz‘나를 ...</t>
+          <t>(평택=연합뉴스) 김지원 기자 = 경기 평택시의 한 아파트 지하에서 불이 나 2살 여아를 포함한 11명이 중경상을 입었다.</t>
         </is>
       </c>
       <c r="F106" s="3" t="inlineStr">
         <is>
-          <t>스포츠동아</t>
+          <t>주요언론</t>
         </is>
       </c>
       <c r="G106" s="3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMibkFVX3lxTE9Ra1M4ZWNJS21PN3QtYnBCU3V4bnZoRm44Z2ZITHR1Z1lkUXZqZ2RVWTN1ZU0xWWRkZkJRVlVvOXQzanpDekVYcnBvWDJ0ekRlWElHZVFmVDVOT0IwWnpBbDlPNzk0WmtGdm1TTGZ3?oc=5</t>
+          <t>https://www.yna.co.kr/view/AKR20261014089151061</t>
         </is>
       </c>
     </row>
@@ -4401,32 +4402,1771 @@
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
+          <t>사회/사건사고</t>
+        </is>
+      </c>
+      <c r="C107" s="2" t="inlineStr">
+        <is>
+          <t>신규 이슈</t>
+        </is>
+      </c>
+      <c r="D107" s="3" t="inlineStr">
+        <is>
+          <t>[게시판] 강남소방서, 서울시의원 '소방관의 하루' 체험 행사</t>
+        </is>
+      </c>
+      <c r="E107" s="3" t="inlineStr">
+        <is>
+          <t>▲ 강남소방서는 강신욱 서울시의원과 지난 9일 '소방관의 하루' 행사를 했다고 14일 밝혔다. 강 시의원이 화재 출동·주택 감지기 설치·산불 훈...</t>
+        </is>
+      </c>
+      <c r="F107" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G107" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014093200004</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>사회/사건사고</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t>신규 이슈</t>
+        </is>
+      </c>
+      <c r="D108" s="3" t="inlineStr">
+        <is>
+          <t>성동구, 가을 중랑천서 '걷고 듣는' 정원 프로그램 운영</t>
+        </is>
+      </c>
+      <c r="E108" s="3" t="inlineStr">
+        <is>
+          <t>(서울=연합뉴스) 정준영 기자 = 서울 성동구(구청장 유보화)는 가을을 맞아 '중랑천 정원투어'와 '중랑천 사운드캠프' 프로그램을 운영한다고 1...</t>
+        </is>
+      </c>
+      <c r="F108" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G108" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014092700004</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="inlineStr">
+        <is>
+          <t>사회/사건사고</t>
+        </is>
+      </c>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t>신규 이슈</t>
+        </is>
+      </c>
+      <c r="D109" s="3" t="inlineStr">
+        <is>
+          <t>[담양소식] 어린이 놀이공간 조성 국비 확보</t>
+        </is>
+      </c>
+      <c r="E109" s="3" t="inlineStr">
+        <is>
+          <t>(담양=연합뉴스) 전남광주통합특별시 담양군은 행정안전부의 '2026년 지역맞춤형 저출산 대응 공모사업'에 선정돼 특별교부세 5억원을 확보했다고 ...</t>
+        </is>
+      </c>
+      <c r="F109" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G109" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014093100054</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>사회/사건사고</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>신규 이슈</t>
+        </is>
+      </c>
+      <c r="D110" s="3" t="inlineStr">
+        <is>
+          <t>'마약 투약 후 시내버스 운전' 40대 기사에 징역 2년 6개월</t>
+        </is>
+      </c>
+      <c r="E110" s="3" t="inlineStr">
+        <is>
+          <t>(안산=연합뉴스) 최해민 기자 = 필로폰을 투약한 채 수많은 시민이 타는 시내버스를 운전한 중국 국적의 40대 버스 기사에게 실형이 선고됐다.</t>
+        </is>
+      </c>
+      <c r="F110" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G110" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014075300061</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B111" s="2" t="inlineStr">
+        <is>
+          <t>사회/사건사고</t>
+        </is>
+      </c>
+      <c r="C111" s="2" t="inlineStr">
+        <is>
+          <t>신규 이슈</t>
+        </is>
+      </c>
+      <c r="D111" s="3" t="inlineStr">
+        <is>
+          <t>전북도, 농기계 임대사업 예산 작년보다 16% 증가</t>
+        </is>
+      </c>
+      <c r="E111" s="3" t="inlineStr">
+        <is>
+          <t>(전주=연합뉴스) 임채두 기자 = 전북특별자치도는 올해 농기계 임대사업에 지난해보다 11억원(16%) 늘어난 78억원을 투입, 농기계 임대 기반...</t>
+        </is>
+      </c>
+      <c r="F111" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G111" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014090400055</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>사회/사건사고</t>
+        </is>
+      </c>
+      <c r="C112" s="2" t="inlineStr">
+        <is>
+          <t>신규 이슈</t>
+        </is>
+      </c>
+      <c r="D112" s="3" t="inlineStr">
+        <is>
+          <t>곡성군, 하와이 교류 연계 고향사랑기부 사업 발굴</t>
+        </is>
+      </c>
+      <c r="E112" s="3" t="inlineStr">
+        <is>
+          <t>(전남광주=연합뉴스) 박철홍 기자 = 전남광주통합특별시 곡성군은 미국 하와이 카운티와의 자매결연을 활용해 청소년 교육 분야 고향사랑기부 사업과 ...</t>
+        </is>
+      </c>
+      <c r="F112" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G112" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014089600054</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B113" s="2" t="inlineStr">
+        <is>
+          <t>사회/사건사고</t>
+        </is>
+      </c>
+      <c r="C113" s="2" t="inlineStr">
+        <is>
+          <t>신규 이슈</t>
+        </is>
+      </c>
+      <c r="D113" s="3" t="inlineStr">
+        <is>
+          <t>우상호 "원주 옛 종축장 부지, 시민 휴식 공간으로 우선 개방"</t>
+        </is>
+      </c>
+      <c r="E113" s="3" t="inlineStr">
+        <is>
+          <t>(춘천=연합뉴스) 이재현 기자 = 30년 가까이 개발계획만 반복된 강원 원주시 반곡동 옛 종축장 부지를 우선 시민 휴식 공간으로 개방하고, 향후...</t>
+        </is>
+      </c>
+      <c r="F113" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G113" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014088700062</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B114" s="2" t="inlineStr">
+        <is>
+          <t>거시경제/비즈니스</t>
+        </is>
+      </c>
+      <c r="C114" s="2" t="inlineStr">
+        <is>
+          <t>🔥 [언론사 집중 보도 (3개사)]</t>
+        </is>
+      </c>
+      <c r="D114" s="3" t="inlineStr">
+        <is>
+          <t>"고객 마음을 훔쳐라"…온·오프 넘나드는 증권가 MTS '전면전'</t>
+        </is>
+      </c>
+      <c r="E114" s="3" t="inlineStr">
+        <is>
+          <t>"고객 마음을 훔쳐라"…온·오프 넘나드는 증권가 MTS '전면전'  연합인포맥스iM증권, MTS 새 단장…내 투자정보 한눈에 본다  뉴시스[게시판] 키움증권, MTS에 신규 국내주식 주문 화면 도입  연합뉴스키움증권, 국내주식 신규 주문 화면 오픈…차트·잔고·ETF 한눈에  전자신문iM...</t>
+        </is>
+      </c>
+      <c r="F114" s="3" t="inlineStr">
+        <is>
+          <t>연합인포맥스</t>
+        </is>
+      </c>
+      <c r="G114" s="3" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE9oWi1hTHRMcW85NnlGU1pWSmZ2a1RiMS00VzhXTGxkbGVudTljV3Ywbzl0V3VxYV9adExGYVF1d0lZUVpXNEliYjVoVVA5b1p4ZnVaWDRNVkIxVlR0U2RLT0FNTnN2VWlTam1vc1VBemw?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B115" s="2" t="inlineStr">
+        <is>
+          <t>거시경제/비즈니스</t>
+        </is>
+      </c>
+      <c r="C115" s="2" t="inlineStr">
+        <is>
+          <t>신규 이슈</t>
+        </is>
+      </c>
+      <c r="D115" s="3" t="inlineStr">
+        <is>
+          <t>삼전닉스 폭락에도 "지금이 저점"…'W자 반등' 전망한 이유 [분석+]</t>
+        </is>
+      </c>
+      <c r="E115" s="3" t="inlineStr">
+        <is>
+          <t>삼전닉스 폭락에도 "지금이 저점"…'W자 반등' 전망한 이유 [분석+]  한국경제“이젠 반도체 미련 버려야?”...내년 증시 주도주 바뀌나  매일경제삼성證 "메모리 가격 상승 둔화해도 이익 성장 가능…'삼전닉스' 매수 유지"  연합인포맥스반도체주 반등 언제쯤…“소부장이 투자 대안”  마...</t>
+        </is>
+      </c>
+      <c r="F115" s="3" t="inlineStr">
+        <is>
+          <t>한국경제</t>
+        </is>
+      </c>
+      <c r="G115" s="3" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTE9vTllzX2VGdExfcjB2aUM4dG8zNVY3TmFLZVQxV3JxSzNqZ3lGX0sxMnRIUjRUNzZBaW9mdEtxM2RQNDVYYTI0eVB6dTNaQURQVEZwZE1LaTJYQQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B116" s="2" t="inlineStr">
+        <is>
+          <t>거시경제/비즈니스</t>
+        </is>
+      </c>
+      <c r="C116" s="2" t="inlineStr">
+        <is>
+          <t>신규 이슈</t>
+        </is>
+      </c>
+      <c r="D116" s="3" t="inlineStr">
+        <is>
+          <t>부활한 '재계 저승사자' 1호 사건…대상·오뚜기·CJ제일제당(종합)</t>
+        </is>
+      </c>
+      <c r="E116" s="3" t="inlineStr">
+        <is>
+          <t>(세종=연합뉴스) 송정은 기자 = 새로 출범한 공정거래위원회 중점조사기획단이 1호 사건으로 식품업체 담합 사건을 조사하고 있다.</t>
+        </is>
+      </c>
+      <c r="F116" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G116" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014091451002</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B117" s="2" t="inlineStr">
+        <is>
+          <t>거시경제/비즈니스</t>
+        </is>
+      </c>
+      <c r="C117" s="2" t="inlineStr">
+        <is>
+          <t>신규 이슈</t>
+        </is>
+      </c>
+      <c r="D117" s="3" t="inlineStr">
+        <is>
+          <t>디지털엑스, 내달 미래에셋증권 본사 센터원으로 이전</t>
+        </is>
+      </c>
+      <c r="E117" s="3" t="inlineStr">
+        <is>
+          <t>(서울=연합뉴스) 유동현 기자 = 미래에셋그룹 가상자산 거래소 디지털엑스가 다음 달 미래에셋증권[006800] 본사로 사무실을 이전한다고 14일...</t>
+        </is>
+      </c>
+      <c r="F117" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G117" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014092600002</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B118" s="2" t="inlineStr">
+        <is>
+          <t>거시경제/비즈니스</t>
+        </is>
+      </c>
+      <c r="C118" s="2" t="inlineStr">
+        <is>
+          <t>신규 이슈</t>
+        </is>
+      </c>
+      <c r="D118" s="3" t="inlineStr">
+        <is>
+          <t>박홍근 "정책기획 역량이 조직 성패 좌우…체질 개선해야"</t>
+        </is>
+      </c>
+      <c r="E118" s="3" t="inlineStr">
+        <is>
+          <t>(세종=연합뉴스) 이대희 기자 = 박홍근 기획예산처 장관은 14일 "정책기획 역량이 조직의 성패를 좌우한다"며 강도 높은 조직체질 개선을 간부들...</t>
+        </is>
+      </c>
+      <c r="F118" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G118" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014092100002</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B119" s="2" t="inlineStr">
+        <is>
+          <t>거시경제/비즈니스</t>
+        </is>
+      </c>
+      <c r="C119" s="2" t="inlineStr">
+        <is>
+          <t>신규 이슈</t>
+        </is>
+      </c>
+      <c r="D119" s="3" t="inlineStr">
+        <is>
+          <t>[1보] 공정위 중점조사기획단 1호 대상·오뚜기·CJ제일제당 현장조사</t>
+        </is>
+      </c>
+      <c r="E119" s="3" t="inlineStr">
+        <is>
+          <t>(</t>
+        </is>
+      </c>
+      <c r="F119" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G119" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014091400002</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B120" s="2" t="inlineStr">
+        <is>
+          <t>거시경제/비즈니스</t>
+        </is>
+      </c>
+      <c r="C120" s="2" t="inlineStr">
+        <is>
+          <t>연결 이슈 (후속)</t>
+        </is>
+      </c>
+      <c r="D120" s="3" t="inlineStr">
+        <is>
+          <t>국고채 금리 일제히 상승…3년물 장중 연 3.883%</t>
+        </is>
+      </c>
+      <c r="E120" s="3" t="inlineStr">
+        <is>
+          <t>(서울=연합뉴스) 14일 국고채 금리가 일제히 상승하고 있다.</t>
+        </is>
+      </c>
+      <c r="F120" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G120" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014091100008</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B121" s="2" t="inlineStr">
+        <is>
+          <t>거시경제/비즈니스</t>
+        </is>
+      </c>
+      <c r="C121" s="2" t="inlineStr">
+        <is>
+          <t>🔥 [언론사 집중 보도 (3개사)]</t>
+        </is>
+      </c>
+      <c r="D121" s="3" t="inlineStr">
+        <is>
+          <t>삼성전자, 기후부 장관에 고효율·저탄소 주거 솔루션 제시</t>
+        </is>
+      </c>
+      <c r="E121" s="3" t="inlineStr">
+        <is>
+          <t>(서울=연합뉴스) 조성흠 기자 = 삼성전자는 14일 김성환 기후에너지환경부 장관에게 히트펌프 방식의 냉난방 솔루션과 인공지능(AI) 기반 에너지...</t>
+        </is>
+      </c>
+      <c r="F121" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G121" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014085100003</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>거시경제/비즈니스</t>
+        </is>
+      </c>
+      <c r="C122" s="2" t="inlineStr">
+        <is>
+          <t>신규 이슈</t>
+        </is>
+      </c>
+      <c r="D122" s="3" t="inlineStr">
+        <is>
+          <t>포천시-차의과학대학, 지역사회 건강증진 업무협약</t>
+        </is>
+      </c>
+      <c r="E122" s="3" t="inlineStr">
+        <is>
+          <t>(포천=연합뉴스) 노승혁 기자 = 경기 포천시보건소는 차의과학대학교 스포츠의학연구원과 '지역사회 건강증진 및 포CHA건강프로젝트 운영을 위한 업...</t>
+        </is>
+      </c>
+      <c r="F122" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G122" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014086500060</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B123" s="2" t="inlineStr">
+        <is>
+          <t>거시경제/비즈니스</t>
+        </is>
+      </c>
+      <c r="C123" s="2" t="inlineStr">
+        <is>
+          <t>신규 이슈</t>
+        </is>
+      </c>
+      <c r="D123" s="3" t="inlineStr">
+        <is>
+          <t>카카오뱅크 "18일 새벽 금융거래 일시 중단…전산시스템 점검"</t>
+        </is>
+      </c>
+      <c r="E123" s="3" t="inlineStr">
+        <is>
+          <t>(서울=연합뉴스) 이도흔 기자 = 카카오뱅크[323410]는 오는 18일 새벽 전산시스템 정기 점검으로 금융거래를 일시 중단한다고 14일 밝혔다...</t>
+        </is>
+      </c>
+      <c r="F123" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G123" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014086400002</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B124" s="2" t="inlineStr">
+        <is>
+          <t>거시경제/비즈니스</t>
+        </is>
+      </c>
+      <c r="C124" s="2" t="inlineStr">
+        <is>
+          <t>신규 이슈</t>
+        </is>
+      </c>
+      <c r="D124" s="3" t="inlineStr">
+        <is>
+          <t>하나은행, 6억달러 규모 달러화 선순위채 발행</t>
+        </is>
+      </c>
+      <c r="E124" s="3" t="inlineStr">
+        <is>
+          <t>(서울=연합뉴스) 채새롬 기자 = 하나은행은 총 6억 달러 규모의 미 달러화 선순위 채권을 발행했다고 14일 밝혔다.</t>
+        </is>
+      </c>
+      <c r="F124" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G124" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014084900002</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B125" s="2" t="inlineStr">
+        <is>
+          <t>거시경제/비즈니스</t>
+        </is>
+      </c>
+      <c r="C125" s="2" t="inlineStr">
+        <is>
+          <t>신규 이슈</t>
+        </is>
+      </c>
+      <c r="D125" s="3" t="inlineStr">
+        <is>
+          <t>반도체산단 입지 용인 처인지역 '사통팔달' 도로망 구축 잰걸음</t>
+        </is>
+      </c>
+      <c r="E125" s="3" t="inlineStr">
+        <is>
+          <t>(용인=연합뉴스) 김광호 기자 = 원삼면과 남사·이동읍 일대에 초대형 반도체 산업단지가 조성 중인 경기 용인시 처인구의 주요 도로망 구축 사업이...</t>
+        </is>
+      </c>
+      <c r="F125" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G125" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014075200061</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B126" s="2" t="inlineStr">
+        <is>
+          <t>거시경제/비즈니스</t>
+        </is>
+      </c>
+      <c r="C126" s="2" t="inlineStr">
+        <is>
+          <t>🔥 [언론사 집중 보도 (3개사)]</t>
+        </is>
+      </c>
+      <c r="D126" s="3" t="inlineStr">
+        <is>
+          <t>[단독] 금융권 비상인데…새마을금고, 해킹 당하고도 60시간 몰랐다</t>
+        </is>
+      </c>
+      <c r="E126" s="3" t="inlineStr">
+        <is>
+          <t>400여명 이름 등 개인정보 유출 외부서 공격 IP 공유받아 인지 금융권 해킹 경계령 내렸지만 계속되는 감독 사각지대 논란새마을금고가 해킹 공격을 당하고도 약 60시간 가까이 이를..</t>
+        </is>
+      </c>
+      <c r="F126" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G126" s="3" t="inlineStr">
+        <is>
+          <t>https://www.mk.co.kr/news/economy/12175452</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B127" s="2" t="inlineStr">
+        <is>
+          <t>세계/국제</t>
+        </is>
+      </c>
+      <c r="C127" s="2" t="inlineStr">
+        <is>
+          <t>신규 이슈</t>
+        </is>
+      </c>
+      <c r="D127" s="3" t="inlineStr">
+        <is>
+          <t>임신 위한 ‘적절한 성관계 횟수’는?…“‘이 시기’ 놓치지 않아야” [라이프+]</t>
+        </is>
+      </c>
+      <c r="E127" s="3" t="inlineStr">
+        <is>
+          <t>임신 위한 ‘적절한 성관계 횟수’는?…“‘이 시기’ 놓치지 않아야” [라이프+]  나우뉴스</t>
+        </is>
+      </c>
+      <c r="F127" s="3" t="inlineStr">
+        <is>
+          <t>나우뉴스</t>
+        </is>
+      </c>
+      <c r="G127" s="3" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE5iTEVvT21uTXFZT251dWVLUFg5Q0VGWnlKaEhhWmpjMUNhTi1ObzdyQ05DcjJNLUpHTXNCbHc5ekxrRFRma2p0S2FSRFBYUUtjS191MVdvNEZ1RG00ZVBxTV9jTmljbW1HQzUtRmdrRWM?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B128" s="2" t="inlineStr">
+        <is>
+          <t>세계/국제</t>
+        </is>
+      </c>
+      <c r="C128" s="2" t="inlineStr">
+        <is>
+          <t>🔥 [언론사 집중 보도 (5개사)]</t>
+        </is>
+      </c>
+      <c r="D128" s="3" t="inlineStr">
+        <is>
+          <t>인니 11년 만에 최악의 산불…연무로 항공 진화 1주일째 난항</t>
+        </is>
+      </c>
+      <c r="E128" s="3" t="inlineStr">
+        <is>
+          <t>인니 11년 만에 최악의 산불…연무로 항공 진화 1주일째 난항  연합뉴스인니 보르네오섬, 오랜 산불에 서식지 잃은 오랑우탄 46마리 구조  뉴시스인니 대규모 산불 연무에 말레이 조호르州 학교 1198곳 최소 16일까지 휴교  아시아투데이[포토] 인니 깨끗한 공기는 언제쯤  뉴스1집단 대...</t>
+        </is>
+      </c>
+      <c r="F128" s="3" t="inlineStr">
+        <is>
+          <t>연합뉴스</t>
+        </is>
+      </c>
+      <c r="G128" s="3" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE9acHV4TGVfM016VEJxMVlXeVNOVWNkMFM3aXBEamE4emhrOGlyeTB3NnRlSG13RUt4dlAza1FVT3NNYi1SMHh1cTh4UmtWY3ZmRGZ2LVY3MVlGdTDSAWBBVV95cUxQNHpFNHBZSUwtU2pZQjh4YXFGR1pDRnpMU3REcUdVOUp4dnlXU09oZ2I0bmRocTRLNk5ReHlMYWRmcWtRLU1DekxTRTVqdWc1X3FTdmJxMGR2U2tfUUNWZnE?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B129" s="2" t="inlineStr">
+        <is>
+          <t>세계/국제</t>
+        </is>
+      </c>
+      <c r="C129" s="2" t="inlineStr">
+        <is>
+          <t>신규 이슈</t>
+        </is>
+      </c>
+      <c r="D129" s="3" t="inlineStr">
+        <is>
+          <t>MLB 휴스턴 감독, 계약 기간 중 시애틀 구단 감독 면접</t>
+        </is>
+      </c>
+      <c r="E129" s="3" t="inlineStr">
+        <is>
+          <t>(서울=연합뉴스) 장현구 기자 = 미국프로야구 메이저리그(MLB) 휴스턴 애스트로스의 조 에스파다 감독이 계약 기간 중 구단의 승낙을 받아 같은...</t>
+        </is>
+      </c>
+      <c r="F129" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G129" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014094100007</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B130" s="2" t="inlineStr">
+        <is>
+          <t>세계/국제</t>
+        </is>
+      </c>
+      <c r="C130" s="2" t="inlineStr">
+        <is>
+          <t>🔥 [언론사 집중 보도 (3개사)]</t>
+        </is>
+      </c>
+      <c r="D130" s="3" t="inlineStr">
+        <is>
+          <t>중국 9월 수출 36.3% 급증…수입은 31.0% 늘어</t>
+        </is>
+      </c>
+      <c r="E130" s="3" t="inlineStr">
+        <is>
+          <t>(상하이=연합뉴스) 차병섭 특파원 = 세계적인 인공지능(AI) 투자 붐 속에 지난달 중국의 수출이 30% 넘게 급증한 것으로 집계됐다.</t>
+        </is>
+      </c>
+      <c r="F130" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G130" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014092900089</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B131" s="2" t="inlineStr">
+        <is>
+          <t>세계/국제</t>
+        </is>
+      </c>
+      <c r="C131" s="2" t="inlineStr">
+        <is>
+          <t>신규 이슈</t>
+        </is>
+      </c>
+      <c r="D131" s="3" t="inlineStr">
+        <is>
+          <t>미 대학서 '동료 음료에 독' 中유학생 도피하다 공항서 체포</t>
+        </is>
+      </c>
+      <c r="E131" s="3" t="inlineStr">
+        <is>
+          <t>(서울=연합뉴스) 김승욱 기자 = 미국 대학교에서 동료 대학원생의 음료에 독극물을 타 중상을 입힌 뒤 중국으로 도피하려던 중국인 유학생이 경찰에...</t>
+        </is>
+      </c>
+      <c r="F131" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G131" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014091800009</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B132" s="2" t="inlineStr">
+        <is>
+          <t>세계/국제</t>
+        </is>
+      </c>
+      <c r="C132" s="2" t="inlineStr">
+        <is>
+          <t>신규 이슈</t>
+        </is>
+      </c>
+      <c r="D132" s="3" t="inlineStr">
+        <is>
+          <t>오라클, 데이터센터용 가스관 승인 신속처리 촉구</t>
+        </is>
+      </c>
+      <c r="E132" s="3" t="inlineStr">
+        <is>
+          <t>(서울=연합뉴스) 설원태 기자 = 오라클은 미국 뉴멕시코주에서 추진중인 대규모데이터센터 구축 프로젝트에 필요한 천연가스관 건설을 신속하게 승인해...</t>
+        </is>
+      </c>
+      <c r="F132" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G132" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014083000009</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B133" s="2" t="inlineStr">
+        <is>
+          <t>세계/국제</t>
+        </is>
+      </c>
+      <c r="C133" s="2" t="inlineStr">
+        <is>
+          <t>신규 이슈</t>
+        </is>
+      </c>
+      <c r="D133" s="3" t="inlineStr">
+        <is>
+          <t>中 9월 생산자물가 5% 올라 4년여만 최고…소비자물가는 0.9%↑</t>
+        </is>
+      </c>
+      <c r="E133" s="3" t="inlineStr">
+        <is>
+          <t>(서울=연합뉴스) 권숙희 기자 = 국제유가와 원자재 비용 상승 속 중국의 지난달 생산자 물가가 가파르게 올라 4년여만에 최고 수준을 기록했다.</t>
+        </is>
+      </c>
+      <c r="F133" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G133" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014088400009</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B134" s="2" t="inlineStr">
+        <is>
+          <t>세계/국제</t>
+        </is>
+      </c>
+      <c r="C134" s="2" t="inlineStr">
+        <is>
+          <t>신규 이슈</t>
+        </is>
+      </c>
+      <c r="D134" s="3" t="inlineStr">
+        <is>
+          <t>반크 '아프리카인이 삶의 주체'인 후원 광고 찾는다</t>
+        </is>
+      </c>
+      <c r="E134" s="3" t="inlineStr">
+        <is>
+          <t>(서울=연합뉴스) 박성진 기자 = 사이버 외교사절단 반크(단장 박기태)가 아프리카 사람들을 외부의 도움을 기다리는 '수혜자'로만 반복해 보여주는...</t>
+        </is>
+      </c>
+      <c r="F134" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G134" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014087500898</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B135" s="2" t="inlineStr">
+        <is>
+          <t>세계/국제</t>
+        </is>
+      </c>
+      <c r="C135" s="2" t="inlineStr">
+        <is>
+          <t>신규 이슈</t>
+        </is>
+      </c>
+      <c r="D135" s="3" t="inlineStr">
+        <is>
+          <t>외국인 인력 부족에 '정원 돌려막기' 나선 日…급식·요양 지원</t>
+        </is>
+      </c>
+      <c r="E135" s="3" t="inlineStr">
+        <is>
+          <t>(도쿄=연합뉴스) 조성미 특파원 = 일본 정부가 체류 허가를 내준 외국인 인력 쿼터의 관리를 강화하면서 일부 업종의 인력 확보에 차질이 빚어지자...</t>
+        </is>
+      </c>
+      <c r="F135" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G135" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014086300073</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B136" s="2" t="inlineStr">
+        <is>
+          <t>세계/국제</t>
+        </is>
+      </c>
+      <c r="C136" s="2" t="inlineStr">
+        <is>
+          <t>🔥 [언론사 집중 보도 (4개사)]</t>
+        </is>
+      </c>
+      <c r="D136" s="3" t="inlineStr">
+        <is>
+          <t>[영상] 해킹에 80도까지 치솟은 냉장고…"다 녹았다" 프랑스 '발칵'</t>
+        </is>
+      </c>
+      <c r="E136" s="3" t="inlineStr">
+        <is>
+          <t>(서울=연합뉴스) 냉장고 신선식품 칸이 텅텅 비었고 냉동고에서도 상품을 찾아볼 수 없습니다. '기술적인 문제로 냉장고 안의 신선식품을 제공할 수...</t>
+        </is>
+      </c>
+      <c r="F136" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G136" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014084300704</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B137" s="2" t="inlineStr">
+        <is>
+          <t>세계/국제</t>
+        </is>
+      </c>
+      <c r="C137" s="2" t="inlineStr">
+        <is>
+          <t>신규 이슈</t>
+        </is>
+      </c>
+      <c r="D137" s="3" t="inlineStr">
+        <is>
+          <t>줘룽타이 대만 총리 "中 패권이 전 세계 반감 불러"</t>
+        </is>
+      </c>
+      <c r="E137" s="3" t="inlineStr">
+        <is>
+          <t>(타이베이=연합뉴스) 김철문 통신원 = 라이칭더 대만 총통의 지난 10일 건국기념일 연설 이후 중국이 군사적, 외교적 압박을 강화하는 가운데 줘...</t>
+        </is>
+      </c>
+      <c r="F137" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G137" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014079900009</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B138" s="2" t="inlineStr">
+        <is>
+          <t>세계/국제</t>
+        </is>
+      </c>
+      <c r="C138" s="2" t="inlineStr">
+        <is>
+          <t>🔥 [언론사 집중 보도 (5개사)]</t>
+        </is>
+      </c>
+      <c r="D138" s="3" t="inlineStr">
+        <is>
+          <t>인니 11년 만에 최악의 산불…연무로 항공 진화 1주일째 난항</t>
+        </is>
+      </c>
+      <c r="E138" s="3" t="inlineStr">
+        <is>
+          <t>(자카르타=연합뉴스) 손현규 특파원 = 11년 만에 최악의 산불로 몸살을 앓는 인도네시아에서 연무로 인해 항공 진화 작업이 1주일 넘게 차질을 ...</t>
+        </is>
+      </c>
+      <c r="F138" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G138" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014083800104</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B139" s="2" t="inlineStr">
+        <is>
+          <t>세계/국제</t>
+        </is>
+      </c>
+      <c r="C139" s="2" t="inlineStr">
+        <is>
+          <t>연결 이슈 (후속)</t>
+        </is>
+      </c>
+      <c r="D139" s="3" t="inlineStr">
+        <is>
+          <t>[영상] 사우디, 후티 연료·군사시설 전격 공습…"공항 피격 보복"</t>
+        </is>
+      </c>
+      <c r="E139" s="3" t="inlineStr">
+        <is>
+          <t>(서울=연합뉴스) 사우디 주도 연합군이 후티 반군 측이 장악한 예멘 수도 사나 등지의 주요 석유 시설과 군사 지원 시설을 전격 공습했습니다.</t>
+        </is>
+      </c>
+      <c r="F139" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G139" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014080700704</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B140" s="2" t="inlineStr">
+        <is>
+          <t>세계/국제</t>
+        </is>
+      </c>
+      <c r="C140" s="2" t="inlineStr">
+        <is>
+          <t>🔥 [언론사 집중 보도 (6개사)]</t>
+        </is>
+      </c>
+      <c r="D140" s="3" t="inlineStr">
+        <is>
+          <t>캐나다 전 부총리 "트럼프, 동맹 압박하려 CEO들 협박"</t>
+        </is>
+      </c>
+      <c r="E140" s="3" t="inlineStr">
+        <is>
+          <t>(서울=연합뉴스) 이성한 기자 = 미국 정부가 동맹국 기업의 최고경영자(CEO)와 비즈니스 리더들을 막후에서 위협하는 방식으로 동맹국을 백악관의...</t>
+        </is>
+      </c>
+      <c r="F140" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G140" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014082500009</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B141" s="2" t="inlineStr">
+        <is>
+          <t>IT/과학/신상품</t>
+        </is>
+      </c>
+      <c r="C141" s="2" t="inlineStr">
+        <is>
+          <t>🔥 [언론사 집중 보도 (4개사)]</t>
+        </is>
+      </c>
+      <c r="D141" s="3" t="inlineStr">
+        <is>
+          <t>코드 이식·AI 실험 전담… MS 엑스박스, R&amp;D 조직 신설</t>
+        </is>
+      </c>
+      <c r="E141" s="3" t="inlineStr">
+        <is>
+          <t>코드 이식·AI 실험 전담… MS 엑스박스, R&amp;D 조직 신설  IT조선엑스박스, 신기술 실험조직 ‘엑스박스 랩스’ 출범  지디넷코리아게임 넘어 디즈니처럼… MS, 엑스박스 엔터 사업부 ‘XP’ 신설  IT조선Xbox, 영화, TV, 라이브 이벤트 및 소비재를 전담하는 새로운 부서 'X...</t>
+        </is>
+      </c>
+      <c r="F141" s="3" t="inlineStr">
+        <is>
+          <t>IT조선</t>
+        </is>
+      </c>
+      <c r="G141" s="3" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE43aDVmbHg3OUM2aTA5clJXZXJIbDFjNGQyclpiLTJ6Ql9HaDJYTHktZkgtQkNhbHVjWi1ENlJ6bkl1QUZ6WEZEZFVBZmw5a3NtREVlMFc4UHNUd0FpTnppaWk4U1JHUDdray14S1FpM3rSAXRBVV95cUxORmZUbmMtYVlXUTNYSWxVUFhyLXlwazE2T1R6X0NjQUZYbm5NQVRXenBtcFR6eFZMa05Xd3AyMVN3VFExOTZYNVJOLVdrSkliN1ZHMFV0TjNVbEJ2SWkzRlBteDdrTnpaaEgybDctbk1wUkMwYg?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B142" s="2" t="inlineStr">
+        <is>
+          <t>IT/과학/신상품</t>
+        </is>
+      </c>
+      <c r="C142" s="2" t="inlineStr">
+        <is>
+          <t>연결 이슈 (후속)</t>
+        </is>
+      </c>
+      <c r="D142" s="3" t="inlineStr">
+        <is>
+          <t>[금주의인물] 프란시스 할전, ‘노벨 물리학상’ 단독 수상</t>
+        </is>
+      </c>
+      <c r="E142" s="3" t="inlineStr">
+        <is>
+          <t>[금주의인물] 프란시스 할전, ‘노벨 물리학상’ 단독 수상  주간한국Google 뉴스에서 헤드라인 및 의견 더보기</t>
+        </is>
+      </c>
+      <c r="F142" s="3" t="inlineStr">
+        <is>
+          <t>주간한국</t>
+        </is>
+      </c>
+      <c r="G142" s="3" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTFBfeGtUZl96V1ZLamFndzNRODRtVTdpRlQyV1g0VE5ZS3BBdlYwWkhGZk92VmxSeDJvLW1mWE9PTWl4VFgzM3p3UC1oTHZOWmZuX1N5M1pfNUQ2ME50dU1VWDNOY0lEeGNkcnJhSVNGUTfSAXRBVV95cUxNMFFsQS1KVzBucVd4Y2JGRTRCdWpOU2c5dkRXY2dRdkJ1Y1phV2FjSzg0Z2dfWUZUTS1NaW1wc3ZySUFhQkY5UU9EOW5KMXVEcVkxNU1yWktpRlBuN1RUWXpGTG4zZWRIOTNMa3ROaENtY05GeQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B143" s="2" t="inlineStr">
+        <is>
+          <t>IT/과학/신상품</t>
+        </is>
+      </c>
+      <c r="C143" s="2" t="inlineStr">
+        <is>
+          <t>🔥 [언론사 집중 보도 (3개사)]</t>
+        </is>
+      </c>
+      <c r="D143" s="3" t="inlineStr">
+        <is>
+          <t>삼성 반도체 부스 찾은 하정우 부위원장 "AI반도체 로드맵 확인"(종합)</t>
+        </is>
+      </c>
+      <c r="E143" s="3" t="inlineStr">
+        <is>
+          <t>(서울=연합뉴스) 김민지 강태우 기자 = 하정우 국가AI전략위원회 부위원장은 14일 서울 코엑스에서 열린 '제28회 반도체대전'(SEDEX 20...</t>
+        </is>
+      </c>
+      <c r="F143" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G143" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014042351003</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B144" s="2" t="inlineStr">
+        <is>
+          <t>IT/과학/신상품</t>
+        </is>
+      </c>
+      <c r="C144" s="2" t="inlineStr">
+        <is>
+          <t>🔥 [언론사 집중 보도 (3개사)]</t>
+        </is>
+      </c>
+      <c r="D144" s="3" t="inlineStr">
+        <is>
+          <t>[옥천소식] 15일 공설시장서 '우리동네 문화장날' 행사</t>
+        </is>
+      </c>
+      <c r="E144" s="3" t="inlineStr">
+        <is>
+          <t>(옥천=연합뉴스) 충북 옥천군은 이달 15일 옥천공설시장에서 '우리동네 문화장날' 행사를 연다고 14일 밝혔다.</t>
+        </is>
+      </c>
+      <c r="F144" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G144" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014091700064</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B145" s="2" t="inlineStr">
+        <is>
+          <t>IT/과학/신상품</t>
+        </is>
+      </c>
+      <c r="C145" s="2" t="inlineStr">
+        <is>
+          <t>신규 이슈</t>
+        </is>
+      </c>
+      <c r="D145" s="3" t="inlineStr">
+        <is>
+          <t>아트광주 22일 개막…12개국 국내외 거장 작품 출품</t>
+        </is>
+      </c>
+      <c r="E145" s="3" t="inlineStr">
+        <is>
+          <t>(전남광주=연합뉴스) 장아름 기자 = 호남권 최대 미술시장인 제17회 광주국제아트페어 '아트광주'가 오는 22일부터 25일까지 전남광주 김대중컨...</t>
+        </is>
+      </c>
+      <c r="F145" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G145" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014089800054</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B146" s="2" t="inlineStr">
+        <is>
+          <t>IT/과학/신상품</t>
+        </is>
+      </c>
+      <c r="C146" s="2" t="inlineStr">
+        <is>
+          <t>신규 이슈</t>
+        </is>
+      </c>
+      <c r="D146" s="3" t="inlineStr">
+        <is>
+          <t>[전남광주소식] 롯데백화점 11월8일까지 김장김치 예약</t>
+        </is>
+      </c>
+      <c r="E146" s="3" t="inlineStr">
+        <is>
+          <t>(전남광주=연합뉴스) 롯데백화점 광주점은 지하 1층 올가매장에서 11월8일까지 김장 김치 사전 예약행사를 한다고 14일 밝혔다.</t>
+        </is>
+      </c>
+      <c r="F146" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G146" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014088000054</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B147" s="2" t="inlineStr">
+        <is>
+          <t>IT/과학/신상품</t>
+        </is>
+      </c>
+      <c r="C147" s="2" t="inlineStr">
+        <is>
+          <t>신규 이슈</t>
+        </is>
+      </c>
+      <c r="D147" s="3" t="inlineStr">
+        <is>
+          <t>말로 지시하면 AI가 광통신망 알아서 설정…'로컬LLM' 기술 확보</t>
+        </is>
+      </c>
+      <c r="E147" s="3" t="inlineStr">
+        <is>
+          <t>(대전=연합뉴스) 김준호 기자 = 한국전자통신연구원(ETRI)은 사용자가 자연어로 원하는 네트워크 동작을 지시하면 대규모언어모델(LLM)이 이를...</t>
+        </is>
+      </c>
+      <c r="F147" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G147" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014087300063</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B148" s="2" t="inlineStr">
+        <is>
+          <t>IT/과학/신상품</t>
+        </is>
+      </c>
+      <c r="C148" s="2" t="inlineStr">
+        <is>
+          <t>신규 이슈</t>
+        </is>
+      </c>
+      <c r="D148" s="3" t="inlineStr">
+        <is>
+          <t>강릉커피거리 350m 노천카페로…21일 커피축제 개막</t>
+        </is>
+      </c>
+      <c r="E148" s="3" t="inlineStr">
+        <is>
+          <t>(강릉=연합뉴스) 유형재 기자 = '제18회 강릉커피축제'가 21∼25일 강릉커피거리와 강릉시 일원에서 열린다.</t>
+        </is>
+      </c>
+      <c r="F148" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G148" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014086200062</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B149" s="2" t="inlineStr">
+        <is>
+          <t>IT/과학/신상품</t>
+        </is>
+      </c>
+      <c r="C149" s="2" t="inlineStr">
+        <is>
+          <t>🔥 [언론사 집중 보도 (5개사)]</t>
+        </is>
+      </c>
+      <c r="D149" s="3" t="inlineStr">
+        <is>
+          <t>괴산군, 굴착기 등 불용 임대농기계 19대 공개 매각</t>
+        </is>
+      </c>
+      <c r="E149" s="3" t="inlineStr">
+        <is>
+          <t>(괴산=연합뉴스) 박재천 기자 = 충북 괴산군은 영농 자재비 상승 등으로 어려움을 겪는 농가들의 경영 부담을 덜어주고 농기계 활용을 극대화하기 ...</t>
+        </is>
+      </c>
+      <c r="F149" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G149" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014083200064</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B150" s="2" t="inlineStr">
+        <is>
           <t>연예/대중문화</t>
         </is>
       </c>
-      <c r="C107" s="2" t="inlineStr">
+      <c r="C150" s="2" t="inlineStr">
+        <is>
+          <t>신규 이슈</t>
+        </is>
+      </c>
+      <c r="D150" s="3" t="inlineStr">
+        <is>
+          <t>문체위, 이임생·이동국 국감증인 의결…암살자(들) 채택은 불발</t>
+        </is>
+      </c>
+      <c r="E150" s="3" t="inlineStr">
+        <is>
+          <t>문체위, 이임생·이동국 국감증인 의결…암살자(들) 채택은 불발  연합뉴스국민의힘 청년당원, 박정희대통령기념관에서 영화 '암살자(들)' 규탄  뉴시스[시론담론] 사실과 진실 사이  제민일보[기고]표현의 자유 뒤에 숨겨진 역사적 책임  경상일보'역사 왜곡' 암살자(들) 왜 보냐고 한 딸이 ...</t>
+        </is>
+      </c>
+      <c r="F150" s="3" t="inlineStr">
+        <is>
+          <t>연합뉴스</t>
+        </is>
+      </c>
+      <c r="G150" s="3" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTFB6ZjR1UU9sRTJ0djlRUTFyby0yeHNKWHNPNGVadEV1dTFiZTQ2VURiLTRKSUZnMnE1NjF0MDMtNFFjQzhIWTRqQ09CUUVFaTFoRENZbm94LXhBM0HSAWBBVV95cUxQdDZMM2dvcE5CeXd2Nkc2NThUWnZLTTQwNFJzamwtWWtiWUVFbThsOVZqc29uZ3Z4M25VZ25Fc29ZQVc3V04xMmRaUHZaY2VLMXZtRnppQVBUT3BtLUtqbEE?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B151" s="2" t="inlineStr">
+        <is>
+          <t>연예/대중문화</t>
+        </is>
+      </c>
+      <c r="C151" s="2" t="inlineStr">
+        <is>
+          <t>🔥 [언론사 집중 보도 (5개사)]</t>
+        </is>
+      </c>
+      <c r="D151" s="3" t="inlineStr">
+        <is>
+          <t>박하선, 6년 만에 SBS 라디오 '씨네타운' 하차…"연기에 집중"</t>
+        </is>
+      </c>
+      <c r="E151" s="3" t="inlineStr">
+        <is>
+          <t>박하선, 6년 만에 SBS 라디오 '씨네타운' 하차…"연기에 집중"  연합뉴스[단독] 박하선, '씨네타운' DJ 6년만에 떠난다…본업 집중  뉴스1박하선, ‘박하선의 씨네타운’ 청취자들에게 작별 인사  스포츠경향박하선, 6년만에 아쉬운 이별 '씨네타운' 떠난다.."연기 집중" [공식] ...</t>
+        </is>
+      </c>
+      <c r="F151" s="3" t="inlineStr">
+        <is>
+          <t>연합뉴스</t>
+        </is>
+      </c>
+      <c r="G151" s="3" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE5LTDRGSEZFSnJlTk9qUnU0ZWVVZXlvczF2WU56TEp5RzR2NlVielBndUE5cjFQeWNjMGF6RGlnT0d0Vkg4clZPVVpiZk0zZ1l3VDA1SG9vb00yZWvSAWBBVV95cUxQNzdVUEdmWTAzRTVDM19CeUFYUWhwS2FfcHhVUVpQdDlEMjF0ZThUYVFTRUpJZEsxX1BMeDZvSTRhMzB5SzNNVUdXdDFxSS11TlpwazhJMzAzV09BTkE4YWU?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B152" s="2" t="inlineStr">
+        <is>
+          <t>연예/대중문화</t>
+        </is>
+      </c>
+      <c r="C152" s="2" t="inlineStr">
         <is>
           <t>🔥 [언론사 집중 보도 (3개사)]</t>
         </is>
       </c>
-      <c r="D107" s="3" t="inlineStr">
-        <is>
-          <t>‘계약결혼’ 음주·흡연 갈등 시작</t>
-        </is>
-      </c>
-      <c r="E107" s="3" t="inlineStr">
-        <is>
-          <t>‘계약결혼’ 음주·흡연 갈등 시작  BNT뉴스'계약결혼' 남편 담배 냄새에 질색 "안대에서도 냄새나"  뉴시스흥행신화 PD도 0%대 굴욕...새 판 짠 남규홍 ‘계약결혼’ 아쉬운 초반 성적표 [SC이슈]  조선일보16기 상철, 암 수술한 영숙에 술 권유 "한 캔 정도는…"  파이낸셜뉴스...</t>
-        </is>
-      </c>
-      <c r="F107" s="3" t="inlineStr">
-        <is>
-          <t>BNT뉴스</t>
-        </is>
-      </c>
-      <c r="G107" s="3" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiZEFVX3lxTE9RbjBZcjlhWHUtcDdJb3V3Q1VlWU9CVTBWSXNzaURtb05heENLNzJ1aHZJM3BqSFBjd2p0WTU0Ym5TODhVSjV5LWxvXzM3LWEyNmlBWVcyRVNhLTRLbEM3VzRpQ1M?oc=5</t>
+      <c r="D152" s="3" t="inlineStr">
+        <is>
+          <t>콘진원, 뉴욕 코믹콘서 Ｋ-게임 알려…340만달러 수출 상담</t>
+        </is>
+      </c>
+      <c r="E152" s="3" t="inlineStr">
+        <is>
+          <t>콘진원, 뉴욕 코믹콘서 Ｋ-게임 알려…340만달러 수출 상담  지디넷코리아[르포] 뉴욕 달군 한국 웹툰…韓작가 사인회에 3시간 대기줄  연합뉴스콘진원, '뉴욕 코믹콘' 韓 공동관 성료…상담액 45억 기록  뉴스핌네이버웹툰, 뉴욕 코믹콘 5만명…'포그랜드' 부스  뉴스1"울버린으로 변신했...</t>
+        </is>
+      </c>
+      <c r="F152" s="3" t="inlineStr">
+        <is>
+          <t>지디넷코리아</t>
+        </is>
+      </c>
+      <c r="G152" s="3" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiVkFVX3lxTFBOQ1U1TGNZQnA2RDlXWm1lUEcwendSV2FKVm5ZTUlXaVZDakhGX0Z3aVB6LUlwUmhlUzRsN2EzMXhGSHJ5aXppNzI3Q1lnTTVBTmxEbXJR?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B153" s="2" t="inlineStr">
+        <is>
+          <t>연예/대중문화</t>
+        </is>
+      </c>
+      <c r="C153" s="2" t="inlineStr">
+        <is>
+          <t>연결 이슈 (후속)</t>
+        </is>
+      </c>
+      <c r="D153" s="3" t="inlineStr">
+        <is>
+          <t>초소형 말 '윌리'·가수 추혁진, 이천시 홍보대사 위촉</t>
+        </is>
+      </c>
+      <c r="E153" s="3" t="inlineStr">
+        <is>
+          <t>(이천=연합뉴스) 김광호 기자 = 경기 이천시는 초소형 말 '윌리'와 가수 추혁진을 시 홍보대사로 위촉했다고 14일 밝혔다.</t>
+        </is>
+      </c>
+      <c r="F153" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G153" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014089900061</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B154" s="2" t="inlineStr">
+        <is>
+          <t>연예/대중문화</t>
+        </is>
+      </c>
+      <c r="C154" s="2" t="inlineStr">
+        <is>
+          <t>🔥 [언론사 집중 보도 (5개사)]</t>
+        </is>
+      </c>
+      <c r="D154" s="3" t="inlineStr">
+        <is>
+          <t>박하선, 6년 만에 SBS 라디오 '씨네타운' 하차…"연기에 집중"</t>
+        </is>
+      </c>
+      <c r="E154" s="3" t="inlineStr">
+        <is>
+          <t>(서울=연합뉴스) 장진리 기자 = 배우 박하선이 다음 달 1일 방송을 끝으로 6년간 진행한 SBS 라디오 파워FM '박하선의 씨네타운'에서 하차...</t>
+        </is>
+      </c>
+      <c r="F154" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G154" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014086700005</t>
         </is>
       </c>
     </row>
@@ -5754,12 +7494,12 @@
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>+31,250.0원 (+15.13%)</t>
+          <t>+31,750.0원 (+15.38%)</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>235,500원</t>
+          <t>236,000원</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
@@ -5769,12 +7509,12 @@
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>229,500원</t>
+          <t>230,000원</t>
         </is>
       </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
-          <t>+9.2%</t>
+          <t>+9.0%</t>
         </is>
       </c>
       <c r="K15" s="3" t="inlineStr">
@@ -5784,7 +7524,7 @@
       </c>
       <c r="L15" s="3" t="inlineStr">
         <is>
-          <t>RSI 38.0로 단기 과매도 구간 진입, 기술적 반등 노림</t>
+          <t>RSI 38.3로 단기 과매도 구간 진입, 기술적 반등 노림</t>
         </is>
       </c>
       <c r="M15" s="3" t="inlineStr">
@@ -5798,21 +7538,21 @@
         </is>
       </c>
       <c r="O15" s="3" t="n">
-        <v>38</v>
+        <v>38.3</v>
       </c>
       <c r="P15" s="3" t="inlineStr">
         <is>
-          <t>-9.4%</t>
+          <t>-9.2%</t>
         </is>
       </c>
       <c r="Q15" s="3" t="inlineStr">
         <is>
-          <t>51.6%</t>
+          <t>51.8%</t>
         </is>
       </c>
       <c r="R15" s="3" t="inlineStr">
         <is>
-          <t>9월 ICT 수출 751억달러 '역대 최대'…반도체가 80% 견인 (연합인포맥스)</t>
+          <t>삼전닉스 폭락에도 "지금이 저점"…'W자 반등' 전망한 이유 [분석+] (한국경제)</t>
         </is>
       </c>
     </row>
@@ -5839,32 +7579,32 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>1,475,000원</t>
+          <t>1,470,000원</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>+372,000.0원 (+33.73%)</t>
+          <t>+367,000.0원 (+33.27%)</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>1,460,000원</t>
+          <t>1,455,500원</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>1,706,000원</t>
+          <t>1,705,500원</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>1,423,500원</t>
+          <t>1,418,500원</t>
         </is>
       </c>
       <c r="J16" s="3" t="inlineStr">
         <is>
-          <t>+16.8%</t>
+          <t>+17.2%</t>
         </is>
       </c>
       <c r="K16" s="3" t="inlineStr">
@@ -5874,7 +7614,7 @@
       </c>
       <c r="L16" s="3" t="inlineStr">
         <is>
-          <t>RSI 34.2로 단기 과매도 구간 진입, 기술적 반등 노림</t>
+          <t>RSI 33.7로 단기 과매도 구간 진입, 기술적 반등 노림</t>
         </is>
       </c>
       <c r="M16" s="3" t="inlineStr">
@@ -5888,16 +7628,16 @@
         </is>
       </c>
       <c r="O16" s="3" t="n">
-        <v>34.2</v>
+        <v>33.7</v>
       </c>
       <c r="P16" s="3" t="inlineStr">
         <is>
-          <t>-15.3%</t>
+          <t>-15.5%</t>
         </is>
       </c>
       <c r="Q16" s="3" t="inlineStr">
         <is>
-          <t>41.4%</t>
+          <t>41.2%</t>
         </is>
       </c>
       <c r="R16" s="3" t="inlineStr">
@@ -5929,17 +7669,17 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>319,500원</t>
+          <t>320,000원</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>-172,000.0원 (-34.99%)</t>
+          <t>-171,500.0원 (-34.89%)</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>313,000원</t>
+          <t>313,500원</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
@@ -5949,12 +7689,12 @@
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>303,500원</t>
+          <t>304,000원</t>
         </is>
       </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
-          <t>+22.2%</t>
+          <t>+22.0%</t>
         </is>
       </c>
       <c r="K17" s="3" t="inlineStr">
@@ -5978,16 +7718,16 @@
         </is>
       </c>
       <c r="O17" s="3" t="n">
-        <v>26.1</v>
+        <v>26.6</v>
       </c>
       <c r="P17" s="3" t="inlineStr">
         <is>
-          <t>-8.6%</t>
+          <t>-8.5%</t>
         </is>
       </c>
       <c r="Q17" s="3" t="inlineStr">
         <is>
-          <t>17.7%</t>
+          <t>17.8%</t>
         </is>
       </c>
       <c r="R17" s="3" t="inlineStr">
@@ -6019,12 +7759,12 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>109,500원</t>
+          <t>110,000원</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>-39,500.0원 (-26.47%)</t>
+          <t>-39,300.0원 (-26.34%)</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
@@ -6039,12 +7779,12 @@
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>104,000원</t>
+          <t>104,500원</t>
         </is>
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>+17.8%</t>
+          <t>+17.5%</t>
         </is>
       </c>
       <c r="K18" s="3" t="inlineStr">
@@ -6068,16 +7808,16 @@
         </is>
       </c>
       <c r="O18" s="3" t="n">
-        <v>33</v>
+        <v>33.5</v>
       </c>
       <c r="P18" s="3" t="inlineStr">
         <is>
-          <t>-5.3%</t>
+          <t>-5.2%</t>
         </is>
       </c>
       <c r="Q18" s="3" t="inlineStr">
         <is>
-          <t>7.1%</t>
+          <t>7.3%</t>
         </is>
       </c>
       <c r="R18" s="3" t="inlineStr">
@@ -6114,7 +7854,7 @@
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>-19,900.0원 (-9.88%)</t>
+          <t>-19,850.0원 (-9.85%)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -6158,7 +7898,7 @@
         </is>
       </c>
       <c r="O19" s="3" t="n">
-        <v>32.6</v>
+        <v>32.7</v>
       </c>
       <c r="P19" s="3" t="inlineStr">
         <is>
@@ -6167,12 +7907,12 @@
       </c>
       <c r="Q19" s="3" t="inlineStr">
         <is>
-          <t>6.4%</t>
+          <t>6.5%</t>
         </is>
       </c>
       <c r="R19" s="3" t="inlineStr">
         <is>
-          <t>최근 특이 뉴스 없음</t>
+          <t>콘진원, 뉴욕 코믹콘서 Ｋ-게임 알려…340만달러 수출 상담 (지디넷코리아)</t>
         </is>
       </c>
     </row>
@@ -6199,17 +7939,17 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>31,900원</t>
+          <t>32,000원</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>-16,200.0원 (-33.68%)</t>
+          <t>-16,100.0원 (-33.47%)</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>31,300원</t>
+          <t>31,400원</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
@@ -6219,12 +7959,12 @@
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>30,300원</t>
+          <t>30,400원</t>
         </is>
       </c>
       <c r="J20" s="3" t="inlineStr">
         <is>
-          <t>+10.8%</t>
+          <t>+10.5%</t>
         </is>
       </c>
       <c r="K20" s="3" t="inlineStr">
@@ -6248,21 +7988,21 @@
         </is>
       </c>
       <c r="O20" s="3" t="n">
-        <v>34.4</v>
+        <v>35.4</v>
       </c>
       <c r="P20" s="3" t="inlineStr">
         <is>
-          <t>-4.4%</t>
+          <t>-4.1%</t>
         </is>
       </c>
       <c r="Q20" s="3" t="inlineStr">
         <is>
-          <t>4.2%</t>
+          <t>4.4%</t>
         </is>
       </c>
       <c r="R20" s="3" t="inlineStr">
         <is>
-          <t>최근 특이 뉴스 없음</t>
+          <t>카카오뱅크 "18일 새벽 금융거래 일시 중단…전산시스템 점검" (주요언론)</t>
         </is>
       </c>
     </row>
@@ -6289,27 +8029,27 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>182,000원</t>
+          <t>182,500원</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>-7,419.049999999988원 (-3.91%)</t>
+          <t>-6,919.049999999988원 (-3.65%)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>178,500원</t>
+          <t>179,000원</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>191,500원</t>
+          <t>192,000원</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>173,000원</t>
+          <t>173,500원</t>
         </is>
       </c>
       <c r="J21" s="3" t="inlineStr">
@@ -6338,16 +8078,16 @@
         </is>
       </c>
       <c r="O21" s="3" t="n">
-        <v>50.3</v>
+        <v>51.3</v>
       </c>
       <c r="P21" s="3" t="inlineStr">
         <is>
-          <t>+1.3%</t>
+          <t>+1.6%</t>
         </is>
       </c>
       <c r="Q21" s="3" t="inlineStr">
         <is>
-          <t>29.4%</t>
+          <t>30.0%</t>
         </is>
       </c>
       <c r="R21" s="3" t="inlineStr">
@@ -6379,17 +8119,17 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>835,000원</t>
+          <t>845,000원</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>-688,000.0원 (-45.17%)</t>
+          <t>-678,000.0원 (-44.52%)</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>818,500원</t>
+          <t>828,000원</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
@@ -6399,12 +8139,12 @@
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>793,000원</t>
+          <t>803,000원</t>
         </is>
       </c>
       <c r="J22" s="3" t="inlineStr">
         <is>
-          <t>+38.9%</t>
+          <t>+37.3%</t>
         </is>
       </c>
       <c r="K22" s="3" t="inlineStr">
@@ -6428,16 +8168,16 @@
         </is>
       </c>
       <c r="O22" s="3" t="n">
-        <v>29.3</v>
+        <v>30.6</v>
       </c>
       <c r="P22" s="3" t="inlineStr">
         <is>
-          <t>-17.5%</t>
+          <t>-16.5%</t>
         </is>
       </c>
       <c r="Q22" s="3" t="inlineStr">
         <is>
-          <t>6.0%</t>
+          <t>7.1%</t>
         </is>
       </c>
       <c r="R22" s="3" t="inlineStr">
@@ -6469,32 +8209,32 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>422,500원</t>
+          <t>424,000원</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>+22,500.0원 (+5.62%)</t>
+          <t>+23,750.0원 (+5.94%)</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>372,000원</t>
+          <t>372,500원</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>422,500원</t>
+          <t>424,000원</t>
         </is>
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>414,000원</t>
+          <t>415,500원</t>
         </is>
       </c>
       <c r="J23" s="3" t="inlineStr">
         <is>
-          <t>+13.5%</t>
+          <t>+13.8%</t>
         </is>
       </c>
       <c r="K23" s="3" t="inlineStr">
@@ -6504,7 +8244,7 @@
       </c>
       <c r="L23" s="3" t="inlineStr">
         <is>
-          <t>RSI 71.1, 20일선 이격도 +13.5%로 단기 과열권, 분할 차익 실현 권고</t>
+          <t>RSI 71.4, 20일선 이격도 +13.8%로 단기 과열권, 분할 차익 실현 권고</t>
         </is>
       </c>
       <c r="M23" s="3" t="inlineStr">
@@ -6518,16 +8258,16 @@
         </is>
       </c>
       <c r="O23" s="3" t="n">
-        <v>71.09999999999999</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="P23" s="3" t="inlineStr">
         <is>
-          <t>+13.5%</t>
+          <t>+13.8%</t>
         </is>
       </c>
       <c r="Q23" s="3" t="inlineStr">
         <is>
-          <t>55.8%</t>
+          <t>56.3%</t>
         </is>
       </c>
       <c r="R23" s="3" t="inlineStr">
@@ -6559,17 +8299,17 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>309,000원</t>
+          <t>310,000원</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>-52,500.0원 (-14.52%)</t>
+          <t>-51,500.0원 (-14.25%)</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>303,000원</t>
+          <t>304,000원</t>
         </is>
       </c>
       <c r="H24" s="3" t="inlineStr">
@@ -6579,12 +8319,12 @@
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>293,500원</t>
+          <t>294,500원</t>
         </is>
       </c>
       <c r="J24" s="3" t="inlineStr">
         <is>
-          <t>+10.3%</t>
+          <t>+9.9%</t>
         </is>
       </c>
       <c r="K24" s="3" t="inlineStr">
@@ -6608,16 +8348,16 @@
         </is>
       </c>
       <c r="O24" s="3" t="n">
-        <v>45.3</v>
+        <v>46</v>
       </c>
       <c r="P24" s="3" t="inlineStr">
         <is>
-          <t>-1.9%</t>
+          <t>-1.6%</t>
         </is>
       </c>
       <c r="Q24" s="3" t="inlineStr">
         <is>
-          <t>12.7%</t>
+          <t>13.1%</t>
         </is>
       </c>
       <c r="R24" s="3" t="inlineStr">
@@ -6712,7 +8452,7 @@
       </c>
       <c r="R25" s="3" t="inlineStr">
         <is>
-          <t>'월가 족집게' 댄 아이브스 "테슬라·스페이스X 내년 합병 가능성 80%" (주요언론)</t>
+          <t>최근 특이 뉴스 없음</t>
         </is>
       </c>
     </row>
@@ -6892,7 +8632,7 @@
       </c>
       <c r="R27" s="3" t="inlineStr">
         <is>
-          <t>'월가 족집게' 댄 아이브스 "테슬라·스페이스X 내년 합병 가능성 80%" (주요언론)</t>
+          <t>최근 특이 뉴스 없음</t>
         </is>
       </c>
     </row>
@@ -7214,12 +8954,12 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>6,123.61</t>
+          <t>6,137.60</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>+88.26 (+1.46%)</t>
+          <t>+102.25 (+1.69%)</t>
         </is>
       </c>
     </row>
@@ -7241,12 +8981,12 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>832.41</t>
+          <t>839.61</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>-4.62 (-0.55%)</t>
+          <t>+2.58 (+0.31%)</t>
         </is>
       </c>
     </row>
@@ -7460,27 +9200,27 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>112,538,000원</t>
+          <t>112,951,000원</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>-0.05%</t>
+          <t>+0.32%</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>111,975,000원</t>
+          <t>112,386,000원</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>121,541,000원</t>
+          <t>121,987,000원</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>110,573,000원</t>
+          <t>110,593,000원</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
@@ -7517,27 +9257,27 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>3,384,000원</t>
+          <t>3,393,000원</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>+0.09%</t>
+          <t>+0.35%</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>3,357,000원</t>
+          <t>3,366,000원</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>3,587,000원</t>
+          <t>3,596,500원</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>3,265,500원</t>
+          <t>3,274,000원</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
@@ -7552,7 +9292,7 @@
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>RSI 46.8로 단기 과매도 구간 진입, 기술적 반등 기대</t>
+          <t>RSI 47.6로 단기 과매도 구간 진입, 기술적 반등 기대</t>
         </is>
       </c>
     </row>
@@ -7574,32 +9314,32 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>145,000원</t>
+          <t>145,600원</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>+0.28%</t>
+          <t>+0.69%</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>143,800원</t>
+          <t>144,400원</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>155,800원</t>
+          <t>155,900원</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>139,900원</t>
+          <t>140,500원</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>+8.3%</t>
+          <t>+7.9%</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
@@ -7609,7 +9349,7 @@
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>RSI 47.3로 단기 과매도 구간 진입, 기술적 반등 기대</t>
+          <t>RSI 48.2로 단기 과매도 구간 진입, 기술적 반등 기대</t>
         </is>
       </c>
     </row>
@@ -7792,7 +9532,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
@@ -7862,7 +9602,7 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
@@ -7871,12 +9611,12 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>일진전기</t>
+          <t>HMM</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>가장 저평가된 전력기기</t>
+          <t>우려도 있지만 너무 잠잠한 주가</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -7891,37 +9631,37 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>변압기 29년 수주 논의 및 전선 상반기 수주 급증 5월 시가총액 약 6.9조원 도달 이후 7월말 2.2조원까지 약 68% 하락. 전선업체들의 수주잔고총계 연간 증가율은 24년 25.4%, 25년 21.2%에서 26년 상반기에만 23.2% 증가. 변압기에 이은 전선 부문의 호황이 확대되는 것을 감안할 때 펀더멘털 문제가 아닌 수급 측면의 주가 하락으로 판단</t>
+          <t>거버넌스 우려로 덮어놓기엔 아까운 실적 글로벌 컨테이너선사들은 가이던스 상향과 함께 주가도 상승했으나 동사 반응은 제한적. 거버넌스 불확실성에도 예상보다 큰 이익 회복에 주목</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>2026-10-14_신한투자증권_일진전기_가장 저평가된 전력기기.pdf</t>
+          <t>2026-10-14_신한투자증권_HMM_우려도 있지만 너무 잠잠한 주가.pdf</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>2,350.8십억원</t>
+          <t>14,179.9십억원</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>252.8십억원</t>
+          <t>2,497.7십억원</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>2,595.2십억원</t>
+          <t>14,293.1십억원</t>
         </is>
       </c>
       <c r="M4" s="3" t="inlineStr">
         <is>
-          <t>271.7십억원</t>
+          <t>1,812.7십억원</t>
         </is>
       </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
-          <t>2026/2027 실적 성장세 및 기업가치 재평가 전망</t>
+          <t>3Q26 매출 4조 802억원(+51%, 이하 YoY) 및 영업이익 1조 42억원(+</t>
         </is>
       </c>
     </row>
@@ -7941,12 +9681,12 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>HMM</t>
+          <t>일진전기</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>우려도 있지만 너무 잠잠한 주가</t>
+          <t>가장 저평가된 전력기기</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -7961,37 +9701,37 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>거버넌스 우려로 덮어놓기엔 아까운 실적 글로벌 컨테이너선사들은 가이던스 상향과 함께 주가도 상승했으나 동사 반응은 제한적. 거버넌스 불확실성에도 예상보다 큰 이익 회복에 주목</t>
+          <t>변압기 29년 수주 논의 및 전선 상반기 수주 급증 5월 시가총액 약 6.9조원 도달 이후 7월말 2.2조원까지 약 68% 하락. 전선업체들의 수주잔고총계 연간 증가율은 24년 25.4%, 25년 21.2%에서 26년 상반기에만 23.2% 증가. 변압기에 이은 전선 부문의 호황이 확대되는 것을 감안할 때 펀더멘털 문제가 아닌 수급 측면의 주가 하락으로 판단</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>2026-10-14_신한투자증권_HMM_우려도 있지만 너무 잠잠한 주가.pdf</t>
+          <t>2026-10-14_신한투자증권_일진전기_가장 저평가된 전력기기.pdf</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>14,179.9십억원</t>
+          <t>2,350.8십억원</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>2,497.7십억원</t>
+          <t>252.8십억원</t>
         </is>
       </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>14,293.1십억원</t>
+          <t>2,595.2십억원</t>
         </is>
       </c>
       <c r="M5" s="3" t="inlineStr">
         <is>
-          <t>1,812.7십억원</t>
+          <t>271.7십억원</t>
         </is>
       </c>
       <c r="N5" s="3" t="inlineStr">
         <is>
-          <t>3Q26 매출 4조 802억원(+51%, 이하 YoY) 및 영업이익 1조 42억원(+</t>
+          <t>2026/2027 실적 성장세 및 기업가치 재평가 전망</t>
         </is>
       </c>
     </row>
@@ -8072,7 +9812,7 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
@@ -8142,7 +9882,7 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -8212,7 +9952,7 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -8282,7 +10022,7 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -8352,7 +10092,7 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
@@ -8426,7 +10166,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -8553,7 +10293,7 @@
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>+2.2%</t>
+          <t>+2.6%</t>
         </is>
       </c>
       <c r="K2" s="3" t="inlineStr">
@@ -8615,7 +10355,7 @@
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>+2.5%</t>
+          <t>+2.7%</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
@@ -8739,7 +10479,7 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>+2.9%</t>
+          <t>+3.2%</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
@@ -8801,12 +10541,12 @@
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>+0.5%</t>
+          <t>+1.7%</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>839,000원</t>
+          <t>849,000원</t>
         </is>
       </c>
       <c r="L6" s="3" t="inlineStr">
@@ -8863,7 +10603,7 @@
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>+4.4%</t>
+          <t>+4.7%</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
@@ -8890,50 +10630,112 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
+          <t>삼성전자</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>005930.KS</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>238,000원</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>235,500원</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>257,000원</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>229,500원</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>⏳ 진행 중 (당일 포지션 구축)</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>+1.3%</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>238,500원</t>
+        </is>
+      </c>
+      <c r="L8" s="3" t="inlineStr">
+        <is>
+          <t>1일차</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
           <t>SK하이닉스</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>000660.KS</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>1,475,000원</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>1,460,000원</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>1,706,000원</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
+      <c r="H9" s="3" t="inlineStr">
         <is>
           <t>1,423,500원</t>
         </is>
       </c>
-      <c r="I8" s="3" t="inlineStr">
+      <c r="I9" s="3" t="inlineStr">
         <is>
           <t>⏳ 진행 중 (당일 포지션 구축)</t>
         </is>
       </c>
-      <c r="J8" s="3" t="inlineStr">
-        <is>
-          <t>+1.0%</t>
-        </is>
-      </c>
-      <c r="K8" s="3" t="inlineStr">
-        <is>
-          <t>1,475,000원</t>
-        </is>
-      </c>
-      <c r="L8" s="3" t="inlineStr">
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>+0.7%</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>1,470,000원</t>
+        </is>
+      </c>
+      <c r="L9" s="3" t="inlineStr">
         <is>
           <t>1일차</t>
         </is>
@@ -9077,7 +10879,7 @@
       <c r="D3" s="3" t="inlineStr"/>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>데스트라 멀티 대체 투자 펀드, 자사주 매입 프로그램 도입·월 배당금 주당 0.115달러로 인상</t>
+          <t>“역시 주주환원은 뒷전입니까”…코스피 자사주 매입, 삼전닉스 뺐더니 줄었다</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
@@ -9087,17 +10889,17 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>데이터투자</t>
+          <t>매일경제 마켓</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 19:52:27 GMT</t>
+          <t>Sun, 11 Oct 2026 11:51:10 GMT</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMic0FVX3lxTE1lemt2YTFaYUFFeVI4cVJZbjFYOHpWLVJmNTUxN3huQlRtYUVHYXplTUpvQktSZFdKenhkMl9PYXlNci1RbHNtTUdQdXgxelpjaEJVbWNjVmFndWFiaV9KZFAxd2ozbVZXVUd4MHFPNlZYT0U?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiUkFVX3lxTE0zXzFYa0xGekFCVWtnODd6QVRIRmp1MnFLcXhBWWVadVdXQWZaY3lGcGg3WUl1dzY4M1R1cTBWV1h1a0JBbXdGV3Y0aC1KV25lRmc?oc=5</t>
         </is>
       </c>
     </row>
@@ -9120,7 +10922,7 @@
       <c r="D4" s="3" t="inlineStr"/>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>“역시 주주환원은 뒷전입니까”…코스피 자사주 매입, 삼전닉스 뺐더니 줄었다</t>
+          <t>데스트라 멀티 대체 투자 펀드, 자사주 매입 프로그램 도입·월 배당금 주당 0.115달러로 인상</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -9130,17 +10932,17 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>매일경제 마켓</t>
+          <t>데이터투자</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>Sun, 11 Oct 2026 11:51:10 GMT</t>
+          <t>Tue, 13 Oct 2026 19:52:27 GMT</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiUkFVX3lxTE0zXzFYa0xGekFCVWtnODd6QVRIRmp1MnFLcXhBWWVadVdXQWZaY3lGcGg3WUl1dzY4M1R1cTBWV1h1a0JBbXdGV3Y0aC1KV25lRmc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMic0FVX3lxTE1lemt2YTFaYUFFeVI4cVJZbjFYOHpWLVJmNTUxN3huQlRtYUVHYXplTUpvQktSZFdKenhkMl9PYXlNci1RbHNtTUdQdXgxelpjaEJVbWNjVmFndWFiaV9KZFAxd2ozbVZXVUd4MHFPNlZYT0U?oc=5</t>
         </is>
       </c>
     </row>
@@ -9372,6 +11174,220 @@
       <c r="I9" s="3" t="inlineStr">
         <is>
           <t>https://news.google.com/rss/articles/CBMic0FVX3lxTE1MVmRGS1NqcEJobXNpM01fNTlJbV9MeFZUeXBTVktGWV9XOWFlMHFET09BeW1rQ1RJdzVCR0I1OXM1UkpxM3Nnazk4RnBPbC1EaGFxM0FpVVpqYzZPRnlGb0plTEwyYmZDSXJXNW8yYmh5M0k?oc=5</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="65" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="5" max="5"/>
+    <col width="65" customWidth="1" min="6" max="6"/>
+    <col width="65" customWidth="1" min="7" max="7"/>
+    <col width="65" customWidth="1" min="8" max="8"/>
+    <col width="65" customWidth="1" min="9" max="9"/>
+    <col width="65" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="53" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>수집일자</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>트랙구분</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>배지</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>스토리제목</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>핵심키워드</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>도입부훅</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>1막_발단현상</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>2막_과거시초타임라인</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>3막_이면의속셈과심리</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>4막_파장과미래변화</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>언론사/출처</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>원문링크</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>경제·사회 딥다이브</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>아! 이래서 그런 거였어</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>🌐 [경제·사회 딥다이브] "아! 이래서 그런 거였어": 트럼프, 동맹 압박하려 CEO들 협박의 숨겨진 비하인드</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>트럼프, 동맹 압박하려 CEO들 협박</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>오늘 언론을 도배한 '트럼프, 동맹 압박하려 CEO들 협박' 뉴스, 겉보기엔 단순한 갈등 같지만 사실은 수년 전부터 시작된 거대한 판의 충돌입니다.</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>오늘 언론사들이 일제히 보도한 사건: **[캐나다 전 부총리 "트럼프, 동맹 압박하려 CEO들 협박"]** 입니다. (서울=연합뉴스) 이성한 기자 = 미국 정부가 동맹국 기업의 최고경영자(CEO)와 비즈니스 리더들을 막후에서 위협하는 방식으로 동맹국을 백악관의...</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>사실 이 문제는 과거 수년 전부터 시장과 정책 당국 간에 누적되어 온 해묵은 과제가 특정 계기를 맞아 수면 위로 폭발한 것입니다.</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>언론 헤드라인이 말해주지 않는 진짜 흑막(돈과 권력의 흐름)은 따로 있습니다. 표면적인 명분 뒤에는 이해관계자들의 치열한 득실 계산과 법·제도의 맹점을 파고든 치밀한 수싸움이 숨겨져 있습니다.</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>이 사건은 일회성 해프닝으로 끝나지 않습니다. 앞으로 한국 경제와 관련 산업의 판도를 바꿀 중요한 분수령이 될 것이며, 우리는 이해관계자들의 다음 행보를 면밀히 주시해야 합니다.</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="L2" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014082500009</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>트렌드·유행 딥다이브</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>요즘 왜 이게 유행할까?</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>🔥 [트렌드·유행 딥다이브] "요즘 왜 이게 유행할까?": 블루 아카이브 품절 대란의 비밀</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>블루 아카이브</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>요즘 SNS와 거리에서 난리 난 '블루 아카이브', 사람들은 도대체 왜 여기에 줄을 서고 열광하는 걸까요?</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>지금 번화가와 온라인 쇼핑몰에서 가장 뜨거운 화두는 단연 **[GS25, '블루 아카이브'와 3차 협업…전국 팝업스토어도 운영]** 입니다. GS25, '블루 아카이브'와 3차 협업…전국 팝업스토어도 운영 매일경제 마켓</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>이 유행의 시초를 거슬러 올라가면 인플루언서와 숏폼(틱톡/릴스) 바이럴이 결정적 계기였습니다: 수영복 입은 문주님, 블루 아카이브에 '람과천청' 업데이트 월요신문 알림음과 배경 음악을 구분하는 블루아카이브 경마 사운드 안내 Calgary Roughnecks...</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>사람들이 지갑을 여는 진짜 심리는 무엇일까요? 단순한 맛이나 디자인을 넘어, '나도 경험해 봤다'는 즉각적인 소속감과 디토(Ditto) 소비 심리가 강력한 기폭제가 되었습니다.</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>이 유행은 단순한 반짝 인기에 그칠까요, 아니면 새로운 일상의 표준이 될까요? 빠르게 바뀌는 트렌드 주기 속에서 관련 업계는 벌써 다음 먹거리 선점에 나섰습니다.</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>매일경제 마켓</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiUkFVX3lxTE5oRlFmSDNxbVRUaEctLWp3SHVvbEtGeFRFajBNUndReGo0QzZNdFBacG1la0ZGR3BScW5qb091eW4xclJOQi1vYk9DVjM4NVd6cnc?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: enhance research selection algorithm, add NASDAQ/SP500, FX diffs, multi-factor quant stock filters, and concise briefing tone
</commit_message>
<xml_diff>
--- a/reports/일자별_누적_데일리_이슈_및_주식_브리핑_마스터.xlsx
+++ b/reports/일자별_누적_데일리_이슈_및_주식_브리핑_마스터.xlsx
@@ -3636,22 +3636,22 @@
       </c>
       <c r="D86" s="3" t="inlineStr">
         <is>
-          <t>한미 국방장관 이달말 첫 대면 가능성...전작권 논의 주목</t>
+          <t>윤석열 선거법 2심, 오는 27일 선고‥국민의힘 '선거비용 397억 원 반환' 달렸다</t>
         </is>
       </c>
       <c r="E86" s="3" t="inlineStr">
         <is>
-          <t>한미 국방장관 이달말 첫 대면 가능성...전작권 논의 주목 YTN 한미 전작권 이견에… SCM, 12월로 이례적 연기 조선일보브런슨 "시간도 하나의 조건"…한미 전작권 전환 협상 난항 예상 뉴스1주한미군사령관 "조건 충족시 전작권 전환 지지‥한반도 다층감지할 것" MBC 뉴스한미, SCM 일정 조율도 ‘삐그덕’…양국 국방장관 이달말 첫 대면 가능성 KBS 뉴스.</t>
+          <t>윤석열 선거법 2심, 오는 27일 선고‥국민의힘 '선거비용 397억 원 반환' 달렸다. MBC 뉴스'국힘 397억 반환' 걸린 尹 재판서 특검 '당선무효형 유지' 요청 MBC 뉴스‘국힘 397억 반환’ 걸린 2심서…윤 "이럴 거면 선거 왜 해" JTBC‘국힘 397억’ 걸린 尹 선거법 2심 27일 선고 동아일보특검, 尹 '여론조사 무상수수' 무죄 판결에 상고…"납득 어려워".</t>
         </is>
       </c>
       <c r="F86" s="3" t="inlineStr">
         <is>
-          <t>YTN</t>
+          <t>MBC 뉴스</t>
         </is>
       </c>
       <c r="G86" s="3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMib0FVX3lxTFByaGg5R3BoUm5yNXVJOENVOXc5cnVCdlpxdldkdFd4WFRVcDBPbmhHTlBPWnJTOUg0Q3FhYVAxV3dTSUVuNTd6N2s0VmxWWlo4NUhja1FtYVFHazRzYmRmZVVNaWtfVm5hZDdRYl9GOA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTFBqVlppeEExSms5RGVjN2ZqY2Y1bXN6ZlV4MTJlcnc3VERVT1BNRDRBZG94Q2xFaGxSZ3JEelJZVk1NNFMzOUt4WW1jOXd2Z0xydXlFajhLM05qZU8xc3RGVlM2NXdteHd1b3FPMjZPdm9UWHFmcjBJ0gF3QVVfeXFMT2FLNS01aG8xbG5qdVpQVl82RmpXVktST0k1VHZ6T2lzdk1lNXJGa1RrV21jZGkxRVUtMzVhdjRFdEF3QUJtRjI0RktXTjhmc2s1YzNLZHpHcDJUZy1Jb2lrYm43ZFpfazFmZUF6OFNtMUJwdEE4M28?oc=5</t>
         </is>
       </c>
     </row>
@@ -3673,22 +3673,22 @@
       </c>
       <c r="D87" s="3" t="inlineStr">
         <is>
-          <t>UST, '청정 원전 해체' 길 열었다…신규 제염제 개발</t>
+          <t>대입 논술시험서 AI안경 쓴 수험생들 적발…시립대 "응시 3년 금지"</t>
         </is>
       </c>
       <c r="E87" s="3" t="inlineStr">
         <is>
-          <t>원자력발전소를 해체할 때 방사성 오염물질은 제거하면서 독성 약품 사용량은 줄이고, 제염 후 남은 폐액까지 하나...</t>
+          <t>대입 논술시험서 AI안경 쓴 수험생들 적발…시립대 "응시 3년 금지" 논술 시험장에 등장한 스마트안경…연세대·시립대서 줄줄이 적발 KBS 뉴스뿔테 안경 아니었어?···연세대 논술 시험장서 ‘스마트 안경’ 적발 주간경향정근식, '스마트 안경' 부정행위 우려에 "교육부 지침 따라 대응" MBC 뉴스수험생들 “이번 수능때 AI 안경 쓸것”… 대학선 방지책 비상 문화일보.</t>
         </is>
       </c>
       <c r="F87" s="3" t="inlineStr">
         <is>
-          <t>주요언론</t>
+          <t>연합뉴스</t>
         </is>
       </c>
       <c r="G87" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261014112100063</t>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTFBkb21vYW14V21SZVNZOVlHaGIyRkJ4TlA5RU9IYkRrekVpOVBSbjlqLWdSZ25mcnVpOUhvS1R5WGpjSGdicm4xSDhCR2xERjduVktqR3RveWJKY03SAWBBVV95cUxObXlQc0RwOFRTSnJaSk9MUTM1S3JsaFlsSUVsc1ZGeWc1SUVjNGFWLUNiWExVc2pTSkpmc1Eyek80WHN3cE9tOHdBZXJIMm5aNno5TGR2bFZ0cml1aEM0WE8?oc=5</t>
         </is>
       </c>
     </row>
@@ -3705,27 +3705,27 @@
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>연결 이슈 (후속)</t>
+          <t>🔥 [언론사 집중 보도 (3개사)]</t>
         </is>
       </c>
       <c r="D88" s="3" t="inlineStr">
         <is>
-          <t>[속보] '1억 공천헌금' 무소속 강선우 의원 1심 징역 2년 6개월 선고</t>
+          <t>"뛰다가 죽음 이를 수도"…황영조가 러너들에 던진 경고</t>
         </is>
       </c>
       <c r="E88" s="3" t="inlineStr">
         <is>
-          <t>[속보] '1억 공천헌금' 무소속 강선우 의원 1심 징역 2년 6개월 선고의 핵심 내용과 시장 반응을 분석한 보도입니다.</t>
+          <t>이를 수도"…황영조가 러너들에 던진 경고 황영조 ’러닝 경고’…“기록·SNS 욕심 보다. 몸 상태 체크“ TV"포기할 줄 아는 사람이 잘 뛰는 사람"...잇따른 마라톤 사고에 황영조 '일침' YTN'서울달리기' 숨진 20대女는 '카이스트 대학원생' 유지원씨 파이낸셜뉴스“그냥 달리고 싶어”…결승선 앞 멈춰진 20대 러너의 꿈 KBS 뉴스.</t>
         </is>
       </c>
       <c r="F88" s="3" t="inlineStr">
         <is>
-          <t>주요언론</t>
+          <t>한국경제</t>
         </is>
       </c>
       <c r="G88" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261014116600004</t>
+          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTFBnZE9PNDVINmZpajNMVEppN3IyZV9KUE1kZE1xcnd1RHlOV2NIWWJiSGFUUW5Ed2F1QkNFNllwY24xY0JUT29VZ3Z6eTJIcGFqZ2hsWk5ocHdfdw?oc=5</t>
         </is>
       </c>
     </row>
@@ -3737,32 +3737,32 @@
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>거시경제/비즈니스</t>
+          <t>사회/사건사고</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>🔥 [언론사 집중 보도 (3개사)]</t>
+          <t>연결 이슈 (후속)</t>
         </is>
       </c>
       <c r="D89" s="3" t="inlineStr">
         <is>
-          <t>"국평 포기합니다"…서울 청약 넣으려다 마음 바꾼 이유</t>
+          <t>‘한동훈 고발장’ 경찰·중수청 접수…‘자녀 허위스펙·부실 수사’ 의혹</t>
         </is>
       </c>
       <c r="E89" s="3" t="inlineStr">
         <is>
-          <t>"국평 포기합니다"…서울 청약 넣으려다. 바꾼 이유 “분양가 무서워 소형으로”…수도권 청약시장 면적별 양극화 심화 매일경제강원 아파트 9월 분양가 제곱미터에 636만 원 KBS 뉴스"국민평형 너무 비싸요"…서울 청약 80% 소형으로 쏠렸다.</t>
+          <t>‘한동훈 고발장’ 경찰·중수청 접수…‘자녀 허위스펙·부실 수사’ 의혹 한겨레시민단체, '딸 허위 스펙 수사무마' 의혹 한동훈 고발 MBC 뉴스 신지호 “한동훈 딸 의혹…민주당, 쓰레기 재활용하나?” KBS 뉴스한동훈, 법무부 장관 재직시 딸 `허위스펙` 수사무마 의혹으로 고발당해 국제신문한동훈이 자초한 3개의 '사법 리스크' OhmyNews.</t>
         </is>
       </c>
       <c r="F89" s="3" t="inlineStr">
         <is>
-          <t>한국경제</t>
+          <t>한겨레</t>
         </is>
       </c>
       <c r="G89" s="3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTFAzR1c3Z3JwcXhPMTlOaHJtQzNmREJhdEpVOGtsZ0ZrTVI0RUVuRVV0aTVuREk4SS01d19keFBlWjhGV0VZb3lKeU84dHlQc1FiQ0RHa2lsOG9RUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMickFVX3lxTE15T3V6NzcweXpta2U4ckpqX05XU21wRlgxQ0ltZ1dlejY5ZGgzbzFvaFF5OTBSZlQwcGRBUW1YWXRQdWV0VWU5Wk44azVOVUFtSzljaXJ0WDVpOWhzWTk4MVZzNEFWQnJucl9ldElENVV0QQ?oc=5</t>
         </is>
       </c>
     </row>
@@ -3774,32 +3774,32 @@
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>거시경제/비즈니스</t>
+          <t>사회/사건사고</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>🔥 [언론사 집중 보도 (7개사)]</t>
+          <t>🔥 [언론사 집중 보도 (3개사)]</t>
         </is>
       </c>
       <c r="D90" s="3" t="inlineStr">
         <is>
-          <t>카카오 '모두의 AI' MAU 500만 목표…과업 완료율로 성과 평가</t>
+          <t>국가원로회의 부산지부, 15일 임시총회…지역 발전방안 논의</t>
         </is>
       </c>
       <c r="E90" s="3" t="inlineStr">
         <is>
-          <t>카카오 '모두의 AI' MAU 500만 목표…과업 완료율로 성과 평가 연합인포맥스 카카오, 웹툰·음원·카카오T에 스테이블코인 결제 연동…소설 원작 AI 애니 제작도 전자신문카톡에 “메시지 정리, 답장 보내줘” 말하면 AI비서가 척척 동아일보카카오 인적분할 앞두고 창사 첫 '그룹 공동 IR' 개최, 계열사 CEO 총출동 비즈니스포스트카카오, AI 시대 ‘신뢰·책임’ 검증 사례 나눈다.</t>
+          <t>각계 원로 인사 모임인 국가원로회의 부산지부는 15일 오전 10시 30분 부산 부산진구 초원농원 양정점에서 임...</t>
         </is>
       </c>
       <c r="F90" s="3" t="inlineStr">
         <is>
-          <t>연합인포맥스</t>
+          <t>주요언론</t>
         </is>
       </c>
       <c r="G90" s="3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE9FREp6R1lfYkJtTEhVUGZqRTdNbXBZbmNUYVpQWDN4c2M0OTZ0TV9OZzJmVW9CZFNITFdtWjNzY1RkTUpmLTYzMWgycEVFbjF6OWRpeGZFdWRjZkN0djBEeXlJVmJnZ1RSbkc4bEl5NDc?oc=5</t>
+          <t>https://www.yna.co.kr/view/AKR20261014122000051</t>
         </is>
       </c>
     </row>
@@ -3816,17 +3816,17 @@
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>🔥 [언론사 집중 보도 (3개사)]</t>
+          <t>연결 이슈 (후속)</t>
         </is>
       </c>
       <c r="D91" s="3" t="inlineStr">
         <is>
-          <t>모건스탠리 "한은, 10월 동결 후 11월 인상…물가 상승 압력"</t>
+          <t>제분업체 6곳, 사료 원료값 8년간 담합…과징금 최대 2100억원</t>
         </is>
       </c>
       <c r="E91" s="3" t="inlineStr">
         <is>
-          <t>모건스탠리는 한국은행이 오는 22일 금융통화위원회에서 기준금리를 연 3.0%로 동결한 후, 11월에 금리를 인...</t>
+          <t>관련매출액 1조4000억원 조사 시작되자 담합 중단 공정위, 임직원 고발 의견대한제분과 CJ제일제당 등 제분업체 6곳이 8년 넘게 사료 원료로 쓰이는 밀가루 부산물의 판매가격을 담..</t>
         </is>
       </c>
       <c r="F91" s="3" t="inlineStr">
@@ -3836,7 +3836,7 @@
       </c>
       <c r="G91" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261014111600008</t>
+          <t>https://www.mk.co.kr/news/economy/12175580</t>
         </is>
       </c>
     </row>
@@ -3848,7 +3848,7 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>세계/국제</t>
+          <t>IT/과학/신상품</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
@@ -3858,22 +3858,22 @@
       </c>
       <c r="D92" s="3" t="inlineStr">
         <is>
-          <t>[속보] 중국 “단둥~신의주 연결 신압록강대교 15일 개통”</t>
+          <t>PS6, PS2와 PS3 게임 지원 전망 나왔다</t>
         </is>
       </c>
       <c r="E92" s="3" t="inlineStr">
         <is>
-          <t>중국 “단둥~신의주 연결 신압록강대교 15일 개통” 한겨레中 신화통신 "북중 신압록강대교, 15일 공식 개통" MBC 뉴스“신압록강대교 내일 정식 개통…북·중, 개통식 합의” KBS 뉴스북·중 잇는 대교 왜 지금 열리나…북미 대화 앞두고 교류 확대? 마켓인완공부터 개통까지 12년···신압록강대교에 반영된 북·중관계 경향신문.</t>
+          <t>PS6, PS2와 PS3 게임 지원 전망 나왔다. 게임와이“어차피 사라질 운명” 사이버커넥트2 대표 디스크 폐지 찬성 게임메카새로운 보도에 따르면 소니는 플레이스테이션 6를 세 가지 구성으로 출시할 계획입니다.</t>
         </is>
       </c>
       <c r="F92" s="3" t="inlineStr">
         <is>
-          <t>한겨레</t>
+          <t>게임와이</t>
         </is>
       </c>
       <c r="G92" s="3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxNSFZBSFp3Q2xBbzYtb29jUHllSzRBdlp0NWtKZVRkcXE0eWd4NUNvMDNqYjBicno3Mk53ZU9YalpGXzhnMW1vS0VuVy1ocEtFOHAxc29OYm93LWljYkN3SzdySlNFYlFRN1lOYk5wZmR4elZDSVJfX2U4bmEwT3hOTW13?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiZ0FVX3lxTFBWN3pmQjJpeUtWZkg5dVBVTUNSYW9zUVV3OXdySkM5NnIzSk5oX0MxMUpsUm55UzdQX2lNaHFpdExPc1VGMHh5UV9SZk1YLUFJOXZ1SFVOOTVNSHpvdDZwTVBPZjg2NUHSAWpBVV95cUxPeGZzYXkzczlJbGRyWG9fSzl5YnhMWFdaT0EzNm5IU19tSGlvTGswSWJZREp3akxKWkxWTzNHR3pDVVBMUXNDenV2UjQ4ZmY1d2NnQkdvdV80UDA2SjcwdDg3TEVpOGtWYXlR?oc=5</t>
         </is>
       </c>
     </row>
@@ -3890,17 +3890,17 @@
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>신규 이슈</t>
+          <t>🔥 [언론사 집중 보도 (5개사)]</t>
         </is>
       </c>
       <c r="D93" s="3" t="inlineStr">
         <is>
-          <t>한미반도체, 반도체대전서 HBM4용 TC 본더 등 선봬</t>
+          <t>GC녹십자, LG CNS와 스마트공장 구축…AI 자동화 추진</t>
         </is>
       </c>
       <c r="E93" s="3" t="inlineStr">
         <is>
-          <t>한미반도체는 14일부터 16일까지 서울 강남구 코엑스에서 열리는 '제28회 반도체대전' 에...</t>
+          <t>GC녹십자가 LG CNS와 인공지능 기반 자동화·자율 운영 스마트 공장 구축을 추진한다.</t>
         </is>
       </c>
       <c r="F93" s="3" t="inlineStr">
@@ -3910,7 +3910,7 @@
       </c>
       <c r="G93" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261014115200003</t>
+          <t>https://www.yna.co.kr/view/AKR20261014121800017</t>
         </is>
       </c>
     </row>
@@ -3925,7 +3925,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S38"/>
+  <dimension ref="A1:S36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3938,7 +3938,7 @@
     <col width="25" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="36" customWidth="1" min="11" max="11"/>
+    <col width="39" customWidth="1" min="11" max="11"/>
     <col width="65" customWidth="1" min="12" max="12"/>
     <col width="34" customWidth="1" min="13" max="13"/>
     <col width="65" customWidth="1" min="14" max="14"/>
@@ -5252,17 +5252,17 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>237,000원</t>
+          <t>236,000원</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>+30,500.0원 (+14.77%)</t>
+          <t>+29,500.0원 (+14.29%)</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>234,500원</t>
+          <t>233,500원</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
@@ -5272,22 +5272,22 @@
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>228,500원</t>
+          <t>227,500원</t>
         </is>
       </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
-          <t>+9.5%</t>
+          <t>+10.0%</t>
         </is>
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>🟢 오늘 단기 매수 (저점 반등)</t>
+          <t>🟢 오늘 단기 매수 (저점 과매도 반등)</t>
         </is>
       </c>
       <c r="L15" s="3" t="inlineStr">
         <is>
-          <t>RSI 37.6로 단기 과매도 구간 진입, 기술적 반등 노림</t>
+          <t>RSI 37.0로 단기 과매도 구간 도달 및 지지선 부근 기술적 반등 기대 (거래량비율 0.66x)</t>
         </is>
       </c>
       <c r="M15" s="3" t="inlineStr">
@@ -5301,26 +5301,26 @@
         </is>
       </c>
       <c r="O15" s="3" t="n">
-        <v>37.6</v>
+        <v>37</v>
       </c>
       <c r="P15" s="3" t="inlineStr">
         <is>
-          <t>-9.6%</t>
+          <t>-10.0%</t>
         </is>
       </c>
       <c r="Q15" s="3" t="inlineStr">
         <is>
-          <t>51.3%</t>
+          <t>51.0%</t>
         </is>
       </c>
       <c r="R15" s="3" t="inlineStr">
         <is>
-          <t>한미반도체, 반도체대전서 HBM4용 TC 본더 등 선봬 (주요언론)</t>
+          <t>[하나증권] 삼성화재: 3Q26 Pre - 단기 실적보다 중요한 것은 (하나증권)</t>
         </is>
       </c>
       <c r="S15" s="3" t="inlineStr">
         <is>
-          <t>[259500.0, 249000.0, 248500.0, 253500.0, 252500.0, 261000.0, 274000.0, 276500.0, 285500.0, 270000.0, 272500.0, 268500.0, 276000.0, 276000.0, 272000.0, 268500.0, 262000.0, 250500.0, 232000.0, 237000.0]</t>
+          <t>[259500.0, 249000.0, 248500.0, 253500.0, 252500.0, 261000.0, 274000.0, 276500.0, 285500.0, 270000.0, 272500.0, 268500.0, 276000.0, 276000.0, 272000.0, 268500.0, 262000.0, 250500.0, 232000.0, 236000.0]</t>
         </is>
       </c>
     </row>
@@ -5347,42 +5347,42 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>1,449,000원</t>
+          <t>1,439,000원</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>+346,000.0원 (+31.37%)</t>
+          <t>+336,000.0원 (+30.46%)</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>1,434,500원</t>
+          <t>1,410,000원</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>1,704,500원</t>
+          <t>1,868,000원</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>1,398,500원</t>
+          <t>1,367,000원</t>
         </is>
       </c>
       <c r="J16" s="3" t="inlineStr">
         <is>
-          <t>+18.8%</t>
+          <t>+32.5%</t>
         </is>
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>🟢 오늘 단기 매수 (저점 반등)</t>
+          <t>관망 (HOLD)</t>
         </is>
       </c>
       <c r="L16" s="3" t="inlineStr">
         <is>
-          <t>RSI 31.9로 단기 과매도 구간 진입, 기술적 반등 노림</t>
+          <t>중립 구간 유지 중</t>
         </is>
       </c>
       <c r="M16" s="3" t="inlineStr">
@@ -5396,16 +5396,16 @@
         </is>
       </c>
       <c r="O16" s="3" t="n">
-        <v>31.9</v>
+        <v>31.2</v>
       </c>
       <c r="P16" s="3" t="inlineStr">
         <is>
-          <t>-16.7%</t>
+          <t>-17.2%</t>
         </is>
       </c>
       <c r="Q16" s="3" t="inlineStr">
         <is>
-          <t>40.4%</t>
+          <t>40.0%</t>
         </is>
       </c>
       <c r="R16" s="3" t="inlineStr">
@@ -5415,7 +5415,7 @@
       </c>
       <c r="S16" s="3" t="inlineStr">
         <is>
-          <t>[1812000.0, 1697000.0, 1690000.0, 1759000.0, 1745000.0, 1857000.0, 1868000.0, 1840000.0, 1862000.0, 1768000.0, 1765000.0, 1776000.0, 1833000.0, 1841000.0, 1773000.0, 1723000.0, 1681000.0, 1605000.0, 1443000.0, 1449000.0]</t>
+          <t>[1812000.0, 1697000.0, 1690000.0, 1759000.0, 1745000.0, 1857000.0, 1868000.0, 1840000.0, 1862000.0, 1768000.0, 1765000.0, 1776000.0, 1833000.0, 1841000.0, 1773000.0, 1723000.0, 1681000.0, 1605000.0, 1443000.0, 1439000.0]</t>
         </is>
       </c>
     </row>
@@ -5442,42 +5442,42 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>318,000원</t>
+          <t>316,000원</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>-173,750.0원 (-35.35%)</t>
+          <t>-175,500.0원 (-35.71%)</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>311,500원</t>
+          <t>299,000원</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>382,500원</t>
+          <t>313,000원</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>302,000원</t>
+          <t>306,500원</t>
         </is>
       </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
-          <t>+22.8%</t>
+          <t>+4.5%</t>
         </is>
       </c>
       <c r="K17" s="3" t="inlineStr">
         <is>
-          <t>⏸️ 관망/보유 (쿨다운 1일차)</t>
+          <t>🔴 단기 비중 축소 (추세 이탈 경고)</t>
         </is>
       </c>
       <c r="L17" s="3" t="inlineStr">
         <is>
-          <t>최근 1일 전(2026-10-13) 단기 매수 추천 이력 존재 ➔ 중복 매수 방지 쿨다운 적용(기존 포지션 분할 보유/관망 권고)</t>
+          <t>주가가 20일선(349,425원)을 하향 이탈하고 이동평균선 역배열 지속. 리스크 관리 차원 비중 축소 권고</t>
         </is>
       </c>
       <c r="M17" s="3" t="inlineStr">
@@ -5491,16 +5491,16 @@
         </is>
       </c>
       <c r="O17" s="3" t="n">
-        <v>24.5</v>
+        <v>22.9</v>
       </c>
       <c r="P17" s="3" t="inlineStr">
         <is>
-          <t>-9.1%</t>
+          <t>-9.6%</t>
         </is>
       </c>
       <c r="Q17" s="3" t="inlineStr">
         <is>
-          <t>17.4%</t>
+          <t>17.1%</t>
         </is>
       </c>
       <c r="R17" s="3" t="inlineStr">
@@ -5510,7 +5510,7 @@
       </c>
       <c r="S17" s="3" t="inlineStr">
         <is>
-          <t>[382500.0, 371500.0, 367000.0, 362000.0, 363000.0, 365000.0, 359000.0, 360500.0, 353500.0, 354500.0, 350000.0, 345000.0, 349000.0, 346500.0, 348000.0, 336000.0, 324500.0, 320000.0, 315000.0, 317750.0]</t>
+          <t>[382500.0, 371500.0, 367000.0, 362000.0, 363000.0, 365000.0, 359000.0, 360500.0, 353500.0, 354500.0, 350000.0, 345000.0, 349000.0, 346500.0, 348000.0, 336000.0, 324500.0, 320000.0, 315000.0, 316000.0]</t>
         </is>
       </c>
     </row>
@@ -5542,7 +5542,7 @@
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>-40,000.0원 (-26.81%)</t>
+          <t>-40,100.0원 (-26.88%)</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
@@ -5562,17 +5562,17 @@
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>+18.3%</t>
+          <t>+18.4%</t>
         </is>
       </c>
       <c r="K18" s="3" t="inlineStr">
         <is>
-          <t>⏸️ 관망/보유 (쿨다운 1일차)</t>
+          <t>관망 (HOLD)</t>
         </is>
       </c>
       <c r="L18" s="3" t="inlineStr">
         <is>
-          <t>최근 1일 전(2026-10-13) 단기 매수 추천 이력 존재 ➔ 중복 매수 방지 쿨다운 적용(기존 포지션 분할 보유/관망 권고)</t>
+          <t>중립 구간 유지 중</t>
         </is>
       </c>
       <c r="M18" s="3" t="inlineStr">
@@ -5586,7 +5586,7 @@
         </is>
       </c>
       <c r="O18" s="3" t="n">
-        <v>31.6</v>
+        <v>31.3</v>
       </c>
       <c r="P18" s="3" t="inlineStr">
         <is>
@@ -5595,7 +5595,7 @@
       </c>
       <c r="Q18" s="3" t="inlineStr">
         <is>
-          <t>6.7%</t>
+          <t>6.6%</t>
         </is>
       </c>
       <c r="R18" s="3" t="inlineStr">
@@ -5605,7 +5605,7 @@
       </c>
       <c r="S18" s="3" t="inlineStr">
         <is>
-          <t>[126600.0, 124200.0, 121800.0, 120700.0, 120900.0, 121900.0, 120000.0, 118500.0, 115400.0, 117600.0, 116000.0, 112800.0, 113300.0, 112900.0, 112600.0, 109600.0, 106800.0, 108100.0, 108300.0, 109200.0]</t>
+          <t>[126600.0, 124200.0, 121800.0, 120700.0, 120900.0, 121900.0, 120000.0, 118500.0, 115400.0, 117600.0, 116000.0, 112800.0, 113300.0, 112900.0, 112600.0, 109600.0, 106800.0, 108100.0, 108300.0, 109100.0]</t>
         </is>
       </c>
     </row>
@@ -5632,42 +5632,42 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>181,500원</t>
+          <t>181,000원</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>-20,100.0원 (-9.98%)</t>
+          <t>-20,600.0원 (-10.22%)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>178,000원</t>
+          <t>169,000원</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>206,500원</t>
+          <t>179,000원</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>172,500원</t>
+          <t>175,500원</t>
         </is>
       </c>
       <c r="J19" s="3" t="inlineStr">
         <is>
-          <t>+16.2%</t>
+          <t>+5.9%</t>
         </is>
       </c>
       <c r="K19" s="3" t="inlineStr">
         <is>
-          <t>⏸️ 관망/보유 (쿨다운 1일차)</t>
+          <t>🔴 단기 비중 축소 (추세 이탈 경고)</t>
         </is>
       </c>
       <c r="L19" s="3" t="inlineStr">
         <is>
-          <t>최근 1일 전(2026-10-13) 단기 매수 추천 이력 존재 ➔ 중복 매수 방지 쿨다운 적용(기존 포지션 분할 보유/관망 권고)</t>
+          <t>주가가 20일선(194,060원)을 하향 이탈하고 이동평균선 역배열 지속. 리스크 관리 차원 비중 축소 권고</t>
         </is>
       </c>
       <c r="M19" s="3" t="inlineStr">
@@ -5681,16 +5681,16 @@
         </is>
       </c>
       <c r="O19" s="3" t="n">
-        <v>32.3</v>
+        <v>31.5</v>
       </c>
       <c r="P19" s="3" t="inlineStr">
         <is>
-          <t>-6.5%</t>
+          <t>-6.8%</t>
         </is>
       </c>
       <c r="Q19" s="3" t="inlineStr">
         <is>
-          <t>6.3%</t>
+          <t>5.9%</t>
         </is>
       </c>
       <c r="R19" s="3" t="inlineStr">
@@ -5700,7 +5700,7 @@
       </c>
       <c r="S19" s="3" t="inlineStr">
         <is>
-          <t>[206500.0, 204000.0, 206000.0, 201500.0, 199000.0, 197700.0, 197900.0, 201000.0, 194700.0, 197700.0, 194800.0, 193700.0, 191200.0, 192200.0, 191100.0, 189000.0, 183800.0, 180500.0, 178000.0, 181400.0]</t>
+          <t>[206500.0, 204000.0, 206000.0, 201500.0, 199000.0, 197700.0, 197900.0, 201000.0, 194700.0, 197700.0, 194800.0, 193700.0, 191200.0, 192200.0, 191100.0, 189000.0, 183800.0, 180500.0, 178000.0, 180900.0]</t>
         </is>
       </c>
     </row>
@@ -5732,12 +5732,12 @@
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>-16,100.0원 (-33.47%)</t>
+          <t>-16,150.0원 (-33.58%)</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>31,400원</t>
+          <t>31,300원</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
@@ -5752,17 +5752,17 @@
       </c>
       <c r="J20" s="3" t="inlineStr">
         <is>
-          <t>+10.5%</t>
+          <t>+10.7%</t>
         </is>
       </c>
       <c r="K20" s="3" t="inlineStr">
         <is>
-          <t>⏸️ 관망/보유 (쿨다운 1일차)</t>
+          <t>관망 (HOLD)</t>
         </is>
       </c>
       <c r="L20" s="3" t="inlineStr">
         <is>
-          <t>최근 1일 전(2026-10-13) 단기 매수 추천 이력 존재 ➔ 중복 매수 방지 쿨다운 적용(기존 포지션 분할 보유/관망 권고)</t>
+          <t>중립 구간 유지 중</t>
         </is>
       </c>
       <c r="M20" s="3" t="inlineStr">
@@ -5776,26 +5776,26 @@
         </is>
       </c>
       <c r="O20" s="3" t="n">
-        <v>35.4</v>
+        <v>34.9</v>
       </c>
       <c r="P20" s="3" t="inlineStr">
         <is>
-          <t>-4.1%</t>
+          <t>-4.3%</t>
         </is>
       </c>
       <c r="Q20" s="3" t="inlineStr">
         <is>
-          <t>4.4%</t>
+          <t>4.3%</t>
         </is>
       </c>
       <c r="R20" s="3" t="inlineStr">
         <is>
-          <t>카카오 '모두의 AI' MAU 500만 목표…과업 완료율로 성과 평가 (연합인포맥스)</t>
+          <t>최근 특이 뉴스 없음</t>
         </is>
       </c>
       <c r="S20" s="3" t="inlineStr">
         <is>
-          <t>[34500.0, 34650.0, 34500.0, 33500.0, 33500.0, 33550.0, 33200.0, 34150.0, 33450.0, 34150.0, 33700.0, 33550.0, 33550.0, 33450.0, 33500.0, 33050.0, 32300.0, 32000.0, 31300.0, 32000.0]</t>
+          <t>[34500.0, 34650.0, 34500.0, 33500.0, 33500.0, 33550.0, 33200.0, 34150.0, 33450.0, 34150.0, 33700.0, 33550.0, 33550.0, 33450.0, 33500.0, 33050.0, 32300.0, 32000.0, 31300.0, 31950.0]</t>
         </is>
       </c>
     </row>
@@ -5822,32 +5822,32 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>181,500원</t>
+          <t>181,000원</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>-8,219.049999999988원 (-4.33%)</t>
+          <t>-8,819.049999999988원 (-4.65%)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>181,500원</t>
+          <t>177,000원</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>190,500원</t>
+          <t>190,000원</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>174,000원</t>
+          <t>172,000원</t>
         </is>
       </c>
       <c r="J21" s="3" t="inlineStr">
         <is>
-          <t>+5.0%</t>
+          <t>+7.1%</t>
         </is>
       </c>
       <c r="K21" s="3" t="inlineStr">
@@ -5871,16 +5871,16 @@
         </is>
       </c>
       <c r="O21" s="3" t="n">
-        <v>48.7</v>
+        <v>47.5</v>
       </c>
       <c r="P21" s="3" t="inlineStr">
         <is>
-          <t>+0.9%</t>
+          <t>+0.6%</t>
         </is>
       </c>
       <c r="Q21" s="3" t="inlineStr">
         <is>
-          <t>28.4%</t>
+          <t>27.7%</t>
         </is>
       </c>
       <c r="R21" s="3" t="inlineStr">
@@ -5890,7 +5890,7 @@
       </c>
       <c r="S21" s="3" t="inlineStr">
         <is>
-          <t>[178200.0, 178800.0, 177500.0, 177200.0, 180300.0, 179400.0, 181400.0, 178500.0, 177400.0, 178300.0, 178900.0, 177700.0, 183600.0, 182600.0, 182400.0, 183500.0, 179600.0, 180400.0, 179700.0, 181400.0]</t>
+          <t>[178200.0, 178800.0, 177500.0, 177200.0, 180300.0, 179400.0, 181400.0, 178500.0, 177400.0, 178300.0, 178900.0, 177700.0, 183600.0, 182600.0, 182400.0, 183500.0, 179600.0, 180400.0, 179700.0, 180800.0]</t>
         </is>
       </c>
     </row>
@@ -5917,42 +5917,42 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>845,000원</t>
+          <t>839,000원</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>-678,000.0원 (-44.52%)</t>
+          <t>-684,000.0원 (-44.91%)</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>828,000원</t>
+          <t>797,000원</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>1,137,000원</t>
+          <t>830,500원</t>
         </is>
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>803,000원</t>
+          <t>814,000원</t>
         </is>
       </c>
       <c r="J22" s="3" t="inlineStr">
         <is>
-          <t>+37.3%</t>
+          <t>+4.2%</t>
         </is>
       </c>
       <c r="K22" s="3" t="inlineStr">
         <is>
-          <t>⏸️ 관망/보유 (쿨다운 1일차)</t>
+          <t>🔴 단기 비중 축소 (추세 이탈 경고)</t>
         </is>
       </c>
       <c r="L22" s="3" t="inlineStr">
         <is>
-          <t>최근 1일 전(2026-10-13) 단기 매수 추천 이력 존재 ➔ 중복 매수 방지 쿨다운 적용(기존 포지션 분할 보유/관망 권고)</t>
+          <t>주가가 20일선(1,012,050원)을 하향 이탈하고 이동평균선 역배열 지속. 리스크 관리 차원 비중 축소 권고</t>
         </is>
       </c>
       <c r="M22" s="3" t="inlineStr">
@@ -5966,16 +5966,16 @@
         </is>
       </c>
       <c r="O22" s="3" t="n">
-        <v>30.6</v>
+        <v>29.6</v>
       </c>
       <c r="P22" s="3" t="inlineStr">
         <is>
-          <t>-16.5%</t>
+          <t>-17.1%</t>
         </is>
       </c>
       <c r="Q22" s="3" t="inlineStr">
         <is>
-          <t>7.1%</t>
+          <t>6.4%</t>
         </is>
       </c>
       <c r="R22" s="3" t="inlineStr">
@@ -5985,7 +5985,7 @@
       </c>
       <c r="S22" s="3" t="inlineStr">
         <is>
-          <t>[1081000.0, 1137000.0, 1063000.0, 1055000.0, 1097000.0, 1078000.0, 1067000.0, 1057000.0, 1021000.0, 1034000.0, 1012000.0, 1007000.0, 1034000.0, 1072000.0, 1023000.0, 972000.0, 891000.0, 862000.0, 839000.0, 845000.0]</t>
+          <t>[1081000.0, 1137000.0, 1063000.0, 1055000.0, 1097000.0, 1078000.0, 1067000.0, 1057000.0, 1021000.0, 1034000.0, 1012000.0, 1007000.0, 1034000.0, 1072000.0, 1023000.0, 972000.0, 891000.0, 862000.0, 839000.0, 839000.0]</t>
         </is>
       </c>
     </row>
@@ -6012,12 +6012,12 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>425,500원</t>
+          <t>426,500원</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>+25,500.0원 (+6.38%)</t>
+          <t>+26,500.0원 (+6.62%)</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -6027,17 +6027,17 @@
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>425,500원</t>
+          <t>426,500원</t>
         </is>
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>417,000원</t>
+          <t>418,000원</t>
         </is>
       </c>
       <c r="J23" s="3" t="inlineStr">
         <is>
-          <t>+14.3%</t>
+          <t>+14.5%</t>
         </is>
       </c>
       <c r="K23" s="3" t="inlineStr">
@@ -6047,7 +6047,7 @@
       </c>
       <c r="L23" s="3" t="inlineStr">
         <is>
-          <t>RSI 71.8, 20일선 이격도 +14.3%로 단기 과열권, 분할 차익 실현 권고</t>
+          <t>RSI 72.0, 20일선 이격도 +14.5%로 단기 과열권 진입. 욕심을 줄이고 분할 차익 실현 권고</t>
         </is>
       </c>
       <c r="M23" s="3" t="inlineStr">
@@ -6061,16 +6061,16 @@
         </is>
       </c>
       <c r="O23" s="3" t="n">
-        <v>71.8</v>
+        <v>72</v>
       </c>
       <c r="P23" s="3" t="inlineStr">
         <is>
-          <t>+14.3%</t>
+          <t>+14.5%</t>
         </is>
       </c>
       <c r="Q23" s="3" t="inlineStr">
         <is>
-          <t>57.1%</t>
+          <t>57.5%</t>
         </is>
       </c>
       <c r="R23" s="3" t="inlineStr">
@@ -6080,7 +6080,7 @@
       </c>
       <c r="S23" s="3" t="inlineStr">
         <is>
-          <t>[360000.0, 351500.0, 365500.0, 367000.0, 365000.0, 364000.0, 352000.0, 350500.0, 351500.0, 364000.0, 352500.0, 357000.0, 360500.0, 371000.0, 390000.0, 391000.0, 401000.0, 398000.0, 410000.0, 425500.0]</t>
+          <t>[360000.0, 351500.0, 365500.0, 367000.0, 365000.0, 364000.0, 352000.0, 350500.0, 351500.0, 364000.0, 352500.0, 357000.0, 360500.0, 371000.0, 390000.0, 391000.0, 401000.0, 398000.0, 410000.0, 426500.0]</t>
         </is>
       </c>
     </row>
@@ -6117,22 +6117,22 @@
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>309,500원</t>
+          <t>303,500원</t>
         </is>
       </c>
       <c r="H24" s="3" t="inlineStr">
         <is>
-          <t>325,000원</t>
+          <t>334,000원</t>
         </is>
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>297,000원</t>
+          <t>294,000원</t>
         </is>
       </c>
       <c r="J24" s="3" t="inlineStr">
         <is>
-          <t>+5.0%</t>
+          <t>+10.1%</t>
         </is>
       </c>
       <c r="K24" s="3" t="inlineStr">
@@ -6202,7 +6202,7 @@
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>$228.52 (약 306,417원)</t>
+          <t>$228.52 (약 305,755원)</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
@@ -6212,22 +6212,22 @@
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>$228.52 (약 306,417원)</t>
+          <t>$223.95 (약 299,640원)</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
-          <t>$239.95 (약 321,738원)</t>
+          <t>$239.95 (약 321,042원)</t>
         </is>
       </c>
       <c r="I25" s="3" t="inlineStr">
         <is>
-          <t>$219.38</t>
+          <t>$217.09</t>
         </is>
       </c>
       <c r="J25" s="3" t="inlineStr">
         <is>
-          <t>+5.0%</t>
+          <t>+7.1%</t>
         </is>
       </c>
       <c r="K25" s="3" t="inlineStr">
@@ -6297,7 +6297,7 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>$341.27 (약 457,602원)</t>
+          <t>$341.27 (약 456,612원)</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
@@ -6307,22 +6307,22 @@
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>$341.27 (약 457,602원)</t>
+          <t>$334.44 (약 447,480원)</t>
         </is>
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
-          <t>$358.33 (약 480,482원)</t>
+          <t>$358.33 (약 479,443원)</t>
         </is>
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>$327.62</t>
+          <t>$324.21</t>
         </is>
       </c>
       <c r="J26" s="3" t="inlineStr">
         <is>
-          <t>+5.0%</t>
+          <t>+7.1%</t>
         </is>
       </c>
       <c r="K26" s="3" t="inlineStr">
@@ -6392,7 +6392,7 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>$375.23 (약 503,138원)</t>
+          <t>$375.23 (약 502,050원)</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
@@ -6402,22 +6402,22 @@
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>$375.23 (약 503,138원)</t>
+          <t>$367.73 (약 492,009원)</t>
         </is>
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>$393.99 (약 528,295원)</t>
+          <t>$393.99 (약 527,152원)</t>
         </is>
       </c>
       <c r="I27" s="3" t="inlineStr">
         <is>
-          <t>$360.22</t>
+          <t>$356.47</t>
         </is>
       </c>
       <c r="J27" s="3" t="inlineStr">
         <is>
-          <t>+5.0%</t>
+          <t>+7.1%</t>
         </is>
       </c>
       <c r="K27" s="3" t="inlineStr">
@@ -6487,7 +6487,7 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>$543.45 (약 728,701원)</t>
+          <t>$543.45 (약 727,125원)</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
@@ -6497,12 +6497,12 @@
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>$514.20 (약 689,480원)</t>
+          <t>$514.20 (약 687,989원)</t>
         </is>
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
-          <t>$543.45 (약 728,701원)</t>
+          <t>$543.45 (약 727,125원)</t>
         </is>
       </c>
       <c r="I28" s="3" t="inlineStr">
@@ -6522,7 +6522,7 @@
       </c>
       <c r="L28" s="3" t="inlineStr">
         <is>
-          <t>RSI 70.7, 20일선 이격도 +5.7%로 단기 과열권, 분할 차익 실현 권고</t>
+          <t>RSI 70.7, 20일선 이격도 +5.7%로 단기 과열권 진입. 욕심을 줄이고 분할 차익 실현 권고</t>
         </is>
       </c>
       <c r="M28" s="3" t="inlineStr">
@@ -6567,12 +6567,12 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>팬오션</t>
+          <t>한미약품</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>028670.KS</t>
+          <t>128940.KS</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
@@ -6582,42 +6582,42 @@
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>7,160원</t>
+          <t>408,000원</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>+1,870.0원 (+35.35%)</t>
+          <t>-93,000.0원 (-18.56%)</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>6,000원</t>
+          <t>404,000원</t>
         </is>
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t>7,160원</t>
+          <t>483,500원</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>7,020원</t>
+          <t>393,500원</t>
         </is>
       </c>
       <c r="J29" s="3" t="inlineStr">
         <is>
-          <t>+19.3%</t>
+          <t>+19.7%</t>
         </is>
       </c>
       <c r="K29" s="3" t="inlineStr">
         <is>
-          <t>🔴 오늘 단기 매도 (과열 차익실현)</t>
+          <t>🟢 오늘 단기 매수 (저점 과매도 반등)</t>
         </is>
       </c>
       <c r="L29" s="3" t="inlineStr">
         <is>
-          <t>RSI 72.1, 20일선 이격도 +19.3%로 단기 과열권, 분할 차익 실현 권고</t>
+          <t>RSI 33.6로 단기 과매도 구간 도달 및 지지선 부근 기술적 반등 기대 (거래량비율 1.63x)</t>
         </is>
       </c>
       <c r="M29" s="3" t="inlineStr">
@@ -6631,16 +6631,16 @@
         </is>
       </c>
       <c r="O29" s="3" t="n">
-        <v>72.09999999999999</v>
+        <v>33.6</v>
       </c>
       <c r="P29" s="3" t="inlineStr">
         <is>
-          <t>+19.3%</t>
+          <t>-17.3%</t>
         </is>
       </c>
       <c r="Q29" s="3" t="inlineStr">
         <is>
-          <t>94.4%</t>
+          <t>30.7%</t>
         </is>
       </c>
       <c r="R29" s="3" t="inlineStr">
@@ -6650,7 +6650,7 @@
       </c>
       <c r="S29" s="3" t="inlineStr">
         <is>
-          <t>[6030.0, 6040.0, 5680.0, 5800.0, 5880.0, 5750.0, 5790.0, 5790.0, 5600.0, 5700.0, 5700.0, 5770.0, 5880.0, 6240.0, 6000.0, 6210.0, 6030.0, 6450.0, 6550.0, 7160.0]</t>
+          <t>[464000.0, 474000.0, 496500.0, 502000.0, 515000.0, 503000.0, 505000.0, 502000.0, 520000.0, 504000.0, 507000.0, 499000.0, 497500.0, 506000.0, 523000.0, 534000.0, 480500.0, 474500.0, 453000.0, 408000.0]</t>
         </is>
       </c>
     </row>
@@ -6662,12 +6662,12 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>한미약품</t>
+          <t>KT</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>128940.KS</t>
+          <t>030200.KS</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
@@ -6677,42 +6677,42 @@
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>415,000원</t>
+          <t>49,800원</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>-86,000.0원 (-17.17%)</t>
+          <t>-14,400.0원 (-22.43%)</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>411,000원</t>
+          <t>49,300원</t>
         </is>
       </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
-          <t>484,000원</t>
+          <t>52,800원</t>
         </is>
       </c>
       <c r="I30" s="3" t="inlineStr">
         <is>
-          <t>400,500원</t>
+          <t>48,100원</t>
         </is>
       </c>
       <c r="J30" s="3" t="inlineStr">
         <is>
-          <t>+17.8%</t>
+          <t>+7.1%</t>
         </is>
       </c>
       <c r="K30" s="3" t="inlineStr">
         <is>
-          <t>🟢 오늘 단기 매수 (저점 반등)</t>
+          <t>🟢 오늘 단기 매수 (저점 과매도 반등)</t>
         </is>
       </c>
       <c r="L30" s="3" t="inlineStr">
         <is>
-          <t>RSI 34.6로 단기 과매도 구간 진입, 기술적 반등 노림</t>
+          <t>RSI 32.1로 단기 과매도 구간 도달 및 지지선 부근 기술적 반등 기대 (거래량비율 0.53x)</t>
         </is>
       </c>
       <c r="M30" s="3" t="inlineStr">
@@ -6726,16 +6726,16 @@
         </is>
       </c>
       <c r="O30" s="3" t="n">
-        <v>34.6</v>
+        <v>32.1</v>
       </c>
       <c r="P30" s="3" t="inlineStr">
         <is>
-          <t>-15.9%</t>
+          <t>-4.5%</t>
         </is>
       </c>
       <c r="Q30" s="3" t="inlineStr">
         <is>
-          <t>32.8%</t>
+          <t>8.0%</t>
         </is>
       </c>
       <c r="R30" s="3" t="inlineStr">
@@ -6745,7 +6745,7 @@
       </c>
       <c r="S30" s="3" t="inlineStr">
         <is>
-          <t>[464000.0, 474000.0, 496500.0, 502000.0, 515000.0, 503000.0, 505000.0, 502000.0, 520000.0, 504000.0, 507000.0, 499000.0, 497500.0, 506000.0, 523000.0, 534000.0, 480500.0, 474500.0, 453000.0, 415000.0]</t>
+          <t>[52700.0, 53200.0, 53000.0, 52800.0, 53400.0, 53000.0, 53100.0, 53100.0, 52700.0, 52900.0, 52900.0, 52300.0, 51800.0, 51900.0, 51500.0, 51300.0, 52100.0, 49900.0, 49750.0, 49800.0]</t>
         </is>
       </c>
     </row>
@@ -6757,12 +6757,12 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>HMM</t>
+          <t>LG유플러스</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>011200.KS</t>
+          <t>032640.KS</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
@@ -6772,42 +6772,42 @@
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>23,400원</t>
+          <t>14,700원</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>+2,400.0원 (+11.43%)</t>
+          <t>-2,770.0원 (-15.86%)</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>21,200원</t>
+          <t>14,400원</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>23,400원</t>
+          <t>15,400원</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
         <is>
-          <t>22,900원</t>
+          <t>14,000원</t>
         </is>
       </c>
       <c r="J31" s="3" t="inlineStr">
         <is>
-          <t>+10.3%</t>
+          <t>+7.1%</t>
         </is>
       </c>
       <c r="K31" s="3" t="inlineStr">
         <is>
-          <t>🔴 오늘 단기 매도 (과열 차익실현)</t>
+          <t>관망 (HOLD)</t>
         </is>
       </c>
       <c r="L31" s="3" t="inlineStr">
         <is>
-          <t>RSI 68.4, 20일선 이격도 +10.3%로 단기 과열권, 분할 차익 실현 권고</t>
+          <t>중립 구간 유지 중</t>
         </is>
       </c>
       <c r="M31" s="3" t="inlineStr">
@@ -6821,16 +6821,16 @@
         </is>
       </c>
       <c r="O31" s="3" t="n">
-        <v>68.40000000000001</v>
+        <v>50.7</v>
       </c>
       <c r="P31" s="3" t="inlineStr">
         <is>
-          <t>+10.3%</t>
+          <t>+0.5%</t>
         </is>
       </c>
       <c r="Q31" s="3" t="inlineStr">
         <is>
-          <t>78.0%</t>
+          <t>17.8%</t>
         </is>
       </c>
       <c r="R31" s="3" t="inlineStr">
@@ -6840,7 +6840,7 @@
       </c>
       <c r="S31" s="3" t="inlineStr">
         <is>
-          <t>[20850.0, 21250.0, 20650.0, 20350.0, 20750.0, 20800.0, 21100.0, 21200.0, 20800.0, 21250.0, 21000.0, 20850.0, 21150.0, 21500.0, 21450.0, 21400.0, 20800.0, 21800.0, 22050.0, 23400.0]</t>
+          <t>[14890.0, 15040.0, 14850.0, 14650.0, 14680.0, 14050.0, 14490.0, 14570.0, 14640.0, 14770.0, 14800.0, 14530.0, 14540.0, 14550.0, 14560.0, 14500.0, 14400.0, 14550.0, 14780.0, 14700.0]</t>
         </is>
       </c>
     </row>
@@ -6852,12 +6852,12 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>일진전기</t>
+          <t>SK텔레콤</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>103590.KS</t>
+          <t>017670.KS</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -6867,42 +6867,42 @@
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>77,000원</t>
+          <t>82,200원</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>-7,300.0원 (-8.66%)</t>
+          <t>-13,300.0원 (-13.93%)</t>
         </is>
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>77,000원</t>
+          <t>81,400원</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr">
         <is>
-          <t>80,800원</t>
+          <t>87,100원</t>
         </is>
       </c>
       <c r="I32" s="3" t="inlineStr">
         <is>
-          <t>73,900원</t>
+          <t>79,300원</t>
         </is>
       </c>
       <c r="J32" s="3" t="inlineStr">
         <is>
-          <t>+5.0%</t>
+          <t>+7.1%</t>
         </is>
       </c>
       <c r="K32" s="3" t="inlineStr">
         <is>
-          <t>관망 (HOLD)</t>
+          <t>🟢 오늘 단기 매수 (저점 과매도 반등)</t>
         </is>
       </c>
       <c r="L32" s="3" t="inlineStr">
         <is>
-          <t>중립 구간 유지 중</t>
+          <t>RSI 38.1로 단기 과매도 구간 도달 및 지지선 부근 기술적 반등 기대 (거래량비율 0.79x)</t>
         </is>
       </c>
       <c r="M32" s="3" t="inlineStr">
@@ -6916,16 +6916,16 @@
         </is>
       </c>
       <c r="O32" s="3" t="n">
-        <v>50.7</v>
+        <v>38.1</v>
       </c>
       <c r="P32" s="3" t="inlineStr">
         <is>
-          <t>-0.9%</t>
+          <t>-5.1%</t>
         </is>
       </c>
       <c r="Q32" s="3" t="inlineStr">
         <is>
-          <t>34.4%</t>
+          <t>35.0%</t>
         </is>
       </c>
       <c r="R32" s="3" t="inlineStr">
@@ -6935,7 +6935,7 @@
       </c>
       <c r="S32" s="3" t="inlineStr">
         <is>
-          <t>[71000.0, 69700.0, 68400.0, 70400.0, 70200.0, 76600.0, 73000.0, 76500.0, 81700.0, 82100.0, 80900.0, 82500.0, 82900.0, 86200.0, 87900.0, 88000.0, 81400.0, 73800.0, 73400.0, 77000.0]</t>
+          <t>[90900.0, 90100.0, 88000.0, 88100.0, 87600.0, 89200.0, 87000.0, 87300.0, 87100.0, 88200.0, 86200.0, 85600.0, 86300.0, 88400.0, 88400.0, 87400.0, 84100.0, 79700.0, 80000.0, 82200.0]</t>
         </is>
       </c>
     </row>
@@ -6947,12 +6947,12 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>현대글로비스</t>
+          <t>일진전기</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>086280.KS</t>
+          <t>103590.KS</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -6962,42 +6962,42 @@
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>185,500원</t>
+          <t>76,000원</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>-33,900.0원 (-15.44%)</t>
+          <t>-8,300.0원 (-9.85%)</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>183,500원</t>
+          <t>74,500원</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>196,500원</t>
+          <t>88,000원</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
         <is>
-          <t>179,000원</t>
+          <t>72,200원</t>
         </is>
       </c>
       <c r="J33" s="3" t="inlineStr">
         <is>
-          <t>+7.1%</t>
+          <t>+18.2%</t>
         </is>
       </c>
       <c r="K33" s="3" t="inlineStr">
         <is>
-          <t>🟢 오늘 단기 매수 (저점 반등)</t>
+          <t>관망 (HOLD)</t>
         </is>
       </c>
       <c r="L33" s="3" t="inlineStr">
         <is>
-          <t>RSI 38.6로 단기 과매도 구간 진입, 기술적 반등 노림</t>
+          <t>중립 구간 유지 중</t>
         </is>
       </c>
       <c r="M33" s="3" t="inlineStr">
@@ -7011,16 +7011,16 @@
         </is>
       </c>
       <c r="O33" s="3" t="n">
-        <v>38.6</v>
+        <v>49.4</v>
       </c>
       <c r="P33" s="3" t="inlineStr">
         <is>
-          <t>-5.9%</t>
+          <t>-2.1%</t>
         </is>
       </c>
       <c r="Q33" s="3" t="inlineStr">
         <is>
-          <t>21.1%</t>
+          <t>33.4%</t>
         </is>
       </c>
       <c r="R33" s="3" t="inlineStr">
@@ -7030,7 +7030,7 @@
       </c>
       <c r="S33" s="3" t="inlineStr">
         <is>
-          <t>[208500.0, 207000.0, 204500.0, 200500.0, 206000.0, 203500.0, 203000.0, 203000.0, 196900.0, 199100.0, 197500.0, 196800.0, 198400.0, 201500.0, 201000.0, 188000.0, 182900.0, 181900.0, 180600.0, 185600.0]</t>
+          <t>[71000.0, 69700.0, 68400.0, 70400.0, 70200.0, 76600.0, 73000.0, 76500.0, 81700.0, 82100.0, 80900.0, 82500.0, 82900.0, 86200.0, 87900.0, 88000.0, 81400.0, 73800.0, 73400.0, 76000.0]</t>
         </is>
       </c>
     </row>
@@ -7042,12 +7042,12 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>삼성화재</t>
+          <t>삼성중공업</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>000810.KS</t>
+          <t>010140.KS</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
@@ -7057,42 +7057,42 @@
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>581,000원</t>
+          <t>19,200원</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>+91,500.0원 (+18.69%)</t>
+          <t>-8,750.0원 (-31.36%)</t>
         </is>
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>575,000원</t>
+          <t>18,800원</t>
         </is>
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>629,000원</t>
+          <t>22,100원</t>
         </is>
       </c>
       <c r="I34" s="3" t="inlineStr">
         <is>
-          <t>560,500원</t>
+          <t>18,200원</t>
         </is>
       </c>
       <c r="J34" s="3" t="inlineStr">
         <is>
-          <t>+9.4%</t>
+          <t>+17.8%</t>
         </is>
       </c>
       <c r="K34" s="3" t="inlineStr">
         <is>
-          <t>🟢 오늘 단기 매수 (저점 반등)</t>
+          <t>관망 (HOLD)</t>
         </is>
       </c>
       <c r="L34" s="3" t="inlineStr">
         <is>
-          <t>RSI 33.5로 단기 과매도 구간 진입, 기술적 반등 노림</t>
+          <t>중립 구간 유지 중</t>
         </is>
       </c>
       <c r="M34" s="3" t="inlineStr">
@@ -7106,16 +7106,16 @@
         </is>
       </c>
       <c r="O34" s="3" t="n">
-        <v>33.5</v>
+        <v>42.7</v>
       </c>
       <c r="P34" s="3" t="inlineStr">
         <is>
-          <t>-9.5%</t>
+          <t>-4.4%</t>
         </is>
       </c>
       <c r="Q34" s="3" t="inlineStr">
         <is>
-          <t>47.9%</t>
+          <t>10.7%</t>
         </is>
       </c>
       <c r="R34" s="3" t="inlineStr">
@@ -7125,7 +7125,7 @@
       </c>
       <c r="S34" s="3" t="inlineStr">
         <is>
-          <t>[686000.0, 675000.0, 661000.0, 661000.0, 666000.0, 648000.0, 651000.0, 655000.0, 648000.0, 661000.0, 653000.0, 633000.0, 626000.0, 626000.0, 635000.0, 629000.0, 612000.0, 622000.0, 612000.0, 581000.0]</t>
+          <t>[21400.0, 22100.0, 20700.0, 20200.0, 21500.0, 20800.0, 20600.0, 20600.0, 20250.0, 20100.0, 19330.0, 19700.0, 19720.0, 19960.0, 19700.0, 19540.0, 18860.0, 18010.0, 18360.0, 19150.0]</t>
         </is>
       </c>
     </row>
@@ -7137,12 +7137,12 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>세아베스틸지주</t>
+          <t>삼성화재</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>001430.KS</t>
+          <t>000810.KS</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
@@ -7152,42 +7152,42 @@
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>43,600원</t>
+          <t>584,000원</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>-24,000.0원 (-35.50%)</t>
+          <t>+94,500.0원 (+19.31%)</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>43,600원</t>
+          <t>578,000원</t>
         </is>
       </c>
       <c r="H35" s="3" t="inlineStr">
         <is>
-          <t>45,800원</t>
+          <t>629,500원</t>
         </is>
       </c>
       <c r="I35" s="3" t="inlineStr">
         <is>
-          <t>41,900원</t>
+          <t>563,500원</t>
         </is>
       </c>
       <c r="J35" s="3" t="inlineStr">
         <is>
-          <t>+5.0%</t>
+          <t>+8.9%</t>
         </is>
       </c>
       <c r="K35" s="3" t="inlineStr">
         <is>
-          <t>관망 (HOLD)</t>
+          <t>🟢 오늘 단기 매수 (저점 과매도 반등)</t>
         </is>
       </c>
       <c r="L35" s="3" t="inlineStr">
         <is>
-          <t>중립 구간 유지 중</t>
+          <t>RSI 34.1로 단기 과매도 구간 도달 및 지지선 부근 기술적 반등 기대 (거래량비율 0.85x)</t>
         </is>
       </c>
       <c r="M35" s="3" t="inlineStr">
@@ -7201,16 +7201,16 @@
         </is>
       </c>
       <c r="O35" s="3" t="n">
-        <v>49.2</v>
+        <v>34.1</v>
       </c>
       <c r="P35" s="3" t="inlineStr">
         <is>
-          <t>-2.1%</t>
+          <t>-9.1%</t>
         </is>
       </c>
       <c r="Q35" s="3" t="inlineStr">
         <is>
-          <t>27.7%</t>
+          <t>48.8%</t>
         </is>
       </c>
       <c r="R35" s="3" t="inlineStr">
@@ -7220,7 +7220,7 @@
       </c>
       <c r="S35" s="3" t="inlineStr">
         <is>
-          <t>[41450.0, 40950.0, 43250.0, 43250.0, 45450.0, 45050.0, 43800.0, 45600.0, 44300.0, 44600.0, 45300.0, 44950.0, 47000.0, 46650.0, 47250.0, 44150.0, 46800.0, 44500.0, 43150.0, 43600.0]</t>
+          <t>[686000.0, 675000.0, 661000.0, 661000.0, 666000.0, 648000.0, 651000.0, 655000.0, 648000.0, 661000.0, 653000.0, 633000.0, 626000.0, 626000.0, 635000.0, 629000.0, 612000.0, 622000.0, 612000.0, 584000.0]</t>
         </is>
       </c>
     </row>
@@ -7232,12 +7232,12 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>한화손해보험</t>
+          <t>휴젤</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>000370.KS</t>
+          <t>145020.KS</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
@@ -7247,42 +7247,42 @@
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>6,440원</t>
+          <t>223,500원</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>-170.0원 (-2.57%)</t>
+          <t>-29,500.0원 (-11.66%)</t>
         </is>
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>6,380원</t>
+          <t>200,000원</t>
         </is>
       </c>
       <c r="H36" s="3" t="inlineStr">
         <is>
-          <t>7,510원</t>
+          <t>223,500원</t>
         </is>
       </c>
       <c r="I36" s="3" t="inlineStr">
         <is>
-          <t>6,210원</t>
+          <t>219,000원</t>
         </is>
       </c>
       <c r="J36" s="3" t="inlineStr">
         <is>
-          <t>+17.8%</t>
+          <t>+11.7%</t>
         </is>
       </c>
       <c r="K36" s="3" t="inlineStr">
         <is>
-          <t>🟢 오늘 단기 매수 (저점 반등)</t>
+          <t>🔴 오늘 단기 매도 (과열 차익실현)</t>
         </is>
       </c>
       <c r="L36" s="3" t="inlineStr">
         <is>
-          <t>RSI 30.7로 단기 과매도 구간 진입, 기술적 반등 노림</t>
+          <t>RSI 19.6, 20일선 이격도 +11.7%로 단기 과열권 진입. 욕심을 줄이고 분할 차익 실현 권고</t>
         </is>
       </c>
       <c r="M36" s="3" t="inlineStr">
@@ -7296,16 +7296,16 @@
         </is>
       </c>
       <c r="O36" s="3" t="n">
-        <v>30.7</v>
+        <v>19.6</v>
       </c>
       <c r="P36" s="3" t="inlineStr">
         <is>
-          <t>-16.0%</t>
+          <t>+11.7%</t>
         </is>
       </c>
       <c r="Q36" s="3" t="inlineStr">
         <is>
-          <t>24.2%</t>
+          <t>41.1%</t>
         </is>
       </c>
       <c r="R36" s="3" t="inlineStr">
@@ -7315,197 +7315,7 @@
       </c>
       <c r="S36" s="3" t="inlineStr">
         <is>
-          <t>[8420.0, 8500.0, 8320.0, 8080.0, 8290.0, 8070.0, 8070.0, 7790.0, 7610.0, 7890.0, 7880.0, 7300.0, 7280.0, 7330.0, 7230.0, 7340.0, 7200.0, 7230.0, 7010.0, 6440.0]</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="inlineStr">
-        <is>
-          <t>휴젤</t>
-        </is>
-      </c>
-      <c r="C37" s="2" t="inlineStr">
-        <is>
-          <t>145020.KS</t>
-        </is>
-      </c>
-      <c r="D37" s="3" t="inlineStr">
-        <is>
-          <t>증권사 공식리서치</t>
-        </is>
-      </c>
-      <c r="E37" s="3" t="inlineStr">
-        <is>
-          <t>223,500원</t>
-        </is>
-      </c>
-      <c r="F37" s="3" t="inlineStr">
-        <is>
-          <t>-29,500.0원 (-11.66%)</t>
-        </is>
-      </c>
-      <c r="G37" s="3" t="inlineStr">
-        <is>
-          <t>221,500원</t>
-        </is>
-      </c>
-      <c r="H37" s="3" t="inlineStr">
-        <is>
-          <t>237,000원</t>
-        </is>
-      </c>
-      <c r="I37" s="3" t="inlineStr">
-        <is>
-          <t>215,500원</t>
-        </is>
-      </c>
-      <c r="J37" s="3" t="inlineStr">
-        <is>
-          <t>+7.1%</t>
-        </is>
-      </c>
-      <c r="K37" s="3" t="inlineStr">
-        <is>
-          <t>🟢 오늘 단기 매수 (저점 반등)</t>
-        </is>
-      </c>
-      <c r="L37" s="3" t="inlineStr">
-        <is>
-          <t>RSI 19.6로 단기 과매도 구간 진입, 기술적 반등 노림</t>
-        </is>
-      </c>
-      <c r="M37" s="3" t="inlineStr">
-        <is>
-          <t>보유 / 중립 (HOLD)</t>
-        </is>
-      </c>
-      <c r="N37" s="3" t="inlineStr">
-        <is>
-          <t>장기 추세 유지</t>
-        </is>
-      </c>
-      <c r="O37" s="3" t="n">
-        <v>19.6</v>
-      </c>
-      <c r="P37" s="3" t="inlineStr">
-        <is>
-          <t>+11.7%</t>
-        </is>
-      </c>
-      <c r="Q37" s="3" t="inlineStr">
-        <is>
-          <t>41.1%</t>
-        </is>
-      </c>
-      <c r="R37" s="3" t="inlineStr">
-        <is>
-          <t>최근 특이 뉴스 없음</t>
-        </is>
-      </c>
-      <c r="S37" s="3" t="inlineStr">
-        <is>
           <t>[236000.0, 231000.0, 232000.0, 235500.0, 231000.0, 231500.0, 214000.0, 206000.0, 190400.0, 187000.0, 186100.0, 183300.0, 179700.0, 180600.0, 180100.0, 181500.0, 183600.0, 182800.0, 180000.0, 169900.0]</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>세아제강</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t>306200.KS</t>
-        </is>
-      </c>
-      <c r="D38" s="3" t="inlineStr">
-        <is>
-          <t>증권사 공식리서치</t>
-        </is>
-      </c>
-      <c r="E38" s="3" t="inlineStr">
-        <is>
-          <t>142,000원</t>
-        </is>
-      </c>
-      <c r="F38" s="3" t="inlineStr">
-        <is>
-          <t>-6,500.0원 (-4.38%)</t>
-        </is>
-      </c>
-      <c r="G38" s="3" t="inlineStr">
-        <is>
-          <t>142,000원</t>
-        </is>
-      </c>
-      <c r="H38" s="3" t="inlineStr">
-        <is>
-          <t>149,000원</t>
-        </is>
-      </c>
-      <c r="I38" s="3" t="inlineStr">
-        <is>
-          <t>136,500원</t>
-        </is>
-      </c>
-      <c r="J38" s="3" t="inlineStr">
-        <is>
-          <t>+5.0%</t>
-        </is>
-      </c>
-      <c r="K38" s="3" t="inlineStr">
-        <is>
-          <t>관망 (HOLD)</t>
-        </is>
-      </c>
-      <c r="L38" s="3" t="inlineStr">
-        <is>
-          <t>중립 구간 유지 중</t>
-        </is>
-      </c>
-      <c r="M38" s="3" t="inlineStr">
-        <is>
-          <t>보유 / 중립 (HOLD)</t>
-        </is>
-      </c>
-      <c r="N38" s="3" t="inlineStr">
-        <is>
-          <t>장기 추세 유지</t>
-        </is>
-      </c>
-      <c r="O38" s="3" t="n">
-        <v>46.2</v>
-      </c>
-      <c r="P38" s="3" t="inlineStr">
-        <is>
-          <t>-3.5%</t>
-        </is>
-      </c>
-      <c r="Q38" s="3" t="inlineStr">
-        <is>
-          <t>39.0%</t>
-        </is>
-      </c>
-      <c r="R38" s="3" t="inlineStr">
-        <is>
-          <t>최근 특이 뉴스 없음</t>
-        </is>
-      </c>
-      <c r="S38" s="3" t="inlineStr">
-        <is>
-          <t>[150600.0, 151400.0, 146900.0, 145300.0, 147400.0, 149600.0, 145200.0, 142700.0, 138200.0, 147500.0, 146200.0, 153200.0, 148300.0, 154600.0, 155100.0, 148500.0, 145200.0, 143500.0, 141300.0, 142000.0]</t>
         </is>
       </c>
     </row>
@@ -7520,14 +7330,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="19" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7737,12 +7547,12 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>6,106.83</t>
+          <t>6,068.91</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>+71.48 (+1.18%)</t>
+          <t>▲ +33.56 (+0.56%)</t>
         </is>
       </c>
     </row>
@@ -7764,12 +7574,12 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>838.62</t>
+          <t>831.05</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>-10.57 (-1.24%)</t>
+          <t>▼ -18.14 (-2.14%)</t>
         </is>
       </c>
     </row>
@@ -7781,22 +7591,22 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>환율</t>
+          <t>증시 지수</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>미국 달러 (USD)</t>
+          <t>나스닥 (NASDAQ)</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>1,340.88</t>
+          <t>27,204.38</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>매매기준율</t>
+          <t>▼ -41.52 (-0.15%)</t>
         </is>
       </c>
     </row>
@@ -7808,22 +7618,22 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>환율</t>
+          <t>증시 지수</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>일본 100엔 (JPY)</t>
+          <t>S&amp;P 500</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>847.01</t>
+          <t>7,805.45</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>100엔 기준</t>
+          <t>▼ -1.79 (-0.02%)</t>
         </is>
       </c>
     </row>
@@ -7840,17 +7650,17 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>유로 (EUR)</t>
+          <t>미국 달러 (USD)</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>1,500.84</t>
+          <t>1,337.98</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>매매기준율</t>
+          <t>▼ -2.15원 (-0.16%)</t>
         </is>
       </c>
     </row>
@@ -7867,17 +7677,71 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
+          <t>일본 100엔 (JPY)</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>842.80</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>▼ -1.30원 (-0.15%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>환율</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>유로 (EUR)</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>1,498.50</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>▼ -1.40원 (-0.09%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>환율</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
           <t>중국 위안 (CNY)</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>199.98</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>매매기준율</t>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>199.96</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>▼ -0.25원 (-0.13%)</t>
         </is>
       </c>
     </row>
@@ -7983,27 +7847,27 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>112,702,000원</t>
+          <t>112,763,000원</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>+0.10%</t>
+          <t>+0.15%</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>112,138,000원</t>
+          <t>112,199,000원</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>121,718,000원</t>
+          <t>121,784,000원</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>110,586,000원</t>
+          <t>110,584,000원</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
@@ -8040,27 +7904,27 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>3,384,000원</t>
+          <t>3,381,000원</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>+0.09%</t>
+          <t>+0.00%</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>3,357,000원</t>
+          <t>3,354,000원</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>3,587,000원</t>
+          <t>3,584,000원</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>3,265,500원</t>
+          <t>3,262,500원</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
@@ -8075,7 +7939,7 @@
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>RSI 46.8로 단기 과매도 구간 진입, 기술적 반등 기대</t>
+          <t>RSI 46.5로 단기 과매도 구간 진입, 기술적 반등 기대</t>
         </is>
       </c>
     </row>
@@ -8097,17 +7961,17 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>145,000원</t>
+          <t>144,700원</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>+0.28%</t>
+          <t>+0.07%</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>143,800원</t>
+          <t>143,500원</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -8117,12 +7981,12 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>139,900원</t>
+          <t>139,600원</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>+8.3%</t>
+          <t>+8.6%</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
@@ -8132,7 +7996,7 @@
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>RSI 47.3로 단기 과매도 구간 진입, 기술적 반등 기대</t>
+          <t>RSI 46.8로 단기 과매도 구간 진입, 기술적 반등 기대</t>
         </is>
       </c>
     </row>
@@ -8153,15 +8017,15 @@
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="47" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="65" customWidth="1" min="8" max="8"/>
     <col width="65" customWidth="1" min="9" max="9"/>
-    <col width="17" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
     <col width="19" customWidth="1" min="11" max="11"/>
-    <col width="17" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
     <col width="19" customWidth="1" min="13" max="13"/>
     <col width="65" customWidth="1" min="14" max="14"/>
   </cols>
@@ -8245,21 +8109,21 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>신한투자증권</t>
+          <t>하나증권</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>팬오션</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>빛을 보기 시작한 포트폴리오 변화</t>
+          <t>컨센서스에 부합</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
@@ -8269,42 +8133,42 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>매수</t>
+          <t>Buy</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>한 단계 진화한 실적, 한 단계 진화할 주가 레벨 수급 영향으로 단기 주가의 변동폭은 과거 대비 커졌으나 우호적인 벌크·탱커 시황 감안 시 중기 우상향 흐름 지속될 것으로 판단. 환율 방향성이원화 환산 실적에 부담이나 펀더멘털에 미치는 영향은 제한적.</t>
+          <t>3Q26 Preview: 컨센서스에 부합하는 실적 전망 SK하이닉스의 26년 3분기 매출액은 99.2조원(YoY +306%, QoQ +25%), 영업이익은 77.9조원(YoY +584%, QoQ +29%)으로 추정한다. 매출액과 영업이익 모두 최근 낮아진 컨센서스에 부합할 전망이다. 환율 가정은 기존대비 5% 하향 조정했고, DRAM 가격은 기존 19%에서 21%로 상향, NAND 가격은 기존 24%에서 17%로 하향했다.</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>2026-10-14_신한투자증권_팬오션_빛을 보기 시작한 포트폴리오 변화.pdf</t>
+          <t>2026-10-14_하나증권_SK하이닉스_컨센서스에 부합.pdf</t>
         </is>
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>7,426.1십억원</t>
+          <t>335,642.4십억원</t>
         </is>
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>726.2십억원</t>
+          <t>258,778.7십억원</t>
         </is>
       </c>
       <c r="L2" s="3" t="inlineStr">
         <is>
-          <t>7,662.9십억원</t>
+          <t>500,127.3십억원</t>
         </is>
       </c>
       <c r="M2" s="3" t="inlineStr">
         <is>
-          <t>742.3십억원</t>
+          <t>405,117.1십억원</t>
         </is>
       </c>
       <c r="N2" s="3" t="inlineStr">
         <is>
-          <t>3Q26 영업이익 2,027억원(+61</t>
+          <t>2026/2027 실적 성장세 및 기업가치 재평가 전망</t>
         </is>
       </c>
     </row>
@@ -8315,7 +8179,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
@@ -8389,17 +8253,17 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>신한투자증권</t>
+          <t>하나증권</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>HMM</t>
+          <t>KT</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>우려도 있지만 너무 잠잠한 주가</t>
+          <t>3Q 프리뷰 - 2027년도 내다본 매수 추천</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -8409,42 +8273,42 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>매수</t>
+          <t>Buy</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>거버넌스 우려로 덮어놓기엔 아까운 실적 글로벌 컨테이너선사들은 가이던스 상향과 함께 주가도 상승했으나 동사 반응은 제한적. 거버넌스 불확실성에도 예상보다.</t>
+          <t>추천 사유는 1) 2027~2028년 장기 실적 전망이 여전히 낙관적이고, 2) 2026년 KT 실적 및 배당 관련 우려가 대부분 주가에 기반영된 상태이며, 3) 2027년 국내에서도 5G 요금제 개편 이슈가 불거질 것임을 감안하면 밸류에이션 매력도가 높고, 4) 연말 이후 국내 시중 금리가 하락 전환한다고 가정 시 배당 매력도 다시 부각될 수 있을 것이며, 5) 스페이스X 통신산업 진출 가능성으로 미국 통신사 주가 하락이 나타난 데 따른 연쇄 반응으로 KT/SKT 주가 하락이 나타났기 때문이다. 주파수 획득, 대주주 적격성 심사 등 국내 규제 상황과 최근 통신업 사업성을 감안 시 스페이스X가 직접 국내에 진출해 국내 통신 3사와 경쟁할 가능성은 희박하다.</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>2026-10-14_신한투자증권_HMM_우려도 있지만 너무 잠잠한 주가.pdf</t>
+          <t>2026-10-14_하나증권_KT_3Q 프리뷰 - 2027년도 내다본 매수 추천.pdf</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>14,179.9십억원</t>
+          <t>27,767.0십억원</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>2,497.7십억원</t>
+          <t>2,050.0십억원</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>14,293.1십억원</t>
+          <t>29,466.9십억원</t>
         </is>
       </c>
       <c r="M4" s="3" t="inlineStr">
         <is>
-          <t>1,812.7십억원</t>
+          <t>2,088.5십억원</t>
         </is>
       </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
-          <t>3Q26 매출 4조 802억원(+51%, 이하 YoY) 및 영업이익 1조 42억원(+</t>
+          <t>연결 영업이익 5,520억원으로 컨센서스와 비슷할 전망</t>
         </is>
       </c>
     </row>
@@ -8455,21 +8319,21 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>신한투자증권</t>
+          <t>하나증권</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>일진전기</t>
+          <t>LG유플러스</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>가장 저평가된 전력기기</t>
+          <t>3Q 프리뷰 - 특별한 대안 없다면 길게 보세요</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -8479,42 +8343,42 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>매수</t>
+          <t>Buy</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>변압기 29년 수주 논의 및 전선 상반기 수주 급증 5월 시가총액 약 6.9조원 도달 이후 7월말 2.2조원까지 약 68% 하락. 전선업체들의 수주잔고총계 연간 증가율은 24년 25.4%, 25년 21.2%에서 26년 상반기에만 23.2% 증가. 변압기에 이은 전선 부문의 호황이 확대되는 것을 감안할 때 펀더멘털 문제가 아닌 수급 측면의 주가 하락으로 판단.</t>
+          <t>매수 투자의견/TP 20,000원 유지, 매도하기보단 배당 감안한 중/장기 매수 추천 LGU+에 대한 투자의견 매수, 12개월 목표주가 20,000원을 유지한다. 추천 사유는 1) 2분기에 이어 3분기에도 우수한 실적을 기록할 것으로 전망됨에 따라 2026년 연간 높은 연결 영업이익 성장 가능성이 높아졌고, 2) 양호한 실적 전망을 바탕으로 2027년도엔 다시 주주환원 증대 기대감이 높아질 전망이며, 3) 조만간 정책 금리 상승이 마무리되고 시중 금리가 하락 전환하면서 연말 이후 4.8%에 달하는 기대배당수익률이 매력적으로 인식될 수 있을 것이기 때문이다. 당장 특별한 재료가 부각될 수 있는 상황은 아니지만 국내 주식 시장이 강한 상승 탄력을 나타나고 있지 않은 점을 감안하면 차라리 매도하기 보단 2027년 초까지 LGU+ 보유 또는 배당을 염두에 둔 신규 매수 진입을 추천한다.</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>2026-10-14_신한투자증권_일진전기_가장 저평가된 전력기기.pdf</t>
+          <t>2026-10-14_하나증권_LG유플러스_3Q 프리뷰 - 특별한 대안 없다면 길게 보세요.pdf</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>2,350.8십억원</t>
+          <t>15,429.4십억원</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>252.8십억원</t>
+          <t>1,144.2십억원</t>
         </is>
       </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>2,595.2십억원</t>
+          <t>16,347.1십억원</t>
         </is>
       </c>
       <c r="M5" s="3" t="inlineStr">
         <is>
-          <t>271.7십억원</t>
+          <t>1,185.5십억원</t>
         </is>
       </c>
       <c r="N5" s="3" t="inlineStr">
         <is>
-          <t>2026/2027 실적 성장세 및 기업가치 재평가 전망</t>
+          <t>연결 영업이익 3,221억원 전망, 4Q 인센티브 반영 고려해도 올해 실적 좋을 것</t>
         </is>
       </c>
     </row>
@@ -8525,21 +8389,21 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>신한투자증권</t>
+          <t>하나증권</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>현대글로비스</t>
+          <t>SK텔레콤</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>환율은 야속하지만 너무 좋은 해운 업황</t>
+          <t>3Q 프리뷰 - DPS 증가 기대감 커지는 계기될 것</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -8549,42 +8413,42 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>매수</t>
+          <t>Buy</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>자동차 밸류체인이지만 해운사이기도 함. 단기 실적 가시성은 다소 낮아졌으나 이익 방향성은 여전히 긍정적. 비계열 고객 호조로 이익 개선이 뚜렷한 사업부를 가진 점은 차별화 포인트.</t>
+          <t>더불어 국내 통신서비스 업종 12개월/10월 Top Pick으로 제시한다. 추천 사유는 1) 3분기 실적도 양호할 전망이라 2026년 연간 연결 영업이익이 2조원에 육박할 전망이고, 2) 2026년 우수한 실적을 바탕으로 DPS가 2024년 수준으로 회귀할 전망이며, 3) 엔트로픽 상장 가치가 당초 기대를 뛰어넘을 것으로 보여 밸류에이션상 저평가 논란이 생겨날 것이고, 4) 금리 인상 기조가 마무리되고 SKT 비과세 배당이 시작되는 2026년 말/2027년 초부터는 수급 개선이 예상되기 때문이다.</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>2026-10-14_신한투자증권_현대글로비스_환율은 야속하지만 너무 좋은 해운 업황.pdf</t>
+          <t>2026-10-14_하나증권_SK텔레콤_3Q 프리뷰 - DPS 증가 기대감 커지는 계기될 것.pdf</t>
         </is>
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>33,217.4십억원</t>
+          <t>17,658.0십억원</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>2,077.2십억원</t>
+          <t>1,950.1십억원</t>
         </is>
       </c>
       <c r="L6" s="3" t="inlineStr">
         <is>
-          <t>34,964.5십억원</t>
+          <t>18,217.8십억원</t>
         </is>
       </c>
       <c r="M6" s="3" t="inlineStr">
         <is>
-          <t>2,408.5십억원</t>
+          <t>2,013.5십억원</t>
         </is>
       </c>
       <c r="N6" s="3" t="inlineStr">
         <is>
-          <t>2026/2027 실적 성장세 및 기업가치 재평가 전망</t>
+          <t>2026년 연간 연결 영업이익이 2조원에 육박할 전망이고, 2) 2026년 우수한 실적을 바탕으</t>
         </is>
       </c>
     </row>
@@ -8599,17 +8463,17 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>하나증권</t>
+          <t>신한투자증권</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>삼성화재</t>
+          <t>일진전기</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>3Q26 Pre - 단기 실적보다 중요한 것은</t>
+          <t>가장 저평가된 전력기기</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
@@ -8619,37 +8483,37 @@
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>Buy</t>
+          <t>매수</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>2026년 3분기 실적은 컨센서스 하회 전망 3분기 연결 지배순이익은 4,863억원으로 컨센서스(5,825억원)를 하회할 것으로 전망한다. 장기보험손익이 사업비 부담 확대로 예상대비 부한 가운데, 증시 부진과 금리 상승에 따른 투자손익 악화도 실적에 부담으로 작용할 것으로 예상한다. [보험손익] 보험손익은 4,006억원(YoY +8.6%, QoQ -27.5%)으로 추정한다.</t>
+          <t>변압기 29년 수주 논의 및 전선 상반기 수주 급증 5월 시가총액 약 6.9조원 도달 이후 7월말 2.2조원까지 약 68% 하락. 전선업체들의 수주잔고총계 연간 증가율은 24년 25.4%, 25년 21.2%에서 26년 상반기에만 23.2% 증가. 변압기에 이은 전선 부문의 호황이 확대되는 것을 감안할 때 펀더멘털 문제가 아닌 수급 측면의 주가 하락으로 판단.</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>2026-10-14_하나증권_삼성화재_3Q26 Pre - 단기 실적보다 중요한 것은.pdf</t>
+          <t>2026-10-14_신한투자증권_일진전기_가장 저평가된 전력기기.pdf</t>
         </is>
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2,350.8십억원</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>3,496십억원</t>
+          <t>252.8십억원</t>
         </is>
       </c>
       <c r="L7" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2,595.2십억원</t>
         </is>
       </c>
       <c r="M7" s="3" t="inlineStr">
         <is>
-          <t>4,566십억원</t>
+          <t>271.7십억원</t>
         </is>
       </c>
       <c r="N7" s="3" t="inlineStr">
@@ -8665,21 +8529,21 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>하나증권</t>
+          <t>DS투자증권</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>세아베스틸지주</t>
+          <t>삼성중공업</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>3분기는 다소 부진하겠지만 4분기부터 회복 기대</t>
+          <t>3Q26 Preview: 증익의 시작점</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -8689,42 +8553,42 @@
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>Buy</t>
+          <t>매수</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>3Q26 주력 자회사들 판매 감소와 스프레드 축소 2026년 3분기 세아베스틸지주의 매출액과 영업이익은 각각 1.0조원(YoY +10.3%, QoQ -10.6%)과 236억원(YoY -12.4%, QoQ -60.6%)으로 영업이익은 시장컨센서스인 398억원을 크게 하회할 것으로 예상된다. 계절적 비수기와 9월 추석 연휴 영향으로 세아베스틸의 특수강 판매는 41.2만톤(YoY +5.0%, QoQ -9.8%)에 그치며 고정비 부담이 확대될 전망이다. 원가 상승분 가격 전가를 위한 노력으로 8월초까지 적극적인 가격 인상을 시도한 결과, 특수강 ASP가 1.6만원/톤 상승이 예상되나 스크랩가격이 이를 상회하는 2.1만원/톤 상승하여 스프레드도 소폭 축소될 전망이다.</t>
+          <t>3Q26 Preview: 영업이익 3,791억원으로 컨센서스 소폭 상회 전망 26년 3분기 실적은 매출액 3.2조원(이하 YoY +22.8%), 영업이익 3,791억원(+59.2%, OPM 11.7%)으로 시장 컨센서스를 10% 상회할 전망이다. 조업일수는 하계 휴가와 추석 연휴 등으로 전분기 대비 9일 감소하나 글로벌 오퍼레이션과 2도크 재가동에 따른 매출 확대가 이를 상쇄하며 탑라인은 전분기 대비 소폭 성장할 것으로 예상된다. 수익성 또한 확대될 예정이다.</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>2026-10-14_하나증권_세아베스틸지주_3분기는 다소 부진하겠지만 4분기부터 회복 기대.pdf</t>
+          <t>2026-10-14_DS투자증권_삼성중공업_3Q26 Preview 증익의 시작점.pdf</t>
         </is>
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>4,116.0십억원</t>
+          <t>10,650십억원</t>
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>140.6십억원</t>
+          <t>862십억원</t>
         </is>
       </c>
       <c r="L8" s="3" t="inlineStr">
         <is>
-          <t>4,496.9십억원</t>
+          <t>12,916십억원</t>
         </is>
       </c>
       <c r="M8" s="3" t="inlineStr">
         <is>
-          <t>223.3십억원</t>
+          <t>1,416십억원</t>
         </is>
       </c>
       <c r="N8" s="3" t="inlineStr">
         <is>
-          <t>3Q26 영업이익 236억원(YoY -</t>
+          <t>3Q26 Preview: 영업이익 3,791억원으로 컨센서스 소폭 상회 전망</t>
         </is>
       </c>
     </row>
@@ -8744,12 +8608,12 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>한화손해보험</t>
+          <t>삼성화재</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>3Q26 Pre - 보험손익 개선세에 주목</t>
+          <t>3Q26 Pre - 단기 실적보다 중요한 것은</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -8764,12 +8628,12 @@
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>2026년 3분기 실적은 컨센서스 소폭 하회 전망 3분기 별도 당기순이익은 903억원으로 컨센서스(939억원)를 소폭 하회할 것으로 전망한다. 증시 부진 및 금리 상승에 따른 투자손익 악화가 예상되나, 보험손익은 전반적으로 개선될 전망이다. [보험손익] 보험손익은 1,377억원(YoY +44.5%, QoQ +35.2%)으로 추정한다.</t>
+          <t>2026년 3분기 실적은 컨센서스 하회 전망 3분기 연결 지배순이익은 4,863억원으로 컨센서스(5,825억원)를 하회할 것으로 전망한다. 장기보험손익이 사업비 부담 확대로 예상대비 부한 가운데, 증시 부진과 금리 상승에 따른 투자손익 악화도 실적에 부담으로 작용할 것으로 예상한다. [보험손익] 보험손익은 4,006억원(YoY +8.6%, QoQ -27.5%)으로 추정한다.</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>2026-10-14_하나증권_한화손해보험_3Q26 Pre - 보험손익 개선세에 주목.pdf</t>
+          <t>2026-10-14_하나증권_삼성화재_3Q26 Pre - 단기 실적보다 중요한 것은.pdf</t>
         </is>
       </c>
       <c r="J9" s="3" t="inlineStr">
@@ -8779,7 +8643,7 @@
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>465십억원</t>
+          <t>3,496십억원</t>
         </is>
       </c>
       <c r="L9" s="3" t="inlineStr">
@@ -8789,7 +8653,7 @@
       </c>
       <c r="M9" s="3" t="inlineStr">
         <is>
-          <t>595십억원</t>
+          <t>4,566십억원</t>
         </is>
       </c>
       <c r="N9" s="3" t="inlineStr">
@@ -8809,17 +8673,17 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>미래에셋증권</t>
+          <t>유안타증권</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>휴젤</t>
+          <t>KT</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>3Q26 Preview: 단기 실적 눈높이 조정</t>
+          <t>바닥 통과, 성장 엔진 점화</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
@@ -8829,42 +8693,42 @@
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>매수</t>
+          <t>Buy</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>3분기 실적은 미국 판매체계 전환 영향으로 부진 휴젤의 3Q26 매출액은 1,009억원(-4.7% YoY), 영업이익 211억원(-55.5% YoY)으로 추정했다. 3Q26 영업이익은 미국 판매체계 전환 영향으로 전년 동기 대비 55.5% 감소할 것으로 보인다. 3분기는 미국 유통사 모델에서 CSO 모델로 전환하는 과정에서 일회성 매출 차감과 비용 증가가 동반되는 구간이었기 때문이다.</t>
+          <t>3Q26 Preview: 일회성 제거시 영업이익 +3% YoY 3Q26 연결 영업수익은 7.1조원(-1.1% YoY), 영업이익은 5,350억원(-0.6% YoY)으로 시장 컨센서스(7.0조원, 5,442억원)에 부합할 전망이다. 부동산 관련 일회성 비용 제거시 영업이익은 +2.8% YoY 증가한 것으로 추정된다. 별도 영업이익은 3,400억원으로 전년과 유사한 수준이 예상된다.</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>2026-10-14_미래에셋증권_휴젤_3Q26 Preview 단기 실적 눈높이 조정.pdf</t>
+          <t>2026-10-14_유안타증권_KT_바닥 통과, 성장 엔진 점화.pdf</t>
         </is>
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>486십억원</t>
+          <t>27,426십억원</t>
         </is>
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>174십억원</t>
+          <t>2,076십억원</t>
         </is>
       </c>
       <c r="L10" s="3" t="inlineStr">
         <is>
-          <t>657십억원</t>
+          <t>27,905십억원</t>
         </is>
       </c>
       <c r="M10" s="3" t="inlineStr">
         <is>
-          <t>272십억원</t>
+          <t>2,256십억원</t>
         </is>
       </c>
       <c r="N10" s="3" t="inlineStr">
         <is>
-          <t>3Q26 매출액은 1,009억원(-4</t>
+          <t>3Q26 Preview: 일회성 제거시 영업이익 +3% YoY</t>
         </is>
       </c>
     </row>
@@ -8875,21 +8739,21 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>하나증권</t>
+          <t>미래에셋증권</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>세아제강</t>
+          <t>휴젤</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>어려운 영업환경!</t>
+          <t>3Q26 Preview: 단기 실적 눈높이 조정</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
@@ -8899,42 +8763,42 @@
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>Buy</t>
+          <t>매수</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>3Q26 내수와 수출 모두 수익성 악화 2026년 3분기 세아제강의 매출액과 영업이익은 각각 4,318억원(YoY +30.2%, QoQ -12.8%)과 195억원(YoY 흑.전, QoQ -44.2%)으로 영업이익은 시장컨센서스인 254억원을 하회할 것으로 예상된다. 3분기 내수 강관 시장은 계절적 비수기와 추석 연휴 영향으로 다소 부진할 것으로 예상되는 가운데 수출의 경우 캐나다. LNG와 같은 프로젝트 덕분에 소폭 증가한 것으로 추정되어 결과적으로 세아제강의 3분기 전체 강관 판매는 22.8만톤(YoY +21.4%, QoQ -6.8%)을 기록할 전망이다.</t>
+          <t>3분기 실적은 미국 판매체계 전환 영향으로 부진 휴젤의 3Q26 매출액은 1,009억원(-4.7% YoY), 영업이익 211억원(-55.5% YoY)으로 추정했다. 3Q26 영업이익은 미국 판매체계 전환 영향으로 전년 동기 대비 55.5% 감소할 것으로 보인다. 3분기는 미국 유통사 모델에서 CSO 모델로 전환하는 과정에서 일회성 매출 차감과 비용 증가가 동반되는 구간이었기 때문이다.</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>2026-10-14_하나증권_세아제강_어려운 영업환경!.pdf</t>
+          <t>2026-10-14_미래에셋증권_휴젤_3Q26 Preview 단기 실적 눈높이 조정.pdf</t>
         </is>
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>1,822.7십억원</t>
+          <t>486십억원</t>
         </is>
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>103.1십억원</t>
+          <t>174십억원</t>
         </is>
       </c>
       <c r="L11" s="3" t="inlineStr">
         <is>
-          <t>1,852.8십억원</t>
+          <t>657십억원</t>
         </is>
       </c>
       <c r="M11" s="3" t="inlineStr">
         <is>
-          <t>124.3십억원</t>
+          <t>272십억원</t>
         </is>
       </c>
       <c r="N11" s="3" t="inlineStr">
         <is>
-          <t>2026년 3분기 세아제강의 매출액과 영업이익은 각각 4,318억원(YoY +30</t>
+          <t>3Q26 매출액은 1,009억원(-4</t>
         </is>
       </c>
     </row>
@@ -8949,20 +8813,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="21" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
     <col width="32" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
@@ -9076,7 +8940,7 @@
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>+1.8%</t>
+          <t>+1.1%</t>
         </is>
       </c>
       <c r="K2" s="3" t="inlineStr">
@@ -9138,7 +9002,7 @@
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>+2.1%</t>
+          <t>+2.0%</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
@@ -9200,7 +9064,7 @@
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>+3.1%</t>
+          <t>+2.7%</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
@@ -9262,7 +9126,7 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>+3.4%</t>
+          <t>+3.2%</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
@@ -9324,7 +9188,7 @@
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>+1.5%</t>
+          <t>+1.0%</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
@@ -9386,7 +9250,7 @@
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>+4.7%</t>
+          <t>+4.6%</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
@@ -9423,12 +9287,12 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>238,500원</t>
+          <t>236,500원</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>236,000원</t>
+          <t>234,000원</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
@@ -9438,7 +9302,7 @@
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>230,000원</t>
+          <t>228,000원</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
@@ -9448,12 +9312,12 @@
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>+0.3%</t>
+          <t>+0.7%</t>
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>236,750원</t>
+          <t>235,750원</t>
         </is>
       </c>
       <c r="L8" s="3" t="inlineStr">
@@ -9475,32 +9339,32 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>한미약품</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>000660.KS</t>
+          <t>128940.KS</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>1,456,000원</t>
+          <t>409,000원</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>1,441,500원</t>
+          <t>405,000원</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>1,705,000원</t>
+          <t>483,500원</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>1,405,000원</t>
+          <t>394,500원</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
@@ -9510,12 +9374,12 @@
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>+0.4%</t>
+          <t>+0.7%</t>
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>1,447,000원</t>
+          <t>408,000원</t>
         </is>
       </c>
       <c r="L9" s="3" t="inlineStr">
@@ -9537,32 +9401,32 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>한미약품</t>
+          <t>KT</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>128940.KS</t>
+          <t>030200.KS</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>417,500원</t>
+          <t>49,800원</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>413,500원</t>
+          <t>49,300원</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>484,000원</t>
+          <t>52,700원</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>403,000원</t>
+          <t>48,000원</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr">
@@ -9572,12 +9436,12 @@
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>+0.5%</t>
+          <t>+1.0%</t>
         </is>
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>415,500원</t>
+          <t>49,800원</t>
         </is>
       </c>
       <c r="L10" s="3" t="inlineStr">
@@ -9599,32 +9463,32 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>현대글로비스</t>
+          <t>SK텔레콤</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>086280.KS</t>
+          <t>017670.KS</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>185,500원</t>
+          <t>82,200원</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>184,000원</t>
+          <t>81,400원</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>197,000원</t>
+          <t>87,100원</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>179,000원</t>
+          <t>79,300원</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
@@ -9634,12 +9498,12 @@
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>+0.9%</t>
+          <t>+1.0%</t>
         </is>
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>185,600원</t>
+          <t>82,200원</t>
         </is>
       </c>
       <c r="L11" s="3" t="inlineStr">
@@ -9671,22 +9535,22 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>581,000원</t>
+          <t>584,000원</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>575,000원</t>
+          <t>578,000원</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>629,000원</t>
+          <t>629,500원</t>
         </is>
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>560,500원</t>
+          <t>563,500원</t>
         </is>
       </c>
       <c r="I12" s="3" t="inlineStr">
@@ -9696,139 +9560,15 @@
       </c>
       <c r="J12" s="3" t="inlineStr">
         <is>
-          <t>+1.2%</t>
+          <t>+1.0%</t>
         </is>
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>582,000원</t>
+          <t>584,000원</t>
         </is>
       </c>
       <c r="L12" s="3" t="inlineStr">
-        <is>
-          <t>1일차</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>한화손해보험</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>000370.KS</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>6,440원</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>6,380원</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>7,510원</t>
-        </is>
-      </c>
-      <c r="H13" s="3" t="inlineStr">
-        <is>
-          <t>6,210원</t>
-        </is>
-      </c>
-      <c r="I13" s="3" t="inlineStr">
-        <is>
-          <t>⏳ 목표가 추적 중 (신규 진입)</t>
-        </is>
-      </c>
-      <c r="J13" s="3" t="inlineStr">
-        <is>
-          <t>+0.9%</t>
-        </is>
-      </c>
-      <c r="K13" s="3" t="inlineStr">
-        <is>
-          <t>6,440원</t>
-        </is>
-      </c>
-      <c r="L13" s="3" t="inlineStr">
-        <is>
-          <t>1일차</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>휴젤</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>145020.KS</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr">
-        <is>
-          <t>223,500원</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>221,500원</t>
-        </is>
-      </c>
-      <c r="G14" s="3" t="inlineStr">
-        <is>
-          <t>237,000원</t>
-        </is>
-      </c>
-      <c r="H14" s="3" t="inlineStr">
-        <is>
-          <t>215,500원</t>
-        </is>
-      </c>
-      <c r="I14" s="3" t="inlineStr">
-        <is>
-          <t>⏳ 목표가 추적 중 (신규 진입)</t>
-        </is>
-      </c>
-      <c r="J14" s="3" t="inlineStr">
-        <is>
-          <t>+0.9%</t>
-        </is>
-      </c>
-      <c r="K14" s="3" t="inlineStr">
-        <is>
-          <t>223,500원</t>
-        </is>
-      </c>
-      <c r="L14" s="3" t="inlineStr">
         <is>
           <t>1일차</t>
         </is>
@@ -10242,7 +9982,7 @@
       <c r="D9" s="3" t="inlineStr"/>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>풍산, 최대주주등 지분율 38.02% 유지, 임원 장내매수로 108주 증가</t>
+          <t>사이먼 쿠케스 박사 측, 페데브코 보통주 14만 7070주 장내 매수…지분율 34.2%로 확대</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -10257,12 +9997,12 @@
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 08:03:15 GMT</t>
+          <t>Tue, 13 Oct 2026 12:14:51 GMT</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMic0FVX3lxTFBCY2RfTnBJdUJVUW5lcFdtUGtuYXhMNmRwNkVmREpRVTdyRUQ3Y2ZfaWFTMUhNVkpSZEdJUGdzMnZ4RWZQSlpwSG9FS2FlV05kaktCSm16clk5Tjg1a0t2MHNmMkw0WHBrdm9fR2lkVXlCODA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMic0FVX3lxTE8wVldLdklzOFE4cnp4RmlPLVJ2LVdveDVQTUV2UjhyTjh1NVhIMG5maUxkelFnUkhEV1ZxdGY2empxS252cDk5QW9ua2EtZ3lRUl94bVA5UEg4b09SZXdMcUk5UnlrbHRpZGU4V1VNYTdzNjQ?oc=5</t>
         </is>
       </c>
     </row>
@@ -10594,32 +10334,32 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>🌐 [경제·사회 심층 리포트] 모두의 AI의 숨겨진 배경과 구조적 쟁점</t>
+          <t>🌐 [경제·사회 심층 리포트] GC녹십자의 숨겨진 배경과 구조적 쟁점</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>모두의 AI</t>
+          <t>GC녹십자</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>단순 뉴스 헤드라인을 넘어선 전후 맥락: '모두의 AI' 이슈가 촉발된 진짜 배경과 이해관계자들의 득실 계산을 분석합니다.</t>
+          <t>단순 뉴스 헤드라인을 넘어선 전후 맥락: 'GC녹십자' 이슈가 촉발된 진짜 배경과 이해관계자들의 득실 계산을 분석합니다.</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>오늘 주요 언론을 통해 집중 조명된 핵심 사안은 바로 **[카카오 '모두의 AI' MAU 500만 목표…과업 완료율로 성과 평가]** 입니다.&lt;br&gt;• &lt;b&gt;핵심 현황:&lt;/b&gt; 카카오 '모두의 AI' MAU 500만 목표…과업 완료율로 성과 평가 연합인포맥스 카카오, 웹툰·음원·카카오T에 스테이블코인 결제 연동…소설 원작 AI 애니 제작도 전자신문카톡에 “메시지 정리, 답장 보내줘” 말하면 AI비서가 척척 동아일보카카오 인적분할 앞두고 창사 첫 '그룹 공동 IR' 개최, 계열사 CEO 총출동 비즈니스포스트카카오, AI 시대 ‘신뢰·책임’ 검증 사례 나눈다.&lt;br&gt;• &lt;b&gt;왜 중요한가:&lt;/b&gt; 단순한 단발성 소식이 아니라 정부 정책, 규제 환경, 기업들의 실질적 손익과 직결되어 시장 전반에 큰 파장을 일으키고 있기 때문입니다.</t>
+          <t>오늘 주요 언론을 통해 집중 조명된 핵심 사안은 바로 **[GC녹십자, LG CNS와 스마트공장 구축…AI 자동화 추진]** 입니다.&lt;br&gt;• &lt;b&gt;핵심 현황:&lt;/b&gt; GC녹십자가 LG CNS와 인공지능 기반 자동화·자율 운영 스마트 공장 구축을 추진한다.&lt;br&gt;• &lt;b&gt;왜 중요한가:&lt;/b&gt; 단순한 단발성 소식이 아니라 정부 정책, 규제 환경, 기업들의 실질적 손익과 직결되어 시장 전반에 큰 파장을 일으키고 있기 때문입니다.</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>이 문제는 오늘 갑자기 발생한 사안이 아니라, 과거부터 축적되어 온 구조적 원인이 있습니다.&lt;br&gt;• &lt;b&gt;과거 배경:&lt;/b&gt; KT컨소시엄, ‘모두의 AI Connect Summit 2026’ 개최 바끄로뉴스. '국민이 체감' 모두의 AI, 이용자 사로잡을 전략은 비즈워치.&lt;br&gt;• &lt;b&gt;결정적 계기:&lt;/b&gt; 잠재되어 있던 제도적 갈등과 시장 환경의 변화가 맞물리면서, 이번 계기를 통해 본격적으로 수면 위로 표출되었습니다.</t>
+          <t>이 문제는 오늘 갑자기 발생한 사안이 아니라, 과거부터 축적되어 온 구조적 원인이 있습니다.&lt;br&gt;• &lt;b&gt;과거 배경:&lt;/b&gt; GC녹십자, 헌터라제 알레르기 유발 항체 정밀 검출 기술 개발 뉴스저널리즘. 어려울 때 GC녹십자 2분기 살린 건, 끈끈한 '피의 힘' 히트뉴스.&lt;br&gt;• &lt;b&gt;결정적 계기:&lt;/b&gt; 잠재되어 있던 제도적 갈등과 시장 환경의 변화가 맞물리면서, 이번 계기를 통해 본격적으로 수면 위로 표출되었습니다.</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>겉으로 보이는 명분 뒤에는 각 주체들의 아주 명확한 '실질적 손익 계산'이 숨어 있습니다.&lt;br&gt;• &lt;b&gt;이해관계 분석:&lt;/b&gt; 통신 3사, 3Q 영업익 1.4조 전망…일회성 비용 털고 AI 성장 가속 매일일보. SKT·KT·카카오, ‘모두의 AI’ 누가 먼저 기선잡나… 베타 서비스 10월 출격, 각축전 ‘점화’ CEO스코어데일리.&lt;br&gt;• &lt;b&gt;핵심 구조:&lt;/b&gt; 규제 당국은 시장 통제력과 정책 주도권을 강화하려 하고, 관련 기업들은 비용 부담을 줄이고 수익성을 지키기 위해 치열한 수싸움을 벌이고 있는 구도입니다.</t>
+          <t>겉으로 보이는 명분 뒤에는 각 주체들의 아주 명확한 '실질적 손익 계산'이 숨어 있습니다.&lt;br&gt;• &lt;b&gt;이해관계 분석:&lt;/b&gt; GC녹십자, 헌터라제 특이 IgE 항체 정밀 분석법 개발…국제학술지 게재 나눔경제뉴스. GC녹십자웰빙, 비만·체형관리까지…'에스테틱' 판 키운다.&lt;br&gt;• &lt;b&gt;핵심 구조:&lt;/b&gt; 규제 당국은 시장 통제력과 정책 주도권을 강화하려 하고, 관련 기업들은 비용 부담을 줄이고 수익성을 지키기 위해 치열한 수싸움을 벌이고 있는 구도입니다.</t>
         </is>
       </c>
       <c r="J2" s="3" t="inlineStr">
@@ -10634,12 +10374,12 @@
       </c>
       <c r="L2" s="3" t="inlineStr">
         <is>
-          <t>연합인포맥스</t>
+          <t>주요언론</t>
         </is>
       </c>
       <c r="M2" s="3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMicEFVX3lxTE9FREp6R1lfYkJtTEhVUGZqRTdNbXBZbmNUYVpQWDN4c2M0OTZ0TV9OZzJmVW9CZFNITFdtWjNzY1RkTUpmLTYzMWgycEVFbjF6OWRpeGZFdWRjZkN0djBEeXlJVmJnZ1RSbkc4bEl5NDc?oc=5</t>
+          <t>https://www.yna.co.kr/view/AKR20261014121800017</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: complete 7-point briefing revamp (DART & crypto page separation, real estate intelligence, enhanced news summary and natural insights)
</commit_message>
<xml_diff>
--- a/reports/일자별_누적_데일리_이슈_및_주식_브리핑_마스터.xlsx
+++ b/reports/일자별_누적_데일리_이슈_및_주식_브리핑_마스터.xlsx
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G93"/>
+  <dimension ref="A1:G95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3631,27 +3631,27 @@
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>연결 이슈 (후속)</t>
+          <t>🔥 [언론사 집중 보도 (3개사)]</t>
         </is>
       </c>
       <c r="D86" s="3" t="inlineStr">
         <is>
-          <t>윤석열 선거법 2심, 오는 27일 선고‥국민의힘 '선거비용 397억 원 반환' 달렸다</t>
+          <t>“신임 비서실장은 임광현”…떠나는 강훈식 마지막 브리핑 [지금뉴스]</t>
         </is>
       </c>
       <c r="E86" s="3" t="inlineStr">
         <is>
-          <t>윤석열 선거법 2심, 오는 27일 선고‥국민의힘 '선거비용 397억 원 반환' 달렸다. MBC 뉴스'국힘 397억 반환' 걸린 尹 재판서 특검 '당선무효형 유지' 요청 MBC 뉴스‘국힘 397억 반환’ 걸린 2심서…윤 "이럴 거면 선거 왜 해" JTBC‘국힘 397억’ 걸린 尹 선거법 2심 27일 선고 동아일보특검, 尹 '여론조사 무상수수' 무죄 판결에 상고…"납득 어려워".</t>
+          <t>“신임 비서실장은 임광현”떠나는 강훈식 마지막 브리핑 KBS 뉴스 신임 대통령 비서실장에 임광현 국세청장 JTBC이 대통령, ‘강훈식 후임’ 새 비서실장에 임광현 국세청장 임명 한겨레안철수 "임광현 비서실장, 보은 인사 결정판처남 대장동 변호사" 뉴스1李 '먹사니즘' 세제 공약 설계한 임광현黨영입인재서 靑비서실장까지 아시아경제.</t>
         </is>
       </c>
       <c r="F86" s="3" t="inlineStr">
         <is>
-          <t>MBC 뉴스</t>
+          <t>KBS 뉴스</t>
         </is>
       </c>
       <c r="G86" s="3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTFBqVlppeEExSms5RGVjN2ZqY2Y1bXN6ZlV4MTJlcnc3VERVT1BNRDRBZG94Q2xFaGxSZ3JEelJZVk1NNFMzOUt4WW1jOXd2Z0xydXlFajhLM05qZU8xc3RGVlM2NXdteHd1b3FPMjZPdm9UWHFmcjBJ0gF3QVVfeXFMT2FLNS01aG8xbG5qdVpQVl82RmpXVktST0k1VHZ6T2lzdk1lNXJGa1RrV21jZGkxRVUtMzVhdjRFdEF3QUJtRjI0RktXTjhmc2s1YzNLZHpHcDJUZy1Jb2lrYm43ZFpfazFmZUF6OFNtMUJwdEE4M28?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTFBOT2xfekhrRnVZc3FfaENuU0xNRUJEczB5Z2RWVjRCLUtheS1VZ2UyUk9GT3J4aHNuclBVS0o5T3FPMFRRYWhwMTYxQWNiUDVQYkd4Ni1XbTdfem8?oc=5</t>
         </is>
       </c>
     </row>
@@ -3668,27 +3668,27 @@
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>신규 이슈</t>
+          <t>연결 이슈 (후속)</t>
         </is>
       </c>
       <c r="D87" s="3" t="inlineStr">
         <is>
-          <t>대입 논술시험서 AI안경 쓴 수험생들 적발…시립대 "응시 3년 금지"</t>
+          <t>인천 흉기난동범 "관심 끌려 범행…힘없어 보이는 사람 골랐다"</t>
         </is>
       </c>
       <c r="E87" s="3" t="inlineStr">
         <is>
-          <t>대입 논술시험서 AI안경 쓴 수험생들 적발…시립대 "응시 3년 금지" 논술 시험장에 등장한 스마트안경…연세대·시립대서 줄줄이 적발 KBS 뉴스뿔테 안경 아니었어?···연세대 논술 시험장서 ‘스마트 안경’ 적발 주간경향정근식, '스마트 안경' 부정행위 우려에 "교육부 지침 따라 대응" MBC 뉴스수험생들 “이번 수능때 AI 안경 쓸것”… 대학선 방지책 비상 문화일보.</t>
+          <t>인천 대형 상업시설에서 흉기를 휘둘러 8명을 다치게 한 50대 남성이 자신의 불만을 사회적으로 알리고 싶어 범.</t>
         </is>
       </c>
       <c r="F87" s="3" t="inlineStr">
         <is>
-          <t>연합뉴스</t>
+          <t>주요언론</t>
         </is>
       </c>
       <c r="G87" s="3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTFBkb21vYW14V21SZVNZOVlHaGIyRkJ4TlA5RU9IYkRrekVpOVBSbjlqLWdSZ25mcnVpOUhvS1R5WGpjSGdicm4xSDhCR2xERjduVktqR3RveWJKY03SAWBBVV95cUxObXlQc0RwOFRTSnJaSk9MUTM1S3JsaFlsSUVsc1ZGeWc1SUVjNGFWLUNiWExVc2pTSkpmc1Eyek80WHN3cE9tOHdBZXJIMm5aNno5TGR2bFZ0cml1aEM0WE8?oc=5</t>
+          <t>https://www.yna.co.kr/view/AKR20261014134000065</t>
         </is>
       </c>
     </row>
@@ -3710,22 +3710,22 @@
       </c>
       <c r="D88" s="3" t="inlineStr">
         <is>
-          <t>"뛰다가 죽음 이를 수도"…황영조가 러너들에 던진 경고</t>
+          <t>'1심 무죄' 前경호처장 2심 징역 1년…尹비화폰 증거인멸 유죄(종합)</t>
         </is>
       </c>
       <c r="E88" s="3" t="inlineStr">
         <is>
-          <t>이를 수도"…황영조가 러너들에 던진 경고 황영조 ’러닝 경고’…“기록·SNS 욕심 보다. 몸 상태 체크“ TV"포기할 줄 아는 사람이 잘 뛰는 사람"...잇따른 마라톤 사고에 황영조 '일침' YTN'서울달리기' 숨진 20대女는 '카이스트 대학원생' 유지원씨 파이낸셜뉴스“그냥 달리고 싶어”…결승선 앞 멈춰진 20대 러너의 꿈 KBS 뉴스.</t>
+          <t>12·3 비상계엄 사태 이후 윤석열 전 대통령 등의 비화폰 정보를 삭제한 혐의로 기소된 박종준 전 대통령 경호.</t>
         </is>
       </c>
       <c r="F88" s="3" t="inlineStr">
         <is>
-          <t>한국경제</t>
+          <t>주요언론</t>
         </is>
       </c>
       <c r="G88" s="3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTFBnZE9PNDVINmZpajNMVEppN3IyZV9KUE1kZE1xcnd1RHlOV2NIWWJiSGFUUW5Ed2F1QkNFNllwY24xY0JUT29VZ3Z6eTJIcGFqZ2hsWk5ocHdfdw?oc=5</t>
+          <t>https://www.yna.co.kr/view/AKR20261014123851004</t>
         </is>
       </c>
     </row>
@@ -3742,27 +3742,27 @@
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>연결 이슈 (후속)</t>
+          <t>신규 이슈</t>
         </is>
       </c>
       <c r="D89" s="3" t="inlineStr">
         <is>
-          <t>‘한동훈 고발장’ 경찰·중수청 접수…‘자녀 허위스펙·부실 수사’ 의혹</t>
+          <t>제주 평화로에서 다중 추돌 교통사고…12대 추정</t>
         </is>
       </c>
       <c r="E89" s="3" t="inlineStr">
         <is>
-          <t>‘한동훈 고발장’ 경찰·중수청 접수…‘자녀 허위스펙·부실 수사’ 의혹 한겨레시민단체, '딸 허위 스펙 수사무마' 의혹 한동훈 고발 MBC 뉴스 신지호 “한동훈 딸 의혹…민주당, 쓰레기 재활용하나?” KBS 뉴스한동훈, 법무부 장관 재직시 딸 `허위스펙` 수사무마 의혹으로 고발당해 국제신문한동훈이 자초한 3개의 '사법 리스크' OhmyNews.</t>
+          <t>14일 오후 3시께 제주시 애월읍 평화로에서 차량 12대 가 잇따라 추돌했다.</t>
         </is>
       </c>
       <c r="F89" s="3" t="inlineStr">
         <is>
-          <t>한겨레</t>
+          <t>주요언론</t>
         </is>
       </c>
       <c r="G89" s="3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMickFVX3lxTE15T3V6NzcweXpta2U4ckpqX05XU21wRlgxQ0ltZ1dlejY5ZGgzbzFvaFF5OTBSZlQwcGRBUW1YWXRQdWV0VWU5Wk44azVOVUFtSzljaXJ0WDVpOWhzWTk4MVZzNEFWQnJucl9ldElENVV0QQ?oc=5</t>
+          <t>https://www.yna.co.kr/view/AKR20261014135000056</t>
         </is>
       </c>
     </row>
@@ -3774,32 +3774,32 @@
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>사회/사건사고</t>
+          <t>거시경제/비즈니스</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>🔥 [언론사 집중 보도 (3개사)]</t>
+          <t>🔥 [언론사 집중 보도 (6개사)]</t>
         </is>
       </c>
       <c r="D90" s="3" t="inlineStr">
         <is>
-          <t>국가원로회의 부산지부, 15일 임시총회…지역 발전방안 논의</t>
+          <t>카카오, ‘모두의 AI’ 연내 공개 예정…월 이용자 500만 명 목표</t>
         </is>
       </c>
       <c r="E90" s="3" t="inlineStr">
         <is>
-          <t>각계 원로 인사 모임인 국가원로회의 부산지부는 15일 오전 10시 30분 부산 부산진구 초원농원 양정점에서 임...</t>
+          <t>카카오, ‘모두의 AI’ 연내 공개 예정월 이용자 500만 명 목표 KBS 뉴스카카오그룹, 인적분할 앞두고 주요 계열사 CEO 함께 모여 ‘첫 공동 IR’ 개최 카카오연말 출시 ‘모두의 AI’“카톡 익숙함. 활용할 것” 마켓 카카오, 웹툰·음원·카카오T에 스테이블코인 결제 연동소설 원작 AI 애니 제작도 전자신문카톡에 “메시지 정리, 답장 보내줘” 말하면 AI비서가 척척.</t>
         </is>
       </c>
       <c r="F90" s="3" t="inlineStr">
         <is>
-          <t>주요언론</t>
+          <t>KBS 뉴스</t>
         </is>
       </c>
       <c r="G90" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261014122000051</t>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE43NnU3MlhmZWZkcEdnRU1abkNDcHdIdG85YU9NZVBqVF90N3BXTHFCVlJIbDZQbkg3RGR5NWltZ29IaXNWNkdIWm1aYzBmLU4wbnVfd1hhVnlwdVk?oc=5</t>
         </is>
       </c>
     </row>
@@ -3816,17 +3816,17 @@
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>연결 이슈 (후속)</t>
+          <t>신규 이슈</t>
         </is>
       </c>
       <c r="D91" s="3" t="inlineStr">
         <is>
-          <t>제분업체 6곳, 사료 원료값 8년간 담합…과징금 최대 2100억원</t>
+          <t>대구 신세계 프리미엄 아울렛 건립 속도…인허가기간 절반 이하로</t>
         </is>
       </c>
       <c r="E91" s="3" t="inlineStr">
         <is>
-          <t>관련매출액 1조4000억원 조사 시작되자 담합 중단 공정위, 임직원 고발 의견대한제분과 CJ제일제당 등 제분업체 6곳이 8년 넘게 사료 원료로 쓰이는 밀가루 부산물의 판매가격을 담..</t>
+          <t>대구시가 신세계사이먼의 '대구 프리미엄 아울렛' 건립을 위한 인허가 기간을 통상의 절반 이하로 줄이는 등 사업.</t>
         </is>
       </c>
       <c r="F91" s="3" t="inlineStr">
@@ -3836,7 +3836,7 @@
       </c>
       <c r="G91" s="3" t="inlineStr">
         <is>
-          <t>https://www.mk.co.kr/news/economy/12175580</t>
+          <t>https://www.yna.co.kr/view/AKR20261014129100053</t>
         </is>
       </c>
     </row>
@@ -3848,32 +3848,32 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>IT/과학/신상품</t>
+          <t>거시경제/비즈니스</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>🔥 [언론사 집중 보도 (3개사)]</t>
+          <t>연결 이슈 (후속)</t>
         </is>
       </c>
       <c r="D92" s="3" t="inlineStr">
         <is>
-          <t>PS6, PS2와 PS3 게임 지원 전망 나왔다</t>
+          <t>토스뱅크, 디지털 취약계층에 노트북 기부</t>
         </is>
       </c>
       <c r="E92" s="3" t="inlineStr">
         <is>
-          <t>PS6, PS2와 PS3 게임 지원 전망 나왔다. 게임와이“어차피 사라질 운명” 사이버커넥트2 대표 디스크 폐지 찬성 게임메카새로운 보도에 따르면 소니는 플레이스테이션 6를 세 가지 구성으로 출시할 계획입니다.</t>
+          <t>토스뱅크가 고령층 문해학습자와 장애인 등 디지털 교육이 필요한 학습자를 지원하기 위해 업무용으로 사용하던 노트북 46대를 기부한다고 14일 밝혔다.</t>
         </is>
       </c>
       <c r="F92" s="3" t="inlineStr">
         <is>
-          <t>게임와이</t>
+          <t>주요언론</t>
         </is>
       </c>
       <c r="G92" s="3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiZ0FVX3lxTFBWN3pmQjJpeUtWZkg5dVBVTUNSYW9zUVV3OXdySkM5NnIzSk5oX0MxMUpsUm55UzdQX2lNaHFpdExPc1VGMHh5UV9SZk1YLUFJOXZ1SFVOOTVNSHpvdDZwTVBPZjg2NUHSAWpBVV95cUxPeGZzYXkzczlJbGRyWG9fSzl5YnhMWFdaT0EzNm5IU19tSGlvTGswSWJZREp3akxKWkxWTzNHR3pDVVBMUXNDenV2UjQ4ZmY1d2NnQkdvdV80UDA2SjcwdDg3TEVpOGtWYXlR?oc=5</t>
+          <t>https://www.mk.co.kr/news/economy/12175659</t>
         </is>
       </c>
     </row>
@@ -3885,22 +3885,22 @@
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>IT/과학/신상품</t>
+          <t>세계/국제</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>🔥 [언론사 집중 보도 (5개사)]</t>
+          <t>신규 이슈</t>
         </is>
       </c>
       <c r="D93" s="3" t="inlineStr">
         <is>
-          <t>GC녹십자, LG CNS와 스마트공장 구축…AI 자동화 추진</t>
+          <t>올해만 10대 선진국 10년물 국채금리 0.81%p 급등</t>
         </is>
       </c>
       <c r="E93" s="3" t="inlineStr">
         <is>
-          <t>GC녹십자가 LG CNS와 인공지능 기반 자동화·자율 운영 스마트 공장 구축을 추진한다.</t>
+          <t>국제 신용평가사 피치는 국채 금리 상승으로 프랑스, 미국, 영국 등 주요 선진국이 채무 부담을 안정적으로 유지.</t>
         </is>
       </c>
       <c r="F93" s="3" t="inlineStr">
@@ -3910,7 +3910,81 @@
       </c>
       <c r="G93" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261014121800017</t>
+          <t>https://www.yna.co.kr/view/AKR20261014133700009</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>연예/대중문화</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>신규 이슈</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="inlineStr">
+        <is>
+          <t>“칼로리에 깜짝” 악뮤 수현도 놀란 ‘최근 유행 디저트’ 정체</t>
+        </is>
+      </c>
+      <c r="E94" s="3" t="inlineStr">
+        <is>
+          <t>“칼로리에 깜짝” 악뮤 수현도 놀란 ‘최근 유행 디저트’ 정체 헬스조선‘30㎏ 감량 이수현’ 콘서트 끝나고 ‘한정선’ 먹자트레이너 “10㎞ 뛰어야” '-30kg' 악뮤 이수현, 콘서트 직후 디저트 흡입트레이너에 "말 걸지 마라" 미주30kg 감량한 이수현, ‘이 음식’ 먹자트레이너 “10km 달려야” 서울신문"3시간 줄 선다고?" 갸우뚱이수현, '한정선' 솔직 후기 -.</t>
+        </is>
+      </c>
+      <c r="F94" s="3" t="inlineStr">
+        <is>
+          <t>헬스조선</t>
+        </is>
+      </c>
+      <c r="G94" s="3" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMif0FVX3lxTFBldDBTc0RkSFJEOVQ5Y2o5bmJIY3gwaGQxZzZvVzZpRHdsX0RCZ3l3NS1oTm5iR0VERmYybWx4NGhSaGRMSFhXdnpPN1l0Y2JpalJ4WGZ0N3V5RHVKX2NUeF92NzVwOV9tenl5WDVyTXpjd281cHVuZmlGUkwzekU?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>연예/대중문화</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>🔥 [언론사 집중 보도 (4개사)]</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="inlineStr">
+        <is>
+          <t>“낙찰가 2400억, 역대 최고가 기대”…반 고흐 '꽃 핀 밤나무' 60년 만에 공개</t>
+        </is>
+      </c>
+      <c r="E95" s="3" t="inlineStr">
+        <is>
+          <t>“낙찰가 2400억, 역대 최고가 기대”반 고흐 '꽃 핀 밤나무' 60년 만에 공개 전자신문낙찰 예상가만 2400억60여 년 만에 공개 반고흐의 ‘꽃 핀 밤나무’ KBS 뉴스고흐 말년작 60년만에 공개내달 경매 2400억원 예상 동아일보홍콩서 60여년 만에 반고흐 '꽃 핀 밤나무' 공개수백명 몰려 60년만에 세상 나온 반고흐 명작'경매가 2400억' 신기록 전망 뉴스1.</t>
+        </is>
+      </c>
+      <c r="F95" s="3" t="inlineStr">
+        <is>
+          <t>전자신문</t>
+        </is>
+      </c>
+      <c r="G95" s="3" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiTkFVX3lxTE80XzRkdG90QUU3QUtFbVJUcEJmNVhja2ZjYnRoY09GRUI3WjJfZzZFY1NkbVlwXzJTYWVUUVpfcG5oTVFENHVXbTFJQTRaZw?oc=5</t>
         </is>
       </c>
     </row>
@@ -5252,17 +5326,17 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>236,000원</t>
+          <t>232,500원</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>+29,500.0원 (+14.29%)</t>
+          <t>+26,000.0원 (+12.59%)</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>233,500원</t>
+          <t>230,000원</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
@@ -5272,12 +5346,12 @@
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>227,500원</t>
+          <t>224,500원</t>
         </is>
       </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
-          <t>+10.0%</t>
+          <t>+11.6%</t>
         </is>
       </c>
       <c r="K15" s="3" t="inlineStr">
@@ -5287,7 +5361,7 @@
       </c>
       <c r="L15" s="3" t="inlineStr">
         <is>
-          <t>RSI 37.0로 단기 과매도 구간 도달 및 지지선 부근 기술적 반등 기대 (거래량비율 0.66x)</t>
+          <t>RSI 34.7로 단기 과매도 구간 도달 및 지지선 부근 기술적 반등 기대 (거래량비율 0.82x)</t>
         </is>
       </c>
       <c r="M15" s="3" t="inlineStr">
@@ -5301,16 +5375,16 @@
         </is>
       </c>
       <c r="O15" s="3" t="n">
-        <v>37</v>
+        <v>34.7</v>
       </c>
       <c r="P15" s="3" t="inlineStr">
         <is>
-          <t>-10.0%</t>
+          <t>-11.3%</t>
         </is>
       </c>
       <c r="Q15" s="3" t="inlineStr">
         <is>
-          <t>51.0%</t>
+          <t>49.7%</t>
         </is>
       </c>
       <c r="R15" s="3" t="inlineStr">
@@ -5320,7 +5394,7 @@
       </c>
       <c r="S15" s="3" t="inlineStr">
         <is>
-          <t>[259500.0, 249000.0, 248500.0, 253500.0, 252500.0, 261000.0, 274000.0, 276500.0, 285500.0, 270000.0, 272500.0, 268500.0, 276000.0, 276000.0, 272000.0, 268500.0, 262000.0, 250500.0, 232000.0, 236000.0]</t>
+          <t>[259500.0, 249000.0, 248500.0, 253500.0, 252500.0, 261000.0, 274000.0, 276500.0, 285500.0, 270000.0, 272500.0, 268500.0, 276000.0, 276000.0, 272000.0, 268500.0, 262000.0, 250500.0, 232000.0, 232500.0]</t>
         </is>
       </c>
     </row>
@@ -5347,17 +5421,17 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>1,439,000원</t>
+          <t>1,419,000원</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>+336,000.0원 (+30.46%)</t>
+          <t>+316,000.0원 (+28.65%)</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>1,410,000원</t>
+          <t>1,390,500원</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
@@ -5367,12 +5441,12 @@
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>1,367,000원</t>
+          <t>1,348,000원</t>
         </is>
       </c>
       <c r="J16" s="3" t="inlineStr">
         <is>
-          <t>+32.5%</t>
+          <t>+34.3%</t>
         </is>
       </c>
       <c r="K16" s="3" t="inlineStr">
@@ -5396,16 +5470,16 @@
         </is>
       </c>
       <c r="O16" s="3" t="n">
-        <v>31.2</v>
+        <v>30.5</v>
       </c>
       <c r="P16" s="3" t="inlineStr">
         <is>
-          <t>-17.2%</t>
+          <t>-18.4%</t>
         </is>
       </c>
       <c r="Q16" s="3" t="inlineStr">
         <is>
-          <t>40.0%</t>
+          <t>39.2%</t>
         </is>
       </c>
       <c r="R16" s="3" t="inlineStr">
@@ -5415,7 +5489,7 @@
       </c>
       <c r="S16" s="3" t="inlineStr">
         <is>
-          <t>[1812000.0, 1697000.0, 1690000.0, 1759000.0, 1745000.0, 1857000.0, 1868000.0, 1840000.0, 1862000.0, 1768000.0, 1765000.0, 1776000.0, 1833000.0, 1841000.0, 1773000.0, 1723000.0, 1681000.0, 1605000.0, 1443000.0, 1439000.0]</t>
+          <t>[1812000.0, 1697000.0, 1690000.0, 1759000.0, 1745000.0, 1857000.0, 1868000.0, 1840000.0, 1862000.0, 1768000.0, 1765000.0, 1776000.0, 1833000.0, 1841000.0, 1773000.0, 1723000.0, 1681000.0, 1605000.0, 1443000.0, 1419000.0]</t>
         </is>
       </c>
     </row>
@@ -5442,32 +5516,32 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>316,000원</t>
+          <t>314,000원</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>-175,500.0원 (-35.71%)</t>
+          <t>-177,500.0원 (-36.11%)</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>299,000원</t>
+          <t>298,500원</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>313,000원</t>
+          <t>311,000원</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>306,500원</t>
+          <t>304,500원</t>
         </is>
       </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
-          <t>+4.5%</t>
+          <t>+4.2%</t>
         </is>
       </c>
       <c r="K17" s="3" t="inlineStr">
@@ -5477,7 +5551,7 @@
       </c>
       <c r="L17" s="3" t="inlineStr">
         <is>
-          <t>주가가 20일선(349,425원)을 하향 이탈하고 이동평균선 역배열 지속. 리스크 관리 차원 비중 축소 권고</t>
+          <t>주가가 20일선(349,325원)을 하향 이탈하고 이동평균선 역배열 지속. 리스크 관리 차원 비중 축소 권고</t>
         </is>
       </c>
       <c r="M17" s="3" t="inlineStr">
@@ -5491,16 +5565,16 @@
         </is>
       </c>
       <c r="O17" s="3" t="n">
-        <v>22.9</v>
+        <v>21.6</v>
       </c>
       <c r="P17" s="3" t="inlineStr">
         <is>
-          <t>-9.6%</t>
+          <t>-10.1%</t>
         </is>
       </c>
       <c r="Q17" s="3" t="inlineStr">
         <is>
-          <t>17.1%</t>
+          <t>16.7%</t>
         </is>
       </c>
       <c r="R17" s="3" t="inlineStr">
@@ -5510,7 +5584,7 @@
       </c>
       <c r="S17" s="3" t="inlineStr">
         <is>
-          <t>[382500.0, 371500.0, 367000.0, 362000.0, 363000.0, 365000.0, 359000.0, 360500.0, 353500.0, 354500.0, 350000.0, 345000.0, 349000.0, 346500.0, 348000.0, 336000.0, 324500.0, 320000.0, 315000.0, 316000.0]</t>
+          <t>[382500.0, 371500.0, 367000.0, 362000.0, 363000.0, 365000.0, 359000.0, 360500.0, 353500.0, 354500.0, 350000.0, 345000.0, 349000.0, 346500.0, 348000.0, 336000.0, 324500.0, 320000.0, 315000.0, 314000.0]</t>
         </is>
       </c>
     </row>
@@ -5537,42 +5611,42 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>109,000원</t>
+          <t>108,500원</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>-40,100.0원 (-26.88%)</t>
+          <t>-40,800.0원 (-27.35%)</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>107,000원</t>
+          <t>101,500원</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>126,500원</t>
+          <t>107,500원</t>
         </is>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>103,500원</t>
+          <t>105,000원</t>
         </is>
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>+18.4%</t>
+          <t>+5.8%</t>
         </is>
       </c>
       <c r="K18" s="3" t="inlineStr">
         <is>
-          <t>관망 (HOLD)</t>
+          <t>🔴 단기 비중 축소 (추세 이탈 경고)</t>
         </is>
       </c>
       <c r="L18" s="3" t="inlineStr">
         <is>
-          <t>중립 구간 유지 중</t>
+          <t>주가가 20일선(115,820원)을 하향 이탈하고 이동평균선 역배열 지속. 리스크 관리 차원 비중 축소 권고</t>
         </is>
       </c>
       <c r="M18" s="3" t="inlineStr">
@@ -5586,16 +5660,16 @@
         </is>
       </c>
       <c r="O18" s="3" t="n">
-        <v>31.3</v>
+        <v>29.3</v>
       </c>
       <c r="P18" s="3" t="inlineStr">
         <is>
-          <t>-5.8%</t>
+          <t>-6.4%</t>
         </is>
       </c>
       <c r="Q18" s="3" t="inlineStr">
         <is>
-          <t>6.6%</t>
+          <t>6.0%</t>
         </is>
       </c>
       <c r="R18" s="3" t="inlineStr">
@@ -5605,7 +5679,7 @@
       </c>
       <c r="S18" s="3" t="inlineStr">
         <is>
-          <t>[126600.0, 124200.0, 121800.0, 120700.0, 120900.0, 121900.0, 120000.0, 118500.0, 115400.0, 117600.0, 116000.0, 112800.0, 113300.0, 112900.0, 112600.0, 109600.0, 106800.0, 108100.0, 108300.0, 109100.0]</t>
+          <t>[126600.0, 124200.0, 121800.0, 120700.0, 120900.0, 121900.0, 120000.0, 118500.0, 115400.0, 117600.0, 116000.0, 112800.0, 113300.0, 112900.0, 112600.0, 109600.0, 106800.0, 108100.0, 108300.0, 108400.0]</t>
         </is>
       </c>
     </row>
@@ -5632,12 +5706,12 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>181,000원</t>
+          <t>180,000원</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>-20,600.0원 (-10.22%)</t>
+          <t>-21,700.0원 (-10.77%)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -5647,17 +5721,17 @@
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>179,000원</t>
+          <t>178,000원</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>175,500원</t>
+          <t>174,500원</t>
         </is>
       </c>
       <c r="J19" s="3" t="inlineStr">
         <is>
-          <t>+5.9%</t>
+          <t>+5.3%</t>
         </is>
       </c>
       <c r="K19" s="3" t="inlineStr">
@@ -5667,7 +5741,7 @@
       </c>
       <c r="L19" s="3" t="inlineStr">
         <is>
-          <t>주가가 20일선(194,060원)을 하향 이탈하고 이동평균선 역배열 지속. 리스크 관리 차원 비중 축소 권고</t>
+          <t>주가가 20일선(194,005원)을 하향 이탈하고 이동평균선 역배열 지속. 리스크 관리 차원 비중 축소 권고</t>
         </is>
       </c>
       <c r="M19" s="3" t="inlineStr">
@@ -5681,16 +5755,16 @@
         </is>
       </c>
       <c r="O19" s="3" t="n">
-        <v>31.5</v>
+        <v>29.8</v>
       </c>
       <c r="P19" s="3" t="inlineStr">
         <is>
-          <t>-6.8%</t>
+          <t>-7.3%</t>
         </is>
       </c>
       <c r="Q19" s="3" t="inlineStr">
         <is>
-          <t>5.9%</t>
+          <t>5.0%</t>
         </is>
       </c>
       <c r="R19" s="3" t="inlineStr">
@@ -5700,7 +5774,7 @@
       </c>
       <c r="S19" s="3" t="inlineStr">
         <is>
-          <t>[206500.0, 204000.0, 206000.0, 201500.0, 199000.0, 197700.0, 197900.0, 201000.0, 194700.0, 197700.0, 194800.0, 193700.0, 191200.0, 192200.0, 191100.0, 189000.0, 183800.0, 180500.0, 178000.0, 180900.0]</t>
+          <t>[206500.0, 204000.0, 206000.0, 201500.0, 199000.0, 197700.0, 197900.0, 201000.0, 194700.0, 197700.0, 194800.0, 193700.0, 191200.0, 192200.0, 191100.0, 189000.0, 183800.0, 180500.0, 178000.0, 179800.0]</t>
         </is>
       </c>
     </row>
@@ -5727,17 +5801,17 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>32,000원</t>
+          <t>31,700원</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>-16,150.0원 (-33.58%)</t>
+          <t>-16,400.0원 (-34.10%)</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>31,300원</t>
+          <t>31,100원</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
@@ -5747,12 +5821,12 @@
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>30,400원</t>
+          <t>30,100원</t>
         </is>
       </c>
       <c r="J20" s="3" t="inlineStr">
         <is>
-          <t>+10.7%</t>
+          <t>+11.5%</t>
         </is>
       </c>
       <c r="K20" s="3" t="inlineStr">
@@ -5776,26 +5850,26 @@
         </is>
       </c>
       <c r="O20" s="3" t="n">
-        <v>34.9</v>
+        <v>32.4</v>
       </c>
       <c r="P20" s="3" t="inlineStr">
         <is>
-          <t>-4.3%</t>
+          <t>-5.0%</t>
         </is>
       </c>
       <c r="Q20" s="3" t="inlineStr">
         <is>
-          <t>4.3%</t>
+          <t>3.7%</t>
         </is>
       </c>
       <c r="R20" s="3" t="inlineStr">
         <is>
-          <t>최근 특이 뉴스 없음</t>
+          <t>카카오, ‘모두의 AI’ 연내 공개 예정…월 이용자 500만 명 목표 (KBS 뉴스)</t>
         </is>
       </c>
       <c r="S20" s="3" t="inlineStr">
         <is>
-          <t>[34500.0, 34650.0, 34500.0, 33500.0, 33500.0, 33550.0, 33200.0, 34150.0, 33450.0, 34150.0, 33700.0, 33550.0, 33550.0, 33450.0, 33500.0, 33050.0, 32300.0, 32000.0, 31300.0, 31950.0]</t>
+          <t>[34500.0, 34650.0, 34500.0, 33500.0, 33500.0, 33550.0, 33200.0, 34150.0, 33450.0, 34150.0, 33700.0, 33550.0, 33550.0, 33450.0, 33500.0, 33050.0, 32300.0, 32000.0, 31300.0, 31700.0]</t>
         </is>
       </c>
     </row>
@@ -5822,27 +5896,27 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>181,000원</t>
+          <t>180,000원</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>-8,819.049999999988원 (-4.65%)</t>
+          <t>-9,719.049999999988원 (-5.13%)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>177,000원</t>
+          <t>176,500원</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>190,000원</t>
+          <t>189,000원</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>172,000원</t>
+          <t>171,000원</t>
         </is>
       </c>
       <c r="J21" s="3" t="inlineStr">
@@ -5871,16 +5945,16 @@
         </is>
       </c>
       <c r="O21" s="3" t="n">
-        <v>47.5</v>
+        <v>45.5</v>
       </c>
       <c r="P21" s="3" t="inlineStr">
         <is>
-          <t>+0.6%</t>
+          <t>+0.1%</t>
         </is>
       </c>
       <c r="Q21" s="3" t="inlineStr">
         <is>
-          <t>27.7%</t>
+          <t>26.6%</t>
         </is>
       </c>
       <c r="R21" s="3" t="inlineStr">
@@ -5890,7 +5964,7 @@
       </c>
       <c r="S21" s="3" t="inlineStr">
         <is>
-          <t>[178200.0, 178800.0, 177500.0, 177200.0, 180300.0, 179400.0, 181400.0, 178500.0, 177400.0, 178300.0, 178900.0, 177700.0, 183600.0, 182600.0, 182400.0, 183500.0, 179600.0, 180400.0, 179700.0, 180800.0]</t>
+          <t>[178200.0, 178800.0, 177500.0, 177200.0, 180300.0, 179400.0, 181400.0, 178500.0, 177400.0, 178300.0, 178900.0, 177700.0, 183600.0, 182600.0, 182400.0, 183500.0, 179600.0, 180400.0, 179700.0, 179900.0]</t>
         </is>
       </c>
     </row>
@@ -6012,32 +6086,32 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>426,500원</t>
+          <t>420,500원</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>+26,500.0원 (+6.62%)</t>
+          <t>+20,500.0원 (+5.12%)</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>372,500원</t>
+          <t>372,000원</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>426,500원</t>
+          <t>420,500원</t>
         </is>
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>418,000원</t>
+          <t>412,000원</t>
         </is>
       </c>
       <c r="J23" s="3" t="inlineStr">
         <is>
-          <t>+14.5%</t>
+          <t>+13.0%</t>
         </is>
       </c>
       <c r="K23" s="3" t="inlineStr">
@@ -6047,7 +6121,7 @@
       </c>
       <c r="L23" s="3" t="inlineStr">
         <is>
-          <t>RSI 72.0, 20일선 이격도 +14.5%로 단기 과열권 진입. 욕심을 줄이고 분할 차익 실현 권고</t>
+          <t>RSI 70.6, 20일선 이격도 +13.0%로 단기 과열권 진입. 욕심을 줄이고 분할 차익 실현 권고</t>
         </is>
       </c>
       <c r="M23" s="3" t="inlineStr">
@@ -6061,16 +6135,16 @@
         </is>
       </c>
       <c r="O23" s="3" t="n">
-        <v>72</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="P23" s="3" t="inlineStr">
         <is>
-          <t>+14.5%</t>
+          <t>+13.0%</t>
         </is>
       </c>
       <c r="Q23" s="3" t="inlineStr">
         <is>
-          <t>57.5%</t>
+          <t>55.0%</t>
         </is>
       </c>
       <c r="R23" s="3" t="inlineStr">
@@ -6080,7 +6154,7 @@
       </c>
       <c r="S23" s="3" t="inlineStr">
         <is>
-          <t>[360000.0, 351500.0, 365500.0, 367000.0, 365000.0, 364000.0, 352000.0, 350500.0, 351500.0, 364000.0, 352500.0, 357000.0, 360500.0, 371000.0, 390000.0, 391000.0, 401000.0, 398000.0, 410000.0, 426500.0]</t>
+          <t>[360000.0, 351500.0, 365500.0, 367000.0, 365000.0, 364000.0, 352000.0, 350500.0, 351500.0, 364000.0, 352500.0, 357000.0, 360500.0, 371000.0, 390000.0, 391000.0, 401000.0, 398000.0, 410000.0, 420500.0]</t>
         </is>
       </c>
     </row>
@@ -6107,17 +6181,17 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>309,500원</t>
+          <t>307,500원</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>-52,000.0원 (-14.38%)</t>
+          <t>-54,000.0원 (-14.94%)</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>303,500원</t>
+          <t>301,500원</t>
         </is>
       </c>
       <c r="H24" s="3" t="inlineStr">
@@ -6127,12 +6201,12 @@
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>294,000원</t>
+          <t>292,000원</t>
         </is>
       </c>
       <c r="J24" s="3" t="inlineStr">
         <is>
-          <t>+10.1%</t>
+          <t>+10.8%</t>
         </is>
       </c>
       <c r="K24" s="3" t="inlineStr">
@@ -6156,16 +6230,16 @@
         </is>
       </c>
       <c r="O24" s="3" t="n">
-        <v>45.7</v>
+        <v>44.2</v>
       </c>
       <c r="P24" s="3" t="inlineStr">
         <is>
-          <t>-1.7%</t>
+          <t>-2.3%</t>
         </is>
       </c>
       <c r="Q24" s="3" t="inlineStr">
         <is>
-          <t>12.9%</t>
+          <t>12.2%</t>
         </is>
       </c>
       <c r="R24" s="3" t="inlineStr">
@@ -6175,7 +6249,7 @@
       </c>
       <c r="S24" s="3" t="inlineStr">
         <is>
-          <t>[334000.0, 326000.0, 332000.0, 326500.0, 326500.0, 323000.0, 317000.0, 317500.0, 311500.0, 316500.0, 304000.0, 306000.0, 306500.0, 311000.0, 318000.0, 307500.0, 306500.0, 299000.0, 299000.0, 309500.0]</t>
+          <t>[334000.0, 326000.0, 332000.0, 326500.0, 326500.0, 323000.0, 317000.0, 317500.0, 311500.0, 316500.0, 304000.0, 306000.0, 306500.0, 311000.0, 318000.0, 307500.0, 306500.0, 299000.0, 299000.0, 307500.0]</t>
         </is>
       </c>
     </row>
@@ -6202,7 +6276,7 @@
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>$228.52 (약 305,755원)</t>
+          <t>$228.52 (약 305,782원)</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
@@ -6212,12 +6286,12 @@
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>$223.95 (약 299,640원)</t>
+          <t>$223.95 (약 299,666원)</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
-          <t>$239.95 (약 321,042원)</t>
+          <t>$239.95 (약 321,071원)</t>
         </is>
       </c>
       <c r="I25" s="3" t="inlineStr">
@@ -6297,7 +6371,7 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>$341.27 (약 456,612원)</t>
+          <t>$341.27 (약 456,653원)</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
@@ -6307,12 +6381,12 @@
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>$334.44 (약 447,480원)</t>
+          <t>$334.44 (약 447,520원)</t>
         </is>
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
-          <t>$358.33 (약 479,443원)</t>
+          <t>$358.33 (약 479,486원)</t>
         </is>
       </c>
       <c r="I26" s="3" t="inlineStr">
@@ -6392,7 +6466,7 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>$375.23 (약 502,050원)</t>
+          <t>$375.23 (약 502,095원)</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
@@ -6402,12 +6476,12 @@
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>$367.73 (약 492,009원)</t>
+          <t>$367.73 (약 492,053원)</t>
         </is>
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>$393.99 (약 527,152원)</t>
+          <t>$393.99 (약 527,200원)</t>
         </is>
       </c>
       <c r="I27" s="3" t="inlineStr">
@@ -6487,7 +6561,7 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>$543.45 (약 727,125원)</t>
+          <t>$543.45 (약 727,190원)</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
@@ -6497,12 +6571,12 @@
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>$514.20 (약 687,989원)</t>
+          <t>$514.20 (약 688,051원)</t>
         </is>
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
-          <t>$543.45 (약 727,125원)</t>
+          <t>$543.45 (약 727,190원)</t>
         </is>
       </c>
       <c r="I28" s="3" t="inlineStr">
@@ -6582,17 +6656,17 @@
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>408,000원</t>
+          <t>403,500원</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>-93,000.0원 (-18.56%)</t>
+          <t>-97,500.0원 (-19.46%)</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>404,000원</t>
+          <t>399,500원</t>
         </is>
       </c>
       <c r="H29" s="3" t="inlineStr">
@@ -6602,12 +6676,12 @@
       </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>393,500원</t>
+          <t>389,500원</t>
         </is>
       </c>
       <c r="J29" s="3" t="inlineStr">
         <is>
-          <t>+19.7%</t>
+          <t>+21.0%</t>
         </is>
       </c>
       <c r="K29" s="3" t="inlineStr">
@@ -6617,7 +6691,7 @@
       </c>
       <c r="L29" s="3" t="inlineStr">
         <is>
-          <t>RSI 33.6로 단기 과매도 구간 도달 및 지지선 부근 기술적 반등 기대 (거래량비율 1.63x)</t>
+          <t>RSI 33.0로 단기 과매도 구간 도달 및 지지선 부근 기술적 반등 기대 (거래량비율 1.99x)</t>
         </is>
       </c>
       <c r="M29" s="3" t="inlineStr">
@@ -6631,16 +6705,16 @@
         </is>
       </c>
       <c r="O29" s="3" t="n">
-        <v>33.6</v>
+        <v>33</v>
       </c>
       <c r="P29" s="3" t="inlineStr">
         <is>
-          <t>-17.3%</t>
+          <t>-18.2%</t>
         </is>
       </c>
       <c r="Q29" s="3" t="inlineStr">
         <is>
-          <t>30.7%</t>
+          <t>29.4%</t>
         </is>
       </c>
       <c r="R29" s="3" t="inlineStr">
@@ -6650,7 +6724,7 @@
       </c>
       <c r="S29" s="3" t="inlineStr">
         <is>
-          <t>[464000.0, 474000.0, 496500.0, 502000.0, 515000.0, 503000.0, 505000.0, 502000.0, 520000.0, 504000.0, 507000.0, 499000.0, 497500.0, 506000.0, 523000.0, 534000.0, 480500.0, 474500.0, 453000.0, 408000.0]</t>
+          <t>[464000.0, 474000.0, 496500.0, 502000.0, 515000.0, 503000.0, 505000.0, 502000.0, 520000.0, 504000.0, 507000.0, 499000.0, 497500.0, 506000.0, 523000.0, 534000.0, 480500.0, 474500.0, 453000.0, 403500.0]</t>
         </is>
       </c>
     </row>
@@ -6677,27 +6751,27 @@
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>49,800원</t>
+          <t>50,200원</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>-14,400.0원 (-22.43%)</t>
+          <t>-14,000.0원 (-21.81%)</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>49,300원</t>
+          <t>49,700원</t>
         </is>
       </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
-          <t>52,800원</t>
+          <t>53,200원</t>
         </is>
       </c>
       <c r="I30" s="3" t="inlineStr">
         <is>
-          <t>48,100원</t>
+          <t>48,400원</t>
         </is>
       </c>
       <c r="J30" s="3" t="inlineStr">
@@ -6712,7 +6786,7 @@
       </c>
       <c r="L30" s="3" t="inlineStr">
         <is>
-          <t>RSI 32.1로 단기 과매도 구간 도달 및 지지선 부근 기술적 반등 기대 (거래량비율 0.53x)</t>
+          <t>RSI 35.8로 단기 과매도 구간 도달 및 지지선 부근 기술적 반등 기대 (거래량비율 0.81x)</t>
         </is>
       </c>
       <c r="M30" s="3" t="inlineStr">
@@ -6726,16 +6800,16 @@
         </is>
       </c>
       <c r="O30" s="3" t="n">
-        <v>32.1</v>
+        <v>35.8</v>
       </c>
       <c r="P30" s="3" t="inlineStr">
         <is>
-          <t>-4.5%</t>
+          <t>-3.8%</t>
         </is>
       </c>
       <c r="Q30" s="3" t="inlineStr">
         <is>
-          <t>8.0%</t>
+          <t>9.9%</t>
         </is>
       </c>
       <c r="R30" s="3" t="inlineStr">
@@ -6745,7 +6819,7 @@
       </c>
       <c r="S30" s="3" t="inlineStr">
         <is>
-          <t>[52700.0, 53200.0, 53000.0, 52800.0, 53400.0, 53000.0, 53100.0, 53100.0, 52700.0, 52900.0, 52900.0, 52300.0, 51800.0, 51900.0, 51500.0, 51300.0, 52100.0, 49900.0, 49750.0, 49800.0]</t>
+          <t>[52700.0, 53200.0, 53000.0, 52800.0, 53400.0, 53000.0, 53100.0, 53100.0, 52700.0, 52900.0, 52900.0, 52300.0, 51800.0, 51900.0, 51500.0, 51300.0, 52100.0, 49900.0, 49750.0, 50200.0]</t>
         </is>
       </c>
     </row>
@@ -6757,12 +6831,12 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>LG유플러스</t>
+          <t>SK텔레콤</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>032640.KS</t>
+          <t>017670.KS</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
@@ -6772,27 +6846,27 @@
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>14,700원</t>
+          <t>81,900원</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>-2,770.0원 (-15.86%)</t>
+          <t>-13,600.0원 (-14.24%)</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>14,400원</t>
+          <t>81,100원</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>15,400원</t>
+          <t>86,800원</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
         <is>
-          <t>14,000원</t>
+          <t>79,000원</t>
         </is>
       </c>
       <c r="J31" s="3" t="inlineStr">
@@ -6802,12 +6876,12 @@
       </c>
       <c r="K31" s="3" t="inlineStr">
         <is>
-          <t>관망 (HOLD)</t>
+          <t>🟢 오늘 단기 매수 (저점 과매도 반등)</t>
         </is>
       </c>
       <c r="L31" s="3" t="inlineStr">
         <is>
-          <t>중립 구간 유지 중</t>
+          <t>RSI 37.3로 단기 과매도 구간 도달 및 지지선 부근 기술적 반등 기대 (거래량비율 0.96x)</t>
         </is>
       </c>
       <c r="M31" s="3" t="inlineStr">
@@ -6821,16 +6895,16 @@
         </is>
       </c>
       <c r="O31" s="3" t="n">
-        <v>50.7</v>
+        <v>37.3</v>
       </c>
       <c r="P31" s="3" t="inlineStr">
         <is>
-          <t>+0.5%</t>
+          <t>-5.4%</t>
         </is>
       </c>
       <c r="Q31" s="3" t="inlineStr">
         <is>
-          <t>17.8%</t>
+          <t>34.6%</t>
         </is>
       </c>
       <c r="R31" s="3" t="inlineStr">
@@ -6840,7 +6914,7 @@
       </c>
       <c r="S31" s="3" t="inlineStr">
         <is>
-          <t>[14890.0, 15040.0, 14850.0, 14650.0, 14680.0, 14050.0, 14490.0, 14570.0, 14640.0, 14770.0, 14800.0, 14530.0, 14540.0, 14550.0, 14560.0, 14500.0, 14400.0, 14550.0, 14780.0, 14700.0]</t>
+          <t>[90900.0, 90100.0, 88000.0, 88100.0, 87600.0, 89200.0, 87000.0, 87300.0, 87100.0, 88200.0, 86200.0, 85600.0, 86300.0, 88400.0, 88400.0, 87400.0, 84100.0, 79700.0, 80000.0, 81900.0]</t>
         </is>
       </c>
     </row>
@@ -6852,12 +6926,12 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>SK텔레콤</t>
+          <t>LG유플러스</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>017670.KS</t>
+          <t>032640.KS</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -6867,27 +6941,27 @@
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>82,200원</t>
+          <t>14,800원</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>-13,300.0원 (-13.93%)</t>
+          <t>-2,700.0원 (-15.46%)</t>
         </is>
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>81,400원</t>
+          <t>14,500원</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr">
         <is>
-          <t>87,100원</t>
+          <t>15,500원</t>
         </is>
       </c>
       <c r="I32" s="3" t="inlineStr">
         <is>
-          <t>79,300원</t>
+          <t>14,000원</t>
         </is>
       </c>
       <c r="J32" s="3" t="inlineStr">
@@ -6897,12 +6971,12 @@
       </c>
       <c r="K32" s="3" t="inlineStr">
         <is>
-          <t>🟢 오늘 단기 매수 (저점 과매도 반등)</t>
+          <t>관망 (HOLD)</t>
         </is>
       </c>
       <c r="L32" s="3" t="inlineStr">
         <is>
-          <t>RSI 38.1로 단기 과매도 구간 도달 및 지지선 부근 기술적 반등 기대 (거래량비율 0.79x)</t>
+          <t>중립 구간 유지 중</t>
         </is>
       </c>
       <c r="M32" s="3" t="inlineStr">
@@ -6916,16 +6990,16 @@
         </is>
       </c>
       <c r="O32" s="3" t="n">
-        <v>38.1</v>
+        <v>52.5</v>
       </c>
       <c r="P32" s="3" t="inlineStr">
         <is>
-          <t>-5.1%</t>
+          <t>+0.9%</t>
         </is>
       </c>
       <c r="Q32" s="3" t="inlineStr">
         <is>
-          <t>35.0%</t>
+          <t>19.2%</t>
         </is>
       </c>
       <c r="R32" s="3" t="inlineStr">
@@ -6935,7 +7009,7 @@
       </c>
       <c r="S32" s="3" t="inlineStr">
         <is>
-          <t>[90900.0, 90100.0, 88000.0, 88100.0, 87600.0, 89200.0, 87000.0, 87300.0, 87100.0, 88200.0, 86200.0, 85600.0, 86300.0, 88400.0, 88400.0, 87400.0, 84100.0, 79700.0, 80000.0, 82200.0]</t>
+          <t>[14890.0, 15040.0, 14850.0, 14650.0, 14680.0, 14050.0, 14490.0, 14570.0, 14640.0, 14770.0, 14800.0, 14530.0, 14540.0, 14550.0, 14560.0, 14500.0, 14400.0, 14550.0, 14780.0, 14770.0]</t>
         </is>
       </c>
     </row>
@@ -6962,17 +7036,17 @@
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>76,000원</t>
+          <t>75,000원</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>-8,300.0원 (-9.85%)</t>
+          <t>-9,300.0원 (-11.03%)</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>74,500원</t>
+          <t>73,500원</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr">
@@ -6982,12 +7056,12 @@
       </c>
       <c r="I33" s="3" t="inlineStr">
         <is>
-          <t>72,200원</t>
+          <t>71,200원</t>
         </is>
       </c>
       <c r="J33" s="3" t="inlineStr">
         <is>
-          <t>+18.2%</t>
+          <t>+19.7%</t>
         </is>
       </c>
       <c r="K33" s="3" t="inlineStr">
@@ -7011,16 +7085,16 @@
         </is>
       </c>
       <c r="O33" s="3" t="n">
-        <v>49.4</v>
+        <v>48</v>
       </c>
       <c r="P33" s="3" t="inlineStr">
         <is>
-          <t>-2.1%</t>
+          <t>-3.3%</t>
         </is>
       </c>
       <c r="Q33" s="3" t="inlineStr">
         <is>
-          <t>33.4%</t>
+          <t>32.5%</t>
         </is>
       </c>
       <c r="R33" s="3" t="inlineStr">
@@ -7030,7 +7104,7 @@
       </c>
       <c r="S33" s="3" t="inlineStr">
         <is>
-          <t>[71000.0, 69700.0, 68400.0, 70400.0, 70200.0, 76600.0, 73000.0, 76500.0, 81700.0, 82100.0, 80900.0, 82500.0, 82900.0, 86200.0, 87900.0, 88000.0, 81400.0, 73800.0, 73400.0, 76000.0]</t>
+          <t>[71000.0, 69700.0, 68400.0, 70400.0, 70200.0, 76600.0, 73000.0, 76500.0, 81700.0, 82100.0, 80900.0, 82500.0, 82900.0, 86200.0, 87900.0, 88000.0, 81400.0, 73800.0, 73400.0, 75000.0]</t>
         </is>
       </c>
     </row>
@@ -7057,12 +7131,12 @@
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>19,200원</t>
+          <t>18,900원</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>-8,750.0원 (-31.36%)</t>
+          <t>-8,960.0원 (-32.11%)</t>
         </is>
       </c>
       <c r="G34" s="3" t="inlineStr">
@@ -7072,27 +7146,27 @@
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>22,100원</t>
+          <t>20,100원</t>
         </is>
       </c>
       <c r="I34" s="3" t="inlineStr">
         <is>
-          <t>18,200원</t>
+          <t>18,300원</t>
         </is>
       </c>
       <c r="J34" s="3" t="inlineStr">
         <is>
-          <t>+17.8%</t>
+          <t>+7.1%</t>
         </is>
       </c>
       <c r="K34" s="3" t="inlineStr">
         <is>
-          <t>관망 (HOLD)</t>
+          <t>🟢 오늘 단기 매수 (저점 과매도 반등)</t>
         </is>
       </c>
       <c r="L34" s="3" t="inlineStr">
         <is>
-          <t>중립 구간 유지 중</t>
+          <t>RSI 40.9로 단기 과매도 구간 도달 및 지지선 부근 기술적 반등 기대 (거래량비율 1.46x)</t>
         </is>
       </c>
       <c r="M34" s="3" t="inlineStr">
@@ -7106,16 +7180,16 @@
         </is>
       </c>
       <c r="O34" s="3" t="n">
-        <v>42.7</v>
+        <v>40.9</v>
       </c>
       <c r="P34" s="3" t="inlineStr">
         <is>
-          <t>-4.4%</t>
+          <t>-5.4%</t>
         </is>
       </c>
       <c r="Q34" s="3" t="inlineStr">
         <is>
-          <t>10.7%</t>
+          <t>9.5%</t>
         </is>
       </c>
       <c r="R34" s="3" t="inlineStr">
@@ -7125,7 +7199,7 @@
       </c>
       <c r="S34" s="3" t="inlineStr">
         <is>
-          <t>[21400.0, 22100.0, 20700.0, 20200.0, 21500.0, 20800.0, 20600.0, 20600.0, 20250.0, 20100.0, 19330.0, 19700.0, 19720.0, 19960.0, 19700.0, 19540.0, 18860.0, 18010.0, 18360.0, 19150.0]</t>
+          <t>[21400.0, 22100.0, 20700.0, 20200.0, 21500.0, 20800.0, 20600.0, 20600.0, 20250.0, 20100.0, 19330.0, 19700.0, 19720.0, 19960.0, 19700.0, 19540.0, 18860.0, 18010.0, 18360.0, 18940.0]</t>
         </is>
       </c>
     </row>
@@ -7152,42 +7226,42 @@
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>584,000원</t>
+          <t>582,000원</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>+94,500.0원 (+19.31%)</t>
+          <t>+92,500.0원 (+18.90%)</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>578,000원</t>
+          <t>553,000원</t>
         </is>
       </c>
       <c r="H35" s="3" t="inlineStr">
         <is>
-          <t>629,500원</t>
+          <t>576,000원</t>
         </is>
       </c>
       <c r="I35" s="3" t="inlineStr">
         <is>
-          <t>563,500원</t>
+          <t>564,500원</t>
         </is>
       </c>
       <c r="J35" s="3" t="inlineStr">
         <is>
-          <t>+8.9%</t>
+          <t>+4.2%</t>
         </is>
       </c>
       <c r="K35" s="3" t="inlineStr">
         <is>
-          <t>🟢 오늘 단기 매수 (저점 과매도 반등)</t>
+          <t>🔴 단기 비중 축소 (추세 이탈 경고)</t>
         </is>
       </c>
       <c r="L35" s="3" t="inlineStr">
         <is>
-          <t>RSI 34.1로 단기 과매도 구간 도달 및 지지선 부근 기술적 반등 기대 (거래량비율 0.85x)</t>
+          <t>주가가 20일선(642,100원)을 하향 이탈하고 이동평균선 역배열 지속. 리스크 관리 차원 비중 축소 권고</t>
         </is>
       </c>
       <c r="M35" s="3" t="inlineStr">
@@ -7201,16 +7275,16 @@
         </is>
       </c>
       <c r="O35" s="3" t="n">
-        <v>34.1</v>
+        <v>33.7</v>
       </c>
       <c r="P35" s="3" t="inlineStr">
         <is>
-          <t>-9.1%</t>
+          <t>-9.4%</t>
         </is>
       </c>
       <c r="Q35" s="3" t="inlineStr">
         <is>
-          <t>48.8%</t>
+          <t>48.2%</t>
         </is>
       </c>
       <c r="R35" s="3" t="inlineStr">
@@ -7220,7 +7294,7 @@
       </c>
       <c r="S35" s="3" t="inlineStr">
         <is>
-          <t>[686000.0, 675000.0, 661000.0, 661000.0, 666000.0, 648000.0, 651000.0, 655000.0, 648000.0, 661000.0, 653000.0, 633000.0, 626000.0, 626000.0, 635000.0, 629000.0, 612000.0, 622000.0, 612000.0, 584000.0]</t>
+          <t>[686000.0, 675000.0, 661000.0, 661000.0, 666000.0, 648000.0, 651000.0, 655000.0, 648000.0, 661000.0, 653000.0, 633000.0, 626000.0, 626000.0, 635000.0, 629000.0, 612000.0, 622000.0, 612000.0, 582000.0]</t>
         </is>
       </c>
     </row>
@@ -7547,12 +7621,12 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>6,068.91</t>
+          <t>5,997.24</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>▲ +33.56 (+0.56%)</t>
+          <t>▼ -38.11 (-0.63%)</t>
         </is>
       </c>
     </row>
@@ -7574,12 +7648,12 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>831.05</t>
+          <t>820.32</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>▼ -18.14 (-2.14%)</t>
+          <t>▼ -28.87 (-3.40%)</t>
         </is>
       </c>
     </row>
@@ -7655,12 +7729,12 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>1,337.98</t>
+          <t>1,338.10</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>▼ -2.15원 (-0.16%)</t>
+          <t>▼ -2.03원 (-0.15%)</t>
         </is>
       </c>
     </row>
@@ -7682,12 +7756,12 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>842.80</t>
+          <t>843.10</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>▼ -1.30원 (-0.15%)</t>
+          <t>▼ -1.00원 (-0.12%)</t>
         </is>
       </c>
     </row>
@@ -7709,12 +7783,12 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>1,498.50</t>
+          <t>1,498.90</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>▼ -1.40원 (-0.09%)</t>
+          <t>▼ -1.00원 (-0.07%)</t>
         </is>
       </c>
     </row>
@@ -7736,12 +7810,12 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>199.96</t>
+          <t>200.02</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>▼ -0.25원 (-0.13%)</t>
+          <t>▼ -0.19원 (-0.10%)</t>
         </is>
       </c>
     </row>
@@ -7847,27 +7921,27 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>112,763,000원</t>
+          <t>112,687,000원</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>+0.15%</t>
+          <t>+0.08%</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>112,199,000원</t>
+          <t>112,124,000원</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>121,784,000원</t>
+          <t>121,702,000원</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>110,584,000원</t>
+          <t>110,580,000원</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
@@ -7939,7 +8013,7 @@
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>RSI 46.5로 단기 과매도 구간 진입, 기술적 반등 기대</t>
+          <t>RSI 46.4로 단기 과매도 구간 진입, 기술적 반등 기대</t>
         </is>
       </c>
     </row>
@@ -7961,17 +8035,17 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>144,700원</t>
+          <t>144,800원</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>+0.07%</t>
+          <t>+0.14%</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>143,500원</t>
+          <t>143,600원</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -7981,12 +8055,12 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>139,600원</t>
+          <t>139,700원</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>+8.6%</t>
+          <t>+8.5%</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
@@ -7996,7 +8070,7 @@
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>RSI 46.8로 단기 과매도 구간 진입, 기술적 반등 기대</t>
+          <t>RSI 47.0로 단기 과매도 구간 진입, 기술적 반등 기대</t>
         </is>
       </c>
     </row>
@@ -8179,7 +8253,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
@@ -8328,12 +8402,12 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>LG유플러스</t>
+          <t>SK텔레콤</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>3Q 프리뷰 - 특별한 대안 없다면 길게 보세요</t>
+          <t>3Q 프리뷰 - DPS 증가 기대감 커지는 계기될 것</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -8348,37 +8422,37 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>매수 투자의견/TP 20,000원 유지, 매도하기보단 배당 감안한 중/장기 매수 추천 LGU+에 대한 투자의견 매수, 12개월 목표주가 20,000원을 유지한다. 추천 사유는 1) 2분기에 이어 3분기에도 우수한 실적을 기록할 것으로 전망됨에 따라 2026년 연간 높은 연결 영업이익 성장 가능성이 높아졌고, 2) 양호한 실적 전망을 바탕으로 2027년도엔 다시 주주환원 증대 기대감이 높아질 전망이며, 3) 조만간 정책 금리 상승이 마무리되고 시중 금리가 하락 전환하면서 연말 이후 4.8%에 달하는 기대배당수익률이 매력적으로 인식될 수 있을 것이기 때문이다. 당장 특별한 재료가 부각될 수 있는 상황은 아니지만 국내 주식 시장이 강한 상승 탄력을 나타나고 있지 않은 점을 감안하면 차라리 매도하기 보단 2027년 초까지 LGU+ 보유 또는 배당을 염두에 둔 신규 매수 진입을 추천한다.</t>
+          <t>더불어 국내 통신서비스 업종 12개월/10월 Top Pick으로 제시한다. 추천 사유는 1) 3분기 실적도 양호할 전망이라 2026년 연간 연결 영업이익이 2조원에 육박할 전망이고, 2) 2026년 우수한 실적을 바탕으로 DPS가 2024년 수준으로 회귀할 전망이며, 3) 엔트로픽 상장 가치가 당초 기대를 뛰어넘을 것으로 보여 밸류에이션상 저평가 논란이 생겨날 것이고, 4) 금리 인상 기조가 마무리되고 SKT 비과세 배당이 시작되는 2026년 말/2027년 초부터는 수급 개선이 예상되기 때문이다.</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>2026-10-14_하나증권_LG유플러스_3Q 프리뷰 - 특별한 대안 없다면 길게 보세요.pdf</t>
+          <t>2026-10-14_하나증권_SK텔레콤_3Q 프리뷰 - DPS 증가 기대감 커지는 계기될 것.pdf</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>15,429.4십억원</t>
+          <t>17,658.0십억원</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>1,144.2십억원</t>
+          <t>1,950.1십억원</t>
         </is>
       </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>16,347.1십억원</t>
+          <t>18,217.8십억원</t>
         </is>
       </c>
       <c r="M5" s="3" t="inlineStr">
         <is>
-          <t>1,185.5십억원</t>
+          <t>2,013.5십억원</t>
         </is>
       </c>
       <c r="N5" s="3" t="inlineStr">
         <is>
-          <t>연결 영업이익 3,221억원 전망, 4Q 인센티브 반영 고려해도 올해 실적 좋을 것</t>
+          <t>2026년 연간 연결 영업이익이 2조원에 육박할 전망이고, 2) 2026년 우수한 실적을 바탕으</t>
         </is>
       </c>
     </row>
@@ -8389,7 +8463,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -8398,12 +8472,12 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>SK텔레콤</t>
+          <t>LG유플러스</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>3Q 프리뷰 - DPS 증가 기대감 커지는 계기될 것</t>
+          <t>3Q 프리뷰 - 특별한 대안 없다면 길게 보세요</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -8418,37 +8492,37 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>더불어 국내 통신서비스 업종 12개월/10월 Top Pick으로 제시한다. 추천 사유는 1) 3분기 실적도 양호할 전망이라 2026년 연간 연결 영업이익이 2조원에 육박할 전망이고, 2) 2026년 우수한 실적을 바탕으로 DPS가 2024년 수준으로 회귀할 전망이며, 3) 엔트로픽 상장 가치가 당초 기대를 뛰어넘을 것으로 보여 밸류에이션상 저평가 논란이 생겨날 것이고, 4) 금리 인상 기조가 마무리되고 SKT 비과세 배당이 시작되는 2026년 말/2027년 초부터는 수급 개선이 예상되기 때문이다.</t>
+          <t>매수 투자의견/TP 20,000원 유지, 매도하기보단 배당 감안한 중/장기 매수 추천 LGU+에 대한 투자의견 매수, 12개월 목표주가 20,000원을 유지한다. 추천 사유는 1) 2분기에 이어 3분기에도 우수한 실적을 기록할 것으로 전망됨에 따라 2026년 연간 높은 연결 영업이익 성장 가능성이 높아졌고, 2) 양호한 실적 전망을 바탕으로 2027년도엔 다시 주주환원 증대 기대감이 높아질 전망이며, 3) 조만간 정책 금리 상승이 마무리되고 시중 금리가 하락 전환하면서 연말 이후 4.8%에 달하는 기대배당수익률이 매력적으로 인식될 수 있을 것이기 때문이다. 당장 특별한 재료가 부각될 수 있는 상황은 아니지만 국내 주식 시장이 강한 상승 탄력을 나타나고 있지 않은 점을 감안하면 차라리 매도하기 보단 2027년 초까지 LGU+ 보유 또는 배당을 염두에 둔 신규 매수 진입을 추천한다.</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>2026-10-14_하나증권_SK텔레콤_3Q 프리뷰 - DPS 증가 기대감 커지는 계기될 것.pdf</t>
+          <t>2026-10-14_하나증권_LG유플러스_3Q 프리뷰 - 특별한 대안 없다면 길게 보세요.pdf</t>
         </is>
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>17,658.0십억원</t>
+          <t>15,429.4십억원</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>1,950.1십억원</t>
+          <t>1,144.2십억원</t>
         </is>
       </c>
       <c r="L6" s="3" t="inlineStr">
         <is>
-          <t>18,217.8십억원</t>
+          <t>16,347.1십억원</t>
         </is>
       </c>
       <c r="M6" s="3" t="inlineStr">
         <is>
-          <t>2,013.5십억원</t>
+          <t>1,185.5십억원</t>
         </is>
       </c>
       <c r="N6" s="3" t="inlineStr">
         <is>
-          <t>2026년 연간 연결 영업이익이 2조원에 육박할 전망이고, 2) 2026년 우수한 실적을 바탕으</t>
+          <t>연결 영업이익 3,221억원 전망, 4Q 인센티브 반영 고려해도 올해 실적 좋을 것</t>
         </is>
       </c>
     </row>
@@ -8813,16 +8887,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="21" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="32" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
@@ -8940,7 +9014,7 @@
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>+1.1%</t>
+          <t>+0.5%</t>
         </is>
       </c>
       <c r="K2" s="3" t="inlineStr">
@@ -9002,7 +9076,7 @@
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>+2.0%</t>
+          <t>+1.2%</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
@@ -9064,7 +9138,7 @@
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>+2.7%</t>
+          <t>+2.2%</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
@@ -9126,7 +9200,7 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>+3.2%</t>
+          <t>+2.4%</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
@@ -9250,7 +9324,7 @@
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>+4.6%</t>
+          <t>+4.1%</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
@@ -9287,22 +9361,22 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>236,500원</t>
+          <t>231,500원</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>234,000원</t>
+          <t>229,000원</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>257,000원</t>
+          <t>256,500원</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>228,000원</t>
+          <t>223,500원</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
@@ -9312,12 +9386,12 @@
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>+0.7%</t>
+          <t>+1.6%</t>
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>235,750원</t>
+          <t>232,750원</t>
         </is>
       </c>
       <c r="L8" s="3" t="inlineStr">
@@ -9339,32 +9413,32 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>한미약품</t>
+          <t>엔비디아 (NVIDIA)</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>128940.KS</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>409,000원</t>
+          <t>$228.52 (약 305,908원)</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>405,000원</t>
+          <t>$228.52 (약 305,908원)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>483,500원</t>
+          <t>$246.80 (약 330,380원)</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>394,500원</t>
+          <t>$219.38</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
@@ -9374,12 +9448,12 @@
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>+0.7%</t>
+          <t>+0.0%</t>
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>408,000원</t>
+          <t>$228.52</t>
         </is>
       </c>
       <c r="L9" s="3" t="inlineStr">
@@ -9401,32 +9475,32 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>KT</t>
+          <t>애플 (Apple)</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>030200.KS</t>
+          <t>AAPL</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>49,800원</t>
+          <t>$341.27 (약 456,841원)</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>49,300원</t>
+          <t>$341.27 (약 456,841원)</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>52,700원</t>
+          <t>$368.57 (약 493,388원)</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>48,000원</t>
+          <t>$327.62</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr">
@@ -9436,12 +9510,12 @@
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>+1.0%</t>
+          <t>+0.0%</t>
         </is>
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>49,800원</t>
+          <t>$341.27</t>
         </is>
       </c>
       <c r="L10" s="3" t="inlineStr">
@@ -9463,32 +9537,32 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>SK텔레콤</t>
+          <t>한미약품</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>017670.KS</t>
+          <t>128940.KS</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>82,200원</t>
+          <t>400,000원</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>81,400원</t>
+          <t>396,000원</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>87,100원</t>
+          <t>483,000원</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>79,300원</t>
+          <t>386,000원</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
@@ -9498,12 +9572,12 @@
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>+1.0%</t>
+          <t>+1.8%</t>
         </is>
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>82,200원</t>
+          <t>403,000원</t>
         </is>
       </c>
       <c r="L11" s="3" t="inlineStr">
@@ -9525,50 +9599,236 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
+          <t>KT</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>030200.KS</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>50,000원</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>49,500원</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>52,900원</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>48,200원</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>⏳ 목표가 추적 중 (신규 진입)</t>
+        </is>
+      </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>+1.4%</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="inlineStr">
+        <is>
+          <t>50,200원</t>
+        </is>
+      </c>
+      <c r="L12" s="3" t="inlineStr">
+        <is>
+          <t>1일차</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>SK텔레콤</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>017670.KS</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>81,600원</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>80,800원</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>86,500원</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>78,700원</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>⏳ 목표가 추적 중 (신규 진입)</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>+1.4%</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>81,900원</t>
+        </is>
+      </c>
+      <c r="L13" s="3" t="inlineStr">
+        <is>
+          <t>1일차</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>삼성중공업</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>010140.KS</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>18,900원</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>18,700원</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>20,000원</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>18,200원</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>⏳ 목표가 추적 중 (신규 진입)</t>
+        </is>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>+1.2%</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t>18,920원</t>
+        </is>
+      </c>
+      <c r="L14" s="3" t="inlineStr">
+        <is>
+          <t>1일차</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
           <t>삼성화재</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="D15" s="3" t="inlineStr">
         <is>
           <t>000810.KS</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>584,000원</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>578,000원</t>
-        </is>
-      </c>
-      <c r="G12" s="3" t="inlineStr">
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>583,000원</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>577,000원</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
         <is>
           <t>629,500원</t>
         </is>
       </c>
-      <c r="H12" s="3" t="inlineStr">
-        <is>
-          <t>563,500원</t>
-        </is>
-      </c>
-      <c r="I12" s="3" t="inlineStr">
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>562,500원</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
         <is>
           <t>⏳ 목표가 추적 중 (신규 진입)</t>
         </is>
       </c>
-      <c r="J12" s="3" t="inlineStr">
-        <is>
-          <t>+1.0%</t>
-        </is>
-      </c>
-      <c r="K12" s="3" t="inlineStr">
-        <is>
-          <t>584,000원</t>
-        </is>
-      </c>
-      <c r="L12" s="3" t="inlineStr">
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>+0.9%</t>
+        </is>
+      </c>
+      <c r="K15" s="3" t="inlineStr">
+        <is>
+          <t>582,000원</t>
+        </is>
+      </c>
+      <c r="L15" s="3" t="inlineStr">
         <is>
           <t>1일차</t>
         </is>
@@ -10334,32 +10594,32 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>🌐 [경제·사회 심층 리포트] GC녹십자의 숨겨진 배경과 구조적 쟁점</t>
+          <t>🌐 [경제·사회 심층 리포트] 카카오의 숨겨진 배경과 구조적 쟁점</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>GC녹십자</t>
+          <t>카카오</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>단순 뉴스 헤드라인을 넘어선 전후 맥락: 'GC녹십자' 이슈가 촉발된 진짜 배경과 이해관계자들의 득실 계산을 분석합니다.</t>
+          <t>단순 뉴스 헤드라인을 넘어선 전후 맥락: '카카오' 이슈가 촉발된 진짜 배경과 이해관계자들의 득실 계산을 분석합니다.</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>오늘 주요 언론을 통해 집중 조명된 핵심 사안은 바로 **[GC녹십자, LG CNS와 스마트공장 구축…AI 자동화 추진]** 입니다.&lt;br&gt;• &lt;b&gt;핵심 현황:&lt;/b&gt; GC녹십자가 LG CNS와 인공지능 기반 자동화·자율 운영 스마트 공장 구축을 추진한다.&lt;br&gt;• &lt;b&gt;왜 중요한가:&lt;/b&gt; 단순한 단발성 소식이 아니라 정부 정책, 규제 환경, 기업들의 실질적 손익과 직결되어 시장 전반에 큰 파장을 일으키고 있기 때문입니다.</t>
+          <t>오늘 주요 언론을 통해 집중 조명된 핵심 사안은 바로 **[카카오, ‘모두의 AI’ 연내 공개 예정…월 이용자 500만 명 목표]** 입니다.&lt;br&gt;• &lt;b&gt;핵심 현황:&lt;/b&gt; 카카오, ‘모두의 AI’ 연내 공개 예정월 이용자 500만 명 목표 KBS 뉴스카카오그룹, 인적분할 앞두고 주요 계열사 CEO 함께 모여 ‘첫 공동 IR’ 개최 카카오연말 출시 ‘모두의 AI’“카톡 익숙함. 활용할 것” 마켓 카카오, 웹툰·음원·카카오T에 스테이블코인 결제 연동소설 원작 AI 애니 제작도 전자신문카톡에 “메시지 정리, 답장 보내줘” 말하면 AI비서가 척척.&lt;br&gt;• &lt;b&gt;왜 중요한가:&lt;/b&gt; 단순한 단발성 소식이 아니라 정부 정책, 규제 환경, 기업들의 실질적 손익과 직결되어 시장 전반에 큰 파장을 일으키고 있기 때문입니다.</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>이 문제는 오늘 갑자기 발생한 사안이 아니라, 과거부터 축적되어 온 구조적 원인이 있습니다.&lt;br&gt;• &lt;b&gt;과거 배경:&lt;/b&gt; GC녹십자, 헌터라제 알레르기 유발 항체 정밀 검출 기술 개발 뉴스저널리즘. 어려울 때 GC녹십자 2분기 살린 건, 끈끈한 '피의 힘' 히트뉴스.&lt;br&gt;• &lt;b&gt;결정적 계기:&lt;/b&gt; 잠재되어 있던 제도적 갈등과 시장 환경의 변화가 맞물리면서, 이번 계기를 통해 본격적으로 수면 위로 표출되었습니다.</t>
+          <t>이 문제는 오늘 갑자기 발생한 사안이 아니라, 과거부터 축적되어 온 구조적 원인이 있습니다.&lt;br&gt;• &lt;b&gt;과거 배경:&lt;/b&gt; 피지컬 AI 시동 건 카카오모빌리티…상생재단서 '카카오' 뗀 이유는? 알림음과 배경 음악을 구분하는 카카오 라인 블록 체인 사운드 안내 Calgary Roughnecks.&lt;br&gt;• &lt;b&gt;결정적 계기:&lt;/b&gt; 잠재되어 있던 제도적 갈등과 시장 환경의 변화가 맞물리면서, 이번 계기를 통해 본격적으로 수면 위로 표출되었습니다.</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>겉으로 보이는 명분 뒤에는 각 주체들의 아주 명확한 '실질적 손익 계산'이 숨어 있습니다.&lt;br&gt;• &lt;b&gt;이해관계 분석:&lt;/b&gt; GC녹십자, 헌터라제 특이 IgE 항체 정밀 분석법 개발…국제학술지 게재 나눔경제뉴스. GC녹십자웰빙, 비만·체형관리까지…'에스테틱' 판 키운다.&lt;br&gt;• &lt;b&gt;핵심 구조:&lt;/b&gt; 규제 당국은 시장 통제력과 정책 주도권을 강화하려 하고, 관련 기업들은 비용 부담을 줄이고 수익성을 지키기 위해 치열한 수싸움을 벌이고 있는 구도입니다.</t>
+          <t>겉으로 보이는 명분 뒤에는 각 주체들의 아주 명확한 '실질적 손익 계산'이 숨어 있습니다.&lt;br&gt;• &lt;b&gt;이해관계 분석:&lt;/b&gt; 카카오 AI, 올해 사회경제적 가치 약 5500억 창출 전망 서울경제. 카카오 AI 사회경제적 가치 연 5506억원…2030년 최대 1.8조원 전망 지디넷코리아.&lt;br&gt;• &lt;b&gt;핵심 구조:&lt;/b&gt; 규제 당국은 시장 통제력과 정책 주도권을 강화하려 하고, 관련 기업들은 비용 부담을 줄이고 수익성을 지키기 위해 치열한 수싸움을 벌이고 있는 구도입니다.</t>
         </is>
       </c>
       <c r="J2" s="3" t="inlineStr">
@@ -10374,12 +10634,12 @@
       </c>
       <c r="L2" s="3" t="inlineStr">
         <is>
-          <t>주요언론</t>
+          <t>KBS 뉴스</t>
         </is>
       </c>
       <c r="M2" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261014121800017</t>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE43NnU3MlhmZWZkcEdnRU1abkNDcHdIdG85YU9NZVBqVF90N3BXTHFCVlJIbDZQbkg3RGR5NWltZ29IaXNWNkdIWm1aYzBmLU4wbnVfd1hhVnlwdVk?oc=5</t>
         </is>
       </c>
     </row>
@@ -10421,7 +10681,7 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>이 유행은 과연 어디서부터 시작되었을까요? 시작점을 추적해 보면 아주 흥미로운 바이럴 계기가 있습니다.&lt;br&gt;• &lt;b&gt;시작 비화:&lt;/b&gt; 수영복 입은 문주님, 블루 아카이브에 '람과천청' 업데이트 월요신문. 알림음과 배경 음악을 구분하는 블루아카이브 경마 사운드 안내 Calgary Roughnecks.&lt;br&gt;• &lt;b&gt;확산 과정:&lt;/b&gt; 초기에는 특정 매니아층 사이의 호기심으로 시작되었으나, 틱톡·릴스 등 숏폼 영상 알고리즘을 타며 '나도 경험해봐야 한다'는 대중적 열풍으로 급격히 번져나갔습니다.</t>
+          <t>이 유행은 과연 어디서부터 시작되었을까요? 시작점을 추적해 보면 아주 흥미로운 바이럴 계기가 있습니다.&lt;br&gt;• &lt;b&gt;시작 비화:&lt;/b&gt; 알림음과 배경 음악을 구분하는 블루아카이브 경마 사운드 안내 Calgary Roughnecks. 수영복 입은 문주님, 블루 아카이브에 '람과천청' 업데이트 월요신문.&lt;br&gt;• &lt;b&gt;확산 과정:&lt;/b&gt; 초기에는 특정 매니아층 사이의 호기심으로 시작되었으나, 틱톡·릴스 등 숏폼 영상 알고리즘을 타며 '나도 경험해봐야 한다'는 대중적 열풍으로 급격히 번져나갔습니다.</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Refactor: complete all-round improvements across dossier, disclosure, pagination and security
</commit_message>
<xml_diff>
--- a/reports/일자별_누적_데일리_이슈_및_주식_브리핑_마스터.xlsx
+++ b/reports/일자별_누적_데일리_이슈_및_주식_브리핑_마스터.xlsx
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G95"/>
+  <dimension ref="A1:G128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -468,7 +468,7 @@
     <col width="32" customWidth="1" min="3" max="3"/>
     <col width="65" customWidth="1" min="4" max="4"/>
     <col width="65" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
     <col width="53" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -3626,7 +3626,7 @@
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>사회/사건사고</t>
+          <t>정치</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
@@ -3636,22 +3636,22 @@
       </c>
       <c r="D86" s="3" t="inlineStr">
         <is>
-          <t>“신임 비서실장은 임광현”…떠나는 강훈식 마지막 브리핑 [지금뉴스]</t>
+          <t>與, 임광현 靑비서실장 발탁에 "국정성과에 속도 낼 적임자"</t>
         </is>
       </c>
       <c r="E86" s="3" t="inlineStr">
         <is>
-          <t>“신임 비서실장은 임광현”떠나는 강훈식 마지막 브리핑 KBS 뉴스 신임 대통령 비서실장에 임광현 국세청장 JTBC이 대통령, ‘강훈식 후임’ 새 비서실장에 임광현 국세청장 임명 한겨레안철수 "임광현 비서실장, 보은 인사 결정판처남 대장동 변호사" 뉴스1李 '먹사니즘' 세제 공약 설계한 임광현黨영입인재서 靑비서실장까지 아시아경제.</t>
+          <t>더불어민주당은 14일 임광현 국세청장이 이재명 정부 청와대 2기 비서실장으로 발탁에 대해 "국민이 피부로 느끼.</t>
         </is>
       </c>
       <c r="F86" s="3" t="inlineStr">
         <is>
-          <t>KBS 뉴스</t>
+          <t>주요언론</t>
         </is>
       </c>
       <c r="G86" s="3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTFBOT2xfekhrRnVZc3FfaENuU0xNRUJEczB5Z2RWVjRCLUtheS1VZ2UyUk9GT3J4aHNuclBVS0o5T3FPMFRRYWhwMTYxQWNiUDVQYkd4Ni1XbTdfem8?oc=5</t>
+          <t>https://www.yna.co.kr/view/AKR20261014144800001</t>
         </is>
       </c>
     </row>
@@ -3663,22 +3663,22 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>사회/사건사고</t>
+          <t>정치</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>연결 이슈 (후속)</t>
+          <t>🔥 [언론사 집중 보도 (3개사)]</t>
         </is>
       </c>
       <c r="D87" s="3" t="inlineStr">
         <is>
-          <t>인천 흉기난동범 "관심 끌려 범행…힘없어 보이는 사람 골랐다"</t>
+          <t>정부, 후티 반군의 사우디 민간시설 공격 규탄…"중단 촉구"</t>
         </is>
       </c>
       <c r="E87" s="3" t="inlineStr">
         <is>
-          <t>인천 대형 상업시설에서 흉기를 휘둘러 8명을 다치게 한 50대 남성이 자신의 불만을 사회적으로 알리고 싶어 범.</t>
+          <t>정부는 최근 후티 반군이 사우디아라비아 수도 리야드에 위치한 국제공항 등 민간 시설을 공격해 다수의 민간인 사.</t>
         </is>
       </c>
       <c r="F87" s="3" t="inlineStr">
@@ -3688,7 +3688,7 @@
       </c>
       <c r="G87" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261014134000065</t>
+          <t>https://www.yna.co.kr/view/AKR20261014148100504</t>
         </is>
       </c>
     </row>
@@ -3700,22 +3700,22 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>사회/사건사고</t>
+          <t>정치</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>🔥 [언론사 집중 보도 (3개사)]</t>
+          <t>신규 이슈</t>
         </is>
       </c>
       <c r="D88" s="3" t="inlineStr">
         <is>
-          <t>'1심 무죄' 前경호처장 2심 징역 1년…尹비화폰 증거인멸 유죄(종합)</t>
+          <t>해군2함대-중부해경청, 서해 안보협력 강화를 위한 MOU 체결</t>
         </is>
       </c>
       <c r="E88" s="3" t="inlineStr">
         <is>
-          <t>12·3 비상계엄 사태 이후 윤석열 전 대통령 등의 비화폰 정보를 삭제한 혐의로 기소된 박종준 전 대통령 경호.</t>
+          <t>해군 제2함대사령부는 14일 중부지방해양경찰청과 서해 안보협력 강화를 위한 양해각서 를 체결했다.</t>
         </is>
       </c>
       <c r="F88" s="3" t="inlineStr">
@@ -3725,7 +3725,7 @@
       </c>
       <c r="G88" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261014123851004</t>
+          <t>https://www.yna.co.kr/view/AKR20261014148400061</t>
         </is>
       </c>
     </row>
@@ -3737,22 +3737,22 @@
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>사회/사건사고</t>
+          <t>정치</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>신규 이슈</t>
+          <t>🔥 [언론사 집중 보도 (4개사)]</t>
         </is>
       </c>
       <c r="D89" s="3" t="inlineStr">
         <is>
-          <t>제주 평화로에서 다중 추돌 교통사고…12대 추정</t>
+          <t>李대통령, 임광현에 "훈식이 형 만큼, 그 이상 해내실 것 기대"</t>
         </is>
       </c>
       <c r="E89" s="3" t="inlineStr">
         <is>
-          <t>14일 오후 3시께 제주시 애월읍 평화로에서 차량 12대 가 잇따라 추돌했다.</t>
+          <t>이재명 대통령은 14일 신임 대통령 비서실장으로 임광현 국세청장을 발탁한 뒤 엑스 에 "임 실장.</t>
         </is>
       </c>
       <c r="F89" s="3" t="inlineStr">
@@ -3762,7 +3762,7 @@
       </c>
       <c r="G89" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261014135000056</t>
+          <t>https://www.yna.co.kr/view/AKR20261014146400001</t>
         </is>
       </c>
     </row>
@@ -3774,32 +3774,32 @@
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>거시경제/비즈니스</t>
+          <t>정치</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>🔥 [언론사 집중 보도 (6개사)]</t>
+          <t>🔥 [언론사 집중 보도 (4개사)]</t>
         </is>
       </c>
       <c r="D90" s="3" t="inlineStr">
         <is>
-          <t>카카오, ‘모두의 AI’ 연내 공개 예정…월 이용자 500만 명 목표</t>
+          <t>李대통령, '경제형 비서실장' 전격 발탁…실용주의로 2년차 돌파</t>
         </is>
       </c>
       <c r="E90" s="3" t="inlineStr">
         <is>
-          <t>카카오, ‘모두의 AI’ 연내 공개 예정월 이용자 500만 명 목표 KBS 뉴스카카오그룹, 인적분할 앞두고 주요 계열사 CEO 함께 모여 ‘첫 공동 IR’ 개최 카카오연말 출시 ‘모두의 AI’“카톡 익숙함. 활용할 것” 마켓 카카오, 웹툰·음원·카카오T에 스테이블코인 결제 연동소설 원작 AI 애니 제작도 전자신문카톡에 “메시지 정리, 답장 보내줘” 말하면 AI비서가 척척.</t>
+          <t>이재명 대통령이 2년 차에 접어든 국정을 보좌할 비서실장으로 14일 경제 관료 출신인 임광현 국세청장을 전격.</t>
         </is>
       </c>
       <c r="F90" s="3" t="inlineStr">
         <is>
-          <t>KBS 뉴스</t>
+          <t>주요언론</t>
         </is>
       </c>
       <c r="G90" s="3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE43NnU3MlhmZWZkcEdnRU1abkNDcHdIdG85YU9NZVBqVF90N3BXTHFCVlJIbDZQbkg3RGR5NWltZ29IaXNWNkdIWm1aYzBmLU4wbnVfd1hhVnlwdVk?oc=5</t>
+          <t>https://www.yna.co.kr/view/AKR20261014138500001</t>
         </is>
       </c>
     </row>
@@ -3811,32 +3811,32 @@
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>거시경제/비즈니스</t>
+          <t>사회/사건사고</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>신규 이슈</t>
+          <t>연결 이슈 (후속)</t>
         </is>
       </c>
       <c r="D91" s="3" t="inlineStr">
         <is>
-          <t>대구 신세계 프리미엄 아울렛 건립 속도…인허가기간 절반 이하로</t>
+          <t>'尹 비화폰 삭제' 박종준 전 경호처장 2심 징역형‥1심 무죄 뒤집혀</t>
         </is>
       </c>
       <c r="E91" s="3" t="inlineStr">
         <is>
-          <t>대구시가 신세계사이먼의 '대구 프리미엄 아울렛' 건립을 위한 인허가 기간을 통상의 절반 이하로 줄이는 등 사업.</t>
+          <t>'尹 비화폰 삭제' 박종준 전 경호처장 2심 징역형‥1심 무죄 뒤집혀.</t>
         </is>
       </c>
       <c r="F91" s="3" t="inlineStr">
         <is>
-          <t>주요언론</t>
+          <t>MBC 뉴스</t>
         </is>
       </c>
       <c r="G91" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261014129100053</t>
+          <t>https://news.google.com/rss/articles/CBMid0FVX3lxTE4yS19JendCbGpWdW11Mll3YnExWWJ4clJpa0lHbXJrUmVPZ2xveC0xN2xCWlJPLVd3anh2dXRla3BRWHFYUmVOLVlVLWhjSjR4ZTFXY0FnXzF4SWIwU1BwOGpFTjBuY3FCMk1OTkVTNmtRcWlueXZv0gF3QVVfeXFMTXZqdlJQeHl1N0hQNFBUZnExVGxSMnY0V1VzYkRpelRUVVR1NXczZlpKcU11QkgzV0NGaUxVMGxVNVpybjJYNjhNYWROVHJLYTVfa0s4ZEZkQkFjRWpGMUtNbm9kbXZIbzFGcjRVU1dCbDBaeU1DMzg?oc=5</t>
         </is>
       </c>
     </row>
@@ -3848,22 +3848,22 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>거시경제/비즈니스</t>
+          <t>사회/사건사고</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>연결 이슈 (후속)</t>
+          <t>신규 이슈</t>
         </is>
       </c>
       <c r="D92" s="3" t="inlineStr">
         <is>
-          <t>토스뱅크, 디지털 취약계층에 노트북 기부</t>
+          <t>대전중리초 체육관 전면보수 특별교부금 확보…교육 인프라 개선</t>
         </is>
       </c>
       <c r="E92" s="3" t="inlineStr">
         <is>
-          <t>토스뱅크가 고령층 문해학습자와 장애인 등 디지털 교육이 필요한 학습자를 지원하기 위해 업무용으로 사용하던 노트북 46대를 기부한다고 14일 밝혔다.</t>
+          <t>더불어민주당 박정현 국회의원 은 대전중리초등학교 체육관 전면 보수 사업을 위한 2026년 교육부.</t>
         </is>
       </c>
       <c r="F92" s="3" t="inlineStr">
@@ -3873,7 +3873,7 @@
       </c>
       <c r="G92" s="3" t="inlineStr">
         <is>
-          <t>https://www.mk.co.kr/news/economy/12175659</t>
+          <t>https://www.yna.co.kr/view/AKR20261014154100063</t>
         </is>
       </c>
     </row>
@@ -3885,22 +3885,22 @@
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>세계/국제</t>
+          <t>사회/사건사고</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>신규 이슈</t>
+          <t>🔥 [언론사 집중 보도 (8개사)]</t>
         </is>
       </c>
       <c r="D93" s="3" t="inlineStr">
         <is>
-          <t>올해만 10대 선진국 10년물 국채금리 0.81%p 급등</t>
+          <t>창원서 제조 AI·스마트공장 통합 'The Next AI×SMATOF' 개막</t>
         </is>
       </c>
       <c r="E93" s="3" t="inlineStr">
         <is>
-          <t>국제 신용평가사 피치는 국채 금리 상승으로 프랑스, 미국, 영국 등 주요 선진국이 채무 부담을 안정적으로 유지.</t>
+          <t>경남도는 14일부터 16일까지 창원컨벤션센터 에서 제조 인공지능 전시회인 'The Next A.</t>
         </is>
       </c>
       <c r="F93" s="3" t="inlineStr">
@@ -3910,7 +3910,7 @@
       </c>
       <c r="G93" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261014133700009</t>
+          <t>https://www.yna.co.kr/view/AKR20261014151200052</t>
         </is>
       </c>
     </row>
@@ -3922,7 +3922,7 @@
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>연예/대중문화</t>
+          <t>사회/사건사고</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
@@ -3932,22 +3932,22 @@
       </c>
       <c r="D94" s="3" t="inlineStr">
         <is>
-          <t>“칼로리에 깜짝” 악뮤 수현도 놀란 ‘최근 유행 디저트’ 정체</t>
+          <t>직원 노동분쟁에 '교비' 쓴 한신대 총장, 횡령 혐의 송치</t>
         </is>
       </c>
       <c r="E94" s="3" t="inlineStr">
         <is>
-          <t>“칼로리에 깜짝” 악뮤 수현도 놀란 ‘최근 유행 디저트’ 정체 헬스조선‘30㎏ 감량 이수현’ 콘서트 끝나고 ‘한정선’ 먹자트레이너 “10㎞ 뛰어야” '-30kg' 악뮤 이수현, 콘서트 직후 디저트 흡입트레이너에 "말 걸지 마라" 미주30kg 감량한 이수현, ‘이 음식’ 먹자트레이너 “10km 달려야” 서울신문"3시간 줄 선다고?" 갸우뚱이수현, '한정선' 솔직 후기 -.</t>
+          <t>한신대학교 강성영 총장이 직원들의 부당해고 등 노동 분쟁에 대응하기 위한 노무사 비용을 교비회계에서 지출한 혐.</t>
         </is>
       </c>
       <c r="F94" s="3" t="inlineStr">
         <is>
-          <t>헬스조선</t>
+          <t>주요언론</t>
         </is>
       </c>
       <c r="G94" s="3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMif0FVX3lxTFBldDBTc0RkSFJEOVQ5Y2o5bmJIY3gwaGQxZzZvVzZpRHdsX0RCZ3l3NS1oTm5iR0VERmYybWx4NGhSaGRMSFhXdnpPN1l0Y2JpalJ4WGZ0N3V5RHVKX2NUeF92NzVwOV9tenl5WDVyTXpjd281cHVuZmlGUkwzekU?oc=5</t>
+          <t>https://www.yna.co.kr/view/AKR20261014153100061</t>
         </is>
       </c>
     </row>
@@ -3959,32 +3959,1253 @@
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
+          <t>사회/사건사고</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>신규 이슈</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="inlineStr">
+        <is>
+          <t>전남교육음악제·초등교원미술작품전 16일 개최</t>
+        </is>
+      </c>
+      <c r="E95" s="3" t="inlineStr">
+        <is>
+          <t>전남광주통합특별시교육청은 가을을 맞아 교육 가족이 함께하는 문화예술행사를 개최한다고 14일 밝혔다.</t>
+        </is>
+      </c>
+      <c r="F95" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G95" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014152400054</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>사회/사건사고</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>신규 이슈</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="inlineStr">
+        <is>
+          <t>[동포의 창] 지구촌동포연대 "사할린 한인에게 음력 달력 선물"</t>
+        </is>
+      </c>
+      <c r="E96" s="3" t="inlineStr">
+        <is>
+          <t>지구촌동포연대 는 러시아 사할린에 거주하는 한인들을 위해 '세상에 하나뿐인 달력 2027'을 제작한다고.</t>
+        </is>
+      </c>
+      <c r="F96" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G96" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014153500371</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>사회/사건사고</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>신규 이슈</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="inlineStr">
+        <is>
+          <t>"횟수보다 방법"…26년 차 치과의사가 전하는 '백년양치질'</t>
+        </is>
+      </c>
+      <c r="E97" s="3" t="inlineStr">
+        <is>
+          <t>"더 열심히 닦을수록 잇몸은 망가집니다. 핵심은 횟수가 아니라 방법입니다.".</t>
+        </is>
+      </c>
+      <c r="F97" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G97" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014152100055</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>사회/사건사고</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>연결 이슈 (후속)</t>
+        </is>
+      </c>
+      <c r="D98" s="3" t="inlineStr">
+        <is>
+          <t>제주 평화로에서 차량 12대 추돌 사고…16명 중경상(종합)</t>
+        </is>
+      </c>
+      <c r="E98" s="3" t="inlineStr">
+        <is>
+          <t>제주 평화로에서 다중 추돌 교통사고가 발생해 16명이 중경상을 입었다.</t>
+        </is>
+      </c>
+      <c r="F98" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G98" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014135051056</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>사회/사건사고</t>
+        </is>
+      </c>
+      <c r="C99" s="2" t="inlineStr">
+        <is>
+          <t>신규 이슈</t>
+        </is>
+      </c>
+      <c r="D99" s="3" t="inlineStr">
+        <is>
+          <t>산림청, 국토부와 소나무재선충 피해목 신속 제거 협의</t>
+        </is>
+      </c>
+      <c r="E99" s="3" t="inlineStr">
+        <is>
+          <t>산림청은 14일 정부세종청사에서 국토교통부와 공동으로 생활권 주변 소나무재선충병 피해목의 신속한 제거를 위한.</t>
+        </is>
+      </c>
+      <c r="F99" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G99" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014149600063</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>사회/사건사고</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
+          <t>신규 이슈</t>
+        </is>
+      </c>
+      <c r="D100" s="3" t="inlineStr">
+        <is>
+          <t>김성주 "리밸런싱 유예 안했다면 매일 8천억 매도…증시 충격"</t>
+        </is>
+      </c>
+      <c r="E100" s="3" t="inlineStr">
+        <is>
+          <t>김성주 국민연금공단 이사장이 올해 초 국내주식 비율 초과에 따른 자산 비중 재조정 작업 을 유예하지.</t>
+        </is>
+      </c>
+      <c r="F100" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G100" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014151100530</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>사회/사건사고</t>
+        </is>
+      </c>
+      <c r="C101" s="2" t="inlineStr">
+        <is>
+          <t>신규 이슈</t>
+        </is>
+      </c>
+      <c r="D101" s="3" t="inlineStr">
+        <is>
+          <t>지식재산처, 기술경찰 수사범위 확대한다…제도 개선 추진</t>
+        </is>
+      </c>
+      <c r="E101" s="3" t="inlineStr">
+        <is>
+          <t>지식재산처는 기술경찰의 수사 범위를 영업비밀 침해를 넘어 국가핵심기술·국가첨단전략기술 유출 범죄까지 확대하는.</t>
+        </is>
+      </c>
+      <c r="F101" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G101" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014151800063</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>사회/사건사고</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t>연결 이슈 (후속)</t>
+        </is>
+      </c>
+      <c r="D102" s="3" t="inlineStr">
+        <is>
+          <t>국공노 "2차 행정기관 이전 대상 공무원 주거·정주대책 필요"</t>
+        </is>
+      </c>
+      <c r="E102" s="3" t="inlineStr">
+        <is>
+          <t>정부가 추진하는 2차 중앙행정기관 이전과 관련해 국가공무원노조 가 이전 공무원에 대한 실질적인 주거·정.</t>
+        </is>
+      </c>
+      <c r="F102" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G102" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014148900063</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="inlineStr">
+        <is>
+          <t>사회/사건사고</t>
+        </is>
+      </c>
+      <c r="C103" s="2" t="inlineStr">
+        <is>
+          <t>신규 이슈</t>
+        </is>
+      </c>
+      <c r="D103" s="3" t="inlineStr">
+        <is>
+          <t>태백 문곡소도동에 '얼굴 없는 천사'…쌀 280㎏ 기부</t>
+        </is>
+      </c>
+      <c r="E103" s="3" t="inlineStr">
+        <is>
+          <t>강원 태백시 문곡소도동에 익명의 주민이 어려운 이웃을 위해 쌀 280㎏을 기부해 훈훈함을 전하고 있다.</t>
+        </is>
+      </c>
+      <c r="F103" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G103" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014150000062</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t>사회/사건사고</t>
+        </is>
+      </c>
+      <c r="C104" s="2" t="inlineStr">
+        <is>
+          <t>신규 이슈</t>
+        </is>
+      </c>
+      <c r="D104" s="3" t="inlineStr">
+        <is>
+          <t>시흥 오이도 해상서 10대 2명 물에 빠져…해경 구조</t>
+        </is>
+      </c>
+      <c r="E104" s="3" t="inlineStr">
+        <is>
+          <t>14일 오후 3시 5분께 경기 시흥시 오이도 빨간등대 인근 해상에서 10대 2명이 물에 빠졌다는 신고가 해경에.</t>
+        </is>
+      </c>
+      <c r="F104" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G104" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014150200065</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="inlineStr">
+        <is>
+          <t>사회/사건사고</t>
+        </is>
+      </c>
+      <c r="C105" s="2" t="inlineStr">
+        <is>
+          <t>신규 이슈</t>
+        </is>
+      </c>
+      <c r="D105" s="3" t="inlineStr">
+        <is>
+          <t>교육부, 12월부터 두달간 유아 레벨테스트 금지 집중점검</t>
+        </is>
+      </c>
+      <c r="E105" s="3" t="inlineStr">
+        <is>
+          <t>교육부는 유아를 대상으로 한 '레벨테스트' 금지 제도가 현장에 안착하도록 점검을 강화하겠다고 14일 밝혔다.</t>
+        </is>
+      </c>
+      <c r="F105" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G105" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014149800530</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t>사회/사건사고</t>
+        </is>
+      </c>
+      <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t>신규 이슈</t>
+        </is>
+      </c>
+      <c r="D106" s="3" t="inlineStr">
+        <is>
+          <t>경기도 버스 노사 교섭 최종 결렬…지노위 조정신청 접수</t>
+        </is>
+      </c>
+      <c r="E106" s="3" t="inlineStr">
+        <is>
+          <t>경기도 버스 노사의 임금 및 단체협약 교섭이 최종 결렬되면서 노조가 지방노동위원회에 노동쟁의 조정을 신청하고.</t>
+        </is>
+      </c>
+      <c r="F106" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G106" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014149500061</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B107" s="2" t="inlineStr">
+        <is>
+          <t>거시경제/비즈니스</t>
+        </is>
+      </c>
+      <c r="C107" s="2" t="inlineStr">
+        <is>
+          <t>🔥 [언론사 집중 보도 (8개사)]</t>
+        </is>
+      </c>
+      <c r="D107" s="3" t="inlineStr">
+        <is>
+          <t>삼성전자 '반도체대전' 참가‥HBM4E 등 AI 반도체 기술 선보인다</t>
+        </is>
+      </c>
+      <c r="E107" s="3" t="inlineStr">
+        <is>
+          <t>삼성전자 '반도체대전' 참가‥HBM4E 등 AI 반도체 기술 선보인다.</t>
+        </is>
+      </c>
+      <c r="F107" s="3" t="inlineStr">
+        <is>
+          <t>MBC 뉴스</t>
+        </is>
+      </c>
+      <c r="G107" s="3" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidEFVX3lxTE9QLWl1VjBqYUpRc3BydE96Y1c1N2JQNUJ4TTdmazF6NmRlb01JaHpYa3NSX2llQkRyUFU3S1JYOUxVbkp3N3VMOUlITWFoUEk2YlpkTDdmUzE3MUJwbG9LclBOQzNYNzkzZnJLcDdveDZKMkFG0gF0QVVfeXFMUG52cWpIVDZJZFNKelIwTmczTFJmVUtRTjVBYlI0ZEJtNkJYWWVYaWVRR1plUFR0M3pQUVZUdmF6RDJRNm5qWjlHNUFzNlZ0d2N6TV8tNm1RUldCMVh3b3l4eWhkdlBUOGMtSVZwMm5YUTlGUzg?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>거시경제/비즈니스</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t>🔥 [언론사 집중 보도 (4개사)]</t>
+        </is>
+      </c>
+      <c r="D108" s="3" t="inlineStr">
+        <is>
+          <t>‘이자만 2700만원’ 이 대통령 아파트 거래…증여세 대상 아닌 이유는?</t>
+        </is>
+      </c>
+      <c r="E108" s="3" t="inlineStr">
+        <is>
+          <t>‘이자만 2700만원’ 이 대통령 아파트 거래증여세 대상 아닌 이유는?</t>
+        </is>
+      </c>
+      <c r="F108" s="3" t="inlineStr">
+        <is>
+          <t>한겨레</t>
+        </is>
+      </c>
+      <c r="G108" s="3" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMickFVX3lxTFA1Nmc0MHpKSV9zMzg1WFBKR3dVRW45aW5lcXVFb3M1V3cydTZ4eXN5Y0ppOWcwc1VGUks1YWdoWEw5TUsxYnp2WWxhQlBrbllRcjgzSURycEpQNkJwWFZhdnNKWTYtQXl2LUpjUS1hQ1lOdw?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="inlineStr">
+        <is>
+          <t>거시경제/비즈니스</t>
+        </is>
+      </c>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t>연결 이슈 (후속)</t>
+        </is>
+      </c>
+      <c r="D109" s="3" t="inlineStr">
+        <is>
+          <t>코스피, 반등 실패…6거래일 연속 내리며 '6천피' 턱걸이(종합)</t>
+        </is>
+      </c>
+      <c r="E109" s="3" t="inlineStr">
+        <is>
+          <t>코스피가 14일 전날 급락을 딛고 상승 출발했지만, 장 후반 들어 하락 전환하며 6거래일 연속 하락세를 이어갔.</t>
+        </is>
+      </c>
+      <c r="F109" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G109" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014138351008</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>거시경제/비즈니스</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>신규 이슈</t>
+        </is>
+      </c>
+      <c r="D110" s="3" t="inlineStr">
+        <is>
+          <t>[동정] 농식품부 장관, 수확기 맞아 사과 재배 농가 방문</t>
+        </is>
+      </c>
+      <c r="E110" s="3" t="inlineStr">
+        <is>
+          <t>▲ 송미령 농림축산식품부 장관은 14일 가을 수확기를 맞아 경남 함양군의 사과 재배 농가를 방문하고, 올해부터 운영 중인 '사과 안정생산 추진단.</t>
+        </is>
+      </c>
+      <c r="F110" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G110" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014059400030</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B111" s="2" t="inlineStr">
+        <is>
+          <t>거시경제/비즈니스</t>
+        </is>
+      </c>
+      <c r="C111" s="2" t="inlineStr">
+        <is>
+          <t>신규 이슈</t>
+        </is>
+      </c>
+      <c r="D111" s="3" t="inlineStr">
+        <is>
+          <t>LS증권, 수요예측서 4천640억 몰려…모집예정액 7배 수준</t>
+        </is>
+      </c>
+      <c r="E111" s="3" t="inlineStr">
+        <is>
+          <t>LS증권 의 무보증사채 수요예측에서 모집예정액의 7배 가까운 자금이 몰렸다.</t>
+        </is>
+      </c>
+      <c r="F111" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G111" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261013159900008</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>세계/국제</t>
+        </is>
+      </c>
+      <c r="C112" s="2" t="inlineStr">
+        <is>
+          <t>신규 이슈</t>
+        </is>
+      </c>
+      <c r="D112" s="3" t="inlineStr">
+        <is>
+          <t>佛 마트 냉장고들 해킹당했다... 온도 50도 폭주 ‘먹거리 테러’</t>
+        </is>
+      </c>
+      <c r="E112" s="3" t="inlineStr">
+        <is>
+          <t>佛 마트 냉장고들 해킹당했다 온도 50도 폭주 ‘먹거리 테러’. 아울러 에펠탑 옆 '슈퍼마켓 냉동고'가 텅 비었다'냉장고 해킹' 덮친 佛파리 가보니.</t>
+        </is>
+      </c>
+      <c r="F112" s="3" t="inlineStr">
+        <is>
+          <t>조선일보</t>
+        </is>
+      </c>
+      <c r="G112" s="3" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxNX3hlMG9oaUR4eWpCTGRxV3d5LWpsVU4wa082NWk0MXZLZWx4aWY3UHo5SUVvc1Jkb0pNdWZtTVMyMkQtbnZUN21Sc05KdjlaMndnS0s4aWZvRmszSTNic3BkbF9HY0Zlb3dwQkF4bVl3bFVOYXJ4M0JLSThaWXpOVV9vaG92M1FlR25KZDFMN3d0eWpZQXRJcElaVXdUdw?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B113" s="2" t="inlineStr">
+        <is>
+          <t>세계/국제</t>
+        </is>
+      </c>
+      <c r="C113" s="2" t="inlineStr">
+        <is>
+          <t>🔥 [언론사 집중 보도 (4개사)]</t>
+        </is>
+      </c>
+      <c r="D113" s="3" t="inlineStr">
+        <is>
+          <t>이란 매체 "미군 드론, 어선 공격해 3명 부상"</t>
+        </is>
+      </c>
+      <c r="E113" s="3" t="inlineStr">
+        <is>
+          <t>김상훈 특파원 = 이란 남부 호르모즈간주 시리크 인근 해상에서 미군의 무인기 공격으로 3명이 부상했다고 반관영.</t>
+        </is>
+      </c>
+      <c r="F113" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G113" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014153200079</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B114" s="2" t="inlineStr">
+        <is>
+          <t>세계/국제</t>
+        </is>
+      </c>
+      <c r="C114" s="2" t="inlineStr">
+        <is>
+          <t>신규 이슈</t>
+        </is>
+      </c>
+      <c r="D114" s="3" t="inlineStr">
+        <is>
+          <t>서울 세계청년대회 성공 기원 음악회…조수미도 무대에</t>
+        </is>
+      </c>
+      <c r="E114" s="3" t="inlineStr">
+        <is>
+          <t>민경락 특파원 = 내년 서울에서 열리는 세계청년대회 의 성공 개최를 기원하는 음악회가 이탈리아 로마에서 열렸다고 주교.</t>
+        </is>
+      </c>
+      <c r="F114" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G114" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014149900109</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B115" s="2" t="inlineStr">
+        <is>
+          <t>세계/국제</t>
+        </is>
+      </c>
+      <c r="C115" s="2" t="inlineStr">
+        <is>
+          <t>🔥 [언론사 집중 보도 (3개사)]</t>
+        </is>
+      </c>
+      <c r="D115" s="3" t="inlineStr">
+        <is>
+          <t>중간선거 앞두고 거칠어진 트럼프의 입…종교·인종 차별까지</t>
+        </is>
+      </c>
+      <c r="E115" s="3" t="inlineStr">
+        <is>
+          <t>달 치러지는 미국 중간선거에서 공화당이 고전할 것이란 전망이 짙어지면서 도널드 트럼프 대통령의 언사가 점.</t>
+        </is>
+      </c>
+      <c r="F115" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G115" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014147100009</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B116" s="2" t="inlineStr">
+        <is>
+          <t>세계/국제</t>
+        </is>
+      </c>
+      <c r="C116" s="2" t="inlineStr">
+        <is>
+          <t>신규 이슈</t>
+        </is>
+      </c>
+      <c r="D116" s="3" t="inlineStr">
+        <is>
+          <t>[쇼츠] 차단봉에 머리 '쿵' 쓰러졌는데…오히려 혼난 남성</t>
+        </is>
+      </c>
+      <c r="E116" s="3" t="inlineStr">
+        <is>
+          <t>12일 인도 타밀나두주 쿠달로르 지역의 한 도로 요금소에서 한 남성이 차단봉에 맞아 쓰러지는 사고가 발생했습니다.</t>
+        </is>
+      </c>
+      <c r="F116" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G116" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014148200704</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B117" s="2" t="inlineStr">
+        <is>
+          <t>세계/국제</t>
+        </is>
+      </c>
+      <c r="C117" s="2" t="inlineStr">
+        <is>
+          <t>신규 이슈</t>
+        </is>
+      </c>
+      <c r="D117" s="3" t="inlineStr">
+        <is>
+          <t>"미국에 할말 하겠다"는 일본. ICC 제재 진의 파악 공들여</t>
+        </is>
+      </c>
+      <c r="E117" s="3" t="inlineStr">
+        <is>
+          <t>일본 정부가 미국의 국제형사재판소 제재 발표와 관련해 ICC에 대한 지지를 강조하면서도 도널드 트럼프.</t>
+        </is>
+      </c>
+      <c r="F117" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G117" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014145800009</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B118" s="2" t="inlineStr">
+        <is>
+          <t>IT/과학/신상품</t>
+        </is>
+      </c>
+      <c r="C118" s="2" t="inlineStr">
+        <is>
+          <t>🔥 [언론사 집중 보도 (5개사)]</t>
+        </is>
+      </c>
+      <c r="D118" s="3" t="inlineStr">
+        <is>
+          <t>엔비디아 RTX 스파크 16일 출격…24GB로 돌리는 740억 파라미터 에이전트 모델 공개</t>
+        </is>
+      </c>
+      <c r="E118" s="3" t="inlineStr">
+        <is>
+          <t>엔비디아 RTX 스파크 16일 출격24GB로 돌리는 740억 파라미터 에이전트 모델 공개. 아울러 DLSS 5, 다음은 '연운'이다 적용 예고 및 성능 개선 진행.</t>
+        </is>
+      </c>
+      <c r="F118" s="3" t="inlineStr">
+        <is>
+          <t>ER 이코노믹리뷰</t>
+        </is>
+      </c>
+      <c r="G118" s="3" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMibEFVX3lxTE5jZnVIcU1McmlHa3Itbm4wYVJPSHlFR2llaFRwUHdBd181c3ZQWjA3czhndkpfQnh1S19rQXpINk1HSTg4ZzhEVHNRTDBlSVJ3M2RoS0Z5MXIzSFpqVFZNT3VfWkNpY1RKY2E4MQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B119" s="2" t="inlineStr">
+        <is>
+          <t>IT/과학/신상품</t>
+        </is>
+      </c>
+      <c r="C119" s="2" t="inlineStr">
+        <is>
+          <t>🔥 [언론사 집중 보도 (5개사)]</t>
+        </is>
+      </c>
+      <c r="D119" s="3" t="inlineStr">
+        <is>
+          <t>‘메트로 2039’ 예약판매 시작, 스토리 확장 DLC·에디션 구성 공개</t>
+        </is>
+      </c>
+      <c r="E119" s="3" t="inlineStr">
+        <is>
+          <t>‘메트로 2039’ 예약판매 시작, 스토리 확장 DLC·에디션 구성 공개.</t>
+        </is>
+      </c>
+      <c r="F119" s="3" t="inlineStr">
+        <is>
+          <t>인벤</t>
+        </is>
+      </c>
+      <c r="G119" s="3" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiXkFVX3lxTE50Ym5RWDNGNjltd0NLMmJTbG5fUldPNW13SHprT1YzYllzSDNnR05DUS0zMVp5dWE0WElMUTlfZWlCdGdpcmRNbktpTTVqMEptUjVkVWo0YTQyRUU0T2c?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B120" s="2" t="inlineStr">
+        <is>
+          <t>IT/과학/신상품</t>
+        </is>
+      </c>
+      <c r="C120" s="2" t="inlineStr">
+        <is>
+          <t>🔥 [언론사 집중 보도 (3개사)]</t>
+        </is>
+      </c>
+      <c r="D120" s="3" t="inlineStr">
+        <is>
+          <t>무게 줄이고 가격 낮췄다…렉트릭, 가성비 도심형 전기자전거 출시</t>
+        </is>
+      </c>
+      <c r="E120" s="3" t="inlineStr">
+        <is>
+          <t>무게 줄이고 가격 낮췄다렉트릭, 가성비 도심형 전기자전거 출시.</t>
+        </is>
+      </c>
+      <c r="F120" s="3" t="inlineStr">
+        <is>
+          <t>디지털투데이</t>
+        </is>
+      </c>
+      <c r="G120" s="3" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMic0FVX3lxTE5TNk9veHRBWmtQZVdPS2NPUEQwVFVKeTRLLWFnc2pYX3hTNHVpbWFqdzJmTmVrdkYtaW05d0VjenRmNTdHLTNJakJyR3QyZHdtRmlnazItR0tLR0lXREFhYVJweXVyU1ZpNlZqeXd3OGM2Ums?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B121" s="2" t="inlineStr">
+        <is>
+          <t>IT/과학/신상품</t>
+        </is>
+      </c>
+      <c r="C121" s="2" t="inlineStr">
+        <is>
+          <t>신규 이슈</t>
+        </is>
+      </c>
+      <c r="D121" s="3" t="inlineStr">
+        <is>
+          <t>한전, 고졸 입사직원 2명 차장 특별승진…"능력·성과 중심"</t>
+        </is>
+      </c>
+      <c r="E121" s="3" t="inlineStr">
+        <is>
+          <t>한국전력은 고졸 전형 입사 직원을 포함해 탁월한 업무성과를 거둔 직원 12명을 특별승진 대상자로 선정했다고 1.</t>
+        </is>
+      </c>
+      <c r="F121" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G121" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014146200003</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>IT/과학/신상품</t>
+        </is>
+      </c>
+      <c r="C122" s="2" t="inlineStr">
+        <is>
+          <t>신규 이슈</t>
+        </is>
+      </c>
+      <c r="D122" s="3" t="inlineStr">
+        <is>
+          <t>엘리시안강촌, '숲속빵시장' 우천 예보에 25일로 연기</t>
+        </is>
+      </c>
+      <c r="E122" s="3" t="inlineStr">
+        <is>
+          <t>강원 춘천 엘리시안강촌에서 열릴 예정이던 '제5회 숲속빵시장'이 우천 예보로 일주일 연기됐다.</t>
+        </is>
+      </c>
+      <c r="F122" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G122" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014152300062</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B123" s="2" t="inlineStr">
+        <is>
+          <t>IT/과학/신상품</t>
+        </is>
+      </c>
+      <c r="C123" s="2" t="inlineStr">
+        <is>
+          <t>연결 이슈 (후속)</t>
+        </is>
+      </c>
+      <c r="D123" s="3" t="inlineStr">
+        <is>
+          <t>미국·영국 등 13개국 서울 집결…양자기술 협력 논의</t>
+        </is>
+      </c>
+      <c r="E123" s="3" t="inlineStr">
+        <is>
+          <t>과학기술정보통신부는 14~16일 서울에서 '제9차 양자기술다자대화'와 '양자기술 산업화 비즈니스 나이트'를 개.</t>
+        </is>
+      </c>
+      <c r="F123" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G123" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014147900017</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B124" s="2" t="inlineStr">
+        <is>
+          <t>IT/과학/신상품</t>
+        </is>
+      </c>
+      <c r="C124" s="2" t="inlineStr">
+        <is>
+          <t>신규 이슈</t>
+        </is>
+      </c>
+      <c r="D124" s="3" t="inlineStr">
+        <is>
+          <t>'경기 스타트업 서밋' 개막…혁신 스타트업-벤처 투자사 매칭</t>
+        </is>
+      </c>
+      <c r="E124" s="3" t="inlineStr">
+        <is>
+          <t>경기도가 주최하고 경기도경제과학진흥원이 주관하는 '2026 경기 스타트업 서밋'이 14일 수원컨벤션센터에서 개.</t>
+        </is>
+      </c>
+      <c r="F124" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G124" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014147000061</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B125" s="2" t="inlineStr">
+        <is>
           <t>연예/대중문화</t>
         </is>
       </c>
-      <c r="C95" s="2" t="inlineStr">
-        <is>
-          <t>🔥 [언론사 집중 보도 (4개사)]</t>
-        </is>
-      </c>
-      <c r="D95" s="3" t="inlineStr">
-        <is>
-          <t>“낙찰가 2400억, 역대 최고가 기대”…반 고흐 '꽃 핀 밤나무' 60년 만에 공개</t>
-        </is>
-      </c>
-      <c r="E95" s="3" t="inlineStr">
-        <is>
-          <t>“낙찰가 2400억, 역대 최고가 기대”반 고흐 '꽃 핀 밤나무' 60년 만에 공개 전자신문낙찰 예상가만 2400억60여 년 만에 공개 반고흐의 ‘꽃 핀 밤나무’ KBS 뉴스고흐 말년작 60년만에 공개내달 경매 2400억원 예상 동아일보홍콩서 60여년 만에 반고흐 '꽃 핀 밤나무' 공개수백명 몰려 60년만에 세상 나온 반고흐 명작'경매가 2400억' 신기록 전망 뉴스1.</t>
-        </is>
-      </c>
-      <c r="F95" s="3" t="inlineStr">
-        <is>
-          <t>전자신문</t>
-        </is>
-      </c>
-      <c r="G95" s="3" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiTkFVX3lxTE80XzRkdG90QUU3QUtFbVJUcEJmNVhja2ZjYnRoY09GRUI3WjJfZzZFY1NkbVlwXzJTYWVUUVpfcG5oTVFENHVXbTFJQTRaZw?oc=5</t>
+      <c r="C125" s="2" t="inlineStr">
+        <is>
+          <t>신규 이슈</t>
+        </is>
+      </c>
+      <c r="D125" s="3" t="inlineStr">
+        <is>
+          <t>김종국, 대만서 ’런닝맨’ 파워 실감..길거리 사진 요청까지 “부러워”(상남자의 여행법)</t>
+        </is>
+      </c>
+      <c r="E125" s="3" t="inlineStr">
+        <is>
+          <t>김종국, 대만서 ’런닝맨’ 파워 실감길거리 사진 요청까지 “부러워”. 아울러 먹뱉 위기22! 들쥐 비주얼에 단체 멘붕 초대형 닭X알 걸린 추성훈ㅋㅋㅋㅋ | #상남자의여행법 EP.02.</t>
+        </is>
+      </c>
+      <c r="F125" s="3" t="inlineStr">
+        <is>
+          <t>조선일보</t>
+        </is>
+      </c>
+      <c r="G125" s="3" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxNTmlJNUxKQTNNV2FMZEZJdU90VmxGYXNVLWdpVTk3VHNrTHdNN0wySjhBWklYU0FfYVN3Q1RCLTdYclFKSHRfWVZndjhFeHJRUERwWlJ4b3d5bmtYdmYyR1NROXV1eURESkVyTkl4OHQtaFcwUVNQMGljYjVFSFFobTFhc2ZqZzlvTHNvSGU0QQ?oc=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B126" s="2" t="inlineStr">
+        <is>
+          <t>연예/대중문화</t>
+        </is>
+      </c>
+      <c r="C126" s="2" t="inlineStr">
+        <is>
+          <t>신규 이슈</t>
+        </is>
+      </c>
+      <c r="D126" s="3" t="inlineStr">
+        <is>
+          <t>[경주소식] KBS 대하드라마 '문무' 성공기원 행사</t>
+        </is>
+      </c>
+      <c r="E126" s="3" t="inlineStr">
+        <is>
+          <t>경북 경주시는 14일 감포읍 문무대왕 해양역사관 앞 광장에서 KBS 대하드라마 '문무'의 성공 기원 행사를 열었다.</t>
+        </is>
+      </c>
+      <c r="F126" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G126" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014153300053</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B127" s="2" t="inlineStr">
+        <is>
+          <t>연예/대중문화</t>
+        </is>
+      </c>
+      <c r="C127" s="2" t="inlineStr">
+        <is>
+          <t>🔥 [언론사 집중 보도 (5개사)]</t>
+        </is>
+      </c>
+      <c r="D127" s="3" t="inlineStr">
+        <is>
+          <t>[방송소식] 웨이브, '더 커뮤니티2' 비하인드 토크 16일 공개</t>
+        </is>
+      </c>
+      <c r="E127" s="3" t="inlineStr">
+        <is>
+          <t>▲ '더 커뮤니티2' 비하인드 토크, 최후 9인 출연 = 웨이브는 오리지널 예능 '더 커뮤니티2: 보이지 않는.</t>
+        </is>
+      </c>
+      <c r="F127" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G127" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014144600005</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B128" s="2" t="inlineStr">
+        <is>
+          <t>연예/대중문화</t>
+        </is>
+      </c>
+      <c r="C128" s="2" t="inlineStr">
+        <is>
+          <t>신규 이슈</t>
+        </is>
+      </c>
+      <c r="D128" s="3" t="inlineStr">
+        <is>
+          <t>[가요소식] BTS '훌리건' 뮤직비디오 1억뷰</t>
+        </is>
+      </c>
+      <c r="E128" s="3" t="inlineStr">
+        <is>
+          <t>▲ BTS '훌리건' 뮤직비디오 1억뷰 = 그룹 방탄소년단 의 '훌리건' 뮤직비디오가.</t>
+        </is>
+      </c>
+      <c r="F128" s="3" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
+      <c r="G128" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yna.co.kr/view/AKR20261014146900005</t>
         </is>
       </c>
     </row>
@@ -3999,7 +5220,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S36"/>
+  <dimension ref="A1:S37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -5326,42 +6547,42 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>232,500원</t>
+          <t>232,000원</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>+26,000.0원 (+12.59%)</t>
+          <t>+25,500원 (+12.35%)</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>230,000원</t>
+          <t>220,500원</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>257,000원</t>
+          <t>229,500원</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>224,500원</t>
+          <t>225,000원</t>
         </is>
       </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
-          <t>+11.6%</t>
+          <t>+4.2%</t>
         </is>
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>🟢 오늘 단기 매수 (저점 과매도 반등)</t>
+          <t>🔴 단기 비중 축소 (악재 주의)</t>
         </is>
       </c>
       <c r="L15" s="3" t="inlineStr">
         <is>
-          <t>RSI 34.7로 단기 과매도 구간 도달 및 지지선 부근 기술적 반등 기대 (거래량비율 0.82x)</t>
+          <t>악재 보도 및 5일 연속 약세(-4% 이상)로 단기 추가 하락 위험</t>
         </is>
       </c>
       <c r="M15" s="3" t="inlineStr">
@@ -5375,26 +6596,26 @@
         </is>
       </c>
       <c r="O15" s="3" t="n">
-        <v>34.7</v>
+        <v>34.4</v>
       </c>
       <c r="P15" s="3" t="inlineStr">
         <is>
-          <t>-11.3%</t>
+          <t>-11.4%</t>
         </is>
       </c>
       <c r="Q15" s="3" t="inlineStr">
         <is>
-          <t>49.7%</t>
+          <t>49.5%</t>
         </is>
       </c>
       <c r="R15" s="3" t="inlineStr">
         <is>
-          <t>[하나증권] 삼성화재: 3Q26 Pre - 단기 실적보다 중요한 것은 (하나증권)</t>
+          <t>삼성전자 '반도체대전' 참가‥HBM4E 등 AI 반도체 기술 선보인다 (MBC 뉴스)</t>
         </is>
       </c>
       <c r="S15" s="3" t="inlineStr">
         <is>
-          <t>[259500.0, 249000.0, 248500.0, 253500.0, 252500.0, 261000.0, 274000.0, 276500.0, 285500.0, 270000.0, 272500.0, 268500.0, 276000.0, 276000.0, 272000.0, 268500.0, 262000.0, 250500.0, 232000.0, 232500.0]</t>
+          <t>[259500.0, 249000.0, 248500.0, 253500.0, 252500.0, 261000.0, 274000.0, 276500.0, 285500.0, 270000.0, 272500.0, 268500.0, 276000.0, 276000.0, 272000.0, 268500.0, 262000.0, 250500.0, 232000.0, 232000.0]</t>
         </is>
       </c>
     </row>
@@ -5426,7 +6647,7 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>+316,000.0원 (+28.65%)</t>
+          <t>+316,000원 (+28.65%)</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
@@ -5484,7 +6705,7 @@
       </c>
       <c r="R16" s="3" t="inlineStr">
         <is>
-          <t>최근 특이 뉴스 없음</t>
+          <t>(마감시황) 코스피, 6,000선 턱걸이…삼전 보합·SK하이닉스 1.66%↓ (뉴스투데이)</t>
         </is>
       </c>
       <c r="S16" s="3" t="inlineStr">
@@ -5516,27 +6737,27 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>314,000원</t>
+          <t>313,500원</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>-177,500.0원 (-36.11%)</t>
+          <t>-178,000원 (-36.22%)</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>298,500원</t>
+          <t>298,000원</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>311,000원</t>
+          <t>310,500원</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>304,500원</t>
+          <t>304,000원</t>
         </is>
       </c>
       <c r="J17" s="3" t="inlineStr">
@@ -5551,7 +6772,7 @@
       </c>
       <c r="L17" s="3" t="inlineStr">
         <is>
-          <t>주가가 20일선(349,325원)을 하향 이탈하고 이동평균선 역배열 지속. 리스크 관리 차원 비중 축소 권고</t>
+          <t>주가가 20일선(349,300원)을 하향 이탈하고 이동평균선 역배열 지속. 리스크 관리 차원 비중 축소 권고</t>
         </is>
       </c>
       <c r="M17" s="3" t="inlineStr">
@@ -5565,16 +6786,16 @@
         </is>
       </c>
       <c r="O17" s="3" t="n">
-        <v>21.6</v>
+        <v>21.5</v>
       </c>
       <c r="P17" s="3" t="inlineStr">
         <is>
-          <t>-10.1%</t>
+          <t>-10.2%</t>
         </is>
       </c>
       <c r="Q17" s="3" t="inlineStr">
         <is>
-          <t>16.7%</t>
+          <t>16.6%</t>
         </is>
       </c>
       <c r="R17" s="3" t="inlineStr">
@@ -5584,7 +6805,7 @@
       </c>
       <c r="S17" s="3" t="inlineStr">
         <is>
-          <t>[382500.0, 371500.0, 367000.0, 362000.0, 363000.0, 365000.0, 359000.0, 360500.0, 353500.0, 354500.0, 350000.0, 345000.0, 349000.0, 346500.0, 348000.0, 336000.0, 324500.0, 320000.0, 315000.0, 314000.0]</t>
+          <t>[382500.0, 371500.0, 367000.0, 362000.0, 363000.0, 365000.0, 359000.0, 360500.0, 353500.0, 354500.0, 350000.0, 345000.0, 349000.0, 346500.0, 348000.0, 336000.0, 324500.0, 320000.0, 315000.0, 313500.0]</t>
         </is>
       </c>
     </row>
@@ -5616,7 +6837,7 @@
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>-40,800.0원 (-27.35%)</t>
+          <t>-40,600원 (-27.21%)</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
@@ -5631,12 +6852,12 @@
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>105,000원</t>
+          <t>105,500원</t>
         </is>
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>+5.8%</t>
+          <t>+6.0%</t>
         </is>
       </c>
       <c r="K18" s="3" t="inlineStr">
@@ -5646,7 +6867,7 @@
       </c>
       <c r="L18" s="3" t="inlineStr">
         <is>
-          <t>주가가 20일선(115,820원)을 하향 이탈하고 이동평균선 역배열 지속. 리스크 관리 차원 비중 축소 권고</t>
+          <t>주가가 20일선(115,830원)을 하향 이탈하고 이동평균선 역배열 지속. 리스크 관리 차원 비중 축소 권고</t>
         </is>
       </c>
       <c r="M18" s="3" t="inlineStr">
@@ -5660,16 +6881,16 @@
         </is>
       </c>
       <c r="O18" s="3" t="n">
-        <v>29.3</v>
+        <v>29.9</v>
       </c>
       <c r="P18" s="3" t="inlineStr">
         <is>
-          <t>-6.4%</t>
+          <t>-6.2%</t>
         </is>
       </c>
       <c r="Q18" s="3" t="inlineStr">
         <is>
-          <t>6.0%</t>
+          <t>6.1%</t>
         </is>
       </c>
       <c r="R18" s="3" t="inlineStr">
@@ -5679,7 +6900,7 @@
       </c>
       <c r="S18" s="3" t="inlineStr">
         <is>
-          <t>[126600.0, 124200.0, 121800.0, 120700.0, 120900.0, 121900.0, 120000.0, 118500.0, 115400.0, 117600.0, 116000.0, 112800.0, 113300.0, 112900.0, 112600.0, 109600.0, 106800.0, 108100.0, 108300.0, 108400.0]</t>
+          <t>[126600.0, 124200.0, 121800.0, 120700.0, 120900.0, 121900.0, 120000.0, 118500.0, 115400.0, 117600.0, 116000.0, 112800.0, 113300.0, 112900.0, 112600.0, 109600.0, 106800.0, 108100.0, 108300.0, 108600.0]</t>
         </is>
       </c>
     </row>
@@ -5706,12 +6927,12 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>180,000원</t>
+          <t>179,500원</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>-21,700.0원 (-10.77%)</t>
+          <t>-22,100원 (-10.97%)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -5721,17 +6942,17 @@
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>178,000원</t>
+          <t>177,500원</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>174,500원</t>
+          <t>174,000원</t>
         </is>
       </c>
       <c r="J19" s="3" t="inlineStr">
         <is>
-          <t>+5.3%</t>
+          <t>+5.0%</t>
         </is>
       </c>
       <c r="K19" s="3" t="inlineStr">
@@ -5741,7 +6962,7 @@
       </c>
       <c r="L19" s="3" t="inlineStr">
         <is>
-          <t>주가가 20일선(194,005원)을 하향 이탈하고 이동평균선 역배열 지속. 리스크 관리 차원 비중 축소 권고</t>
+          <t>주가가 20일선(193,985원)을 하향 이탈하고 이동평균선 역배열 지속. 리스크 관리 차원 비중 축소 권고</t>
         </is>
       </c>
       <c r="M19" s="3" t="inlineStr">
@@ -5755,16 +6976,16 @@
         </is>
       </c>
       <c r="O19" s="3" t="n">
-        <v>29.8</v>
+        <v>29.1</v>
       </c>
       <c r="P19" s="3" t="inlineStr">
         <is>
-          <t>-7.3%</t>
+          <t>-7.5%</t>
         </is>
       </c>
       <c r="Q19" s="3" t="inlineStr">
         <is>
-          <t>5.0%</t>
+          <t>4.7%</t>
         </is>
       </c>
       <c r="R19" s="3" t="inlineStr">
@@ -5774,7 +6995,7 @@
       </c>
       <c r="S19" s="3" t="inlineStr">
         <is>
-          <t>[206500.0, 204000.0, 206000.0, 201500.0, 199000.0, 197700.0, 197900.0, 201000.0, 194700.0, 197700.0, 194800.0, 193700.0, 191200.0, 192200.0, 191100.0, 189000.0, 183800.0, 180500.0, 178000.0, 179800.0]</t>
+          <t>[206500.0, 204000.0, 206000.0, 201500.0, 199000.0, 197700.0, 197900.0, 201000.0, 194700.0, 197700.0, 194800.0, 193700.0, 191200.0, 192200.0, 191100.0, 189000.0, 183800.0, 180500.0, 178000.0, 179400.0]</t>
         </is>
       </c>
     </row>
@@ -5806,7 +7027,7 @@
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>-16,400.0원 (-34.10%)</t>
+          <t>-16,400원 (-34.10%)</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
@@ -5864,7 +7085,7 @@
       </c>
       <c r="R20" s="3" t="inlineStr">
         <is>
-          <t>카카오, ‘모두의 AI’ 연내 공개 예정…월 이용자 500만 명 목표 (KBS 뉴스)</t>
+          <t>최근 특이 뉴스 없음</t>
         </is>
       </c>
       <c r="S20" s="3" t="inlineStr">
@@ -5901,12 +7122,12 @@
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>-9,719.049999999988원 (-5.13%)</t>
+          <t>-9,819원 (-5.18%)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>176,500원</t>
+          <t>176,000원</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
@@ -5945,16 +7166,16 @@
         </is>
       </c>
       <c r="O21" s="3" t="n">
-        <v>45.5</v>
+        <v>45.2</v>
       </c>
       <c r="P21" s="3" t="inlineStr">
         <is>
-          <t>+0.1%</t>
+          <t>+0.0%</t>
         </is>
       </c>
       <c r="Q21" s="3" t="inlineStr">
         <is>
-          <t>26.6%</t>
+          <t>26.4%</t>
         </is>
       </c>
       <c r="R21" s="3" t="inlineStr">
@@ -5964,7 +7185,7 @@
       </c>
       <c r="S21" s="3" t="inlineStr">
         <is>
-          <t>[178200.0, 178800.0, 177500.0, 177200.0, 180300.0, 179400.0, 181400.0, 178500.0, 177400.0, 178300.0, 178900.0, 177700.0, 183600.0, 182600.0, 182400.0, 183500.0, 179600.0, 180400.0, 179700.0, 179900.0]</t>
+          <t>[178200.0, 178800.0, 177500.0, 177200.0, 180300.0, 179400.0, 181400.0, 178500.0, 177400.0, 178300.0, 178900.0, 177700.0, 183600.0, 182600.0, 182400.0, 183500.0, 179600.0, 180400.0, 179700.0, 179800.0]</t>
         </is>
       </c>
     </row>
@@ -5991,12 +7212,12 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>839,000원</t>
+          <t>842,000원</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>-684,000.0원 (-44.91%)</t>
+          <t>-681,000원 (-44.71%)</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
@@ -6006,17 +7227,17 @@
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>830,500원</t>
+          <t>833,500원</t>
         </is>
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>814,000원</t>
+          <t>816,500원</t>
         </is>
       </c>
       <c r="J22" s="3" t="inlineStr">
         <is>
-          <t>+4.2%</t>
+          <t>+4.6%</t>
         </is>
       </c>
       <c r="K22" s="3" t="inlineStr">
@@ -6026,7 +7247,7 @@
       </c>
       <c r="L22" s="3" t="inlineStr">
         <is>
-          <t>주가가 20일선(1,012,050원)을 하향 이탈하고 이동평균선 역배열 지속. 리스크 관리 차원 비중 축소 권고</t>
+          <t>주가가 20일선(1,012,200원)을 하향 이탈하고 이동평균선 역배열 지속. 리스크 관리 차원 비중 축소 권고</t>
         </is>
       </c>
       <c r="M22" s="3" t="inlineStr">
@@ -6040,16 +7261,16 @@
         </is>
       </c>
       <c r="O22" s="3" t="n">
-        <v>29.6</v>
+        <v>30.1</v>
       </c>
       <c r="P22" s="3" t="inlineStr">
         <is>
-          <t>-17.1%</t>
+          <t>-16.8%</t>
         </is>
       </c>
       <c r="Q22" s="3" t="inlineStr">
         <is>
-          <t>6.4%</t>
+          <t>6.8%</t>
         </is>
       </c>
       <c r="R22" s="3" t="inlineStr">
@@ -6059,7 +7280,7 @@
       </c>
       <c r="S22" s="3" t="inlineStr">
         <is>
-          <t>[1081000.0, 1137000.0, 1063000.0, 1055000.0, 1097000.0, 1078000.0, 1067000.0, 1057000.0, 1021000.0, 1034000.0, 1012000.0, 1007000.0, 1034000.0, 1072000.0, 1023000.0, 972000.0, 891000.0, 862000.0, 839000.0, 839000.0]</t>
+          <t>[1081000.0, 1137000.0, 1063000.0, 1055000.0, 1097000.0, 1078000.0, 1067000.0, 1057000.0, 1021000.0, 1034000.0, 1012000.0, 1007000.0, 1034000.0, 1072000.0, 1023000.0, 972000.0, 891000.0, 862000.0, 839000.0, 842000.0]</t>
         </is>
       </c>
     </row>
@@ -6086,12 +7307,12 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>420,500원</t>
+          <t>422,000원</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>+20,500.0원 (+5.12%)</t>
+          <t>+22,000원 (+5.50%)</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -6101,17 +7322,17 @@
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>420,500원</t>
+          <t>422,000원</t>
         </is>
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>412,000원</t>
+          <t>413,500원</t>
         </is>
       </c>
       <c r="J23" s="3" t="inlineStr">
         <is>
-          <t>+13.0%</t>
+          <t>+13.4%</t>
         </is>
       </c>
       <c r="K23" s="3" t="inlineStr">
@@ -6121,7 +7342,7 @@
       </c>
       <c r="L23" s="3" t="inlineStr">
         <is>
-          <t>RSI 70.6, 20일선 이격도 +13.0%로 단기 과열권 진입. 욕심을 줄이고 분할 차익 실현 권고</t>
+          <t>RSI 71.0, 20일선 이격도 +13.4%로 단기 과열권 진입. 욕심을 줄이고 분할 차익 실현 권고</t>
         </is>
       </c>
       <c r="M23" s="3" t="inlineStr">
@@ -6135,16 +7356,16 @@
         </is>
       </c>
       <c r="O23" s="3" t="n">
-        <v>70.59999999999999</v>
+        <v>71</v>
       </c>
       <c r="P23" s="3" t="inlineStr">
         <is>
-          <t>+13.0%</t>
+          <t>+13.4%</t>
         </is>
       </c>
       <c r="Q23" s="3" t="inlineStr">
         <is>
-          <t>55.0%</t>
+          <t>55.6%</t>
         </is>
       </c>
       <c r="R23" s="3" t="inlineStr">
@@ -6154,7 +7375,7 @@
       </c>
       <c r="S23" s="3" t="inlineStr">
         <is>
-          <t>[360000.0, 351500.0, 365500.0, 367000.0, 365000.0, 364000.0, 352000.0, 350500.0, 351500.0, 364000.0, 352500.0, 357000.0, 360500.0, 371000.0, 390000.0, 391000.0, 401000.0, 398000.0, 410000.0, 420500.0]</t>
+          <t>[360000.0, 351500.0, 365500.0, 367000.0, 365000.0, 364000.0, 352000.0, 350500.0, 351500.0, 364000.0, 352500.0, 357000.0, 360500.0, 371000.0, 390000.0, 391000.0, 401000.0, 398000.0, 410000.0, 422000.0]</t>
         </is>
       </c>
     </row>
@@ -6181,17 +7402,17 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>307,500원</t>
+          <t>309,000원</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>-54,000.0원 (-14.94%)</t>
+          <t>-52,500원 (-14.52%)</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>301,500원</t>
+          <t>303,000원</t>
         </is>
       </c>
       <c r="H24" s="3" t="inlineStr">
@@ -6201,12 +7422,12 @@
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>292,000원</t>
+          <t>293,500원</t>
         </is>
       </c>
       <c r="J24" s="3" t="inlineStr">
         <is>
-          <t>+10.8%</t>
+          <t>+10.3%</t>
         </is>
       </c>
       <c r="K24" s="3" t="inlineStr">
@@ -6230,16 +7451,16 @@
         </is>
       </c>
       <c r="O24" s="3" t="n">
-        <v>44.2</v>
+        <v>45.3</v>
       </c>
       <c r="P24" s="3" t="inlineStr">
         <is>
-          <t>-2.3%</t>
+          <t>-1.9%</t>
         </is>
       </c>
       <c r="Q24" s="3" t="inlineStr">
         <is>
-          <t>12.2%</t>
+          <t>12.7%</t>
         </is>
       </c>
       <c r="R24" s="3" t="inlineStr">
@@ -6249,7 +7470,7 @@
       </c>
       <c r="S24" s="3" t="inlineStr">
         <is>
-          <t>[334000.0, 326000.0, 332000.0, 326500.0, 326500.0, 323000.0, 317000.0, 317500.0, 311500.0, 316500.0, 304000.0, 306000.0, 306500.0, 311000.0, 318000.0, 307500.0, 306500.0, 299000.0, 299000.0, 307500.0]</t>
+          <t>[334000.0, 326000.0, 332000.0, 326500.0, 326500.0, 323000.0, 317000.0, 317500.0, 311500.0, 316500.0, 304000.0, 306000.0, 306500.0, 311000.0, 318000.0, 307500.0, 306500.0, 299000.0, 299000.0, 309000.0]</t>
         </is>
       </c>
     </row>
@@ -6276,22 +7497,22 @@
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>$228.52 (약 305,782원)</t>
+          <t>$228.52 (약 305,131원)</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>+39.21000000000001$ (+20.71%)</t>
+          <t>+39.21$ (+20.71%)</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>$223.95 (약 299,666원)</t>
+          <t>$223.95 (약 299,028원)</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
-          <t>$239.95 (약 321,071원)</t>
+          <t>$239.95 (약 320,387원)</t>
         </is>
       </c>
       <c r="I25" s="3" t="inlineStr">
@@ -6339,7 +7560,7 @@
       </c>
       <c r="R25" s="3" t="inlineStr">
         <is>
-          <t>최근 특이 뉴스 없음</t>
+          <t>엔비디아 RTX 스파크 16일 출격…24GB로 돌리는 740억 파라미터 에이전트 모델 공개 (ER 이코노믹리뷰)</t>
         </is>
       </c>
       <c r="S25" s="3" t="inlineStr">
@@ -6371,7 +7592,7 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>$341.27 (약 456,653원)</t>
+          <t>$341.27 (약 455,680원)</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
@@ -6381,12 +7602,12 @@
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>$334.44 (약 447,520원)</t>
+          <t>$334.44 (약 446,567원)</t>
         </is>
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
-          <t>$358.33 (약 479,486원)</t>
+          <t>$358.33 (약 478,464원)</t>
         </is>
       </c>
       <c r="I26" s="3" t="inlineStr">
@@ -6466,22 +7687,22 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>$375.23 (약 502,095원)</t>
+          <t>$375.23 (약 501,025원)</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>+22.810000000000002$ (+6.47%)</t>
+          <t>+22.81$ (+6.47%)</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>$367.73 (약 492,053원)</t>
+          <t>$367.73 (약 491,005원)</t>
         </is>
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>$393.99 (약 527,200원)</t>
+          <t>$393.99 (약 526,077원)</t>
         </is>
       </c>
       <c r="I27" s="3" t="inlineStr">
@@ -6561,22 +7782,22 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>$543.45 (약 727,190원)</t>
+          <t>$543.45 (약 725,641원)</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>+159.08000000000004$ (+41.39%)</t>
+          <t>+159.08$ (+41.39%)</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>$514.20 (약 688,051원)</t>
+          <t>$514.20 (약 686,585원)</t>
         </is>
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
-          <t>$543.45 (약 727,190원)</t>
+          <t>$543.45 (약 725,641원)</t>
         </is>
       </c>
       <c r="I28" s="3" t="inlineStr">
@@ -6656,17 +7877,17 @@
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>403,500원</t>
+          <t>404,500원</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>-97,500.0원 (-19.46%)</t>
+          <t>-96,500원 (-19.26%)</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>399,500원</t>
+          <t>400,500원</t>
         </is>
       </c>
       <c r="H29" s="3" t="inlineStr">
@@ -6676,12 +7897,12 @@
       </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>389,500원</t>
+          <t>390,500원</t>
         </is>
       </c>
       <c r="J29" s="3" t="inlineStr">
         <is>
-          <t>+21.0%</t>
+          <t>+20.7%</t>
         </is>
       </c>
       <c r="K29" s="3" t="inlineStr">
@@ -6691,7 +7912,7 @@
       </c>
       <c r="L29" s="3" t="inlineStr">
         <is>
-          <t>RSI 33.0로 단기 과매도 구간 도달 및 지지선 부근 기술적 반등 기대 (거래량비율 1.99x)</t>
+          <t>RSI 33.1로 단기 과매도 구간 도달 및 지지선 부근 기술적 반등 기대 (거래량비율 2.11x)</t>
         </is>
       </c>
       <c r="M29" s="3" t="inlineStr">
@@ -6705,16 +7926,16 @@
         </is>
       </c>
       <c r="O29" s="3" t="n">
-        <v>33</v>
+        <v>33.1</v>
       </c>
       <c r="P29" s="3" t="inlineStr">
         <is>
-          <t>-18.2%</t>
+          <t>-18.0%</t>
         </is>
       </c>
       <c r="Q29" s="3" t="inlineStr">
         <is>
-          <t>29.4%</t>
+          <t>29.7%</t>
         </is>
       </c>
       <c r="R29" s="3" t="inlineStr">
@@ -6724,7 +7945,7 @@
       </c>
       <c r="S29" s="3" t="inlineStr">
         <is>
-          <t>[464000.0, 474000.0, 496500.0, 502000.0, 515000.0, 503000.0, 505000.0, 502000.0, 520000.0, 504000.0, 507000.0, 499000.0, 497500.0, 506000.0, 523000.0, 534000.0, 480500.0, 474500.0, 453000.0, 403500.0]</t>
+          <t>[464000.0, 474000.0, 496500.0, 502000.0, 515000.0, 503000.0, 505000.0, 502000.0, 520000.0, 504000.0, 507000.0, 499000.0, 497500.0, 506000.0, 523000.0, 534000.0, 480500.0, 474500.0, 453000.0, 404500.0]</t>
         </is>
       </c>
     </row>
@@ -6751,27 +7972,27 @@
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>50,200원</t>
+          <t>49,900원</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>-14,000.0원 (-21.81%)</t>
+          <t>-14,300원 (-22.27%)</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>49,700원</t>
+          <t>49,400원</t>
         </is>
       </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
-          <t>53,200원</t>
+          <t>52,900원</t>
         </is>
       </c>
       <c r="I30" s="3" t="inlineStr">
         <is>
-          <t>48,400원</t>
+          <t>48,200원</t>
         </is>
       </c>
       <c r="J30" s="3" t="inlineStr">
@@ -6786,7 +8007,7 @@
       </c>
       <c r="L30" s="3" t="inlineStr">
         <is>
-          <t>RSI 35.8로 단기 과매도 구간 도달 및 지지선 부근 기술적 반등 기대 (거래량비율 0.81x)</t>
+          <t>RSI 33.1로 단기 과매도 구간 도달 및 지지선 부근 기술적 반등 기대 (거래량비율 0.99x)</t>
         </is>
       </c>
       <c r="M30" s="3" t="inlineStr">
@@ -6800,16 +8021,16 @@
         </is>
       </c>
       <c r="O30" s="3" t="n">
-        <v>35.8</v>
+        <v>33.1</v>
       </c>
       <c r="P30" s="3" t="inlineStr">
         <is>
-          <t>-3.8%</t>
+          <t>-4.3%</t>
         </is>
       </c>
       <c r="Q30" s="3" t="inlineStr">
         <is>
-          <t>9.9%</t>
+          <t>8.5%</t>
         </is>
       </c>
       <c r="R30" s="3" t="inlineStr">
@@ -6819,7 +8040,7 @@
       </c>
       <c r="S30" s="3" t="inlineStr">
         <is>
-          <t>[52700.0, 53200.0, 53000.0, 52800.0, 53400.0, 53000.0, 53100.0, 53100.0, 52700.0, 52900.0, 52900.0, 52300.0, 51800.0, 51900.0, 51500.0, 51300.0, 52100.0, 49900.0, 49750.0, 50200.0]</t>
+          <t>[52700.0, 53200.0, 53000.0, 52800.0, 53400.0, 53000.0, 53100.0, 53100.0, 52700.0, 52900.0, 52900.0, 52300.0, 51800.0, 51900.0, 51500.0, 51300.0, 52100.0, 49900.0, 49750.0, 49900.0]</t>
         </is>
       </c>
     </row>
@@ -6851,7 +8072,7 @@
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>-13,600.0원 (-14.24%)</t>
+          <t>-13,600원 (-14.24%)</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
@@ -6881,7 +8102,7 @@
       </c>
       <c r="L31" s="3" t="inlineStr">
         <is>
-          <t>RSI 37.3로 단기 과매도 구간 도달 및 지지선 부근 기술적 반등 기대 (거래량비율 0.96x)</t>
+          <t>RSI 37.3로 단기 과매도 구간 도달 및 지지선 부근 기술적 반등 기대 (거래량비율 1.17x)</t>
         </is>
       </c>
       <c r="M31" s="3" t="inlineStr">
@@ -6941,22 +8162,22 @@
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>14,800원</t>
+          <t>14,700원</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>-2,700.0원 (-15.46%)</t>
+          <t>-2,770원 (-15.86%)</t>
         </is>
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>14,500원</t>
+          <t>14,400원</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr">
         <is>
-          <t>15,500원</t>
+          <t>15,400원</t>
         </is>
       </c>
       <c r="I32" s="3" t="inlineStr">
@@ -6990,16 +8211,16 @@
         </is>
       </c>
       <c r="O32" s="3" t="n">
-        <v>52.5</v>
+        <v>50.7</v>
       </c>
       <c r="P32" s="3" t="inlineStr">
         <is>
-          <t>+0.9%</t>
+          <t>+0.5%</t>
         </is>
       </c>
       <c r="Q32" s="3" t="inlineStr">
         <is>
-          <t>19.2%</t>
+          <t>17.8%</t>
         </is>
       </c>
       <c r="R32" s="3" t="inlineStr">
@@ -7009,7 +8230,7 @@
       </c>
       <c r="S32" s="3" t="inlineStr">
         <is>
-          <t>[14890.0, 15040.0, 14850.0, 14650.0, 14680.0, 14050.0, 14490.0, 14570.0, 14640.0, 14770.0, 14800.0, 14530.0, 14540.0, 14550.0, 14560.0, 14500.0, 14400.0, 14550.0, 14780.0, 14770.0]</t>
+          <t>[14890.0, 15040.0, 14850.0, 14650.0, 14680.0, 14050.0, 14490.0, 14570.0, 14640.0, 14770.0, 14800.0, 14530.0, 14540.0, 14550.0, 14560.0, 14500.0, 14400.0, 14550.0, 14780.0, 14700.0]</t>
         </is>
       </c>
     </row>
@@ -7021,12 +8242,12 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>일진전기</t>
+          <t>삼성화재</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>103590.KS</t>
+          <t>000810.KS</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -7036,42 +8257,42 @@
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>75,000원</t>
+          <t>582,000원</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>-9,300.0원 (-11.03%)</t>
+          <t>+92,500원 (+18.90%)</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>73,500원</t>
+          <t>553,000원</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>88,000원</t>
+          <t>576,000원</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
         <is>
-          <t>71,200원</t>
+          <t>564,500원</t>
         </is>
       </c>
       <c r="J33" s="3" t="inlineStr">
         <is>
-          <t>+19.7%</t>
+          <t>+4.2%</t>
         </is>
       </c>
       <c r="K33" s="3" t="inlineStr">
         <is>
-          <t>관망 (HOLD)</t>
+          <t>🔴 단기 비중 축소 (추세 이탈 경고)</t>
         </is>
       </c>
       <c r="L33" s="3" t="inlineStr">
         <is>
-          <t>중립 구간 유지 중</t>
+          <t>주가가 20일선(642,100원)을 하향 이탈하고 이동평균선 역배열 지속. 리스크 관리 차원 비중 축소 권고</t>
         </is>
       </c>
       <c r="M33" s="3" t="inlineStr">
@@ -7085,16 +8306,16 @@
         </is>
       </c>
       <c r="O33" s="3" t="n">
-        <v>48</v>
+        <v>33.7</v>
       </c>
       <c r="P33" s="3" t="inlineStr">
         <is>
-          <t>-3.3%</t>
+          <t>-9.4%</t>
         </is>
       </c>
       <c r="Q33" s="3" t="inlineStr">
         <is>
-          <t>32.5%</t>
+          <t>48.2%</t>
         </is>
       </c>
       <c r="R33" s="3" t="inlineStr">
@@ -7104,7 +8325,7 @@
       </c>
       <c r="S33" s="3" t="inlineStr">
         <is>
-          <t>[71000.0, 69700.0, 68400.0, 70400.0, 70200.0, 76600.0, 73000.0, 76500.0, 81700.0, 82100.0, 80900.0, 82500.0, 82900.0, 86200.0, 87900.0, 88000.0, 81400.0, 73800.0, 73400.0, 75000.0]</t>
+          <t>[686000.0, 675000.0, 661000.0, 661000.0, 666000.0, 648000.0, 651000.0, 655000.0, 648000.0, 661000.0, 653000.0, 633000.0, 626000.0, 626000.0, 635000.0, 629000.0, 612000.0, 622000.0, 612000.0, 582000.0]</t>
         </is>
       </c>
     </row>
@@ -7116,12 +8337,12 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>삼성중공업</t>
+          <t>휴젤</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>010140.KS</t>
+          <t>145020.KS</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
@@ -7131,42 +8352,42 @@
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>18,900원</t>
+          <t>223,500원</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>-8,960.0원 (-32.11%)</t>
+          <t>-29,500원 (-11.66%)</t>
         </is>
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>18,800원</t>
+          <t>200,000원</t>
         </is>
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>20,100원</t>
+          <t>223,500원</t>
         </is>
       </c>
       <c r="I34" s="3" t="inlineStr">
         <is>
-          <t>18,300원</t>
+          <t>219,000원</t>
         </is>
       </c>
       <c r="J34" s="3" t="inlineStr">
         <is>
-          <t>+7.1%</t>
+          <t>+11.7%</t>
         </is>
       </c>
       <c r="K34" s="3" t="inlineStr">
         <is>
-          <t>🟢 오늘 단기 매수 (저점 과매도 반등)</t>
+          <t>🔴 오늘 단기 매도 (과열 차익실현)</t>
         </is>
       </c>
       <c r="L34" s="3" t="inlineStr">
         <is>
-          <t>RSI 40.9로 단기 과매도 구간 도달 및 지지선 부근 기술적 반등 기대 (거래량비율 1.46x)</t>
+          <t>RSI 19.6, 20일선 이격도 +11.7%로 단기 과열권 진입. 욕심을 줄이고 분할 차익 실현 권고</t>
         </is>
       </c>
       <c r="M34" s="3" t="inlineStr">
@@ -7180,16 +8401,16 @@
         </is>
       </c>
       <c r="O34" s="3" t="n">
-        <v>40.9</v>
+        <v>19.6</v>
       </c>
       <c r="P34" s="3" t="inlineStr">
         <is>
-          <t>-5.4%</t>
+          <t>+11.7%</t>
         </is>
       </c>
       <c r="Q34" s="3" t="inlineStr">
         <is>
-          <t>9.5%</t>
+          <t>41.1%</t>
         </is>
       </c>
       <c r="R34" s="3" t="inlineStr">
@@ -7199,7 +8420,7 @@
       </c>
       <c r="S34" s="3" t="inlineStr">
         <is>
-          <t>[21400.0, 22100.0, 20700.0, 20200.0, 21500.0, 20800.0, 20600.0, 20600.0, 20250.0, 20100.0, 19330.0, 19700.0, 19720.0, 19960.0, 19700.0, 19540.0, 18860.0, 18010.0, 18360.0, 18940.0]</t>
+          <t>[236000.0, 231000.0, 232000.0, 235500.0, 231000.0, 231500.0, 214000.0, 206000.0, 190400.0, 187000.0, 186100.0, 183300.0, 179700.0, 180600.0, 180100.0, 181500.0, 183600.0, 182800.0, 180000.0, 169900.0]</t>
         </is>
       </c>
     </row>
@@ -7211,12 +8432,12 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>삼성화재</t>
+          <t>일진전기</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>000810.KS</t>
+          <t>103590.KS</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
@@ -7226,42 +8447,42 @@
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>582,000원</t>
+          <t>74,900원</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>+92,500.0원 (+18.90%)</t>
+          <t>-9,400원 (-11.15%)</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>553,000원</t>
+          <t>73,400원</t>
         </is>
       </c>
       <c r="H35" s="3" t="inlineStr">
         <is>
-          <t>576,000원</t>
+          <t>88,000원</t>
         </is>
       </c>
       <c r="I35" s="3" t="inlineStr">
         <is>
-          <t>564,500원</t>
+          <t>71,200원</t>
         </is>
       </c>
       <c r="J35" s="3" t="inlineStr">
         <is>
-          <t>+4.2%</t>
+          <t>+19.9%</t>
         </is>
       </c>
       <c r="K35" s="3" t="inlineStr">
         <is>
-          <t>🔴 단기 비중 축소 (추세 이탈 경고)</t>
+          <t>관망 (HOLD)</t>
         </is>
       </c>
       <c r="L35" s="3" t="inlineStr">
         <is>
-          <t>주가가 20일선(642,100원)을 하향 이탈하고 이동평균선 역배열 지속. 리스크 관리 차원 비중 축소 권고</t>
+          <t>중립 구간 유지 중</t>
         </is>
       </c>
       <c r="M35" s="3" t="inlineStr">
@@ -7275,16 +8496,16 @@
         </is>
       </c>
       <c r="O35" s="3" t="n">
-        <v>33.7</v>
+        <v>47.8</v>
       </c>
       <c r="P35" s="3" t="inlineStr">
         <is>
-          <t>-9.4%</t>
+          <t>-3.5%</t>
         </is>
       </c>
       <c r="Q35" s="3" t="inlineStr">
         <is>
-          <t>48.2%</t>
+          <t>32.4%</t>
         </is>
       </c>
       <c r="R35" s="3" t="inlineStr">
@@ -7294,7 +8515,7 @@
       </c>
       <c r="S35" s="3" t="inlineStr">
         <is>
-          <t>[686000.0, 675000.0, 661000.0, 661000.0, 666000.0, 648000.0, 651000.0, 655000.0, 648000.0, 661000.0, 653000.0, 633000.0, 626000.0, 626000.0, 635000.0, 629000.0, 612000.0, 622000.0, 612000.0, 582000.0]</t>
+          <t>[71000.0, 69700.0, 68400.0, 70400.0, 70200.0, 76600.0, 73000.0, 76500.0, 81700.0, 82100.0, 80900.0, 82500.0, 82900.0, 86200.0, 87900.0, 88000.0, 81400.0, 73800.0, 73400.0, 74900.0]</t>
         </is>
       </c>
     </row>
@@ -7306,12 +8527,12 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>휴젤</t>
+          <t>효성중공업</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>145020.KS</t>
+          <t>298040.KS</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
@@ -7321,42 +8542,42 @@
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>223,500원</t>
+          <t>2,135,000원</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>-29,500.0원 (-11.66%)</t>
+          <t>-907,000원 (-29.82%)</t>
         </is>
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>200,000원</t>
+          <t>2,028,000원</t>
         </is>
       </c>
       <c r="H36" s="3" t="inlineStr">
         <is>
-          <t>223,500원</t>
+          <t>2,113,500원</t>
         </is>
       </c>
       <c r="I36" s="3" t="inlineStr">
         <is>
-          <t>219,000원</t>
+          <t>2,071,000원</t>
         </is>
       </c>
       <c r="J36" s="3" t="inlineStr">
         <is>
-          <t>+11.7%</t>
+          <t>+4.2%</t>
         </is>
       </c>
       <c r="K36" s="3" t="inlineStr">
         <is>
-          <t>🔴 오늘 단기 매도 (과열 차익실현)</t>
+          <t>🔴 단기 비중 축소 (추세 이탈 경고)</t>
         </is>
       </c>
       <c r="L36" s="3" t="inlineStr">
         <is>
-          <t>RSI 19.6, 20일선 이격도 +11.7%로 단기 과열권 진입. 욕심을 줄이고 분할 차익 실현 권고</t>
+          <t>주가가 20일선(2,701,200원)을 하향 이탈하고 이동평균선 역배열 지속. 리스크 관리 차원 비중 축소 권고</t>
         </is>
       </c>
       <c r="M36" s="3" t="inlineStr">
@@ -7370,16 +8591,16 @@
         </is>
       </c>
       <c r="O36" s="3" t="n">
-        <v>19.6</v>
+        <v>26.2</v>
       </c>
       <c r="P36" s="3" t="inlineStr">
         <is>
-          <t>+11.7%</t>
+          <t>-21.0%</t>
         </is>
       </c>
       <c r="Q36" s="3" t="inlineStr">
         <is>
-          <t>41.1%</t>
+          <t>20.2%</t>
         </is>
       </c>
       <c r="R36" s="3" t="inlineStr">
@@ -7389,7 +8610,102 @@
       </c>
       <c r="S36" s="3" t="inlineStr">
         <is>
-          <t>[236000.0, 231000.0, 232000.0, 235500.0, 231000.0, 231500.0, 214000.0, 206000.0, 190400.0, 187000.0, 186100.0, 183300.0, 179700.0, 180600.0, 180100.0, 181500.0, 183600.0, 182800.0, 180000.0, 169900.0]</t>
+          <t>[2854000.0, 2803000.0, 2689000.0, 2806000.0, 2861000.0, 2915000.0, 2917000.0, 2901000.0, 2896000.0, 2780000.0, 2804000.0, 2773000.0, 2822000.0, 2785000.0, 2807000.0, 2588000.0, 2494000.0, 2242000.0, 2152000.0, 2135000.0]</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>삼성중공업</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>010140.KS</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>증권사 공식리서치</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>19,000원</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>-8,950원 (-32.08%)</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>18,800원</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr">
+        <is>
+          <t>20,100원</t>
+        </is>
+      </c>
+      <c r="I37" s="3" t="inlineStr">
+        <is>
+          <t>18,300원</t>
+        </is>
+      </c>
+      <c r="J37" s="3" t="inlineStr">
+        <is>
+          <t>+7.1%</t>
+        </is>
+      </c>
+      <c r="K37" s="3" t="inlineStr">
+        <is>
+          <t>🟢 오늘 단기 매수 (저점 과매도 반등)</t>
+        </is>
+      </c>
+      <c r="L37" s="3" t="inlineStr">
+        <is>
+          <t>RSI 41.0로 단기 과매도 구간 도달 및 지지선 부근 기술적 반등 기대 (거래량비율 1.7x)</t>
+        </is>
+      </c>
+      <c r="M37" s="3" t="inlineStr">
+        <is>
+          <t>보유 / 중립 (HOLD)</t>
+        </is>
+      </c>
+      <c r="N37" s="3" t="inlineStr">
+        <is>
+          <t>장기 추세 유지</t>
+        </is>
+      </c>
+      <c r="O37" s="3" t="n">
+        <v>41</v>
+      </c>
+      <c r="P37" s="3" t="inlineStr">
+        <is>
+          <t>-5.3%</t>
+        </is>
+      </c>
+      <c r="Q37" s="3" t="inlineStr">
+        <is>
+          <t>9.6%</t>
+        </is>
+      </c>
+      <c r="R37" s="3" t="inlineStr">
+        <is>
+          <t>최근 특이 뉴스 없음</t>
+        </is>
+      </c>
+      <c r="S37" s="3" t="inlineStr">
+        <is>
+          <t>[21400.0, 22100.0, 20700.0, 20200.0, 21500.0, 20800.0, 20600.0, 20600.0, 20250.0, 20100.0, 19330.0, 19700.0, 19720.0, 19960.0, 19700.0, 19540.0, 18860.0, 18010.0, 18360.0, 18950.0]</t>
         </is>
       </c>
     </row>
@@ -7621,12 +8937,12 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>5,997.24</t>
+          <t>6,008.81</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>▼ -38.11 (-0.63%)</t>
+          <t>▼ -26.54 (-0.44%)</t>
         </is>
       </c>
     </row>
@@ -7648,12 +8964,12 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>820.32</t>
+          <t>823.88</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>▼ -28.87 (-3.40%)</t>
+          <t>▼ -13.15 (-1.57%)</t>
         </is>
       </c>
     </row>
@@ -7729,12 +9045,12 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>1,338.10</t>
+          <t>1,335.25</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>▼ -2.03원 (-0.15%)</t>
+          <t>▼ -4.88원 (-0.36%)</t>
         </is>
       </c>
     </row>
@@ -7756,12 +9072,12 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>843.10</t>
+          <t>841.40</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>▼ -1.00원 (-0.12%)</t>
+          <t>▼ -2.70원 (-0.32%)</t>
         </is>
       </c>
     </row>
@@ -7783,12 +9099,12 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>1,498.90</t>
+          <t>1,495.50</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>▼ -1.00원 (-0.07%)</t>
+          <t>▼ -4.40원 (-0.29%)</t>
         </is>
       </c>
     </row>
@@ -7810,12 +9126,12 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>200.02</t>
+          <t>199.60</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>▼ -0.19원 (-0.10%)</t>
+          <t>▼ -0.62원 (-0.31%)</t>
         </is>
       </c>
     </row>
@@ -7921,27 +9237,27 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>112,687,000원</t>
+          <t>112,550,000원</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>+0.08%</t>
+          <t>-0.04%</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>112,124,000원</t>
+          <t>111,987,000원</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>121,702,000원</t>
+          <t>121,554,000원</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>110,580,000원</t>
+          <t>110,574,000원</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
@@ -7978,27 +9294,27 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>3,381,000원</t>
+          <t>3,380,000원</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>+0.00%</t>
+          <t>-0.03%</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>3,354,000원</t>
+          <t>3,353,000원</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>3,584,000원</t>
+          <t>3,583,000원</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>3,262,500원</t>
+          <t>3,261,500원</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
@@ -8013,7 +9329,7 @@
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>RSI 46.4로 단기 과매도 구간 진입, 기술적 반등 기대</t>
+          <t>RSI 46.5로 단기 과매도 구간 진입, 기술적 반등 기대</t>
         </is>
       </c>
     </row>
@@ -8312,7 +9628,7 @@
       </c>
       <c r="N3" s="3" t="inlineStr">
         <is>
-          <t>3Q26 실적은 연결기준 매출액 3,794억원(YoY+4</t>
+          <t>3Q26 실적은 연결기준 매출액 3,794억원(YoY+4)</t>
         </is>
       </c>
     </row>
@@ -8537,17 +9853,17 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>신한투자증권</t>
+          <t>하나증권</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>일진전기</t>
+          <t>삼성화재</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>가장 저평가된 전력기기</t>
+          <t>3Q26 Pre - 단기 실적보다 중요한 것은</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
@@ -8557,37 +9873,37 @@
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>매수</t>
+          <t>Buy</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>변압기 29년 수주 논의 및 전선 상반기 수주 급증 5월 시가총액 약 6.9조원 도달 이후 7월말 2.2조원까지 약 68% 하락. 전선업체들의 수주잔고총계 연간 증가율은 24년 25.4%, 25년 21.2%에서 26년 상반기에만 23.2% 증가. 변압기에 이은 전선 부문의 호황이 확대되는 것을 감안할 때 펀더멘털 문제가 아닌 수급 측면의 주가 하락으로 판단.</t>
+          <t>2026년 3분기 실적은 컨센서스 하회 전망 3분기 연결 지배순이익은 4,863억원으로 컨센서스(5,825억원)를 하회할 것으로 전망한다. 장기보험손익이 사업비 부담 확대로 예상대비 부한 가운데, 증시 부진과 금리 상승에 따른 투자손익 악화도 실적에 부담으로 작용할 것으로 예상한다. [보험손익] 보험손익은 4,006억원(YoY +8.6%, QoQ -27.5%)으로 추정한다.</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>2026-10-14_신한투자증권_일진전기_가장 저평가된 전력기기.pdf</t>
+          <t>2026-10-14_하나증권_삼성화재_3Q26 Pre - 단기 실적보다 중요한 것은.pdf</t>
         </is>
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>2,350.8십억원</t>
+          <t>-</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>252.8십억원</t>
+          <t>3,496십억원</t>
         </is>
       </c>
       <c r="L7" s="3" t="inlineStr">
         <is>
-          <t>2,595.2십억원</t>
+          <t>-</t>
         </is>
       </c>
       <c r="M7" s="3" t="inlineStr">
         <is>
-          <t>271.7십억원</t>
+          <t>4,566십억원</t>
         </is>
       </c>
       <c r="N7" s="3" t="inlineStr">
@@ -8607,17 +9923,17 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>DS투자증권</t>
+          <t>미래에셋증권</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>삼성중공업</t>
+          <t>휴젤</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>3Q26 Preview: 증익의 시작점</t>
+          <t>3Q26 Preview: 단기 실적 눈높이 조정</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -8632,37 +9948,37 @@
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>3Q26 Preview: 영업이익 3,791억원으로 컨센서스 소폭 상회 전망 26년 3분기 실적은 매출액 3.2조원(이하 YoY +22.8%), 영업이익 3,791억원(+59.2%, OPM 11.7%)으로 시장 컨센서스를 10% 상회할 전망이다. 조업일수는 하계 휴가와 추석 연휴 등으로 전분기 대비 9일 감소하나 글로벌 오퍼레이션과 2도크 재가동에 따른 매출 확대가 이를 상쇄하며 탑라인은 전분기 대비 소폭 성장할 것으로 예상된다. 수익성 또한 확대될 예정이다.</t>
+          <t>3분기 실적은 미국 판매체계 전환 영향으로 부진 휴젤의 3Q26 매출액은 1,009억원(-4.7% YoY), 영업이익 211억원(-55.5% YoY)으로 추정했다. 3Q26 영업이익은 미국 판매체계 전환 영향으로 전년 동기 대비 55.5% 감소할 것으로 보인다. 3분기는 미국 유통사 모델에서 CSO 모델로 전환하는 과정에서 일회성 매출 차감과 비용 증가가 동반되는 구간이었기 때문이다.</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>2026-10-14_DS투자증권_삼성중공업_3Q26 Preview 증익의 시작점.pdf</t>
+          <t>2026-10-14_미래에셋증권_휴젤_3Q26 Preview 단기 실적 눈높이 조정.pdf</t>
         </is>
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>10,650십억원</t>
+          <t>486십억원</t>
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>862십억원</t>
+          <t>174십억원</t>
         </is>
       </c>
       <c r="L8" s="3" t="inlineStr">
         <is>
-          <t>12,916십억원</t>
+          <t>657십억원</t>
         </is>
       </c>
       <c r="M8" s="3" t="inlineStr">
         <is>
-          <t>1,416십억원</t>
+          <t>272십억원</t>
         </is>
       </c>
       <c r="N8" s="3" t="inlineStr">
         <is>
-          <t>3Q26 Preview: 영업이익 3,791억원으로 컨센서스 소폭 상회 전망</t>
+          <t>3Q26 매출액은 1,009억원(-4)</t>
         </is>
       </c>
     </row>
@@ -8673,21 +9989,21 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>하나증권</t>
+          <t>신한투자증권</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>삼성화재</t>
+          <t>일진전기</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>3Q26 Pre - 단기 실적보다 중요한 것은</t>
+          <t>가장 저평가된 전력기기</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -8697,37 +10013,37 @@
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Buy</t>
+          <t>매수</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>2026년 3분기 실적은 컨센서스 하회 전망 3분기 연결 지배순이익은 4,863억원으로 컨센서스(5,825억원)를 하회할 것으로 전망한다. 장기보험손익이 사업비 부담 확대로 예상대비 부한 가운데, 증시 부진과 금리 상승에 따른 투자손익 악화도 실적에 부담으로 작용할 것으로 예상한다. [보험손익] 보험손익은 4,006억원(YoY +8.6%, QoQ -27.5%)으로 추정한다.</t>
+          <t>변압기 29년 수주 논의 및 전선 상반기 수주 급증 5월 시가총액 약 6.9조원 도달 이후 7월말 2.2조원까지 약 68% 하락. 전선업체들의 수주잔고총계 연간 증가율은 24년 25.4%, 25년 21.2%에서 26년 상반기에만 23.2% 증가. 변압기에 이은 전선 부문의 호황이 확대되는 것을 감안할 때 펀더멘털 문제가 아닌 수급 측면의 주가 하락으로 판단.</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>2026-10-14_하나증권_삼성화재_3Q26 Pre - 단기 실적보다 중요한 것은.pdf</t>
+          <t>2026-10-14_신한투자증권_일진전기_가장 저평가된 전력기기.pdf</t>
         </is>
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2,350.8십억원</t>
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>3,496십억원</t>
+          <t>252.8십억원</t>
         </is>
       </c>
       <c r="L9" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2,595.2십억원</t>
         </is>
       </c>
       <c r="M9" s="3" t="inlineStr">
         <is>
-          <t>4,566십억원</t>
+          <t>271.7십억원</t>
         </is>
       </c>
       <c r="N9" s="3" t="inlineStr">
@@ -8743,21 +10059,21 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>유안타증권</t>
+          <t>미래에셋증권</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>KT</t>
+          <t>효성중공업</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>바닥 통과, 성장 엔진 점화</t>
+          <t>중장기 카탈리스트는 여전히 유효</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
@@ -8767,42 +10083,42 @@
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>Buy</t>
+          <t>매수</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>3Q26 Preview: 일회성 제거시 영업이익 +3% YoY 3Q26 연결 영업수익은 7.1조원(-1.1% YoY), 영업이익은 5,350억원(-0.6% YoY)으로 시장 컨센서스(7.0조원, 5,442억원)에 부합할 전망이다. 부동산 관련 일회성 비용 제거시 영업이익은 +2.8% YoY 증가한 것으로 추정된다. 별도 영업이익은 3,400억원으로 전년과 유사한 수준이 예상된다.</t>
+          <t>3Q26 Preview: 매출 인식 지연으로 컨센서스 하회 전망 동사의 3Q26 매출액은 1조 7,438억원(+7.4% YoY, 컨센서스 8.7% 하회), 영업이익은 2,816억원(+16.2% YoY, 컨센서스 10.6% 하회)을 전망한다. 컨센서스 하회는 2분기에 이어 중공업 부문의 일부 출하 물량에 대한 매출 인식이 지연된 데 기인한다. 중동향 물량은 지정학적 리스크로 선적 확보에 차질이 발생하고 있으며, 미국향 물량은 고객사 변전설비 부지의 준비 지연으로 제품 인도가 이연되고 있는 것으로 파악된다.</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>2026-10-14_유안타증권_KT_바닥 통과, 성장 엔진 점화.pdf</t>
+          <t>2026-10-14_미래에셋증권_효성중공업_중장기 카탈리스트는 여전히 유효.pdf</t>
         </is>
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>27,426십억원</t>
+          <t>-</t>
         </is>
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>2,076십억원</t>
+          <t>-</t>
         </is>
       </c>
       <c r="L10" s="3" t="inlineStr">
         <is>
-          <t>27,905십억원</t>
+          <t>-</t>
         </is>
       </c>
       <c r="M10" s="3" t="inlineStr">
         <is>
-          <t>2,256십억원</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N10" s="3" t="inlineStr">
         <is>
-          <t>3Q26 Preview: 일회성 제거시 영업이익 +3% YoY</t>
+          <t>2026/2027 실적 성장세 및 기업가치 재평가 전망</t>
         </is>
       </c>
     </row>
@@ -8813,21 +10129,21 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>미래에셋증권</t>
+          <t>DS투자증권</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>휴젤</t>
+          <t>삼성중공업</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>3Q26 Preview: 단기 실적 눈높이 조정</t>
+          <t>3Q26 Preview: 증익의 시작점</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
@@ -8842,37 +10158,37 @@
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>3분기 실적은 미국 판매체계 전환 영향으로 부진 휴젤의 3Q26 매출액은 1,009억원(-4.7% YoY), 영업이익 211억원(-55.5% YoY)으로 추정했다. 3Q26 영업이익은 미국 판매체계 전환 영향으로 전년 동기 대비 55.5% 감소할 것으로 보인다. 3분기는 미국 유통사 모델에서 CSO 모델로 전환하는 과정에서 일회성 매출 차감과 비용 증가가 동반되는 구간이었기 때문이다.</t>
+          <t>3Q26 Preview: 영업이익 3,791억원으로 컨센서스 소폭 상회 전망 26년 3분기 실적은 매출액 3.2조원(이하 YoY +22.8%), 영업이익 3,791억원(+59.2%, OPM 11.7%)으로 시장 컨센서스를 10% 상회할 전망이다. 조업일수는 하계 휴가와 추석 연휴 등으로 전분기 대비 9일 감소하나 글로벌 오퍼레이션과 2도크 재가동에 따른 매출 확대가 이를 상쇄하며 탑라인은 전분기 대비 소폭 성장할 것으로 예상된다. 수익성 또한 확대될 예정이다.</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>2026-10-14_미래에셋증권_휴젤_3Q26 Preview 단기 실적 눈높이 조정.pdf</t>
+          <t>2026-10-14_DS투자증권_삼성중공업_3Q26 Preview 증익의 시작점.pdf</t>
         </is>
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>486십억원</t>
+          <t>10,650십억원</t>
         </is>
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>174십억원</t>
+          <t>862십억원</t>
         </is>
       </c>
       <c r="L11" s="3" t="inlineStr">
         <is>
-          <t>657십억원</t>
+          <t>12,916십억원</t>
         </is>
       </c>
       <c r="M11" s="3" t="inlineStr">
         <is>
-          <t>272십억원</t>
+          <t>1,416십억원</t>
         </is>
       </c>
       <c r="N11" s="3" t="inlineStr">
         <is>
-          <t>3Q26 매출액은 1,009억원(-4</t>
+          <t>3Q26 Preview: 영업이익 3,791억원으로 컨센서스 소폭 상회 전망</t>
         </is>
       </c>
     </row>
@@ -8887,16 +10203,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L15"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="21" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="25" customWidth="1" min="5" max="5"/>
-    <col width="25" customWidth="1" min="6" max="6"/>
-    <col width="25" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="32" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
@@ -9076,7 +10392,7 @@
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>+1.2%</t>
+          <t>+1.5%</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
@@ -9138,7 +10454,7 @@
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>+2.2%</t>
+          <t>+1.9%</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
@@ -9200,7 +10516,7 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>+2.4%</t>
+          <t>+2.3%</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
@@ -9262,7 +10578,7 @@
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>+1.0%</t>
+          <t>+1.4%</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
@@ -9324,7 +10640,7 @@
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>+4.1%</t>
+          <t>+4.4%</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
@@ -9351,32 +10667,32 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>삼성전자</t>
+          <t>한미약품</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>005930.KS</t>
+          <t>128940.KS</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>231,500원</t>
+          <t>404,500원</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>229,000원</t>
+          <t>400,500원</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>256,500원</t>
+          <t>483,500원</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>223,500원</t>
+          <t>390,500원</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
@@ -9386,12 +10702,12 @@
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>+1.6%</t>
+          <t>+1.0%</t>
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>232,750원</t>
+          <t>404,500원</t>
         </is>
       </c>
       <c r="L8" s="3" t="inlineStr">
@@ -9413,32 +10729,32 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>엔비디아 (NVIDIA)</t>
+          <t>KT</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>030200.KS</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>$228.52 (약 305,908원)</t>
+          <t>49,900원</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>$228.52 (약 305,908원)</t>
+          <t>49,400원</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>$246.80 (약 330,380원)</t>
+          <t>52,900원</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>$219.38</t>
+          <t>48,200원</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
@@ -9448,12 +10764,12 @@
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>+0.0%</t>
+          <t>+1.0%</t>
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>$228.52</t>
+          <t>49,900원</t>
         </is>
       </c>
       <c r="L9" s="3" t="inlineStr">
@@ -9475,32 +10791,32 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>애플 (Apple)</t>
+          <t>SK텔레콤</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>AAPL</t>
+          <t>017670.KS</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>$341.27 (약 456,841원)</t>
+          <t>81,900원</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>$341.27 (약 456,841원)</t>
+          <t>81,100원</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>$368.57 (약 493,388원)</t>
+          <t>86,800원</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>$327.62</t>
+          <t>79,000원</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr">
@@ -9510,12 +10826,12 @@
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>+0.0%</t>
+          <t>+1.0%</t>
         </is>
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>$341.27</t>
+          <t>81,900원</t>
         </is>
       </c>
       <c r="L10" s="3" t="inlineStr">
@@ -9537,32 +10853,32 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>한미약품</t>
+          <t>삼성중공업</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>128940.KS</t>
+          <t>010140.KS</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>400,000원</t>
+          <t>19,000원</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>396,000원</t>
+          <t>18,800원</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>483,000원</t>
+          <t>20,100원</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>386,000원</t>
+          <t>18,300원</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
@@ -9572,263 +10888,15 @@
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>+1.8%</t>
+          <t>+0.8%</t>
         </is>
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>403,000원</t>
+          <t>18,950원</t>
         </is>
       </c>
       <c r="L11" s="3" t="inlineStr">
-        <is>
-          <t>1일차</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>KT</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>030200.KS</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>50,000원</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>49,500원</t>
-        </is>
-      </c>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t>52,900원</t>
-        </is>
-      </c>
-      <c r="H12" s="3" t="inlineStr">
-        <is>
-          <t>48,200원</t>
-        </is>
-      </c>
-      <c r="I12" s="3" t="inlineStr">
-        <is>
-          <t>⏳ 목표가 추적 중 (신규 진입)</t>
-        </is>
-      </c>
-      <c r="J12" s="3" t="inlineStr">
-        <is>
-          <t>+1.4%</t>
-        </is>
-      </c>
-      <c r="K12" s="3" t="inlineStr">
-        <is>
-          <t>50,200원</t>
-        </is>
-      </c>
-      <c r="L12" s="3" t="inlineStr">
-        <is>
-          <t>1일차</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>SK텔레콤</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>017670.KS</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>81,600원</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>80,800원</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>86,500원</t>
-        </is>
-      </c>
-      <c r="H13" s="3" t="inlineStr">
-        <is>
-          <t>78,700원</t>
-        </is>
-      </c>
-      <c r="I13" s="3" t="inlineStr">
-        <is>
-          <t>⏳ 목표가 추적 중 (신규 진입)</t>
-        </is>
-      </c>
-      <c r="J13" s="3" t="inlineStr">
-        <is>
-          <t>+1.4%</t>
-        </is>
-      </c>
-      <c r="K13" s="3" t="inlineStr">
-        <is>
-          <t>81,900원</t>
-        </is>
-      </c>
-      <c r="L13" s="3" t="inlineStr">
-        <is>
-          <t>1일차</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>삼성중공업</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>010140.KS</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr">
-        <is>
-          <t>18,900원</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>18,700원</t>
-        </is>
-      </c>
-      <c r="G14" s="3" t="inlineStr">
-        <is>
-          <t>20,000원</t>
-        </is>
-      </c>
-      <c r="H14" s="3" t="inlineStr">
-        <is>
-          <t>18,200원</t>
-        </is>
-      </c>
-      <c r="I14" s="3" t="inlineStr">
-        <is>
-          <t>⏳ 목표가 추적 중 (신규 진입)</t>
-        </is>
-      </c>
-      <c r="J14" s="3" t="inlineStr">
-        <is>
-          <t>+1.2%</t>
-        </is>
-      </c>
-      <c r="K14" s="3" t="inlineStr">
-        <is>
-          <t>18,920원</t>
-        </is>
-      </c>
-      <c r="L14" s="3" t="inlineStr">
-        <is>
-          <t>1일차</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>삼성화재</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>000810.KS</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr">
-        <is>
-          <t>583,000원</t>
-        </is>
-      </c>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>577,000원</t>
-        </is>
-      </c>
-      <c r="G15" s="3" t="inlineStr">
-        <is>
-          <t>629,500원</t>
-        </is>
-      </c>
-      <c r="H15" s="3" t="inlineStr">
-        <is>
-          <t>562,500원</t>
-        </is>
-      </c>
-      <c r="I15" s="3" t="inlineStr">
-        <is>
-          <t>⏳ 목표가 추적 중 (신규 진입)</t>
-        </is>
-      </c>
-      <c r="J15" s="3" t="inlineStr">
-        <is>
-          <t>+0.9%</t>
-        </is>
-      </c>
-      <c r="K15" s="3" t="inlineStr">
-        <is>
-          <t>582,000원</t>
-        </is>
-      </c>
-      <c r="L15" s="3" t="inlineStr">
         <is>
           <t>1일차</t>
         </is>
@@ -9854,7 +10922,7 @@
     <col width="19" customWidth="1" min="4" max="4"/>
     <col width="65" customWidth="1" min="5" max="5"/>
     <col width="65" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
     <col width="32" customWidth="1" min="8" max="8"/>
     <col width="53" customWidth="1" min="9" max="9"/>
   </cols>
@@ -9969,10 +11037,14 @@
           <t>자사주 취득</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr"/>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>엘컴텍</t>
+        </is>
+      </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>“역시 주주환원은 뒷전입니까”…코스피 자사주 매입, 삼전닉스 뺐더니 줄었다</t>
+          <t>엘컴텍, 20억원 규모 자사주 취득 결정</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
@@ -9982,17 +11054,17 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>매일경제 마켓</t>
+          <t>데이터투자</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>Sun, 11 Oct 2026 11:51:10 GMT</t>
+          <t>Tue, 13 Oct 2026 07:22:52 GMT</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiUkFVX3lxTE0zXzFYa0xGekFCVWtnODd6QVRIRmp1MnFLcXhBWWVadVdXQWZaY3lGcGg3WUl1dzY4M1R1cTBWV1h1a0JBbXdGV3Y0aC1KV25lRmc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMickFVX3lxTE13UXpQT2FyUjBQSkpSdFNtQVpJOHFGMExaeDFtajBra1h5dHl5S2dMbUV5TUdmMzFYZkF6b1RmSTd0TVk1NUZCOGN1Y1pWS3d1Rk50WmRUS19XZkJISzdJX3k1YXpPU2V3X3FhNkloOWs1QQ?oc=5</t>
         </is>
       </c>
     </row>
@@ -10012,10 +11084,14 @@
           <t>자사주 취득</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr"/>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>더핑크퐁컴퍼니</t>
+        </is>
+      </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>데스트라 멀티 대체 투자 펀드, 자사주 매입 프로그램 도입·월 배당금 주당 0.115달러로 인상</t>
+          <t>더핑크퐁컴퍼니, 50억원 규모 자사주 취득 신탁계약 해지 결정</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -10030,12 +11106,12 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 19:52:27 GMT</t>
+          <t>Tue, 13 Oct 2026 05:43:38 GMT</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMic0FVX3lxTE1lemt2YTFaYUFFeVI4cVJZbjFYOHpWLVJmNTUxN3huQlRtYUVHYXplTUpvQktSZFdKenhkMl9PYXlNci1RbHNtTUdQdXgxelpjaEJVbWNjVmFndWFiaV9KZFAxd2ozbVZXVUd4MHFPNlZYT0U?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMic0FVX3lxTE1MVmRGS1NqcEJobXNpM01fNTlJbV9MeFZUeXBTVktGWV9XOWFlMHFET09BeW1rQ1RJdzVCR0I1OXM1UkpxM3Nnazk4RnBPbC1EaGFxM0FpVVpqYzZPRnlGb0plTEwyYmZDSXJXNW8yYmh5M0k?oc=5</t>
         </is>
       </c>
     </row>
@@ -10055,10 +11131,14 @@
           <t>자사주 취득</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr"/>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>메디앙스</t>
+        </is>
+      </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>AZZ, 연간 실적 가이던스 상향…2000만 달러 규모 자사주 매입</t>
+          <t>메디앙스, 10억원 규모 자사주 취득 결정</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -10073,12 +11153,12 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 20:20:27 GMT</t>
+          <t>Mon, 12 Oct 2026 05:39:56 GMT</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMickFVX3lxTE9QR3MyNXVOWndYaXJsdTF5Z2NaQnlGUVRFanBlUjhmN1U0TDNCMXNUZ2RrNTRselZhSGtXTW9YMUJGVWtvSTdDdFhCVVN6ZTVCcTZ0WnlkeUNsRTZlMGZBXzJnSnkxZ1Z3NjI5MlF0N0N3dw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMic0FVX3lxTE1TRmxBdndpdk9HTXZRTzdxNF8wSWpxQklLcDBRQks1TmxUSm4xRU9zVzRCSkxLZ3RUYy1JbS1vZXhhSnRxMXRJZnNGVHJLdkwyZzNTZTlLUWlCb0xkQUpnSWtnVURLcExLaGtWOTFMcnV6cGM?oc=5</t>
         </is>
       </c>
     </row>
@@ -10090,42 +11170,42 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>💎 자사주 취득 (주가 부양)</t>
+          <t>🏛️ 대주주/임원 장내매수 (책임경영)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>자사주 취득</t>
+          <t>내부자 매수</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>트러스트</t>
+          <t>회장</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>선라이즈 리얼티 트러스트, 2000만 달러 자사주 매입 프로그램 승인</t>
+          <t>원종석 신영증권 회장, 5거래일간 자사주 30억 장내 매수</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>기업 자금 투입으로 유통 물량 흡수 및 강력한 주가 바닥 지지 신호</t>
+          <t>내부 사정을 가장 잘 아는 경영진의 직접 매수로 기업가치 저평가 방증</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>데이터투자</t>
+          <t>더팩트</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 12:13:59 GMT</t>
+          <t>Thu, 11 Jun 2026 07:00:00 GMT</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMic0FVX3lxTE1fQmV2cFR2OFA5M1B6UXE3NF83TmRrd2lGSE1QelFpZWFMUDhZT1lHWHJYUnFBcmtKNUJmRWlwRTU3ME1ydno4cmpDMnpWMTF0Q09HQ0dmOVVubFFIYXNWZ1FhWlRZaEp3dk4xcHd2TmdFQ00?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTE5tYTBhV0h3WkQzbG5SbklZMW16enV2UWxnZHlkYzFjYmhYaVNQclkyYWxQM1VDTjdWYVhuMHNXRklUMGsyT2F0ck5EZkhSWGlUX2I2MmxjUENKUdIBVEFVX3lxTE1RcVhPeC1tU2FoTThuWHFyMnJFa2VSRm91eUs3dFQ5YmU2Y25BVzF2cHFycEN5UmYxTDdxWGZBM2p4ZVFFX1NwblFIMWU5cGEtcGxqZQ?oc=5</t>
         </is>
       </c>
     </row>
@@ -10137,42 +11217,42 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>💎 자사주 취득 (주가 부양)</t>
+          <t>📈 대규모 단일판매·공급계약</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>자사주 취득</t>
+          <t>대규모 수주</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>아웃렛</t>
+          <t>스피어</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>올리스 바겐 아웃렛, 5억 달러 규모 신규 자사주 매입 승인</t>
+          <t>[속보] 스피어, 285억원 규모 특수합금 공급계약…지난해 매출액 대비 29.84%</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>기업 자금 투입으로 유통 물량 흡수 및 강력한 주가 바닥 지지 신호</t>
+          <t>매출액 직결 확정 계약으로 향후 분기 실적 퀀텀점프 기대</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>데이터투자</t>
+          <t>CBC뉴스</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 11:09:56 GMT</t>
+          <t>Wed, 14 Oct 2026 05:49:26 GMT</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMic0FVX3lxTE5nZklvLUJYTTRmYUtlSnZGdWgzaE9aeExETGVnWDF1dXpLTGVMWWpSSEdodW1WMkprQW5oeEMxV0xtM0pIcndVZDVhVk5UWnIwcFNyMlI2X0hjb2M3UHBXME5sRGFCN0pYdDJWTEstSmpqVE0?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiaEFVX3lxTFBVR0NZZ25tdjlPRnB3TFQ4UXpFNVZaTWJPaVBfWWZhRUVVWnpiRk5fWDFJM2staGx2NEhsZ1pHWVRINjBDZng3bFBZMGtQeUdWWi0xN2xROWU3ejNMNHJObmpuSjQ2TTJy?oc=5</t>
         </is>
       </c>
     </row>
@@ -10184,42 +11264,42 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>💎 자사주 취득 (주가 부양)</t>
+          <t>📈 대규모 단일판매·공급계약</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>자사주 취득</t>
+          <t>대규모 수주</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>엘컴텍</t>
+          <t>우진아이엔에스</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>엘컴텍, 20억원 규모 자사주 취득 결정</t>
+          <t>우진아이엔에스, 144억원 규모 공급계약 체결… 매출의 8.74%</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>기업 자금 투입으로 유통 물량 흡수 및 강력한 주가 바닥 지지 신호</t>
+          <t>매출액 직결 확정 계약으로 향후 분기 실적 퀀텀점프 기대</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>데이터투자</t>
+          <t>CEO경제신문</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 07:22:52 GMT</t>
+          <t>Wed, 14 Oct 2026 01:10:42 GMT</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMickFVX3lxTE13UXpQT2FyUjBQSkpSdFNtQVpJOHFGMExaeDFtajBra1h5dHl5S2dMbUV5TUdmMzFYZkF6b1RmSTd0TVk1NUZCOGN1Y1pWS3d1Rk50WmRUS19XZkJISzdJX3k1YXpPU2V3X3FhNkloOWs1QQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMibEFVX3lxTE9OMkc3SVNncl9rSWxrMjZmMFE5ZGJTaGxrem9zb2t3ZzlGYWFhcFo0dHNNMVlWa0tuVE1zeG9MOTlKRThmVS1rR3Fqb3pVNUJjQUs3MElsVFNqaHozeExqNllLbERJbHdKT0RnUA?oc=5</t>
         </is>
       </c>
     </row>
@@ -10231,38 +11311,42 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>🏛️ 대주주/임원 장내매수 (책임경영)</t>
+          <t>📈 대규모 단일판매·공급계약</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>내부자 매수</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr"/>
+          <t>대규모 수주</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>LS머트리얼즈</t>
+        </is>
+      </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>사이먼 쿠케스 박사 측, 페데브코 보통주 14만 7070주 장내 매수…지분율 34.2%로 확대</t>
+          <t>[공시 Pick] LS머트리얼즈, 美 연료전지용 UC 공급계약에 주가 강세…증시 급락 속 ‘역주행’</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>내부 사정을 가장 잘 아는 경영진의 직접 매수로 기업가치 저평가 방증</t>
+          <t>매출액 직결 확정 계약으로 향후 분기 실적 퀀텀점프 기대</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>데이터투자</t>
+          <t>뉴스투데이</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>Tue, 13 Oct 2026 12:14:51 GMT</t>
+          <t>Tue, 13 Oct 2026 01:48:00 GMT</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMic0FVX3lxTE8wVldLdklzOFE4cnp4RmlPLVJ2LVdveDVQTUV2UjhyTjh1NVhIMG5maUxkelFnUkhEV1ZxdGY2empxS252cDk5QW9ua2EtZ3lRUl94bVA5UEg4b09SZXdMcUk5UnlrbHRpZGU4V1VNYTdzNjQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiXkFVX3lxTFBQTWoxNDVLVWtBTXVoS3MtWmFpd1UwMG9FYkVLM0EtcWhTbThJZFVkOWdVekxQMEpNR2ZMTklDQTZHdWpZU3BJSkJpTUQ2TnNVcW8weHFGM1pEVnBqNlE?oc=5</t>
         </is>
       </c>
     </row>
@@ -10498,14 +11582,14 @@
     <col width="25" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="65" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
     <col width="65" customWidth="1" min="6" max="6"/>
     <col width="65" customWidth="1" min="7" max="7"/>
     <col width="65" customWidth="1" min="8" max="8"/>
     <col width="65" customWidth="1" min="9" max="9"/>
     <col width="65" customWidth="1" min="10" max="10"/>
     <col width="65" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
     <col width="53" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
@@ -10594,32 +11678,32 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>🌐 [경제·사회 심층 리포트] 카카오의 숨겨진 배경과 구조적 쟁점</t>
+          <t>🌐 [경제·사회 심층 리포트] 반도체대전의 숨겨진 배경과 구조적 쟁점</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>카카오</t>
+          <t>반도체대전</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>단순 뉴스 헤드라인을 넘어선 전후 맥락: '카카오' 이슈가 촉발된 진짜 배경과 이해관계자들의 득실 계산을 분석합니다.</t>
+          <t>단순 뉴스 헤드라인을 넘어선 전후 맥락: '반도체대전' 이슈가 촉발된 진짜 배경과 이해관계자들의 득실 계산을 분석합니다.</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>오늘 주요 언론을 통해 집중 조명된 핵심 사안은 바로 **[카카오, ‘모두의 AI’ 연내 공개 예정…월 이용자 500만 명 목표]** 입니다.&lt;br&gt;• &lt;b&gt;핵심 현황:&lt;/b&gt; 카카오, ‘모두의 AI’ 연내 공개 예정월 이용자 500만 명 목표 KBS 뉴스카카오그룹, 인적분할 앞두고 주요 계열사 CEO 함께 모여 ‘첫 공동 IR’ 개최 카카오연말 출시 ‘모두의 AI’“카톡 익숙함. 활용할 것” 마켓 카카오, 웹툰·음원·카카오T에 스테이블코인 결제 연동소설 원작 AI 애니 제작도 전자신문카톡에 “메시지 정리, 답장 보내줘” 말하면 AI비서가 척척.&lt;br&gt;• &lt;b&gt;왜 중요한가:&lt;/b&gt; 단순한 단발성 소식이 아니라 정부 정책, 규제 환경, 기업들의 실질적 손익과 직결되어 시장 전반에 큰 파장을 일으키고 있기 때문입니다.</t>
+          <t>오늘 주요 언론을 통해 집중 조명된 핵심 사안은 바로 **[삼성전자 '반도체대전' 참가‥HBM4E 등 AI 반도체 기술 선보인다]** 입니다.&lt;br&gt;• &lt;b&gt;핵심 현황:&lt;/b&gt; 삼성전자 '반도체대전' 참가‥HBM4E 등 AI 반도체 기술 선보인다.&lt;br&gt;• &lt;b&gt;왜 중요한가:&lt;/b&gt; 단순한 단발성 소식이 아니라 정부 정책, 규제 환경, 기업들의 실질적 손익과 직결되어 시장 전반에 큰 파장을 일으키고 있기 때문입니다.</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>이 문제는 오늘 갑자기 발생한 사안이 아니라, 과거부터 축적되어 온 구조적 원인이 있습니다.&lt;br&gt;• &lt;b&gt;과거 배경:&lt;/b&gt; 피지컬 AI 시동 건 카카오모빌리티…상생재단서 '카카오' 뗀 이유는? 알림음과 배경 음악을 구분하는 카카오 라인 블록 체인 사운드 안내 Calgary Roughnecks.&lt;br&gt;• &lt;b&gt;결정적 계기:&lt;/b&gt; 잠재되어 있던 제도적 갈등과 시장 환경의 변화가 맞물리면서, 이번 계기를 통해 본격적으로 수면 위로 표출되었습니다.</t>
+          <t>이 문제는 오늘 갑자기 발생한 사안이 아니라, 과거부터 축적되어 온 구조적 원인이 있습니다.&lt;br&gt;• &lt;b&gt;과거 배경:&lt;/b&gt; 신성이엔지, 반도체대전서 클린룸 기술 공개...해외시장 공략 확대 헬로티. KTC, ‘제28회 반도체대전’ 참가… 시스템반도체·미래차 전장부품 신뢰성 검증 인프라 공개 기계신문.&lt;br&gt;• &lt;b&gt;결정적 계기:&lt;/b&gt; 잠재되어 있던 제도적 갈등과 시장 환경의 변화가 맞물리면서, 이번 계기를 통해 본격적으로 수면 위로 표출되었습니다.</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>겉으로 보이는 명분 뒤에는 각 주체들의 아주 명확한 '실질적 손익 계산'이 숨어 있습니다.&lt;br&gt;• &lt;b&gt;이해관계 분석:&lt;/b&gt; 카카오 AI, 올해 사회경제적 가치 약 5500억 창출 전망 서울경제. 카카오 AI 사회경제적 가치 연 5506억원…2030년 최대 1.8조원 전망 지디넷코리아.&lt;br&gt;• &lt;b&gt;핵심 구조:&lt;/b&gt; 규제 당국은 시장 통제력과 정책 주도권을 강화하려 하고, 관련 기업들은 비용 부담을 줄이고 수익성을 지키기 위해 치열한 수싸움을 벌이고 있는 구도입니다.</t>
+          <t>겉으로 보이는 명분 뒤에는 각 주체들의 아주 명확한 '실질적 손익 계산'이 숨어 있습니다.&lt;br&gt;• &lt;b&gt;이해관계 분석:&lt;/b&gt; 반도체대전, 기술 전시 넘어 채용까지…삼성·SK하이닉스 등 300개사 집결 매일일보. ② 반도체 쏠림이 위험하다고?…“올해 코스피 이익 증가분 90%가 반도체" - 조선비즈 Chosunbiz.&lt;br&gt;• &lt;b&gt;핵심 구조:&lt;/b&gt; 규제 당국은 시장 통제력과 정책 주도권을 강화하려 하고, 관련 기업들은 비용 부담을 줄이고 수익성을 지키기 위해 치열한 수싸움을 벌이고 있는 구도입니다.</t>
         </is>
       </c>
       <c r="J2" s="3" t="inlineStr">
@@ -10629,17 +11713,17 @@
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>📌 **구조적 수혜(Structural Beneficiary)**: 단기적 유행이 아닌, 국가 정책이나 글로벌 지정학적 공급망 재편에 따라 수년간 장기적인 성장을 누리게 되는 산업 생태계 현상입니다.</t>
+          <t>📌 **HBM(고대역폭 메모리)**: D램을 수직으로 높게 쌓아 데이터 처리 속도를 획기적으로 끌어올린 인공지능(AI) 그래픽처리장치(GPU) 필수 탑재 메모리입니다.</t>
         </is>
       </c>
       <c r="L2" s="3" t="inlineStr">
         <is>
-          <t>KBS 뉴스</t>
+          <t>MBC 뉴스</t>
         </is>
       </c>
       <c r="M2" s="3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE43NnU3MlhmZWZkcEdnRU1abkNDcHdIdG85YU9NZVBqVF90N3BXTHFCVlJIbDZQbkg3RGR5NWltZ29IaXNWNkdIWm1aYzBmLU4wbnVfd1hhVnlwdVk?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMidEFVX3lxTE9QLWl1VjBqYUpRc3BydE96Y1c1N2JQNUJ4TTdmazF6NmRlb01JaHpYa3NSX2llQkRyUFU3S1JYOUxVbkp3N3VMOUlITWFoUEk2YlpkTDdmUzE3MUJwbG9LclBOQzNYNzkzZnJLcDdveDZKMkFG0gF0QVVfeXFMUG52cWpIVDZJZFNKelIwTmczTFJmVUtRTjVBYlI0ZEJtNkJYWWVYaWVRR1plUFR0M3pQUVZUdmF6RDJRNm5qWjlHNUFzNlZ0d2N6TV8tNm1RUldCMVh3b3l4eWhkdlBUOGMtSVZwMm5YUTlGUzg?oc=5</t>
         </is>
       </c>
     </row>
@@ -10661,32 +11745,32 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>🔥 [트렌드 &amp; 소비 인사이트] 블루 아카이브 열풍의 배경과 소비 심리 분석</t>
+          <t>🔥 [트렌드 &amp; 소비 인사이트] 시오라 열풍의 배경과 소비 심리 분석</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>블루 아카이브</t>
+          <t>시오라</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>요즘 왜 난리일까? '블루 아카이브' 품절 대란과 오픈런 이면에 숨은 소비 심리와 바이럴 구조를 짚어봅니다.</t>
+          <t>요즘 왜 난리일까? '시오라' 품절 대란과 오픈런 이면에 숨은 소비 심리와 바이럴 구조를 짚어봅니다.</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>지금 거리와 SNS에서 소비자들이 가장 열광하고 있는 화제의 중심은 단연 **[GS25, '블루 아카이브'와 3차 협업…전국 팝업스토어도 운영]** 입니다.&lt;br&gt;• &lt;b&gt;트렌드 현황:&lt;/b&gt; GS25, '블루 아카이브'와 3차 협업…전국 팝업스토어도 운영 매일경제 마켓.&lt;br&gt;• &lt;b&gt;열풍의 온도:&lt;/b&gt; 매장 문이 열리기 전부터 줄을 서는 '오픈런'과 온라인 품절 사태가 잇따르며, 단순한 유행을 넘어 하나의 강력한 문화적 현상으로 자리 잡았습니다.</t>
+          <t>지금 거리와 SNS에서 소비자들이 가장 열광하고 있는 화제의 중심은 단연 **[시오라, 성수동 팝업스토어 오픈…슬로우에이징 스킨케어 선보여]** 입니다.&lt;br&gt;• &lt;b&gt;트렌드 현황:&lt;/b&gt; 시오라, 성수동 팝업스토어 오픈…슬로우에이징 스킨케어 선보여 중앙일보.&lt;br&gt;• &lt;b&gt;열풍의 온도:&lt;/b&gt; 매장 문이 열리기 전부터 줄을 서는 '오픈런'과 온라인 품절 사태가 잇따르며, 단순한 유행을 넘어 하나의 강력한 문화적 현상으로 자리 잡았습니다.</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>이 유행은 과연 어디서부터 시작되었을까요? 시작점을 추적해 보면 아주 흥미로운 바이럴 계기가 있습니다.&lt;br&gt;• &lt;b&gt;시작 비화:&lt;/b&gt; 알림음과 배경 음악을 구분하는 블루아카이브 경마 사운드 안내 Calgary Roughnecks. 수영복 입은 문주님, 블루 아카이브에 '람과천청' 업데이트 월요신문.&lt;br&gt;• &lt;b&gt;확산 과정:&lt;/b&gt; 초기에는 특정 매니아층 사이의 호기심으로 시작되었으나, 틱톡·릴스 등 숏폼 영상 알고리즘을 타며 '나도 경험해봐야 한다'는 대중적 열풍으로 급격히 번져나갔습니다.</t>
+          <t>이 유행은 과연 어디서부터 시작되었을까요? 시작점을 추적해 보면 아주 흥미로운 바이럴 계기가 있습니다.&lt;br&gt;• &lt;b&gt;시작 비화:&lt;/b&gt; 호남오페라단 '달하 비취시오라, 정읍사' - 지역사 예술적 부각, 감동 무대 전북일보 인터넷신문. ‘달하, 비취시오라’와 창작오페라를 위한 제언 서울문화투데이.&lt;br&gt;• &lt;b&gt;확산 과정:&lt;/b&gt; 초기에는 특정 매니아층 사이의 호기심으로 시작되었으나, 틱톡·릴스 등 숏폼 영상 알고리즘을 타며 '나도 경험해봐야 한다'는 대중적 열풍으로 급격히 번져나갔습니다.</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>소비자들이 기꺼이 시간과 비용을 들여 줄을 서는 심리적 이유를 쉽게 풀어보았습니다.&lt;br&gt;• &lt;b&gt;소비 심리:&lt;/b&gt; 넥슨 '블루 아카이브' 모집 BM 개편한다, 4분기 글로벌 적용 게임뷰. 생성형 AI와의 공존 ③ 넥슨게임즈 김용하 본부장 게임메카.&lt;br&gt;• &lt;b&gt;심리적 기제:&lt;/b&gt; 단순히 제품의 기능 때문이 아니라, '희소한 트렌드를 남들보다 빠르게 경험하고 인증했다'는 심리적 만족감과 소속감(디토 소비 및 포모 심리)이 지갑을 열게 만드는 핵심 동기입니다.</t>
+          <t>소비자들이 기꺼이 시간과 비용을 들여 줄을 서는 심리적 이유를 쉽게 풀어보았습니다.&lt;br&gt;• &lt;b&gt;소비 심리:&lt;/b&gt; 시오라, 성수동 팝업 통해 오프라인 시장 공략 세계비즈.&lt;br&gt;• &lt;b&gt;심리적 기제:&lt;/b&gt; 단순히 제품의 기능 때문이 아니라, '희소한 트렌드를 남들보다 빠르게 경험하고 인증했다'는 심리적 만족감과 소속감(디토 소비 및 포모 심리)이 지갑을 열게 만드는 핵심 동기입니다.</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">
@@ -10701,12 +11785,12 @@
       </c>
       <c r="L3" s="3" t="inlineStr">
         <is>
-          <t>매일경제 마켓</t>
+          <t>중앙일보</t>
         </is>
       </c>
       <c r="M3" s="3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiUkFVX3lxTE5oRlFmSDNxbVRUaEctLWp3SHVvbEtGeFRFajBNUndReGo0QzZNdFBacG1la0ZGR3BScW5qb091eW4xclJOQi1vYk9DVjM4NVd6cnc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiVkFVX3lxTE4wV1Y5MTVqUTFlVHpha3BmY201YjVydFgydlFybzU3VTh0MmxneTJ6TGwwT1dWVURpRjFaaVFZWjNSYVU1ZEx3UDRmSTM3VWhJTVN0WWd3?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>